<commit_message>
Add MikroTik shipment-geography analysis with Comtrade data and regional entry priorities
- MikroTik出货地分析与区域切入优先级_2026-09.md: re-derives MikroTik's
  export geography from UN Comtrade (Latvia HS 851762, 2024, 60 partners,
  90.9% coverage), corrects the Claude-chat estimates (LatAm/N. America
  overstated, UAE/HK hubs missed), adds US-vs-EU tariff landed-cost
  comparison and a country priority list (T1/T2/T3) with per-country
  playbooks mapped to the four customer types
- Workbook: new sheets 'MikroTik出口地(Comtrade2024)' (country table +
  region SUMIF summary) and '落地价与关税' (editable landed-cost calculator)

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -9,9 +9,11 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="替代对照表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MikroTik关键事实(实测)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SmartByte关键SKU" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原Excel数据修正" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MikroTik出口地(Comtrade2024)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="落地价与关税" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MikroTik关键事实(实测)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SmartByte关键SKU" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原Excel数据修正" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +22,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="+0%;-0%"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -37,7 +42,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,6 +52,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -62,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -75,6 +85,23 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -513,6 +540,13 @@
       <c r="A7" t="inlineStr">
         <is>
           <t>SmartByte = 价格表 2026.09.01–2026.12.30 未税 RMB 进价（for Simon）。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MikroTik 出口地数据 = UN Comtrade 2024（见 'MikroTik出口地(Comtrade2024)' sheet）；MikroTik 营收 2023/2024/2025 = €401.6M / €326.7M / €344.6M（Lursoft）。</t>
         </is>
       </c>
     </row>
@@ -1753,6 +1787,2364 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G78"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="45" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>说明：UN Comtrade，Reporter=Latvia(428)，HS 851762（交换/路由设备），Export，2024，FOB USD。MikroTik 占拉脱维亚该税号出口 3/4 以上，可视为 MikroTik 分销商进货地图。全球合计 USD 422,324,814。</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>排名</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>国家/地区</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>M49 代码</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>区域</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>出口额 USD</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>占全球 %</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>842</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>北美</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>50994438</v>
+      </c>
+      <c r="F3" s="8">
+        <f>E3/422324814</f>
+        <v/>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>对华关税约 37.5%（2026-09）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>阿联酋(转口枢纽)</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>784</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>中东/土耳其</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>43018484</v>
+      </c>
+      <c r="F4" s="8">
+        <f>E4/422324814</f>
+        <v/>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>转口枢纽→中东/非洲/南亚</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>616</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>34368342</v>
+      </c>
+      <c r="F5" s="8">
+        <f>E5/422324814</f>
+        <v/>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>欧洲第一 MikroTik 国</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>立陶宛(波罗的海分销枢纽)</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>440</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>32525290</v>
+      </c>
+      <c r="F6" s="8">
+        <f>E6/422324814</f>
+        <v/>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>波罗的海分销枢纽</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>203</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>21822977</v>
+      </c>
+      <c r="F7" s="8">
+        <f>E7/422324814</f>
+        <v/>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>WISP 密度极高</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>276</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>16002618</v>
+      </c>
+      <c r="F8" s="8">
+        <f>E8/422324814</f>
+        <v/>
+      </c>
+      <c r="G8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>中国香港(转口枢纽)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>344</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>15962714</v>
+      </c>
+      <c r="F9" s="8">
+        <f>E9/422324814</f>
+        <v/>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>转口枢纽→东南亚/南亚</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>南非</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>710</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>非洲</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>11426199</v>
+      </c>
+      <c r="F10" s="8">
+        <f>E10/422324814</f>
+        <v/>
+      </c>
+      <c r="G10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>印度尼西亚</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>360</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>11250898</v>
+      </c>
+      <c r="F11" s="8">
+        <f>E11/422324814</f>
+        <v/>
+      </c>
+      <c r="G11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>哈萨克斯坦</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>398</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>独联体/中亚</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>10925270</v>
+      </c>
+      <c r="F12" s="8">
+        <f>E12/422324814</f>
+        <v/>
+      </c>
+      <c r="G12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>826</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>8784753</v>
+      </c>
+      <c r="F13" s="8">
+        <f>E13/422324814</f>
+        <v/>
+      </c>
+      <c r="G13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>爱沙尼亚</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>233</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>8754532</v>
+      </c>
+      <c r="F14" s="8">
+        <f>E14/422324814</f>
+        <v/>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>波罗的海分销枢纽</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>804</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>8206878</v>
+      </c>
+      <c r="F15" s="8">
+        <f>E15/422324814</f>
+        <v/>
+      </c>
+      <c r="G15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>380</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>8186541</v>
+      </c>
+      <c r="F16" s="8">
+        <f>E16/422324814</f>
+        <v/>
+      </c>
+      <c r="G16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>土耳其</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>792</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>中东/土耳其</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>7652474</v>
+      </c>
+      <c r="F17" s="8">
+        <f>E17/422324814</f>
+        <v/>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>你已有 NMS 客户</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>724</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>7284155</v>
+      </c>
+      <c r="F18" s="8">
+        <f>E18/422324814</f>
+        <v/>
+      </c>
+      <c r="G18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>528</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>6532562</v>
+      </c>
+      <c r="F19" s="8">
+        <f>E19/422324814</f>
+        <v/>
+      </c>
+      <c r="G19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>巴西</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>76</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>拉美</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>5655456</v>
+      </c>
+      <c r="F20" s="8">
+        <f>E20/422324814</f>
+        <v/>
+      </c>
+      <c r="G20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>奥地利</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>40</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>4567730</v>
+      </c>
+      <c r="F21" s="8">
+        <f>E21/422324814</f>
+        <v/>
+      </c>
+      <c r="G21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>新加坡</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>702</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>4496379</v>
+      </c>
+      <c r="F22" s="8">
+        <f>E22/422324814</f>
+        <v/>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>转口枢纽</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>中国大陆</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>156</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>4493322</v>
+      </c>
+      <c r="F23" s="8">
+        <f>E23/422324814</f>
+        <v/>
+      </c>
+      <c r="G23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>124</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>北美</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>4469245</v>
+      </c>
+      <c r="F24" s="8">
+        <f>E24/422324814</f>
+        <v/>
+      </c>
+      <c r="G24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>哥伦比亚</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>170</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>拉美</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>3752926</v>
+      </c>
+      <c r="F25" s="8">
+        <f>E25/422324814</f>
+        <v/>
+      </c>
+      <c r="G25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>保加利亚</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>100</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>3606615</v>
+      </c>
+      <c r="F26" s="8">
+        <f>E26/422324814</f>
+        <v/>
+      </c>
+      <c r="G26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>澳大利亚</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>36</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>3596152</v>
+      </c>
+      <c r="F27" s="8">
+        <f>E27/422324814</f>
+        <v/>
+      </c>
+      <c r="G27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>匈牙利</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>348</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>3207035</v>
+      </c>
+      <c r="F28" s="8">
+        <f>E28/422324814</f>
+        <v/>
+      </c>
+      <c r="G28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>瑞典</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>752</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>3137243</v>
+      </c>
+      <c r="F29" s="8">
+        <f>E29/422324814</f>
+        <v/>
+      </c>
+      <c r="G29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>越南</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>704</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>2733552</v>
+      </c>
+      <c r="F30" s="8">
+        <f>E30/422324814</f>
+        <v/>
+      </c>
+      <c r="G30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>智利</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>152</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>拉美</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>2721330</v>
+      </c>
+      <c r="F31" s="8">
+        <f>E31/422324814</f>
+        <v/>
+      </c>
+      <c r="G31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>秘鲁</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>604</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>拉美</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="n">
+        <v>2713158</v>
+      </c>
+      <c r="F32" s="8">
+        <f>E32/422324814</f>
+        <v/>
+      </c>
+      <c r="G32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>泰国</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>764</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="n">
+        <v>2464546</v>
+      </c>
+      <c r="F33" s="8">
+        <f>E33/422324814</f>
+        <v/>
+      </c>
+      <c r="G33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>300</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="n">
+        <v>2308883</v>
+      </c>
+      <c r="F34" s="8">
+        <f>E34/422324814</f>
+        <v/>
+      </c>
+      <c r="G34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>丹麦</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>208</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="n">
+        <v>2239002</v>
+      </c>
+      <c r="F35" s="8">
+        <f>E35/422324814</f>
+        <v/>
+      </c>
+      <c r="G35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>墨西哥</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>484</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>拉美</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>2183194</v>
+      </c>
+      <c r="F36" s="8">
+        <f>E36/422324814</f>
+        <v/>
+      </c>
+      <c r="G36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>阿根廷</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>32</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>拉美</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="n">
+        <v>1858335</v>
+      </c>
+      <c r="F37" s="8">
+        <f>E37/422324814</f>
+        <v/>
+      </c>
+      <c r="G37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>罗马尼亚</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>642</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="n">
+        <v>1844544</v>
+      </c>
+      <c r="F38" s="8">
+        <f>E38/422324814</f>
+        <v/>
+      </c>
+      <c r="G38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>新西兰</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>554</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="n">
+        <v>1696031</v>
+      </c>
+      <c r="F39" s="8">
+        <f>E39/422324814</f>
+        <v/>
+      </c>
+      <c r="G39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>孟加拉国</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>50</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="n">
+        <v>1099842</v>
+      </c>
+      <c r="F40" s="8">
+        <f>E40/422324814</f>
+        <v/>
+      </c>
+      <c r="G40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>斯洛伐克</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>703</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="n">
+        <v>1068939</v>
+      </c>
+      <c r="F41" s="8">
+        <f>E41/422324814</f>
+        <v/>
+      </c>
+      <c r="G41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>塞尔维亚</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>688</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="n">
+        <v>1057170</v>
+      </c>
+      <c r="F42" s="8">
+        <f>E42/422324814</f>
+        <v/>
+      </c>
+      <c r="G42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>马来西亚</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>458</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="n">
+        <v>996768</v>
+      </c>
+      <c r="F43" s="8">
+        <f>E43/422324814</f>
+        <v/>
+      </c>
+      <c r="G43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>斯洛文尼亚</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>705</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="n">
+        <v>951791</v>
+      </c>
+      <c r="F44" s="8">
+        <f>E44/422324814</f>
+        <v/>
+      </c>
+      <c r="G44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>肯尼亚</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>404</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>非洲</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="n">
+        <v>934046</v>
+      </c>
+      <c r="F45" s="8">
+        <f>E45/422324814</f>
+        <v/>
+      </c>
+      <c r="G45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>葡萄牙</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>620</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="n">
+        <v>927187</v>
+      </c>
+      <c r="F46" s="8">
+        <f>E46/422324814</f>
+        <v/>
+      </c>
+      <c r="G46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>克罗地亚</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>191</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="n">
+        <v>881827</v>
+      </c>
+      <c r="F47" s="8">
+        <f>E47/422324814</f>
+        <v/>
+      </c>
+      <c r="G47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>芬兰</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>246</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="n">
+        <v>843078</v>
+      </c>
+      <c r="F48" s="8">
+        <f>E48/422324814</f>
+        <v/>
+      </c>
+      <c r="G48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>乌兹别克斯坦</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>860</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>独联体/中亚</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="n">
+        <v>802640</v>
+      </c>
+      <c r="F49" s="8">
+        <f>E49/422324814</f>
+        <v/>
+      </c>
+      <c r="G49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>沙特</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>682</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>中东/土耳其</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="n">
+        <v>800914</v>
+      </c>
+      <c r="F50" s="8">
+        <f>E50/422324814</f>
+        <v/>
+      </c>
+      <c r="G50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>比利时</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>56</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="n">
+        <v>706207</v>
+      </c>
+      <c r="F51" s="8">
+        <f>E51/422324814</f>
+        <v/>
+      </c>
+      <c r="G51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>巴基斯坦</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>586</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="n">
+        <v>632718</v>
+      </c>
+      <c r="F52" s="8">
+        <f>E52/422324814</f>
+        <v/>
+      </c>
+      <c r="G52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>格鲁吉亚</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>268</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>独联体/中亚</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="n">
+        <v>612616</v>
+      </c>
+      <c r="F53" s="8">
+        <f>E53/422324814</f>
+        <v/>
+      </c>
+      <c r="G53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>中国台湾</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>490</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="n">
+        <v>601808</v>
+      </c>
+      <c r="F54" s="8">
+        <f>E54/422324814</f>
+        <v/>
+      </c>
+      <c r="G54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>阿尔巴尼亚</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>8</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="n">
+        <v>551402</v>
+      </c>
+      <c r="F55" s="8">
+        <f>E55/422324814</f>
+        <v/>
+      </c>
+      <c r="G55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>韩国</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>410</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="n">
+        <v>465113</v>
+      </c>
+      <c r="F56" s="8">
+        <f>E56/422324814</f>
+        <v/>
+      </c>
+      <c r="G56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>392</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="n">
+        <v>430801</v>
+      </c>
+      <c r="F57" s="8">
+        <f>E57/422324814</f>
+        <v/>
+      </c>
+      <c r="G57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>菲律宾</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>608</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="n">
+        <v>381036</v>
+      </c>
+      <c r="F58" s="8">
+        <f>E58/422324814</f>
+        <v/>
+      </c>
+      <c r="G58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>爱尔兰</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>372</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="n">
+        <v>357037</v>
+      </c>
+      <c r="F59" s="8">
+        <f>E59/422324814</f>
+        <v/>
+      </c>
+      <c r="G59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>58</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>埃及</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>818</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>非洲</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="n">
+        <v>345877</v>
+      </c>
+      <c r="F60" s="8">
+        <f>E60/422324814</f>
+        <v/>
+      </c>
+      <c r="G60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>以色列</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>376</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>中东/土耳其</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="n">
+        <v>273731</v>
+      </c>
+      <c r="F61" s="8">
+        <f>E61/422324814</f>
+        <v/>
+      </c>
+      <c r="G61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>阿塞拜疆</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>31</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>独联体/中亚</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="n">
+        <v>273435</v>
+      </c>
+      <c r="F62" s="8">
+        <f>E62/422324814</f>
+        <v/>
+      </c>
+      <c r="G62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>尼日利亚</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>566</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>非洲</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="n">
+        <v>265052</v>
+      </c>
+      <c r="F63" s="8">
+        <f>E63/422324814</f>
+        <v/>
+      </c>
+      <c r="G63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>62</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>安哥拉</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>24</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>非洲</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="n">
+        <v>93579</v>
+      </c>
+      <c r="F64" s="8">
+        <f>E64/422324814</f>
+        <v/>
+      </c>
+      <c r="G64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>63</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>白俄罗斯</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>112</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>独联体/中亚</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="n">
+        <v>3144</v>
+      </c>
+      <c r="F65" s="8">
+        <f>E65/422324814</f>
+        <v/>
+      </c>
+      <c r="G65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>其他未查询国家（合计约 90 国）</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr"/>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" s="7">
+        <f>422324814-SUM(E3:E65)</f>
+        <v/>
+      </c>
+      <c r="F66" s="8">
+        <f>E66/422324814</f>
+        <v/>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>余量</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="inlineStr"/>
+      <c r="B67" s="1" t="inlineStr">
+        <is>
+          <t>全球合计</t>
+        </is>
+      </c>
+      <c r="C67" s="1" t="inlineStr"/>
+      <c r="D67" s="1" t="inlineStr"/>
+      <c r="E67" s="9" t="n">
+        <v>422324814</v>
+      </c>
+      <c r="F67" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" s="1" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="inlineStr">
+        <is>
+          <t>区域汇总</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="inlineStr"/>
+      <c r="B70" s="1" t="inlineStr">
+        <is>
+          <t>区域</t>
+        </is>
+      </c>
+      <c r="C70" s="1" t="inlineStr"/>
+      <c r="D70" s="1" t="inlineStr"/>
+      <c r="E70" s="1" t="inlineStr">
+        <is>
+          <t>出口额 USD</t>
+        </is>
+      </c>
+      <c r="F70" s="1" t="inlineStr">
+        <is>
+          <t>占全球 %</t>
+        </is>
+      </c>
+      <c r="G70" s="1" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr"/>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" s="7">
+        <f>SUMIF(D3:D65,"欧洲",E3:E65)</f>
+        <v/>
+      </c>
+      <c r="F71" s="8">
+        <f>E71/422324814</f>
+        <v/>
+      </c>
+      <c r="G71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr"/>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>北美</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" s="7">
+        <f>SUMIF(D3:D65,"北美",E3:E65)</f>
+        <v/>
+      </c>
+      <c r="F72" s="8">
+        <f>E72/422324814</f>
+        <v/>
+      </c>
+      <c r="G72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr"/>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>中东/土耳其</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" s="7">
+        <f>SUMIF(D3:D65,"中东/土耳其",E3:E65)</f>
+        <v/>
+      </c>
+      <c r="F73" s="8">
+        <f>E73/422324814</f>
+        <v/>
+      </c>
+      <c r="G73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr"/>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" s="7">
+        <f>SUMIF(D3:D65,"亚太",E3:E65)</f>
+        <v/>
+      </c>
+      <c r="F74" s="8">
+        <f>E74/422324814</f>
+        <v/>
+      </c>
+      <c r="G74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr"/>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>拉美</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" s="7">
+        <f>SUMIF(D3:D65,"拉美",E3:E65)</f>
+        <v/>
+      </c>
+      <c r="F75" s="8">
+        <f>E75/422324814</f>
+        <v/>
+      </c>
+      <c r="G75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr"/>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>非洲</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" s="7">
+        <f>SUMIF(D3:D65,"非洲",E3:E65)</f>
+        <v/>
+      </c>
+      <c r="F76" s="8">
+        <f>E76/422324814</f>
+        <v/>
+      </c>
+      <c r="G76" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr"/>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>独联体/中亚</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" s="7">
+        <f>SUMIF(D3:D65,"独联体/中亚",E3:E65)</f>
+        <v/>
+      </c>
+      <c r="F77" s="8">
+        <f>E77/422324814</f>
+        <v/>
+      </c>
+      <c r="G77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr"/>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>其他未查询国家</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" s="7">
+        <f>422324814-SUM(E3:E65)</f>
+        <v/>
+      </c>
+      <c r="F78" s="8">
+        <f>E78/422324814</f>
+        <v/>
+      </c>
+      <c r="G78" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>落地价计算器（不含 VAT）。黄色格可改。美国关税 2025–2026 变动频繁，报价前按 HTS 8517.62.0020 现查。</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>参数</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>值</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>你的售价 USD (EXW/FOB)</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>海运摊销 USD/台</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>对比：CRS326 MSRP</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>对比：CSS326 MSRP</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>目的地</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>中国产 HS 8517.62 关税</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>依据（2026-09）</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>落地价 USD</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>vs CRS326</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>vs CSS326</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>打法</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>欧盟</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>ITA 信息技术协定 0%</t>
+        </is>
+      </c>
+      <c r="D9" s="3">
+        <f>ROUND(($B$3+$B$4)*(1+B9),0)</f>
+        <v/>
+      </c>
+      <c r="E9" s="14">
+        <f>D9/$B$5-1</f>
+        <v/>
+      </c>
+      <c r="F9" s="14">
+        <f>D9/$B$6-1</f>
+        <v/>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>价格+功能双打</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>ITA 0%；UKCA 你已有</t>
+        </is>
+      </c>
+      <c r="D10" s="3">
+        <f>ROUND(($B$3+$B$4)*(1+B10),0)</f>
+        <v/>
+      </c>
+      <c r="E10" s="14">
+        <f>D10/$B$5-1</f>
+        <v/>
+      </c>
+      <c r="F10" s="14">
+        <f>D10/$B$6-1</f>
+        <v/>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>价格+功能双打</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>美国（现状）</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>301 List 3 25% + 2026-07-24 起强迫劳动分级中国档 12.5%</t>
+        </is>
+      </c>
+      <c r="D11" s="3">
+        <f>ROUND(($B$3+$B$4)*(1+B11),0)</f>
+        <v/>
+      </c>
+      <c r="E11" s="14">
+        <f>D11/$B$5-1</f>
+        <v/>
+      </c>
+      <c r="F11" s="14">
+        <f>D11/$B$6-1</f>
+        <v/>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>只卖差异化：工业/PoE++/ERPS/串口/5年保修</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>美国（若叠加 10% 对华互惠层）</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="n">
+        <v>0.475</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>部分来源称对华 10% 互惠层仍在（至 2026-11-10），报关行确认</t>
+        </is>
+      </c>
+      <c r="D12" s="3">
+        <f>ROUND(($B$3+$B$4)*(1+B12),0)</f>
+        <v/>
+      </c>
+      <c r="E12" s="14">
+        <f>D12/$B$5-1</f>
+        <v/>
+      </c>
+      <c r="F12" s="14">
+        <f>D12/$B$6-1</f>
+        <v/>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>澳大利亚</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>ChAFTA 0%；需 RCM</t>
+        </is>
+      </c>
+      <c r="D13" s="3">
+        <f>ROUND(($B$3+$B$4)*(1+B13),0)</f>
+        <v/>
+      </c>
+      <c r="E13" s="14">
+        <f>D13/$B$5-1</f>
+        <v/>
+      </c>
+      <c r="F13" s="14">
+        <f>D13/$B$6-1</f>
+        <v/>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>价格+功能</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>阿联酋</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>GCC 统一关税 5%（部分 IT 设备 0%）</t>
+        </is>
+      </c>
+      <c r="D14" s="3">
+        <f>ROUND(($B$3+$B$4)*(1+B14),0)</f>
+        <v/>
+      </c>
+      <c r="E14" s="14">
+        <f>D14/$B$5-1</f>
+        <v/>
+      </c>
+      <c r="F14" s="14">
+        <f>D14/$B$6-1</f>
+        <v/>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>枢纽分销商 house brand</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>MFN 0%，无 301</t>
+        </is>
+      </c>
+      <c r="D15" s="3">
+        <f>ROUND(($B$3+$B$4)*(1+B15),0)</f>
+        <v/>
+      </c>
+      <c r="E15" s="14">
+        <f>D15/$B$5-1</f>
+        <v/>
+      </c>
+      <c r="F15" s="14">
+        <f>D15/$B$6-1</f>
+        <v/>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>随美国客户但价格优势保留</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>土耳其</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>欧盟关税同盟，ITA 0%（另有本地附加税，需核）</t>
+        </is>
+      </c>
+      <c r="D16" s="3">
+        <f>ROUND(($B$3+$B$4)*(1+B16),0)</f>
+        <v/>
+      </c>
+      <c r="E16" s="14">
+        <f>D16/$B$5-1</f>
+        <v/>
+      </c>
+      <c r="F16" s="14">
+        <f>D16/$B$6-1</f>
+        <v/>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>复制 NMS 案例</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>负数 = 比 MikroTik 便宜；正数 = 比 MikroTik 贵。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2313,7 +4705,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3131,7 +5523,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3228,7 +5620,6 @@
           <t>$119</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3246,7 +5637,6 @@
           <t>$209</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3264,7 +5654,6 @@
           <t>$489</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">

</xml_diff>

<commit_message>
Add full MikroTik-customer playbook (spec matrices, adjacent competitors, country playbooks, talk tracks)
- MikroTik类客户全量作战手册_2026-09.md: consolidated deep-dive without
  tariff considerations — MikroTik line-up by segment, adjacent brands
  (TP-Link Omada, Ubiquiti, Teltonika, PLANET, ORing, China-direct),
  8 spec matrices (hardware/L2/L3/security/management/PoE/industrial/
  ecosystem), country playbooks, 4 customer battle cards, talk tracks,
  15 objection handlers, email/LinkedIn templates, demo script,
  promotion plan, OEM tiers, pricing ladder, supplier asks, risks,
  full MikroTik lineup appendix
- Workbook: new sheets '竞品全景' and 'MikroTik全产品线'

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -9,11 +9,13 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="替代对照表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MikroTik出口地(Comtrade2024)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="落地价与关税" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MikroTik关键事实(实测)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SmartByte关键SKU" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原Excel数据修正" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="竞品全景" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MikroTik全产品线" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MikroTik出口地(Comtrade2024)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="落地价与关税" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MikroTik关键事实(实测)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SmartByte关键SKU" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原Excel数据修正" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1787,6 +1789,3016 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:M15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>品牌</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>代表型号</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>≈价格 USD</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>价格来源</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>定位</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>强项</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>弱项</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>ERPS</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>OEM</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>工业线</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>保修</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>对你的威胁</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>你的打法</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>CSS326-24G-2S+RM</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>159</v>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>官网 ✅</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>傻瓜 Web 24 口</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>价格、品牌、-20~70°C</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>无 CLI/SSH/LLDP/Trap，SNMP 只读，250 VLAN/32 ACL</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>1 年</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>全面碾压</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>CRS326-24G-2S+RM</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>209</v>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>官网 ✅</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS 24 口</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS 生态、API/REST/脚本、QinQ/MSTP/L3 卸载、-40~60°C</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>无 ERPS、无 PoE-out、2×SFP+、1 年保修</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>1 年</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>补空白：ERPS/PoE++/工业/OEM，价格低 1/3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>CRS328-24P-4S+RM</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>489</v>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>官网 ✅</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>24 PoE af/at 450W</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>被动+标准 PoE、4×SFP+</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>无 bt、-20~60°C、无 PoE 看门狗</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>1 年</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>PoE 管理 + 工业款 + 价格</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>CRS354-48G-4S+2Q+RM</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>599</v>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>官网 ✅</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>48 口 + 40G</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>2×QSFP+ 40G</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>QCA9531 650MHz/64MB，L3 极弱</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>1 年</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>无 40G 则用 LT-S8352XG</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>CRS418-8P-8G-2S+RM</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>449</v>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>抓取 *</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>新方向：强 CPU 混合路由交换</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>2.2GHz 四核、L3 卸载、可当路由器/CAPsMAN、双 AC</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>价格、-20°C</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>1 年</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>不碰</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>TP-Link Omada</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>SG3428X</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>零售 ≈259–367</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>商业 L2+ 24G+4×SFP+</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>有 ERPS、OAM、sFlow、DDM、CLI、Omada 云、终身有限保修、渠道广</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>0~50°C、无工业线、不能 OEM、无 DI/DO</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>终身有限</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>24 口只做敲门 SKU；用工业/PoE++/OEM 赚钱</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>TP-Link Omada</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>SG3428XMP</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>480</v>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>零售 ≈</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>24 PoE+ 384W + 4×SFP+</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>终身有限</t>
+        </is>
+      </c>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Ubiquiti UniFi</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>USW-24</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>250</v>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>零售 ≈219–295</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>L2 24G + 2×SFP 1G</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>UI/控制器、品牌</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>控制器依赖、无 SFP+、无 ERPS、无 QinQ</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>1 年</t>
+        </is>
+      </c>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>对不想被控制器绑定的客户</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Ubiquiti UniFi</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>USW-Pro-24</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>399</v>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>store.ui.com</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>L3 24G + 2×SFP+</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>UI/控制器、L3</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>同上，价格高</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>1 年</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>价格 1/3 + CLI/SNMP/ERPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Teltonika Networks</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>TSW212</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>129</v>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>MSRP</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>工业 8G + 2×SFP 管理型</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>价格、RMS 云、PROFINET/EtherNet-IP/MRP、7–57V、与 MikroTik 同渠道</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>8K MAC/512KB 缓存、无 10G、无 ERPS、无 PoE++、无 QinQ/MSTP 级 L2+</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>否(MRP)</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>2 年</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG：4×10G、ERPS、16K/12Mbit、PoE++、DI/DO、5 年</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>PLANET</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>IGS-5225-8P4S</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>790</v>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>零售 757–828</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>工业 8 PoE+ + 2 SFP + 2×2.5G SFP</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>ERPS &lt;10ms、MSTP、Modbus TCP、1588 透传、-40~75、TAA</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>价格 5–7×、交期</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>有限</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>5 年</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>'PLANET 的功能，MikroTik 的价格'</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>IGS-9084GP 类</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>≈900–1200</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>工业标杆</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>O-Ring &lt;30ms、ERPS、EN50155、IP67、UL</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>价格 8–10×</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>5 年</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>低</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>让出铁路/IP67/UL 项目</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>中国直供</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Utepo/ONV/HRUI/UNIPOE</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>低你 10–30%</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>低价管理/非管理</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>价格、目录大</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>软件弱、CLI 不规范、MIB 缺、文档差、无欧美支持</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>部分</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>1–3 年</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>不比裸价：Marvell+CLI+MIB+固件迭代+保修</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>SmartByte (经你)</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>130</v>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>售价（进价 ≈100）</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>商业 L2+ 24G+4×SFP+</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>4×10G、Cisco CLI、SNMPv3+Trap+私有 MIB、MQTT、ERPS、QinQ、480 ACL、双分区、OEM No MOQ、3 年</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>0~50°C、无 API/云、品牌弱</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>是（LT-IS 线）</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>3 年 / 工业 5 年</t>
+        </is>
+      </c>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J51"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>说明：来自仓库 MikroTik_L2Plus_Switches.xlsx 去重后 49 款（抓取值，可能有误）；'实测价' 列为 2026-09 官网核实值。</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>型号</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>抓取价格</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>实测价 ✅</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>端口配置</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>交换芯片</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>OS</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>工作温度</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>PoE 输出</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>PoE 预算</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>分段/备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>CRS106-1C-5S</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>$89.00</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>1x Combo (GbE/SFP), 5x SFP (1G)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>QCA8511</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7 / SwOS</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to +60°C</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>CRS112-8G-4S-IN</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>$119.00</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>8x GbE RJ45, 4x SFP (1G)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>QCA8513</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7 / SwOS</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to +60°C</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>CRS112-8P-4S-IN</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>$209.00</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>8x GbE RJ45, 4x SFP</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>QCA8511</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to 60°C</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>PoE (802.3af)</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>CRS210-8G-2S+IN</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>$229.00</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>8x GbE RJ45, 2x SFP+</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>QCA8519-AC2C</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>PoE (802.3af)</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr"/>
+      <c r="J6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>CRS212-1G-10S-1S+IN</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>$219.00</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>1x GbE RJ45, 10x SFP, 1x SFP+</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>QCA8519</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr"/>
+      <c r="I7" s="3" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>CRS304-4XG-IN</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>$199.00</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>4x 10GbE RJ45</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>98DX2528</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>PoE (802.3af)</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>CRS305-1G-4S+IN</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>$149.00</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>1x GbE RJ45, 4x SFP+</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>98DX3236</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS / SwitchOS</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>PoE (802.3af)</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>CRS305-1G-4S+OUT</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>$229.00</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>98DX226S</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7 / SwOS</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>PoE (802.3af)</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>CRS309-1G-8S+IN</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>$269.00</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>1x GbE RJ45, 8x SFP+</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>98DX8208</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS / SwitchOS</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>PoE (802.3af)</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>全光/高速，不打</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>CRS310-1G-5S-4S+IN</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>$199.00</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>1x GbE RJ45, 5x SFP, 5x SFP+</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>98DX226S</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7 / SwitchOS</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>PoE (802.3af)</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>CRS310-1G-5S-4S+OUT</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>$249.00</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>5x SFP+</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>98DX226S</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7 / SwitchOS</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>PoE (802.3af)</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr"/>
+      <c r="J13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>CRS310-8G+2S+IN</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>$149.00</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>8x 2.5GbE RJ45, 2x SFP+ (10G)</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>98DX226S</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7 / SwOS</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to +60°C</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>CRS312-4C+8XG</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>$349.00</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>4x Combo (10G SFP+/RJ45), 8x 10GbE RJ45</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>98DX8212</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7 / SwOS</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to +60°C</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
+      <c r="I15" s="3" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>全光/高速，不打</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>CRS312-4C+8XG-RM</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>$699.00</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>8x 10GbE RJ45, 4x Combo</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>98DX8212</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7 / SwitchOS</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>-30°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr"/>
+      <c r="I16" s="3" t="inlineStr"/>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>全光/高速，不打</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>CRS317-1G-16S+RM</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>$499.00</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>10x GbE RJ45, 16x SFP+</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>98DX8216</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS / SwitchOS</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to 60°C</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr"/>
+      <c r="I17" s="3" t="inlineStr"/>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>全光/高速，不打</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>CRS318-16P-2S+OUT</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>$279.00</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>16x GbE RJ45</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>98DX226S</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS / SwitchOS</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>PoE (802.3af)</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr"/>
+      <c r="J18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>CRS318-16P-2S+RM</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>$329.00</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>16x GbE RJ45 (PoE-out), 2x SFP+ (10G)</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>98DX3236</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7 / SwOS</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to +60°C</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>PoE+ (802.3af/at/bt)</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>300 W</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>CRS318-1F</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>$169.00</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>15x 100M Fiber</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>98DX224S</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS / SwitchOS</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Passive PoE</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr"/>
+      <c r="J20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>CRS318-1Fi-15Fr-2S</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>$225.00</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>15x 100M Fiber, 1x 1G Fiber, 2x SFP</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>98DX3236</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7 / SwOS</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to +70°C</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr"/>
+      <c r="I21" s="3" t="inlineStr"/>
+      <c r="J21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>CRS320-8P-8B-4S+RM</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>$489.00</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>17x GbE RJ45, 4x SFP+</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>98DX226S</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7 / SwitchOS</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>-10°C to 50°C</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>PoE+ (802.3bt)</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr"/>
+      <c r="J22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>CRS326-24G-2S+IN</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>$199.00</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>24x GbE RJ45, 2x SFP+ (10G)</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>98DX3236</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7 / SwOS</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to +60°C</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr"/>
+      <c r="I23" s="3" t="inlineStr"/>
+      <c r="J23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>CRS326-24G-2S+RM</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>$219.00</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>209</v>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>24x GbE RJ45, 2x SFP+ (10G)</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>98DX3236</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7 / SwOS</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to +60°C</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr"/>
+      <c r="I24" s="3" t="inlineStr"/>
+      <c r="J24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>CRS326-24S+2Q+RM</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>$599.00</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>24x SFP+</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>98DX8332</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7 / SwitchOS</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to 60°C</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr"/>
+      <c r="I25" s="3" t="inlineStr"/>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>全光/高速，不打</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>CRS326-4C+20G+2Q+RM</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>$999.00</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>5x GbE RJ45, 20x 2.5GbE, 4x Combo</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>98DX8332</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to 60°C</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr"/>
+      <c r="I26" s="3" t="inlineStr"/>
+      <c r="J26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>CRS326-4C+20G+2S+RM</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>$239.00</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>4x Combo (GbE/SFP), 20x GbE RJ45, 2x SFP+ (10G)</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>98DX3236</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7 / SwOS</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to +60°C</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr"/>
+      <c r="I27" s="3" t="inlineStr"/>
+      <c r="J27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>CRS328-24P-4S+RM</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>$489.00</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>489</v>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>24x GbE RJ45, 4x SFP+</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>98DX3236</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS / SwitchOS</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to 60°C</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>PoE (802.3af)</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr"/>
+      <c r="J28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>CRS328-4C-20S-4S+RM</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>$449.00</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>4x Combo, 20x SFP, 4x SFP+</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>98DX3236</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS / SwitchOS</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to 60°C</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr"/>
+      <c r="I29" s="3" t="inlineStr"/>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>全光/高速，不打</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>CRS332-32S+RM</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>$749.00</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>32x SFP+ (10G), 6x Combo (SFP+/RJ45)</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>98DX8332</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7 / SwOS</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to +60°C</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr"/>
+      <c r="I30" s="3" t="inlineStr"/>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>全光/高速，不打</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>CRS354-48G-4S+2Q+RM</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>$599.00</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>599</v>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>48x GbE RJ45, 4x SFP+</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>98DX3257</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7 / SwitchOS</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to 60°C</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr"/>
+      <c r="I31" s="3" t="inlineStr"/>
+      <c r="J31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>CRS354-48P-4S+2Q+RM</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>$999.00</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>4x SFP+</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>98DX3257</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7 / SwitchOS</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to 60°C</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>PoE (802.3af)</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr"/>
+      <c r="J32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>CRS418-8P-8G-2S+5</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>$499.00</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>16x GbE RJ45, 2x SFP+</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>98DX226S</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>PoE (802.3af)</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr"/>
+      <c r="J33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>CRS418-8P-8G-2S+RM</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>$449.00</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr"/>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>16x GbE RJ45, 2x SFP+</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>98DX226S</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>PoE (802.3af)</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr"/>
+      <c r="J34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>CRS504-4XQ-IN</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>$799.00</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>4x QSFP28</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>98DX4310</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr"/>
+      <c r="I35" s="3" t="inlineStr"/>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>全光/高速，不打</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>CRS504-4XQ-OUT</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>$899.00</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr"/>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>100x GbE RJ45, 4x QSFP28</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>98DX4310</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>PoE+ (802.3bt)</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr"/>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>全光/高速，不打</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>CRS510-8XS-2XQ-IN</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>$999.00</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>8x SFP+, 2x QSFP28</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>98DX4310</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr"/>
+      <c r="I37" s="3" t="inlineStr"/>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>全光/高速，不打</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>CRS518-16XS-2XQ-RM</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>$1595.00</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr"/>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>16x SFP+, 2x QSFP28</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>98DX8525</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr"/>
+      <c r="I38" s="3" t="inlineStr"/>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>全光/高速，不打</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>CRS520-4XS-16XQ-RM</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>$2195.00</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>100x GbE RJ45, 4x SFP+, 16x QSFP28</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>98CX8410</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to 50°C</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr"/>
+      <c r="I39" s="3" t="inlineStr"/>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>全光/高速，不打</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>CRS804-4DDQ-</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>$1295.00</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr"/>
+      <c r="D40" s="3" t="inlineStr"/>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>98DX7335</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>-10°C to 60°C</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr"/>
+      <c r="I40" s="3" t="inlineStr"/>
+      <c r="J40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>CRS812-8DS-2DQ-2DDQ-RM</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>$1295.00</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>98DX7335</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS v7</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>-10°C to 50°C</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr"/>
+      <c r="I41" s="3" t="inlineStr"/>
+      <c r="J41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>CSS106-1G-4P-1S</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>$55.95</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr"/>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>260x GbE RJ45</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>QCA8337</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik SwOS</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>Passive PoE</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr"/>
+      <c r="J42" s="3" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>CSS106-5G-1S</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>$39.95</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>5x GbE RJ45</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>QCA8337</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik SwOS</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Passive PoE</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr"/>
+      <c r="J43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>CSS318-16G-2S+IN</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>$139.00</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr"/>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>16x GbE RJ45, 2x SFP+</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>98DX2518</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>SwOS</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr"/>
+      <c r="I44" s="3" t="inlineStr"/>
+      <c r="J44" s="3" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>CSS326-24G-2S+RM</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>$199.00</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="n">
+        <v>159</v>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>24x GbE RJ45, 2x SFP+ (10G)</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>98DX3236</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>SwOS</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to +60°C</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr"/>
+      <c r="I45" s="3" t="inlineStr"/>
+      <c r="J45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>CSS606-1G-2G</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>$139.00</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr"/>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>3x GbE RJ45</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>88E6193X</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>SwOS</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>Passive PoE</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>Built for th…</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>CSS610-1G</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>$139.00</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr"/>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>88E6193X</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>SwitchOS Lite</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Passive PoE</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr"/>
+      <c r="J47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>CSS610-1Gi-7R-2S+OUT</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>$99.00</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr"/>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>1x GbE RJ45, 7x 100M Fiber (Reverse PoE), 2x SFP+ (10G)</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>98DX3236</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>SwOS</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to +70°C</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr"/>
+      <c r="I48" s="3" t="inlineStr"/>
+      <c r="J48" s="3" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>CSS610-8G-2S+IN</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>$119.00</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="n">
+        <v>119</v>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>8x GbE RJ45, 2x SFP+</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>88E6193X</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>SwitchOS Lite</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>-20°C to 60°C</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>Passive PoE</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr"/>
+      <c r="J49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>CSS610-8P-2S+IN</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>$229.00</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr"/>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>2x SFP+</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>88E6193X</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>SwitchOS Lite</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>PoE (802.3af)</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>of 140 W</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>CSS610-8P-2S+OUT</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>$199.00</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>8x GbE RJ45</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>88E6193</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>SwOS Lite</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>-40°C to 70°C</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>PoE (802.3af)</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr"/>
+      <c r="J51" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2017,7 +5029,6 @@
         <f>E8/422324814</f>
         <v/>
       </c>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -2073,7 +5084,6 @@
         <f>E10/422324814</f>
         <v/>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -2099,7 +5109,6 @@
         <f>E11/422324814</f>
         <v/>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2125,7 +5134,6 @@
         <f>E12/422324814</f>
         <v/>
       </c>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -2151,7 +5159,6 @@
         <f>E13/422324814</f>
         <v/>
       </c>
-      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -2207,7 +5214,6 @@
         <f>E15/422324814</f>
         <v/>
       </c>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2233,7 +5239,6 @@
         <f>E16/422324814</f>
         <v/>
       </c>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2289,7 +5294,6 @@
         <f>E18/422324814</f>
         <v/>
       </c>
-      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2315,7 +5319,6 @@
         <f>E19/422324814</f>
         <v/>
       </c>
-      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -2341,7 +5344,6 @@
         <f>E20/422324814</f>
         <v/>
       </c>
-      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -2367,7 +5369,6 @@
         <f>E21/422324814</f>
         <v/>
       </c>
-      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -2423,7 +5424,6 @@
         <f>E23/422324814</f>
         <v/>
       </c>
-      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2449,7 +5449,6 @@
         <f>E24/422324814</f>
         <v/>
       </c>
-      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2475,7 +5474,6 @@
         <f>E25/422324814</f>
         <v/>
       </c>
-      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2501,7 +5499,6 @@
         <f>E26/422324814</f>
         <v/>
       </c>
-      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2527,7 +5524,6 @@
         <f>E27/422324814</f>
         <v/>
       </c>
-      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2553,7 +5549,6 @@
         <f>E28/422324814</f>
         <v/>
       </c>
-      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2579,7 +5574,6 @@
         <f>E29/422324814</f>
         <v/>
       </c>
-      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2605,7 +5599,6 @@
         <f>E30/422324814</f>
         <v/>
       </c>
-      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2631,7 +5624,6 @@
         <f>E31/422324814</f>
         <v/>
       </c>
-      <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2657,7 +5649,6 @@
         <f>E32/422324814</f>
         <v/>
       </c>
-      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2683,7 +5674,6 @@
         <f>E33/422324814</f>
         <v/>
       </c>
-      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2709,7 +5699,6 @@
         <f>E34/422324814</f>
         <v/>
       </c>
-      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2735,7 +5724,6 @@
         <f>E35/422324814</f>
         <v/>
       </c>
-      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2761,7 +5749,6 @@
         <f>E36/422324814</f>
         <v/>
       </c>
-      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2787,7 +5774,6 @@
         <f>E37/422324814</f>
         <v/>
       </c>
-      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2813,7 +5799,6 @@
         <f>E38/422324814</f>
         <v/>
       </c>
-      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2839,7 +5824,6 @@
         <f>E39/422324814</f>
         <v/>
       </c>
-      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2865,7 +5849,6 @@
         <f>E40/422324814</f>
         <v/>
       </c>
-      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2891,7 +5874,6 @@
         <f>E41/422324814</f>
         <v/>
       </c>
-      <c r="G41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2917,7 +5899,6 @@
         <f>E42/422324814</f>
         <v/>
       </c>
-      <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2943,7 +5924,6 @@
         <f>E43/422324814</f>
         <v/>
       </c>
-      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2969,7 +5949,6 @@
         <f>E44/422324814</f>
         <v/>
       </c>
-      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2995,7 +5974,6 @@
         <f>E45/422324814</f>
         <v/>
       </c>
-      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -3021,7 +5999,6 @@
         <f>E46/422324814</f>
         <v/>
       </c>
-      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -3047,7 +6024,6 @@
         <f>E47/422324814</f>
         <v/>
       </c>
-      <c r="G47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -3073,7 +6049,6 @@
         <f>E48/422324814</f>
         <v/>
       </c>
-      <c r="G48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -3099,7 +6074,6 @@
         <f>E49/422324814</f>
         <v/>
       </c>
-      <c r="G49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -3125,7 +6099,6 @@
         <f>E50/422324814</f>
         <v/>
       </c>
-      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -3151,7 +6124,6 @@
         <f>E51/422324814</f>
         <v/>
       </c>
-      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -3177,7 +6149,6 @@
         <f>E52/422324814</f>
         <v/>
       </c>
-      <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -3203,7 +6174,6 @@
         <f>E53/422324814</f>
         <v/>
       </c>
-      <c r="G53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -3229,7 +6199,6 @@
         <f>E54/422324814</f>
         <v/>
       </c>
-      <c r="G54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -3255,7 +6224,6 @@
         <f>E55/422324814</f>
         <v/>
       </c>
-      <c r="G55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -3281,7 +6249,6 @@
         <f>E56/422324814</f>
         <v/>
       </c>
-      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -3307,7 +6274,6 @@
         <f>E57/422324814</f>
         <v/>
       </c>
-      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -3333,7 +6299,6 @@
         <f>E58/422324814</f>
         <v/>
       </c>
-      <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -3359,7 +6324,6 @@
         <f>E59/422324814</f>
         <v/>
       </c>
-      <c r="G59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -3385,7 +6349,6 @@
         <f>E60/422324814</f>
         <v/>
       </c>
-      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -3411,7 +6374,6 @@
         <f>E61/422324814</f>
         <v/>
       </c>
-      <c r="G61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -3437,7 +6399,6 @@
         <f>E62/422324814</f>
         <v/>
       </c>
-      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -3463,7 +6424,6 @@
         <f>E63/422324814</f>
         <v/>
       </c>
-      <c r="G63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -3489,7 +6449,6 @@
         <f>E64/422324814</f>
         <v/>
       </c>
-      <c r="G64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -3515,17 +6474,13 @@
         <f>E65/422324814</f>
         <v/>
       </c>
-      <c r="G65" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr"/>
       <c r="B66" t="inlineStr">
         <is>
           <t>其他未查询国家（合计约 90 国）</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr"/>
-      <c r="D66" t="inlineStr"/>
       <c r="E66" s="7">
         <f>422324814-SUM(E3:E65)</f>
         <v/>
@@ -3586,14 +6541,11 @@
       <c r="G70" s="1" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr"/>
       <c r="B71" t="inlineStr">
         <is>
           <t>欧洲</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr"/>
-      <c r="D71" t="inlineStr"/>
       <c r="E71" s="7">
         <f>SUMIF(D3:D65,"欧洲",E3:E65)</f>
         <v/>
@@ -3602,17 +6554,13 @@
         <f>E71/422324814</f>
         <v/>
       </c>
-      <c r="G71" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr"/>
       <c r="B72" t="inlineStr">
         <is>
           <t>北美</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr"/>
-      <c r="D72" t="inlineStr"/>
       <c r="E72" s="7">
         <f>SUMIF(D3:D65,"北美",E3:E65)</f>
         <v/>
@@ -3621,17 +6569,13 @@
         <f>E72/422324814</f>
         <v/>
       </c>
-      <c r="G72" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr"/>
       <c r="B73" t="inlineStr">
         <is>
           <t>中东/土耳其</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr"/>
-      <c r="D73" t="inlineStr"/>
       <c r="E73" s="7">
         <f>SUMIF(D3:D65,"中东/土耳其",E3:E65)</f>
         <v/>
@@ -3640,17 +6584,13 @@
         <f>E73/422324814</f>
         <v/>
       </c>
-      <c r="G73" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr"/>
       <c r="B74" t="inlineStr">
         <is>
           <t>亚太</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr"/>
-      <c r="D74" t="inlineStr"/>
       <c r="E74" s="7">
         <f>SUMIF(D3:D65,"亚太",E3:E65)</f>
         <v/>
@@ -3659,17 +6599,13 @@
         <f>E74/422324814</f>
         <v/>
       </c>
-      <c r="G74" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr"/>
       <c r="B75" t="inlineStr">
         <is>
           <t>拉美</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr"/>
-      <c r="D75" t="inlineStr"/>
       <c r="E75" s="7">
         <f>SUMIF(D3:D65,"拉美",E3:E65)</f>
         <v/>
@@ -3678,17 +6614,13 @@
         <f>E75/422324814</f>
         <v/>
       </c>
-      <c r="G75" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr"/>
       <c r="B76" t="inlineStr">
         <is>
           <t>非洲</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr"/>
-      <c r="D76" t="inlineStr"/>
       <c r="E76" s="7">
         <f>SUMIF(D3:D65,"非洲",E3:E65)</f>
         <v/>
@@ -3697,17 +6629,13 @@
         <f>E76/422324814</f>
         <v/>
       </c>
-      <c r="G76" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr"/>
       <c r="B77" t="inlineStr">
         <is>
           <t>独联体/中亚</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr"/>
-      <c r="D77" t="inlineStr"/>
       <c r="E77" s="7">
         <f>SUMIF(D3:D65,"独联体/中亚",E3:E65)</f>
         <v/>
@@ -3716,17 +6644,13 @@
         <f>E77/422324814</f>
         <v/>
       </c>
-      <c r="G77" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr"/>
       <c r="B78" t="inlineStr">
         <is>
           <t>其他未查询国家</t>
         </is>
       </c>
-      <c r="C78" t="inlineStr"/>
-      <c r="D78" t="inlineStr"/>
       <c r="E78" s="7">
         <f>422324814-SUM(E3:E65)</f>
         <v/>
@@ -3735,7 +6659,6 @@
         <f>E78/422324814</f>
         <v/>
       </c>
-      <c r="G78" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3745,7 +6668,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4139,7 +7062,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4705,7 +7628,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5523,7 +8446,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Add Marvell-brand landscape sheet and development-cadence KPI sheet to workbook
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -1,21 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="参数" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="替代对照表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="竞品全景" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MikroTik全产品线" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MikroTik出口地(Comtrade2024)" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="落地价与关税" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MikroTik关键事实(实测)" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SmartByte关键SKU" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="原Excel数据修正" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="参数" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="替代对照表" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="竞品全景" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Marvell品牌全景" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="MikroTik全产品线" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="开发系统-节奏与KPI" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="MikroTik出口地(Comtrade2024)" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="落地价与关税" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MikroTik关键事实(实测)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="SmartByte关键SKU" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="原Excel数据修正" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -557,6 +559,1027 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>系列</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>型号</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>描述</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>进价 RMB</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>≈USD</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>售价 USD (+加价率)</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>商业 L2+</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>24G + 4×SFP+ 1/2.5/10G；0~50°C；3年</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>710</v>
+      </c>
+      <c r="E2" s="3">
+        <f>IF(D2="","",ROUND(D2/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F2" s="3">
+        <f>IF(D2="","",ROUND(D2/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>对标 CSS326/CRS326 主力</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>商业 L2+</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>24×PoE + 4×SFP+ 10G；280W</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>1010</v>
+      </c>
+      <c r="E3" s="3">
+        <f>IF(D3="","",ROUND(D3/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F3" s="3">
+        <f>IF(D3="","",ROUND(D3/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>对标 CRS328-24P（预算差）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>商业 L2+</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>24G + 4×1G/2.5G SFP</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>460</v>
+      </c>
+      <c r="E4" s="3">
+        <f>IF(D4="","",ROUND(D4/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F4" s="3">
+        <f>IF(D4="","",ROUND(D4/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>商业 L2+</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>24×PoE + 4×2.5G SFP；440W</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E5" s="3">
+        <f>IF(D5="","",ROUND(D5/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F5" s="3">
+        <f>IF(D5="","",ROUND(D5/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>商业 L2+</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8310G-2GX8GT</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>8G + 2×2.5G SFP</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>380</v>
+      </c>
+      <c r="E6" s="3">
+        <f>IF(D6="","",ROUND(D6/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F6" s="3">
+        <f>IF(D6="","",ROUND(D6/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>成本回落前暂停出货</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>商业 L2+</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8310GP-2GX8GT</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>8×PoE(120W) + 2×2.5G SFP</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>450</v>
+      </c>
+      <c r="E7" s="3">
+        <f>IF(D7="","",ROUND(D7/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F7" s="3">
+        <f>IF(D7="","",ROUND(D7/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>商业 L2+</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8352XG-4XS48GT</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>48G + 4×SFP+ 10G</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>1470</v>
+      </c>
+      <c r="E8" s="3">
+        <f>IF(D8="","",ROUND(D8/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F8" s="3">
+        <f>IF(D8="","",ROUND(D8/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>商业 L2+</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8352XGP-4XS48GT</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>48×PoE + 4×SFP+ 10G；440W/850W</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>1870</v>
+      </c>
+      <c r="E9" s="3">
+        <f>IF(D9="","",ROUND(D9/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F9" s="3">
+        <f>IF(D9="","",ROUND(D9/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>商业 L3</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8528XG-4XS24GT</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>24G + 4×SFP+；L3 (RIP/OSPF/IS-IS/BGP/VRRP)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E10" s="3">
+        <f>IF(D10="","",ROUND(D10/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F10" s="3">
+        <f>IF(D10="","",ROUND(D10/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>PoE 版 1900</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>商业 L3</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8528XG-4XS16GX8GC</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>16×SFP + 8 Combo + 4×SFP+；L3</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>2100</v>
+      </c>
+      <c r="E11" s="3">
+        <f>IF(D11="","",ROUND(D11/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F11" s="3">
+        <f>IF(D11="","",ROUND(D11/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>商业 L3</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8552XG-4XS48GT</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>48G + 4×SFP+；L3</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>2600</v>
+      </c>
+      <c r="E12" s="3">
+        <f>IF(D12="","",ROUND(D12/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F12" s="3">
+        <f>IF(D12="","",ROUND(D12/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>PoE 版 3100</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>工业 L2+</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6306G-2GX4GT</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>4G + 2×SFP；DIN；-40~75°C；5年</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>660</v>
+      </c>
+      <c r="E13" s="3">
+        <f>IF(D13="","",ROUND(D13/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F13" s="3">
+        <f>IF(D13="","",ROUND(D13/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>PoE 720 / PoE++ 820；Frank 6口对位</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>工业 L2+</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G-2GX8GT</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>8G + 2×2.5G SFP</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>700</v>
+      </c>
+      <c r="E14" s="3">
+        <f>IF(D14="","",ROUND(D14/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F14" s="3">
+        <f>IF(D14="","",ROUND(D14/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>PoE 780 / PoE++ 880</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>工业 L2+</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312G-4GX8GT</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>8G + 4×2.5G SFP</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>740</v>
+      </c>
+      <c r="E15" s="3">
+        <f>IF(D15="","",ROUND(D15/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F15" s="3">
+        <f>IF(D15="","",ROUND(D15/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>PoE 820 / -2BT 920；Frank 12口对位</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>工业 L2+</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>8G + 4×SFP+ 10G</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="E16" s="3">
+        <f>IF(D16="","",ROUND(D16/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F16" s="3">
+        <f>IF(D16="","",ROUND(D16/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>PoE 920 / -2BT 1020</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>工业 L2+</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312GP-4GX8GT-8BT</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>8×90W PoE++ (480W) + 4×2.5G SFP；52–57VDC</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3">
+        <f>IF(D17="","",ROUND(D17/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F17" s="3">
+        <f>IF(D17="","",ROUND(D17/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>价格表未列，官网有；询价</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>工业 L2+</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6316XG-4XS4GX8GT</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>8G + 4×SFP + 4×SFP+</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>1400</v>
+      </c>
+      <c r="E18" s="3">
+        <f>IF(D18="","",ROUND(D18/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F18" s="3">
+        <f>IF(D18="","",ROUND(D18/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>工业 L2+</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6318G-2GX16GT</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>16G + 2×SFP</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>1180</v>
+      </c>
+      <c r="E19" s="3">
+        <f>IF(D19="","",ROUND(D19/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F19" s="3">
+        <f>IF(D19="","",ROUND(D19/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>PoE 1340</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>工业 L2+</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6318XGP-2XS16GT</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>16×PoE + 2×SFP+</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>1660</v>
+      </c>
+      <c r="E20" s="3">
+        <f>IF(D20="","",ROUND(D20/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F20" s="3">
+        <f>IF(D20="","",ROUND(D20/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>工业 L2+ DI/DO/RS485</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6320G-4GX16GT-D</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>16G + 4×SFP + DI/DO/RS485</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>1560</v>
+      </c>
+      <c r="E21" s="3">
+        <f>IF(D21="","",ROUND(D21/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F21" s="3">
+        <f>IF(D21="","",ROUND(D21/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>PoE 1760 / -4BT 1960；ITS/SCADA 场景</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>工业 L2+ DI/DO/RS485</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6328XG-4XS24GT-D</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>24G + 4×SFP+ 10G + DI/DO/RS485</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>1960</v>
+      </c>
+      <c r="E22" s="3">
+        <f>IF(D22="","",ROUND(D22/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F22" s="3">
+        <f>IF(D22="","",ROUND(D22/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>PoE 2200 / -4BT 2400</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>工业 L2+ DI/DO/RS485</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6328XG-4XS16GX8GC-D</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>16×SFP + 8 Combo + 4×SFP+ + DI/DO</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>2650</v>
+      </c>
+      <c r="E23" s="3">
+        <f>IF(D23="","",ROUND(D23/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F23" s="3">
+        <f>IF(D23="","",ROUND(D23/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>vs CRS328-4C-20S-4S+ $299：MikroTik 更便宜</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>工业 Bypass</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS63xx-FBP 系列</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>光纤 Bypass 管理型</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>960</v>
+      </c>
+      <c r="E24" s="3">
+        <f>IF(D24="","",ROUND(D24/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F24" s="3">
+        <f>IF(D24="","",ROUND(D24/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>960–1640</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>工业 L3</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS65xx 系列</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>工业 L3</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>1900</v>
+      </c>
+      <c r="E25" s="3">
+        <f>IF(D25="","",ROUND(D25/参数!$B$2,0))</f>
+        <v/>
+      </c>
+      <c r="F25" s="3">
+        <f>IF(D25="","",ROUND(D25/参数!$B$2*(1+参数!$B$3),0))</f>
+        <v/>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>1900–3100</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>型号</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>原 Excel 值</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>官网实测值</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CSS326-24G-2S+RM 芯片</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>98DX3236</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>98DX3216</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>离线库写错</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CSS610-8G-2S+IN 芯片</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>98DX3236 / 88E6193X 两行</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>88E6193X</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>离线库与在线抓取不一致</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CSS610-8G-2S+IN 价格</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>$89 / $119</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>$119</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CRS326-24G-2S+RM 价格</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>$219</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>$209</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CRS328-24P-4S+RM 价格</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>$499 / $489</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>$489</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CRS320-8P-8B-4S+RM 价格</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>$299 / $489</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>待核实</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>两行不一致</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>RB260GSP</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>端口写成 260x GbE</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>5×GbE + 1×SFP</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>正则解析错误行，建议删除</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>整体</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>72 行含十余行重复</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>按 product_code 去重，以在线值为准</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>两种 URL slug 抓了两遍</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2797,6 +3820,2004 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>品牌</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>国家/地区</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>类型</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Marvell证据</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>主战场</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>关系</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>切入点</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>拉脱维亚(欧盟)</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>✅ 官方文档列 98DX3236/3257/226S/2528/8332/4310</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>WISP/中小企业/工业</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>主要对标</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>ERPS/PoE++/工业/贴牌补其空白</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Allied Telesis</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>日本/新西兰，美国总部 WA</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>✅ 内核补丁支持 98DX3236/3336/4251（作者 @alliedtelesis.co.nz）</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>欧美企业接入 L2/L3</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>竞品+最大替换池</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>老型号 EOL 替换、抢其渠道</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>A-替换</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Edgecore(Accton)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>台湾</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>ODM/白牌</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>✅ SAF51001I 规格书标注 8×GbE through 98DX3236</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>数据中心/白牌</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>旁证(台湾体系熟Marvell)</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>不做主攻</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>PLANET Technology</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>台湾</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>○ 混合(Realtek/Marvell)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>工业/商业/电力/安防</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>头号对标</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>抄规格与文档、抢渠道</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>A-渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Moxa</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>台湾</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>铁路/电力/海事</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>高端锚</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>只打备件/扩容/项目配套</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>EtherWAN</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>台湾</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>工业/ITS/安防</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>竞品</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>抢 ITS 项目位置</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>台湾</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>工业/ITS/铁路</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>竞品</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>让出铁路/IP67/UL 项目</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>CTC Union</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>台湾</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>品牌商(自有厂)</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>○ 官网明示 in-house R&amp;D and factory</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>电信接入/工业, EN50155/IEC61850-3</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>竞品</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>关注 EOL 与运营商项目</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Lantech</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>台湾</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>工业 PoE/EN50155/E-mark</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>竞品,欧洲渠道密</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>抢渠道</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Volktek</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>台湾</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>ODM+品牌</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>● ODM 常用 Marvell 平台</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>工业/企业</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>第二供应源参考</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>对标其工业线成本</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Korenix</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>台湾</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>工业无线+交换</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>竞品(小)</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>观察</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Zyxel</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>台湾</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>○ 混合</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>商业/SMB, Nebula 云</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>竞品(云强)</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>避开云正面</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>D-Link</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>台湾</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>○ 混合</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>商业/消费/SMB</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>竞品+最大 EOL 池</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>EOL 替换重点</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>B-替换</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Advantech (EKI)</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>台湾</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>工业/嵌入式</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>竞品</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>项目配套</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Nexcom/ATOP/ICP DAS/Axiomtek</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>台湾</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>工业垂直/嵌入式</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>细分竞品</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>关注行业项目</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>CTS/Handlink/Unex/Ruby Tech/Proscend</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>台湾</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>ODM/电信接入</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>欧美运营商</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>潜在 ODM 伙伴</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>台湾产线备份</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Hirschmann (Belden)</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>工业标杆 Profinet/EN50155</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>高端锚(5-10×)</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>老项目扩容/备件/非核心网段</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Westermo (Beijer)</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>瑞典</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>● 历史平台含 Marvell</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>铁路/电力/能源 WeOS</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>高端锚</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>抢交期长的项目</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Phoenix Contact / Weidmüller / Helmholz</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>工业自动化</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>渠道型竞品</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>做其以太网模块补充</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Lancom</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>中小企业/政府/教育,云管理</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>竞品(德渠道第一梯队)</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>避开云,打本地/私有部署</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>INSYS icom / Welotec / MB connect line</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>工业远程维护</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>细分</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>配套交换机机会</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>MPL / NetModule</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>瑞士</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>高可靠/车载/铁路</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>高端锚</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>让出</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Teltonika Networks</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>立陶宛</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>○ TSW212 MSRP $129</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>工业 8G+2SFP, RMS 云</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>价格型直接对手</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>4×10G/ERPS/PoE++/DI-DO/5年保</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Nedis</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>分销商自有品牌</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>自有品牌分销, SKU 数万</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>⭐ OEM 客户池</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>无MOQ+定制UI</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Deltaco</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>瑞典</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>分销商自有品牌</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>北欧自有品牌</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>⭐ OEM 客户池</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>无MOQ+定制UI</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>LogiLink (2direct)</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>分销商自有品牌</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>自有品牌分销</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>⭐ OEM 客户池</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>无MOQ+定制UI</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Intellinet (IC Intracom)</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>美国/德国</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>分销商自有品牌</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>自有品牌网络配件</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>⭐ OEM 客户池</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>无MOQ+定制UI</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Equip / LevelOne</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>德国/台湾</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>分销商自有品牌</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>自有品牌,交换机线完整</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>⭐ OEM 客户池</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>无MOQ+定制UI</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Conrad / Reichelt / Distrelec</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>德/德/瑞士</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>大分销+自有品牌</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>分销招商采购</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>⭐ OEM 客户池</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>供应商入驻+自有品牌项目</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>StarTech.com</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>自有品牌巨头</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>配件/网络/工业</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>⭐ OEM 客户池</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>低MOQ+定制</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>ComNet (ACRE)</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>安防传输品牌</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>安防专用传输</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>竞品+互补</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>安防项目</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Antaira</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>美国(台系ODM)</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>工业,价格中低</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>直接对手</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>同价位比规格与质保</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Transition Networks</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>工业/电信接入</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>竞品</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>项目配套</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Red Lion / N-Tron / Sixnet</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>美国(HMS)</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>工业自动化</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>竞品</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>配套</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>GarrettCom (Belden)</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>工业现场/变电站</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>高端锚</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>备件/扩容</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Cambium cnMatrix</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>WISP + 云管理</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>竞品</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>WISP 场景正面打</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Ubiquiti UniFi</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>✘ Realtek(RTL93xx)</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>企业/SMB/控制器</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>最大价格对手</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>打'不想被控制器锁定'+CLI/SNMP/ERPS</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Netgear</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>商业 + AV 线(M4250/M4300)</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>竞品</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>避开 AV 线</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Perle Systems</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>工业+串口服务器+媒转</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>竞品+互补</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>RS485/DI-DO + PoE++ 补其空白</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>NEC UNIVERGE</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>● 高概率</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>政企</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>观察</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>东南亚存量替换</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Yamaha/Buffalo/Contec/Omron</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>中小企业/工业</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>观察</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Ubiquoss / DZS(Dasan)</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>韩国</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>运营商接入</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>观察</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>RAD / Telco Systems(Ribbon) / Siklu</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>以色列</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>运营商/无线</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>观察</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>MRO-TEK / Syrotech</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>印度</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>本地网络</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>中长线</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>PLI 本地化/散件</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Intelbras</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>巴西</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>品牌商(大量中国OEM)</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>安防/网络巨头</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>⭐ 潜在客户</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>外采补线</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Datacom / Furukawa 拉美</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>巴西</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>品牌商</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>运营商/企业</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>中长线</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4793,7 +7814,793 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>周期</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>动作</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>数量/频率</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>负责人</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>看什么数</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>每日</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>新进名单+打分入池</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>15-20 家</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>开发</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>新增名单</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>宁可精准300不要垃圾3000</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>每日</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn 邀请</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>15-20（每周总量≤100）</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>开发</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>接受率≥35%</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>新号前两周每天≤10</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>每日</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>首触/跟进</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>20-30</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>开发</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>回复率</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn+邮件混合</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>每日</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>处理回复</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>2 小时内</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>开发</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>超过2小时转化率腰斩</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>每日</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>更新 CRM / 明日跟进</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>下班前</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>开发</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>客户不得停在'已触达'&gt;21天</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>每周二/四</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>内容发布</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>各 1 条</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>内容</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>互动率</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>技术型 &gt; 广告型</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>每周五</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>漏斗复盘</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>1 小时</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>负责人</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>全漏斗</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>砍掉最差管道的10%动作</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>每周五</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>周报</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>1 篇</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>负责人</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>见手册附录A</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>每月</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>A 类深挖（找老板/技术总监）</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>30 家</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>开发</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>A类池 40-60 家</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>定制化技术资料</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>每月</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>线上 demo / POC 复盘</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>2 次</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>技术</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>POC 通过率</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>每月</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>案例或技术文章</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>1 篇</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>内容</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>累计12篇/年</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>每月</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>渠道价格与竞品复核</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>1 次</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>负责人</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>每季</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>展会或客户拜访</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>1 次</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>负责人</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>有效名片数</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>会前40家预约会</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>每季</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>产品-市场匹配回顾</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>1 次</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>负责人</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>缺口台账频次</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>同一需求出现3次→向SmartByte提案</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>每年</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>展会</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>2-3 次</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>负责人</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>MUM / embedded world / Intertraffic 优先</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>每年</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>与 SmartByte 年度共创会</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>1 次</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>负责人</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>新品转化数</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>把客户缺口变明年新品</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>指标</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>起步期(月)</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>稳定期(月)</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>新增名单</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>300-400</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>200-300</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>触达次数</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>500-600</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>400-500</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr"/>
+      <c r="F21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn 邀请</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>250-300</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>200-250</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>邮件发送</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>400-600</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>400-600</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr"/>
+      <c r="F23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>邀请接受率</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>≥35%</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>邮件回复率</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>≥6%</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr"/>
+      <c r="F25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>月度漏斗</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>400触达→30回复→8技术对话→6样机→8报价→1-2首单</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+      <c r="F26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>12个月目标</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>新客户15-25家(OEM 3-5家) / 出货8-15k台 / 复购率≥50%</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>预算 轻模式</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>≈ US$27k/年</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>预算 标准模式</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>≈ US$87k/年（含参展+本地BD）</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>ROI门槛</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>1个OEM客户 = 年3k台 × 毛利$15 = $45k</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr"/>
+      <c r="F30" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6668,7 +10475,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7062,7 +10869,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7626,1025 +11433,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G25"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>系列</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>型号</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>描述</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>进价 RMB</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>≈USD</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>售价 USD (+加价率)</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>备注</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>商业 L2+</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>LT-S8328XG-4XS24GT-S</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>24G + 4×SFP+ 1/2.5/10G；0~50°C；3年</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>710</v>
-      </c>
-      <c r="E2" s="3">
-        <f>IF(D2="","",ROUND(D2/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F2" s="3">
-        <f>IF(D2="","",ROUND(D2/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>对标 CSS326/CRS326 主力</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>商业 L2+</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>LT-S8328XGP-4XS24GT-S</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>24×PoE + 4×SFP+ 10G；280W</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>1010</v>
-      </c>
-      <c r="E3" s="3">
-        <f>IF(D3="","",ROUND(D3/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F3" s="3">
-        <f>IF(D3="","",ROUND(D3/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>对标 CRS328-24P（预算差）</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>商业 L2+</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>LT-S8328G-4GX24GT-S</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>24G + 4×1G/2.5G SFP</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>460</v>
-      </c>
-      <c r="E4" s="3">
-        <f>IF(D4="","",ROUND(D4/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F4" s="3">
-        <f>IF(D4="","",ROUND(D4/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G4" s="3" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>商业 L2+</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>LT-S8328GP-4GX24GT</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>24×PoE + 4×2.5G SFP；440W</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>1200</v>
-      </c>
-      <c r="E5" s="3">
-        <f>IF(D5="","",ROUND(D5/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F5" s="3">
-        <f>IF(D5="","",ROUND(D5/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G5" s="3" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>商业 L2+</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>LT-S8310G-2GX8GT</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>8G + 2×2.5G SFP</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>380</v>
-      </c>
-      <c r="E6" s="3">
-        <f>IF(D6="","",ROUND(D6/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F6" s="3">
-        <f>IF(D6="","",ROUND(D6/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>成本回落前暂停出货</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>商业 L2+</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>LT-S8310GP-2GX8GT</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>8×PoE(120W) + 2×2.5G SFP</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>450</v>
-      </c>
-      <c r="E7" s="3">
-        <f>IF(D7="","",ROUND(D7/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F7" s="3">
-        <f>IF(D7="","",ROUND(D7/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G7" s="3" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>商业 L2+</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>LT-S8352XG-4XS48GT</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>48G + 4×SFP+ 10G</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="n">
-        <v>1470</v>
-      </c>
-      <c r="E8" s="3">
-        <f>IF(D8="","",ROUND(D8/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F8" s="3">
-        <f>IF(D8="","",ROUND(D8/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>商业 L2+</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>LT-S8352XGP-4XS48GT</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>48×PoE + 4×SFP+ 10G；440W/850W</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>1870</v>
-      </c>
-      <c r="E9" s="3">
-        <f>IF(D9="","",ROUND(D9/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F9" s="3">
-        <f>IF(D9="","",ROUND(D9/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>商业 L3</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>LT-S8528XG-4XS24GT</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>24G + 4×SFP+；L3 (RIP/OSPF/IS-IS/BGP/VRRP)</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>1500</v>
-      </c>
-      <c r="E10" s="3">
-        <f>IF(D10="","",ROUND(D10/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F10" s="3">
-        <f>IF(D10="","",ROUND(D10/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>PoE 版 1900</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>商业 L3</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>LT-S8528XG-4XS16GX8GC</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>16×SFP + 8 Combo + 4×SFP+；L3</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>2100</v>
-      </c>
-      <c r="E11" s="3">
-        <f>IF(D11="","",ROUND(D11/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F11" s="3">
-        <f>IF(D11="","",ROUND(D11/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>商业 L3</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>LT-S8552XG-4XS48GT</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>48G + 4×SFP+；L3</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>2600</v>
-      </c>
-      <c r="E12" s="3">
-        <f>IF(D12="","",ROUND(D12/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F12" s="3">
-        <f>IF(D12="","",ROUND(D12/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>PoE 版 3100</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>工业 L2+</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>LT-IS6306G-2GX4GT</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>4G + 2×SFP；DIN；-40~75°C；5年</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="n">
-        <v>660</v>
-      </c>
-      <c r="E13" s="3">
-        <f>IF(D13="","",ROUND(D13/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F13" s="3">
-        <f>IF(D13="","",ROUND(D13/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>PoE 720 / PoE++ 820；Frank 6口对位</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>工业 L2+</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>LT-IS6310G-2GX8GT</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>8G + 2×2.5G SFP</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>700</v>
-      </c>
-      <c r="E14" s="3">
-        <f>IF(D14="","",ROUND(D14/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F14" s="3">
-        <f>IF(D14="","",ROUND(D14/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>PoE 780 / PoE++ 880</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>工业 L2+</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>LT-IS6312G-4GX8GT</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>8G + 4×2.5G SFP</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="n">
-        <v>740</v>
-      </c>
-      <c r="E15" s="3">
-        <f>IF(D15="","",ROUND(D15/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F15" s="3">
-        <f>IF(D15="","",ROUND(D15/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>PoE 820 / -2BT 920；Frank 12口对位</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>工业 L2+</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>LT-IS6312XG-4XS8GT</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>8G + 4×SFP+ 10G</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>840</v>
-      </c>
-      <c r="E16" s="3">
-        <f>IF(D16="","",ROUND(D16/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F16" s="3">
-        <f>IF(D16="","",ROUND(D16/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>PoE 920 / -2BT 1020</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>工业 L2+</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>LT-IS6312GP-4GX8GT-8BT</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>8×90W PoE++ (480W) + 4×2.5G SFP；52–57VDC</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="n"/>
-      <c r="E17" s="3">
-        <f>IF(D17="","",ROUND(D17/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F17" s="3">
-        <f>IF(D17="","",ROUND(D17/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>价格表未列，官网有；询价</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>工业 L2+</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>LT-IS6316XG-4XS4GX8GT</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>8G + 4×SFP + 4×SFP+</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>1400</v>
-      </c>
-      <c r="E18" s="3">
-        <f>IF(D18="","",ROUND(D18/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F18" s="3">
-        <f>IF(D18="","",ROUND(D18/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G18" s="3" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>工业 L2+</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>LT-IS6318G-2GX16GT</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>16G + 2×SFP</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>1180</v>
-      </c>
-      <c r="E19" s="3">
-        <f>IF(D19="","",ROUND(D19/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F19" s="3">
-        <f>IF(D19="","",ROUND(D19/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>PoE 1340</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>工业 L2+</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>LT-IS6318XGP-2XS16GT</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>16×PoE + 2×SFP+</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="n">
-        <v>1660</v>
-      </c>
-      <c r="E20" s="3">
-        <f>IF(D20="","",ROUND(D20/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F20" s="3">
-        <f>IF(D20="","",ROUND(D20/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>工业 L2+ DI/DO/RS485</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>LT-IS6320G-4GX16GT-D</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>16G + 4×SFP + DI/DO/RS485</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="n">
-        <v>1560</v>
-      </c>
-      <c r="E21" s="3">
-        <f>IF(D21="","",ROUND(D21/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F21" s="3">
-        <f>IF(D21="","",ROUND(D21/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>PoE 1760 / -4BT 1960；ITS/SCADA 场景</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>工业 L2+ DI/DO/RS485</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>LT-IS6328XG-4XS24GT-D</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>24G + 4×SFP+ 10G + DI/DO/RS485</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="n">
-        <v>1960</v>
-      </c>
-      <c r="E22" s="3">
-        <f>IF(D22="","",ROUND(D22/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F22" s="3">
-        <f>IF(D22="","",ROUND(D22/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>PoE 2200 / -4BT 2400</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>工业 L2+ DI/DO/RS485</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>LT-IS6328XG-4XS16GX8GC-D</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>16×SFP + 8 Combo + 4×SFP+ + DI/DO</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>2650</v>
-      </c>
-      <c r="E23" s="3">
-        <f>IF(D23="","",ROUND(D23/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F23" s="3">
-        <f>IF(D23="","",ROUND(D23/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>vs CRS328-4C-20S-4S+ $299：MikroTik 更便宜</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>工业 Bypass</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>LT-IS63xx-FBP 系列</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>光纤 Bypass 管理型</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="n">
-        <v>960</v>
-      </c>
-      <c r="E24" s="3">
-        <f>IF(D24="","",ROUND(D24/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F24" s="3">
-        <f>IF(D24="","",ROUND(D24/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>960–1640</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>工业 L3</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>LT-IS65xx 系列</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>工业 L3</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="n">
-        <v>1900</v>
-      </c>
-      <c r="E25" s="3">
-        <f>IF(D25="","",ROUND(D25/参数!$B$2,0))</f>
-        <v/>
-      </c>
-      <c r="F25" s="3">
-        <f>IF(D25="","",ROUND(D25/参数!$B$2*(1+参数!$B$3),0))</f>
-        <v/>
-      </c>
-      <c r="G25" s="3" t="inlineStr">
-        <is>
-          <t>1900–3100</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>型号</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>原 Excel 值</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>官网实测值</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>说明</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>CSS326-24G-2S+RM 芯片</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>98DX3236</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>98DX3216</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>离线库写错</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>CSS610-8G-2S+IN 芯片</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>98DX3236 / 88E6193X 两行</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>88E6193X</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>离线库与在线抓取不一致</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>CSS610-8G-2S+IN 价格</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>$89 / $119</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>$119</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>CRS326-24G-2S+RM 价格</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>$219</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>$209</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>CRS328-24P-4S+RM 价格</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>$499 / $489</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>$489</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>CRS320-8P-8B-4S+RM 价格</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>$299 / $489</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>待核实</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>两行不一致</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>RB260GSP</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>端口写成 260x GbE</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>5×GbE + 1×SFP</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>正则解析错误行，建议删除</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>整体</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>72 行含十余行重复</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>按 product_code 去重，以在线值为准</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>两种 URL slug 抓了两遍</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add A-class account quick-reference and compliance checklist sheets to workbook
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11,13 +11,15 @@
     <sheet name="替代对照表" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="竞品全景" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Marvell品牌全景" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="MikroTik全产品线" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="开发系统-节奏与KPI" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="MikroTik出口地(Comtrade2024)" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="落地价与关税" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MikroTik关键事实(实测)" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="SmartByte关键SKU" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="原Excel数据修正" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="A类客户速查" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="MikroTik全产品线" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="合规文件清单" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="开发系统-节奏与KPI" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="MikroTik出口地(Comtrade2024)" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="落地价与关税" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="MikroTik关键事实(实测)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="SmartByte关键SKU" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="原Excel数据修正" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -565,6 +567,966 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>落地价计算器（不含 VAT）。黄色格可改。美国关税 2025–2026 变动频繁，报价前按 HTS 8517.62.0020 现查。</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>参数</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>值</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>你的售价 USD (EXW/FOB)</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>海运摊销 USD/台</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>对比：CRS326 MSRP</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>对比：CSS326 MSRP</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>目的地</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>中国产 HS 8517.62 关税</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>依据（2026-09）</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>落地价 USD</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>vs CRS326</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>vs CSS326</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>打法</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>欧盟</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>ITA 信息技术协定 0%</t>
+        </is>
+      </c>
+      <c r="D9" s="3">
+        <f>ROUND(($B$3+$B$4)*(1+B9),0)</f>
+        <v/>
+      </c>
+      <c r="E9" s="14">
+        <f>D9/$B$5-1</f>
+        <v/>
+      </c>
+      <c r="F9" s="14">
+        <f>D9/$B$6-1</f>
+        <v/>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>价格+功能双打</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>ITA 0%；UKCA 你已有</t>
+        </is>
+      </c>
+      <c r="D10" s="3">
+        <f>ROUND(($B$3+$B$4)*(1+B10),0)</f>
+        <v/>
+      </c>
+      <c r="E10" s="14">
+        <f>D10/$B$5-1</f>
+        <v/>
+      </c>
+      <c r="F10" s="14">
+        <f>D10/$B$6-1</f>
+        <v/>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>价格+功能双打</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>美国（现状）</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>301 List 3 25% + 2026-07-24 起强迫劳动分级中国档 12.5%</t>
+        </is>
+      </c>
+      <c r="D11" s="3">
+        <f>ROUND(($B$3+$B$4)*(1+B11),0)</f>
+        <v/>
+      </c>
+      <c r="E11" s="14">
+        <f>D11/$B$5-1</f>
+        <v/>
+      </c>
+      <c r="F11" s="14">
+        <f>D11/$B$6-1</f>
+        <v/>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>只卖差异化：工业/PoE++/ERPS/串口/5年保修</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>美国（若叠加 10% 对华互惠层）</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="n">
+        <v>0.475</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>部分来源称对华 10% 互惠层仍在（至 2026-11-10），报关行确认</t>
+        </is>
+      </c>
+      <c r="D12" s="3">
+        <f>ROUND(($B$3+$B$4)*(1+B12),0)</f>
+        <v/>
+      </c>
+      <c r="E12" s="14">
+        <f>D12/$B$5-1</f>
+        <v/>
+      </c>
+      <c r="F12" s="14">
+        <f>D12/$B$6-1</f>
+        <v/>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>澳大利亚</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>ChAFTA 0%；需 RCM</t>
+        </is>
+      </c>
+      <c r="D13" s="3">
+        <f>ROUND(($B$3+$B$4)*(1+B13),0)</f>
+        <v/>
+      </c>
+      <c r="E13" s="14">
+        <f>D13/$B$5-1</f>
+        <v/>
+      </c>
+      <c r="F13" s="14">
+        <f>D13/$B$6-1</f>
+        <v/>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>价格+功能</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>阿联酋</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>GCC 统一关税 5%（部分 IT 设备 0%）</t>
+        </is>
+      </c>
+      <c r="D14" s="3">
+        <f>ROUND(($B$3+$B$4)*(1+B14),0)</f>
+        <v/>
+      </c>
+      <c r="E14" s="14">
+        <f>D14/$B$5-1</f>
+        <v/>
+      </c>
+      <c r="F14" s="14">
+        <f>D14/$B$6-1</f>
+        <v/>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>枢纽分销商 house brand</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>MFN 0%，无 301</t>
+        </is>
+      </c>
+      <c r="D15" s="3">
+        <f>ROUND(($B$3+$B$4)*(1+B15),0)</f>
+        <v/>
+      </c>
+      <c r="E15" s="14">
+        <f>D15/$B$5-1</f>
+        <v/>
+      </c>
+      <c r="F15" s="14">
+        <f>D15/$B$6-1</f>
+        <v/>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>随美国客户但价格优势保留</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>土耳其</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>欧盟关税同盟，ITA 0%（另有本地附加税，需核）</t>
+        </is>
+      </c>
+      <c r="D16" s="3">
+        <f>ROUND(($B$3+$B$4)*(1+B16),0)</f>
+        <v/>
+      </c>
+      <c r="E16" s="14">
+        <f>D16/$B$5-1</f>
+        <v/>
+      </c>
+      <c r="F16" s="14">
+        <f>D16/$B$6-1</f>
+        <v/>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>复制 NMS 案例</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>负数 = 比 MikroTik 便宜；正数 = 比 MikroTik 贵。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>项目</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>CSS326-24G-2S+RM</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>CRS326-24G-2S+RM</t>
+        </is>
+      </c>
+      <c r="D1" s="5" t="inlineStr">
+        <is>
+          <t>CRS328-24P-4S+RM</t>
+        </is>
+      </c>
+      <c r="E1" s="5" t="inlineStr">
+        <is>
+          <t>CSS610-8G-2S+IN</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>来源</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>MSRP</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>$159</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>$209</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>$489</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>$119</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>mikrotik.com 产品页 2026-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>操作系统</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>SwOS only (v2.19)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS L5 / SwOS 双启动 (7.24.4)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS L5 / SwOS 双启动</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>SwOS Lite (v2.21)</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>交换芯片</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>98DX3216</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>98DX3236</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>98DX3236</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>88E6193X</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>CPU / RAM / Flash</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>— / — / 2MB</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>ARM 2×800MHz / 512MB / 16MB</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>ARM 1×800MHz / 512MB / 16MB</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>— / — / 64KB</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>端口</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>24G + 2×SFP+</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>24G + 2×SFP+</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>24×PoE-out af/at + 4×SFP+</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>8G + 2×SFP+</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>PoE-out</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>450W 总预算(3×150W/8口)，30W/口，无 802.3bt</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Console</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>RJ45</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>RJ45</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>温度</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>-20~70°C</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>-40~60°C</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>-20~60°C</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>-20~60°C</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>供电</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>10–30V DC jack / 被动 PoE-in</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>10–30V DC jack / 被动 PoE-in</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>内置 500W PSU</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>12–57V DC / 被动 PoE-in</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>认证</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>CE, EAC, RoHS</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>CE, EAC, RoHS</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>CE, EAC, RoHS</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>CE, EAC, RoHS</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>同上（均无 UL/FCC 列出）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>MTBF</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>~200k h @25°C</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>~200k h</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>~200k h</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>~200k h</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>软件更新承诺</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>产品寿命或≥5年免费更新</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>同左</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>同左</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>同左</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>同上</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>SwOS 限制(CSS/SwOS 模式)</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>仅 RSTP；≤250 VLAN；≤32 ACL；16 LAG；IGMP snooping；只有入向限速；仅 Web 管理(无 CLI/SSH)；无默认网关；仅 IPv4；无 LLDP(MNDP)；SNMP v1/v2c 只读、无 Trap</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>同 CSS326 (SwOS Lite 更弱)</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>help.mikrotik.com SwOS CRS3xx/CSS3xx 手册</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS on CRS3xx 能力</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>单硬件 bridge；STP/RSTP/MSTP 硬件；Q-in-Q 802.1ad 硬件卸载(v6.43+)；LACP/balance-xor 硬件；switch-rule ACL；L3 HW offload 基础路由(98DX3236)，不支持 NAT/Fasttrack 卸载，需在 HW 路由与 HW 防火墙间二选一</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>同左</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>help.mikrotik.com CRS3xx &amp; L3 HW Offloading</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>ERPS G.8032</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>无（论坛 feature request 自 2013 年起未实现，用户反映大环 RSTP 收敛 ~4s）</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>无</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>forum.mikrotik.com/t/71183, /t/84795</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS 强项(承认)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>API、REST API(v7.1+)、脚本、Winbox、The Dude、bandwidth-test/traffic-generator、LLDP/CDP/MNDP</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>同左</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>RouterOS 文档</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1377,7 +2339,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5818,6 +6780,684 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>公司</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>国家</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>主入口/联系方式</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>现有交换机线</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>⭐缺口</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>首推 SKU</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>第一句话钩子</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>最大风险</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Digital Data Communications (LevelOne/equip)</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>德国 Dortmund</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn（Group CEO Amanda Chen）+ 官网；制造在台湾&amp;中国</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>LevelOne PoE 交换机/媒转/AP，多为非管理与 web-smart</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>缺可管理 L2+ / L3 汇聚 / 工业宽温</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG + LT-IS6312XG</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>你们的 PoE 线最强，但停在 web-smart</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>他们自己也做 ODM 服务，可能视你为竞争</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>2direct GmbH (LogiLink)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>德国 Schalksmühle</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>官网 kontakt；Langenstück 5, D-58579</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>LogiLink 网络线以配件/非管理为主</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>缺可管理 L2+ 与工业线</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>全系贴牌阶梯</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>你们公开说做 OEM 项目</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>价格敏感，需给阶梯价</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>⭐⭐⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Nedis</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>nedis.com/en-us/business/become-a-partner 表单</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>8口千兆非管理(NSWH8P100BK)、8口PoE 150W(GS-1008P)、部分贴 Edimax</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>几乎只有非管理/SOHO</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>8/16/24口 PoE+ 贴牌</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>你们贴牌覆盖所有品类，交换机只有非管理</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>决策慢，需走品类经理</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>⭐⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Distrelec (RS Group, 自有品牌 RND)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>瑞士/欧洲</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Supplier onboarding</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>RND 以无源/仪器/元件为主</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>缺有源网络（可管理/工业以太网）</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>工业线 + 可管理</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>RND 缺有源网络这一层</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>供应商准入流程长</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>⭐⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Conrad Electronic</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>platform.conrad.de → Become a Seller（Mirakl 平台，已有650+卖家）</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>分销 + 自有品牌</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>需德语内容/EAN/CE/WEEE/LUCID</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>自有品牌上架（最快出单）</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>4-8周即可上平台出单</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>需德语产品数据与德国合规号</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>⭐⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>IC Intracom (Intellinet/Manhattan)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>德国 Halver / 美国 FL</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>sales@intellinetnetwork.eu；+49 2353 7007 0；WEEE DE40753042 / LUCID DE2489084505093</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Intellinet 可管理偏少，多为非管理与 web-smart PoE</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>缺可管理 L2+ / PoE++ / 工业</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>可管理 L2+ + 工业线</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>你们亚洲有 QC、欧盟合规号齐全，沟通成本最低</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>他们已有亚洲供应</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>⭐⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Deltaco (DistIT → Aurdel)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>瑞典</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>官网 B2B</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>含 switches/转换器/光纤，偏北欧零售 SOHO</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>可管理 PoE 与工业线薄弱</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>北欧 PoE+ / 工业线</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>从台湾进口到自有品牌的这条路我们熟</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>集团合并期，决策链变化</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>StarTech.com</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>加拿大多伦多</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>官网供应商入口（⚠️ 不要发冷邮件，CASL）</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>IES61002POE / IES81000PoE(TAA) / IESC1G50UP / IES1G52UPDIN / IES5102 —— 全部非管理</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>没有可管理工业交换机、无 PoE++、无环网</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>可管理工业线</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>你们的工业交换机全是非管理型</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>⚠️ TAA SKU 不能碰（中国原产）</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Intelbras</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>巴西</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Amilcar Scheffer（网络方案与产品总监）/ Elton Thiesen（企业线经理）</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>SG 5204 MR L2+、S3028G-PB Max(L3,380W)、SG 2404 PoE L2+ 等；与 H3C 合作本地化生产</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>接入层低价位 / PoE++ / 工业宽温；SKD/CKD 机会</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>接入层 + SKD/CKD 散件</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>H3C 覆盖核心，接入层与本地组装是空间</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>H3C 关系深；需葡语与 ANATEL 确认</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>⭐</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Antaira</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>美国(台系供应链)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>其合作方：Switch SFP(UK)、Things Embedded</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>工业以太网为主</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>同价位下规格与质保</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>4×10G + PoE++ + ERPS</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>项目要更大规格时他们够不着</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>主要是竞品；打其渠道</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>ComNet (ACRE)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>美国 Danbury CT</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>+1 203 796 5300；comnetcustomercare@acresecurity.com</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>光纤/铜缆/无线传输，有限终身质保，IEC61850-3 产品线</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>ITS/电力集成商渠道；非核心网段第二供应源</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>ITS 与电力项目配套</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>打其下游集成商</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>美国本土制造，本地保护</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Teltonika Networks</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>立陶宛</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>其各国分销商（如英国 Diamond 分销商 Millbeck）</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>TSW202/TSW212（8×GE+2SFP，8K MAC/512KB，MSRP $129），开放 SDK 可自写固件</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>无 10G 上行、无 PoE++、无 ERPS、只有 8 口</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG 正面对冲</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>8 口以上他们没有</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>有 SDK + RMS 云，工程师粘性高</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -7814,7 +9454,1073 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>文件/证书</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>适用地区</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>必备性</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>谁出具</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>你目前状态</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>怎么补</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>对客户的价值</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>EN 55032 / EN 55035 EMC 测试报告</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>EU/UK</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>必备</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>第三方实验室</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>需向 SmartByte 要带型号的完整报告</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>向工厂索取原件，核对型号/日期/实验室资质</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>CE 与 UKCA 的技术基础</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>EN IEC 62368-1 安全测试报告（LVD）</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>EU/UK</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>必备</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>第三方实验室</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>需确认是 62368-1 而非 60950-1</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>索取；若仍是旧标准需补测</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>客户合规部第一件事就是查这个</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>RoHS 10 项检测报告 + EN IEC 63000 技术文档</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>EU/UK</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>必备</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>实验室</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>有声明，需报告原件</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>索取报告原件</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>无报告=无 CE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>REACH SVHC 声明 / SCIP 通报数据</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>必备</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>供应链</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>⚠️ SCIP 多半没有</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>要 SVHC 清单；&gt;0.1% 需物料数据</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>缺少会被海关/市场监管拦下</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>EU DoC（欧盟符合性声明）模板</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>必备</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>制造商（贴牌客户）</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>需工厂提供可改写模板</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>向工厂要模板 + 客户签署</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>没有 DoC 就不能贴 CE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>EU Authorised Representative（欧盟授权代表）</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>必备（非欧盟制造商）</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>客户指定</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>由客户承担</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>可协助对接第三方 AR 服务（增值）</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>OEM 谈判最常见的断点</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>WEEE 注册号（DE stiftung ear / FR / IT / ES / NL / SE / PL BDO）</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>EU各国</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>必备</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>客户（品牌方）</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>客户持有</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>我们提供型号重量与材料拆分数据</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>没有注册号不能在该国销售</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>包装法：德国 VerpackG LUCID + 双元系统；法国 EPR；PPWR (EU)2025/40</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>必备</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>客户</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>客户持有</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>我们提供包装材料与重量数据</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>德国查得最严</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>ErP (EU)2019/1782 外置电源能效（等同 DoE Level VI）</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>EU/US</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>带适配器时必备</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>实验室</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>需确认适配器证书</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>索取适配器证书</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>外置电源没证=整机不能上架</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>CRA (EU)2024/2847 技术文档（交换机=Annex III Class I）</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>2027-12-11 起必备</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>制造商（客户）+ 我们提供输入</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>⚠️ 基本空白</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>SBOM + 漏洞政策 + 更新承诺 + EN 18031 路线图</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>⭐ 2026-2027 最有杀伤力的差异化</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>SBOM（SPDX / CycloneDX）</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>EU/UK/US</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>CRA 必备</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>工厂</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>⚠️ 没有</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>向工厂索取并约定每版更新</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>客户合规部无法自行生成</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>漏洞处理政策（接收渠道/响应SLA/协调披露）</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>CRA 必备</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>工厂 + 我们</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>⚠️ 没有</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>起草 policy + security@ 邮箱 + 响应时限</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>24h/72h 通报义务的基础</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>固件签名 / 安全启动说明</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>CRA 安全默认要求</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>工厂</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>需确认</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>向工厂确认并出书面说明</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Class I 自评估的关键项</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>固件更新支持期承诺（建议≥5年）</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>EU/全球</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>商业必备</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>你 + 工厂</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>需书面化</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>写进合同附件</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>大客户问卷必问</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>EN 18031 系列符合性路线图</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>决定能否走 Module A 自评</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>第三方/自评</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>⚠️ 没有</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>做差距分析（gap analysis）</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>有则可自评（省钱），无则第三方评估（费钱）</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>UKCA + UK Responsible Person + UK DoC</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>必备</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>客户 + 我们协助</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>CE 在英有过渡安排（以英国政府公告为准）</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>按 UKCA 要求准备，UKRP 由客户指定</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>英国客户必查</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>FCC Part 15B SDoC（Class A/B）</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>必备</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>实验室/供方自我声明</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>有 FCC</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>核对 Class A/B 与型号</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>无则不能进美国</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>UL / ETL 62368-1</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>美国/加拿大</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>事实必备（非联邦强制）</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>第三方</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>⚠️ 还没有</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>按首单量谈判分摊送测费用</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>分销商与验收方几乎必要求</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>ISED ICES-003 + CSA/cUL/ETL 安全标志</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>必备</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>第三方</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>需确认</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>ICES-003 通常可沿用 FCC 报告；安全标志需补</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>魁北克还需法语标签（Bill 96）</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>TAA 合规（美国联邦采购）</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>政府项目必备</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>❌ 中国原产不可能 TAA</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>不碰政府单，只做商用渠道</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>提前说清，避免浪费时间</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>NDAA 889 排除声明（非华为/中兴/海康/大华等）</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>关键项目必备</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>你出具</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>可出具</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>准备一份标准声明</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Marvell 方案不在受限清单</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>EN 50155（轨交）/ IEC 61850-3（电力）/ IEC 62443-4-2（工控安全）/ EN 45545-2 / E-mark</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>EU 行业</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>项目要求</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>第三方</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>❌ 基本没有</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>短期不做铁路/车载；攻工厂/ITS/CCTV/楼宇</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>坦诚说明，不要硬接</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>产品重量与材料拆分表（WEEE 申报用）</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>必备</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>工厂</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>需索取</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>逐型号整理成表</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>客户申报 WEEE 的必需输入</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>ISO 9001 / ISO 14001 证书</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>全球</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>大客户问卷必问</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>工厂</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>需索取</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>索取证书与审核报告摘要</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>问卷里的第一道门槛</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>产品责任保险</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>EU/US</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>大客户常要求</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>客户/双方</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>需确认</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>客户投保或双方共保</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>贴牌客户作为制造商通常需要</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8600,7 +11306,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10473,964 +13179,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>落地价计算器（不含 VAT）。黄色格可改。美国关税 2025–2026 变动频繁，报价前按 HTS 8517.62.0020 现查。</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>参数</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>值</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>你的售价 USD (EXW/FOB)</t>
-        </is>
-      </c>
-      <c r="B3" s="11" t="n">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>海运摊销 USD/台</t>
-        </is>
-      </c>
-      <c r="B4" s="11" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>对比：CRS326 MSRP</t>
-        </is>
-      </c>
-      <c r="B5" s="11" t="n">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>对比：CSS326 MSRP</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="n">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>目的地</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>中国产 HS 8517.62 关税</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>依据（2026-09）</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>落地价 USD</t>
-        </is>
-      </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>vs CRS326</t>
-        </is>
-      </c>
-      <c r="F8" s="12" t="inlineStr">
-        <is>
-          <t>vs CSS326</t>
-        </is>
-      </c>
-      <c r="G8" s="12" t="inlineStr">
-        <is>
-          <t>打法</t>
-        </is>
-      </c>
-      <c r="H8" s="12" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>欧盟</t>
-        </is>
-      </c>
-      <c r="B9" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>ITA 信息技术协定 0%</t>
-        </is>
-      </c>
-      <c r="D9" s="3">
-        <f>ROUND(($B$3+$B$4)*(1+B9),0)</f>
-        <v/>
-      </c>
-      <c r="E9" s="14">
-        <f>D9/$B$5-1</f>
-        <v/>
-      </c>
-      <c r="F9" s="14">
-        <f>D9/$B$6-1</f>
-        <v/>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>价格+功能双打</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>英国</t>
-        </is>
-      </c>
-      <c r="B10" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>ITA 0%；UKCA 你已有</t>
-        </is>
-      </c>
-      <c r="D10" s="3">
-        <f>ROUND(($B$3+$B$4)*(1+B10),0)</f>
-        <v/>
-      </c>
-      <c r="E10" s="14">
-        <f>D10/$B$5-1</f>
-        <v/>
-      </c>
-      <c r="F10" s="14">
-        <f>D10/$B$6-1</f>
-        <v/>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>价格+功能双打</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>美国（现状）</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>301 List 3 25% + 2026-07-24 起强迫劳动分级中国档 12.5%</t>
-        </is>
-      </c>
-      <c r="D11" s="3">
-        <f>ROUND(($B$3+$B$4)*(1+B11),0)</f>
-        <v/>
-      </c>
-      <c r="E11" s="14">
-        <f>D11/$B$5-1</f>
-        <v/>
-      </c>
-      <c r="F11" s="14">
-        <f>D11/$B$6-1</f>
-        <v/>
-      </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>只卖差异化：工业/PoE++/ERPS/串口/5年保修</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>美国（若叠加 10% 对华互惠层）</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="n">
-        <v>0.475</v>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>部分来源称对华 10% 互惠层仍在（至 2026-11-10），报关行确认</t>
-        </is>
-      </c>
-      <c r="D12" s="3">
-        <f>ROUND(($B$3+$B$4)*(1+B12),0)</f>
-        <v/>
-      </c>
-      <c r="E12" s="14">
-        <f>D12/$B$5-1</f>
-        <v/>
-      </c>
-      <c r="F12" s="14">
-        <f>D12/$B$6-1</f>
-        <v/>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>同上</t>
-        </is>
-      </c>
-      <c r="H12" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>澳大利亚</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>ChAFTA 0%；需 RCM</t>
-        </is>
-      </c>
-      <c r="D13" s="3">
-        <f>ROUND(($B$3+$B$4)*(1+B13),0)</f>
-        <v/>
-      </c>
-      <c r="E13" s="14">
-        <f>D13/$B$5-1</f>
-        <v/>
-      </c>
-      <c r="F13" s="14">
-        <f>D13/$B$6-1</f>
-        <v/>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>价格+功能</t>
-        </is>
-      </c>
-      <c r="H13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>阿联酋</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>GCC 统一关税 5%（部分 IT 设备 0%）</t>
-        </is>
-      </c>
-      <c r="D14" s="3">
-        <f>ROUND(($B$3+$B$4)*(1+B14),0)</f>
-        <v/>
-      </c>
-      <c r="E14" s="14">
-        <f>D14/$B$5-1</f>
-        <v/>
-      </c>
-      <c r="F14" s="14">
-        <f>D14/$B$6-1</f>
-        <v/>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>枢纽分销商 house brand</t>
-        </is>
-      </c>
-      <c r="H14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>加拿大</t>
-        </is>
-      </c>
-      <c r="B15" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>MFN 0%，无 301</t>
-        </is>
-      </c>
-      <c r="D15" s="3">
-        <f>ROUND(($B$3+$B$4)*(1+B15),0)</f>
-        <v/>
-      </c>
-      <c r="E15" s="14">
-        <f>D15/$B$5-1</f>
-        <v/>
-      </c>
-      <c r="F15" s="14">
-        <f>D15/$B$6-1</f>
-        <v/>
-      </c>
-      <c r="G15" s="3" t="inlineStr">
-        <is>
-          <t>随美国客户但价格优势保留</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>土耳其</t>
-        </is>
-      </c>
-      <c r="B16" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>欧盟关税同盟，ITA 0%（另有本地附加税，需核）</t>
-        </is>
-      </c>
-      <c r="D16" s="3">
-        <f>ROUND(($B$3+$B$4)*(1+B16),0)</f>
-        <v/>
-      </c>
-      <c r="E16" s="14">
-        <f>D16/$B$5-1</f>
-        <v/>
-      </c>
-      <c r="F16" s="14">
-        <f>D16/$B$6-1</f>
-        <v/>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>复制 NMS 案例</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>负数 = 比 MikroTik 便宜；正数 = 比 MikroTik 贵。</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="inlineStr">
-        <is>
-          <t>项目</t>
-        </is>
-      </c>
-      <c r="B1" s="5" t="inlineStr">
-        <is>
-          <t>CSS326-24G-2S+RM</t>
-        </is>
-      </c>
-      <c r="C1" s="5" t="inlineStr">
-        <is>
-          <t>CRS326-24G-2S+RM</t>
-        </is>
-      </c>
-      <c r="D1" s="5" t="inlineStr">
-        <is>
-          <t>CRS328-24P-4S+RM</t>
-        </is>
-      </c>
-      <c r="E1" s="5" t="inlineStr">
-        <is>
-          <t>CSS610-8G-2S+IN</t>
-        </is>
-      </c>
-      <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>来源</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>MSRP</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>$159</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>$209</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>$489</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>$119</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>mikrotik.com 产品页 2026-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>操作系统</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>SwOS only (v2.19)</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>RouterOS L5 / SwOS 双启动 (7.24.4)</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>RouterOS L5 / SwOS 双启动</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>SwOS Lite (v2.21)</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>同上</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>交换芯片</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>98DX3216</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>98DX3236</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>98DX3236</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>88E6193X</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>同上</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>CPU / RAM / Flash</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>— / — / 2MB</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>ARM 2×800MHz / 512MB / 16MB</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>ARM 1×800MHz / 512MB / 16MB</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>— / — / 64KB</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>同上</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>端口</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>24G + 2×SFP+</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>24G + 2×SFP+</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>24×PoE-out af/at + 4×SFP+</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>8G + 2×SFP+</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>同上</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>PoE-out</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>450W 总预算(3×150W/8口)，30W/口，无 802.3bt</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>同上</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Console</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>RJ45</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>RJ45</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>同上</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>温度</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>-20~70°C</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>-40~60°C</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>-20~60°C</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>-20~60°C</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>同上</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>供电</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>10–30V DC jack / 被动 PoE-in</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>10–30V DC jack / 被动 PoE-in</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>内置 500W PSU</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>12–57V DC / 被动 PoE-in</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>同上</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>认证</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>CE, EAC, RoHS</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>CE, EAC, RoHS</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>CE, EAC, RoHS</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>CE, EAC, RoHS</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>同上（均无 UL/FCC 列出）</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>MTBF</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>~200k h @25°C</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>~200k h</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>~200k h</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>~200k h</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>同上</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>软件更新承诺</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>产品寿命或≥5年免费更新</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>同左</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>同左</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>同左</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>同上</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>SwOS 限制(CSS/SwOS 模式)</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>仅 RSTP；≤250 VLAN；≤32 ACL；16 LAG；IGMP snooping；只有入向限速；仅 Web 管理(无 CLI/SSH)；无默认网关；仅 IPv4；无 LLDP(MNDP)；SNMP v1/v2c 只读、无 Trap</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr">
-        <is>
-          <t>同 CSS326 (SwOS Lite 更弱)</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>help.mikrotik.com SwOS CRS3xx/CSS3xx 手册</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>RouterOS on CRS3xx 能力</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>单硬件 bridge；STP/RSTP/MSTP 硬件；Q-in-Q 802.1ad 硬件卸载(v6.43+)；LACP/balance-xor 硬件；switch-rule ACL；L3 HW offload 基础路由(98DX3236)，不支持 NAT/Fasttrack 卸载，需在 HW 路由与 HW 防火墙间二选一</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>同左</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>help.mikrotik.com CRS3xx &amp; L3 HW Offloading</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>ERPS G.8032</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>无（论坛 feature request 自 2013 年起未实现，用户反映大环 RSTP 收敛 ~4s）</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>无</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>forum.mikrotik.com/t/71183, /t/84795</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>RouterOS 强项(承认)</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>API、REST API(v7.1+)、脚本、Winbox、The Dude、bandwidth-test/traffic-generator、LLDP/CDP/MNDP</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>同左</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>RouterOS 文档</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add key-account deep-dive with neutral-shipping playbook and SmartByte pricing ladder
Rewritten for a small trader: micro budgets (2k/5k/10k USD), neutral/OEM
shipping with US 19 U.S.C. 1304 and EU 2019/1020 origin-marking limits,
Taiwan brands used only as a lead-source signal (reverse-lookup search
strings), seven concrete routes into well-known own-brand distributors,
six deep account profiles (ASSMANN/DIGITUS, DDC LevelOne, 2direct LogiLink,
Nedis, IC Intracom, Intos InLine incl. verified addresses, phone, named
contacts), second-tier target list, full SmartByte price-to-sell ladder,
90-day plan and KP-hunting SOP
- Workbook: new sheet '重点客户配货表'

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -12,14 +12,15 @@
     <sheet name="竞品全景" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Marvell品牌全景" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="A类客户速查" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="MikroTik全产品线" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="合规文件清单" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="开发系统-节奏与KPI" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="MikroTik出口地(Comtrade2024)" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="落地价与关税" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="MikroTik关键事实(实测)" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="SmartByte关键SKU" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="原Excel数据修正" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="重点客户配货表" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="MikroTik全产品线" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="合规文件清单" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="开发系统-节奏与KPI" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="MikroTik出口地(Comtrade2024)" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="落地价与关税" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="MikroTik关键事实(实测)" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="SmartByte关键SKU" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="原Excel数据修正" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -567,6 +568,1881 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G78"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="45" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>说明：UN Comtrade，Reporter=Latvia(428)，HS 851762（交换/路由设备），Export，2024，FOB USD。MikroTik 占拉脱维亚该税号出口 3/4 以上，可视为 MikroTik 分销商进货地图。全球合计 USD 422,324,814。</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>排名</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>国家/地区</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>M49 代码</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>区域</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>出口额 USD</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>占全球 %</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>842</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>北美</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>50994438</v>
+      </c>
+      <c r="F3" s="8">
+        <f>E3/422324814</f>
+        <v/>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>对华关税约 37.5%（2026-09）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>阿联酋(转口枢纽)</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>784</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>中东/土耳其</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>43018484</v>
+      </c>
+      <c r="F4" s="8">
+        <f>E4/422324814</f>
+        <v/>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>转口枢纽→中东/非洲/南亚</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>616</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>34368342</v>
+      </c>
+      <c r="F5" s="8">
+        <f>E5/422324814</f>
+        <v/>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>欧洲第一 MikroTik 国</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>立陶宛(波罗的海分销枢纽)</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>440</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>32525290</v>
+      </c>
+      <c r="F6" s="8">
+        <f>E6/422324814</f>
+        <v/>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>波罗的海分销枢纽</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>203</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>21822977</v>
+      </c>
+      <c r="F7" s="8">
+        <f>E7/422324814</f>
+        <v/>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>WISP 密度极高</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>276</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>16002618</v>
+      </c>
+      <c r="F8" s="8">
+        <f>E8/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>中国香港(转口枢纽)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>344</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>15962714</v>
+      </c>
+      <c r="F9" s="8">
+        <f>E9/422324814</f>
+        <v/>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>转口枢纽→东南亚/南亚</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>南非</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>710</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>非洲</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>11426199</v>
+      </c>
+      <c r="F10" s="8">
+        <f>E10/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>印度尼西亚</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>360</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>11250898</v>
+      </c>
+      <c r="F11" s="8">
+        <f>E11/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>哈萨克斯坦</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>398</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>独联体/中亚</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>10925270</v>
+      </c>
+      <c r="F12" s="8">
+        <f>E12/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>826</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>8784753</v>
+      </c>
+      <c r="F13" s="8">
+        <f>E13/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>爱沙尼亚</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>233</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>8754532</v>
+      </c>
+      <c r="F14" s="8">
+        <f>E14/422324814</f>
+        <v/>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>波罗的海分销枢纽</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>804</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>8206878</v>
+      </c>
+      <c r="F15" s="8">
+        <f>E15/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>380</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>8186541</v>
+      </c>
+      <c r="F16" s="8">
+        <f>E16/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>土耳其</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>792</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>中东/土耳其</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>7652474</v>
+      </c>
+      <c r="F17" s="8">
+        <f>E17/422324814</f>
+        <v/>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>你已有 NMS 客户</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>724</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="n">
+        <v>7284155</v>
+      </c>
+      <c r="F18" s="8">
+        <f>E18/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>528</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>6532562</v>
+      </c>
+      <c r="F19" s="8">
+        <f>E19/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>巴西</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>76</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>拉美</t>
+        </is>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>5655456</v>
+      </c>
+      <c r="F20" s="8">
+        <f>E20/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>奥地利</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>40</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>4567730</v>
+      </c>
+      <c r="F21" s="8">
+        <f>E21/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>新加坡</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>702</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>4496379</v>
+      </c>
+      <c r="F22" s="8">
+        <f>E22/422324814</f>
+        <v/>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>转口枢纽</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>中国大陆</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>156</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>4493322</v>
+      </c>
+      <c r="F23" s="8">
+        <f>E23/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>124</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>北美</t>
+        </is>
+      </c>
+      <c r="E24" s="7" t="n">
+        <v>4469245</v>
+      </c>
+      <c r="F24" s="8">
+        <f>E24/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>哥伦比亚</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>170</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>拉美</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>3752926</v>
+      </c>
+      <c r="F25" s="8">
+        <f>E25/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>保加利亚</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>100</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>3606615</v>
+      </c>
+      <c r="F26" s="8">
+        <f>E26/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>澳大利亚</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>36</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>3596152</v>
+      </c>
+      <c r="F27" s="8">
+        <f>E27/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>匈牙利</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>348</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="n">
+        <v>3207035</v>
+      </c>
+      <c r="F28" s="8">
+        <f>E28/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>瑞典</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>752</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="n">
+        <v>3137243</v>
+      </c>
+      <c r="F29" s="8">
+        <f>E29/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>越南</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>704</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>2733552</v>
+      </c>
+      <c r="F30" s="8">
+        <f>E30/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>智利</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>152</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>拉美</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>2721330</v>
+      </c>
+      <c r="F31" s="8">
+        <f>E31/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>秘鲁</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>604</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>拉美</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="n">
+        <v>2713158</v>
+      </c>
+      <c r="F32" s="8">
+        <f>E32/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>泰国</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>764</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="n">
+        <v>2464546</v>
+      </c>
+      <c r="F33" s="8">
+        <f>E33/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>300</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="n">
+        <v>2308883</v>
+      </c>
+      <c r="F34" s="8">
+        <f>E34/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>丹麦</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>208</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="n">
+        <v>2239002</v>
+      </c>
+      <c r="F35" s="8">
+        <f>E35/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>墨西哥</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>484</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>拉美</t>
+        </is>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>2183194</v>
+      </c>
+      <c r="F36" s="8">
+        <f>E36/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>阿根廷</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>32</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>拉美</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="n">
+        <v>1858335</v>
+      </c>
+      <c r="F37" s="8">
+        <f>E37/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>罗马尼亚</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>642</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E38" s="7" t="n">
+        <v>1844544</v>
+      </c>
+      <c r="F38" s="8">
+        <f>E38/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>新西兰</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>554</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="n">
+        <v>1696031</v>
+      </c>
+      <c r="F39" s="8">
+        <f>E39/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>孟加拉国</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>50</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="n">
+        <v>1099842</v>
+      </c>
+      <c r="F40" s="8">
+        <f>E40/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>斯洛伐克</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>703</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="n">
+        <v>1068939</v>
+      </c>
+      <c r="F41" s="8">
+        <f>E41/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>塞尔维亚</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>688</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E42" s="7" t="n">
+        <v>1057170</v>
+      </c>
+      <c r="F42" s="8">
+        <f>E42/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>马来西亚</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>458</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="n">
+        <v>996768</v>
+      </c>
+      <c r="F43" s="8">
+        <f>E43/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>斯洛文尼亚</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>705</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E44" s="7" t="n">
+        <v>951791</v>
+      </c>
+      <c r="F44" s="8">
+        <f>E44/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>肯尼亚</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>404</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>非洲</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="n">
+        <v>934046</v>
+      </c>
+      <c r="F45" s="8">
+        <f>E45/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>葡萄牙</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>620</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E46" s="7" t="n">
+        <v>927187</v>
+      </c>
+      <c r="F46" s="8">
+        <f>E46/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>克罗地亚</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>191</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="n">
+        <v>881827</v>
+      </c>
+      <c r="F47" s="8">
+        <f>E47/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>芬兰</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>246</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="n">
+        <v>843078</v>
+      </c>
+      <c r="F48" s="8">
+        <f>E48/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>乌兹别克斯坦</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>860</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>独联体/中亚</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="n">
+        <v>802640</v>
+      </c>
+      <c r="F49" s="8">
+        <f>E49/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>沙特</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>682</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>中东/土耳其</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="n">
+        <v>800914</v>
+      </c>
+      <c r="F50" s="8">
+        <f>E50/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>比利时</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>56</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="n">
+        <v>706207</v>
+      </c>
+      <c r="F51" s="8">
+        <f>E51/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>巴基斯坦</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>586</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="n">
+        <v>632718</v>
+      </c>
+      <c r="F52" s="8">
+        <f>E52/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>格鲁吉亚</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>268</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>独联体/中亚</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="n">
+        <v>612616</v>
+      </c>
+      <c r="F53" s="8">
+        <f>E53/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>中国台湾</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>490</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="n">
+        <v>601808</v>
+      </c>
+      <c r="F54" s="8">
+        <f>E54/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>阿尔巴尼亚</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>8</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="n">
+        <v>551402</v>
+      </c>
+      <c r="F55" s="8">
+        <f>E55/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>韩国</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>410</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="n">
+        <v>465113</v>
+      </c>
+      <c r="F56" s="8">
+        <f>E56/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>392</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="n">
+        <v>430801</v>
+      </c>
+      <c r="F57" s="8">
+        <f>E57/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>菲律宾</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>608</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="n">
+        <v>381036</v>
+      </c>
+      <c r="F58" s="8">
+        <f>E58/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>爱尔兰</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>372</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="n">
+        <v>357037</v>
+      </c>
+      <c r="F59" s="8">
+        <f>E59/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>58</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>埃及</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>818</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>非洲</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="n">
+        <v>345877</v>
+      </c>
+      <c r="F60" s="8">
+        <f>E60/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>以色列</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>376</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>中东/土耳其</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="n">
+        <v>273731</v>
+      </c>
+      <c r="F61" s="8">
+        <f>E61/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>阿塞拜疆</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>31</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>独联体/中亚</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="n">
+        <v>273435</v>
+      </c>
+      <c r="F62" s="8">
+        <f>E62/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>尼日利亚</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>566</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>非洲</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="n">
+        <v>265052</v>
+      </c>
+      <c r="F63" s="8">
+        <f>E63/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>62</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>安哥拉</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>24</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>非洲</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="n">
+        <v>93579</v>
+      </c>
+      <c r="F64" s="8">
+        <f>E64/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>63</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>白俄罗斯</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>112</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>独联体/中亚</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="n">
+        <v>3144</v>
+      </c>
+      <c r="F65" s="8">
+        <f>E65/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>其他未查询国家（合计约 90 国）</t>
+        </is>
+      </c>
+      <c r="E66" s="7">
+        <f>422324814-SUM(E3:E65)</f>
+        <v/>
+      </c>
+      <c r="F66" s="8">
+        <f>E66/422324814</f>
+        <v/>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>余量</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="inlineStr"/>
+      <c r="B67" s="1" t="inlineStr">
+        <is>
+          <t>全球合计</t>
+        </is>
+      </c>
+      <c r="C67" s="1" t="inlineStr"/>
+      <c r="D67" s="1" t="inlineStr"/>
+      <c r="E67" s="9" t="n">
+        <v>422324814</v>
+      </c>
+      <c r="F67" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" s="1" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="inlineStr">
+        <is>
+          <t>区域汇总</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="inlineStr"/>
+      <c r="B70" s="1" t="inlineStr">
+        <is>
+          <t>区域</t>
+        </is>
+      </c>
+      <c r="C70" s="1" t="inlineStr"/>
+      <c r="D70" s="1" t="inlineStr"/>
+      <c r="E70" s="1" t="inlineStr">
+        <is>
+          <t>出口额 USD</t>
+        </is>
+      </c>
+      <c r="F70" s="1" t="inlineStr">
+        <is>
+          <t>占全球 %</t>
+        </is>
+      </c>
+      <c r="G70" s="1" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>欧洲</t>
+        </is>
+      </c>
+      <c r="E71" s="7">
+        <f>SUMIF(D3:D65,"欧洲",E3:E65)</f>
+        <v/>
+      </c>
+      <c r="F71" s="8">
+        <f>E71/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>北美</t>
+        </is>
+      </c>
+      <c r="E72" s="7">
+        <f>SUMIF(D3:D65,"北美",E3:E65)</f>
+        <v/>
+      </c>
+      <c r="F72" s="8">
+        <f>E72/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>中东/土耳其</t>
+        </is>
+      </c>
+      <c r="E73" s="7">
+        <f>SUMIF(D3:D65,"中东/土耳其",E3:E65)</f>
+        <v/>
+      </c>
+      <c r="F73" s="8">
+        <f>E73/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>亚太</t>
+        </is>
+      </c>
+      <c r="E74" s="7">
+        <f>SUMIF(D3:D65,"亚太",E3:E65)</f>
+        <v/>
+      </c>
+      <c r="F74" s="8">
+        <f>E74/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>拉美</t>
+        </is>
+      </c>
+      <c r="E75" s="7">
+        <f>SUMIF(D3:D65,"拉美",E3:E65)</f>
+        <v/>
+      </c>
+      <c r="F75" s="8">
+        <f>E75/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>非洲</t>
+        </is>
+      </c>
+      <c r="E76" s="7">
+        <f>SUMIF(D3:D65,"非洲",E3:E65)</f>
+        <v/>
+      </c>
+      <c r="F76" s="8">
+        <f>E76/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>独联体/中亚</t>
+        </is>
+      </c>
+      <c r="E77" s="7">
+        <f>SUMIF(D3:D65,"独联体/中亚",E3:E65)</f>
+        <v/>
+      </c>
+      <c r="F77" s="8">
+        <f>E77/422324814</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>其他未查询国家</t>
+        </is>
+      </c>
+      <c r="E78" s="7">
+        <f>422324814-SUM(E3:E65)</f>
+        <v/>
+      </c>
+      <c r="F78" s="8">
+        <f>E78/422324814</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -955,7 +2831,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1521,7 +3397,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2339,7 +4215,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7458,6 +9334,965 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>类别</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>SmartByte型号</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>关键规格</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>¥未税(2026.09.01-12.30)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>$进价(7.1)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>$建议卖价(+30%)</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>⭐主推客户</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>商业L2+ 走量</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>24×GE + 4×1G/2.5G SFP（AC5爆款）</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>460</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>2direct / Nedis</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>商业L2+</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8310GP-2GX8GT</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>8×GE PoE + 4 SFP，120W</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>450</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>82</v>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Nedis / Intos</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>商业L2+</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>24×GE PoE + 4 SFP，280W</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>750</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>106</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>138</v>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>2direct / Intos</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>商业L2+</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>24×GE PoE + 4 SFP，440W</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>1200</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>169</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>220</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Intos（对标其380W款）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>商业L2+ ⭐</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>24×GE + 4×10G SFP+（AC5爆款）</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>710</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>130</v>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>ASSMANN / Nedis / IC Intracom</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>商业L2+ ⭐</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>24×GE PoE + 4×10G SFP+，280W</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>1010</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>142</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>185</v>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>ASSMANN / IC Intracom</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>商业L2+</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8352G-4GX48GT</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>48×GE + 4 SFP</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>1320</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>186</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>242</v>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>DDC / Intos</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>商业L2+</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8352GP-4GX48GT</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>48×GE PoE + 4 SFP，440W</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>1720</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>242</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>315</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>DDC</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>商业L2+</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8352XG-4XS48GT</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>48×GE + 4×10G SFP+</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>1470</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>207</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>269</v>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>DDC</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>商业L2+</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8352XGP-4XS48GT</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>48×GE PoE + 4×10G，440W/850W</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>1870</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>263</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>342</v>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>DDC / Intos</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>商业L3</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8528XG-4XS24GT</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>L3，24×GE + 4×10G</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>211</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>274</v>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>DDC（他们没有L3）</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>商业L3</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8528XGP-4XS24GT</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>L3 PoE，400W</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>1900</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>268</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>348</v>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>DDC</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>商业L3</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8552XG-4XS48GT</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>L3 48×GE + 4×10G</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>2600</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>366</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>476</v>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>DDC</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>商业L3</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8552XGP-4XS48GT</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>L3 48×GE PoE，400W</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>3100</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>437</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>568</v>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>IC Intracom（试探高端）</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>工业L2+</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6306GP-2GX4GT</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>4×GE PoE + 2 SFP，DC12~58V</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>720</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>101</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>132</v>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>工业入门</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>工业L2+</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310GP-2GX8GT</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>8×GE PoE + 2 SFP</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>780</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>110</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>143</v>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>2direct / Nedis</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>工业L2+</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312GP-4GX8GT</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>8×GE PoE + 4 SFP</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>820</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>115</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>工业走量</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>工业L2+</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6318GP-2GX16GT</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>16×GE PoE + 2 SFP</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>1340</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>189</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>245</v>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>集成商</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>工业L2+</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6320GP-4GX16GT-D</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>16×GE PoE + DI/DO/RS485</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>1760</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>248</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>322</v>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>IC Intracom / ITS集成商</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>工业L2+</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6328GP-4GX24GT</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>24×GE PoE + DI/DO/RS485</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>1900</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>268</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>348</v>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>ITS / 电力配套</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>工业L2+ 10G ⭐</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>8×GE + 4×10G SFP+，-40~75℃</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>840</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>118</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>154</v>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>ASSMANN / Intos</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>工业L2+ 10G ⭐</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>8×GE PoE + 4×10G SFP+</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>920</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>130</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>169</v>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Intos / 工业PoE项目</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>工业L2+ 10G</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT-2BT</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>+ PoE++（1-2口）</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>1020</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>144</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>187</v>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>PoE++ 场景</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>工业L2+ 10G</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6318XGP-2XS16GT</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>16×GE PoE + 2×10G</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>1660</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>234</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>304</v>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>集成商</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>工业L2+ 10G</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6320XG-4XS8GX8GT-D</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>8×GE + 8 SFP + 4×10G，DI/DO/RS485</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>1780</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>251</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>326</v>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>ITS 机柜</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>工业L2+ 10G</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6328XGP-4XS24GT</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>24×GE PoE + 4×10G</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>2200</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>310</v>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>403</v>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>DDC</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>工业L2+ 10G</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6328XGP-4XS24GT-4BT</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>+ PoE++（1-4口）</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>2400</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>338</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>439</v>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>PoE++ 场景</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>工业L3</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6520XGP-4XS16GT</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>L3 16×GE PoE + 4×10G</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>2510</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>354</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>460</v>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>工业L3项目</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>工业L3</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6528XGP-4XS24GT</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>L3 24×GE PoE + 4×10G</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>2700</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>380</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>494</v>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>工业L3项目</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -9454,7 +12289,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10520,7 +13355,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11304,1879 +14139,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G78"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="45" customHeight="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>说明：UN Comtrade，Reporter=Latvia(428)，HS 851762（交换/路由设备），Export，2024，FOB USD。MikroTik 占拉脱维亚该税号出口 3/4 以上，可视为 MikroTik 分销商进货地图。全球合计 USD 422,324,814。</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>排名</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>国家/地区</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>M49 代码</t>
-        </is>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>区域</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>出口额 USD</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>占全球 %</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="inlineStr">
-        <is>
-          <t>备注</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>美国</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>842</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>北美</t>
-        </is>
-      </c>
-      <c r="E3" s="7" t="n">
-        <v>50994438</v>
-      </c>
-      <c r="F3" s="8">
-        <f>E3/422324814</f>
-        <v/>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>对华关税约 37.5%（2026-09）</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>阿联酋(转口枢纽)</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>784</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>中东/土耳其</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="n">
-        <v>43018484</v>
-      </c>
-      <c r="F4" s="8">
-        <f>E4/422324814</f>
-        <v/>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>转口枢纽→中东/非洲/南亚</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>波兰</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>616</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="n">
-        <v>34368342</v>
-      </c>
-      <c r="F5" s="8">
-        <f>E5/422324814</f>
-        <v/>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>欧洲第一 MikroTik 国</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>立陶宛(波罗的海分销枢纽)</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>440</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>32525290</v>
-      </c>
-      <c r="F6" s="8">
-        <f>E6/422324814</f>
-        <v/>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>波罗的海分销枢纽</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>捷克</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>203</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="n">
-        <v>21822977</v>
-      </c>
-      <c r="F7" s="8">
-        <f>E7/422324814</f>
-        <v/>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>WISP 密度极高</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>德国</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>276</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>16002618</v>
-      </c>
-      <c r="F8" s="8">
-        <f>E8/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>中国香港(转口枢纽)</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>344</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>亚太</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="n">
-        <v>15962714</v>
-      </c>
-      <c r="F9" s="8">
-        <f>E9/422324814</f>
-        <v/>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>转口枢纽→东南亚/南亚</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>南非</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>710</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>非洲</t>
-        </is>
-      </c>
-      <c r="E10" s="7" t="n">
-        <v>11426199</v>
-      </c>
-      <c r="F10" s="8">
-        <f>E10/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>印度尼西亚</t>
-        </is>
-      </c>
-      <c r="C11" t="n">
-        <v>360</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>亚太</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="n">
-        <v>11250898</v>
-      </c>
-      <c r="F11" s="8">
-        <f>E11/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>10</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>哈萨克斯坦</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>398</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>独联体/中亚</t>
-        </is>
-      </c>
-      <c r="E12" s="7" t="n">
-        <v>10925270</v>
-      </c>
-      <c r="F12" s="8">
-        <f>E12/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>11</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>英国</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>826</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="n">
-        <v>8784753</v>
-      </c>
-      <c r="F13" s="8">
-        <f>E13/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>12</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>爱沙尼亚</t>
-        </is>
-      </c>
-      <c r="C14" t="n">
-        <v>233</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="n">
-        <v>8754532</v>
-      </c>
-      <c r="F14" s="8">
-        <f>E14/422324814</f>
-        <v/>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>波罗的海分销枢纽</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>13</v>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>乌克兰</t>
-        </is>
-      </c>
-      <c r="C15" t="n">
-        <v>804</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="n">
-        <v>8206878</v>
-      </c>
-      <c r="F15" s="8">
-        <f>E15/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>14</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>意大利</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>380</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E16" s="7" t="n">
-        <v>8186541</v>
-      </c>
-      <c r="F16" s="8">
-        <f>E16/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>15</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>土耳其</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>792</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>中东/土耳其</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="n">
-        <v>7652474</v>
-      </c>
-      <c r="F17" s="8">
-        <f>E17/422324814</f>
-        <v/>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>你已有 NMS 客户</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>16</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>西班牙</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>724</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="n">
-        <v>7284155</v>
-      </c>
-      <c r="F18" s="8">
-        <f>E18/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>17</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>荷兰</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>528</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E19" s="7" t="n">
-        <v>6532562</v>
-      </c>
-      <c r="F19" s="8">
-        <f>E19/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>18</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>巴西</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>76</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>拉美</t>
-        </is>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>5655456</v>
-      </c>
-      <c r="F20" s="8">
-        <f>E20/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>19</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>奥地利</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>40</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="n">
-        <v>4567730</v>
-      </c>
-      <c r="F21" s="8">
-        <f>E21/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>20</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>新加坡</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>702</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>亚太</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="n">
-        <v>4496379</v>
-      </c>
-      <c r="F22" s="8">
-        <f>E22/422324814</f>
-        <v/>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>转口枢纽</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>21</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>中国大陆</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>156</v>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>亚太</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="n">
-        <v>4493322</v>
-      </c>
-      <c r="F23" s="8">
-        <f>E23/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>22</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>加拿大</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>124</v>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>北美</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="n">
-        <v>4469245</v>
-      </c>
-      <c r="F24" s="8">
-        <f>E24/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>23</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>哥伦比亚</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>170</v>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>拉美</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="n">
-        <v>3752926</v>
-      </c>
-      <c r="F25" s="8">
-        <f>E25/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>24</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>保加利亚</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>100</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="n">
-        <v>3606615</v>
-      </c>
-      <c r="F26" s="8">
-        <f>E26/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>25</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>澳大利亚</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>36</v>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>亚太</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="n">
-        <v>3596152</v>
-      </c>
-      <c r="F27" s="8">
-        <f>E27/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>26</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>匈牙利</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>348</v>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="n">
-        <v>3207035</v>
-      </c>
-      <c r="F28" s="8">
-        <f>E28/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>27</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>瑞典</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>752</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="n">
-        <v>3137243</v>
-      </c>
-      <c r="F29" s="8">
-        <f>E29/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>28</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>越南</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>704</v>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>亚太</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="n">
-        <v>2733552</v>
-      </c>
-      <c r="F30" s="8">
-        <f>E30/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>29</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>智利</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>152</v>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>拉美</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="n">
-        <v>2721330</v>
-      </c>
-      <c r="F31" s="8">
-        <f>E31/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>30</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>秘鲁</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>604</v>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>拉美</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="n">
-        <v>2713158</v>
-      </c>
-      <c r="F32" s="8">
-        <f>E32/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>31</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>泰国</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>764</v>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>亚太</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="n">
-        <v>2464546</v>
-      </c>
-      <c r="F33" s="8">
-        <f>E33/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>32</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>希腊</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>300</v>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E34" s="7" t="n">
-        <v>2308883</v>
-      </c>
-      <c r="F34" s="8">
-        <f>E34/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>33</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>丹麦</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>208</v>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="n">
-        <v>2239002</v>
-      </c>
-      <c r="F35" s="8">
-        <f>E35/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>34</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>墨西哥</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>484</v>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>拉美</t>
-        </is>
-      </c>
-      <c r="E36" s="7" t="n">
-        <v>2183194</v>
-      </c>
-      <c r="F36" s="8">
-        <f>E36/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>35</v>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>阿根廷</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>32</v>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>拉美</t>
-        </is>
-      </c>
-      <c r="E37" s="7" t="n">
-        <v>1858335</v>
-      </c>
-      <c r="F37" s="8">
-        <f>E37/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>36</v>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>罗马尼亚</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>642</v>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E38" s="7" t="n">
-        <v>1844544</v>
-      </c>
-      <c r="F38" s="8">
-        <f>E38/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>37</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>新西兰</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>554</v>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>亚太</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="n">
-        <v>1696031</v>
-      </c>
-      <c r="F39" s="8">
-        <f>E39/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>38</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>孟加拉国</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>50</v>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>亚太</t>
-        </is>
-      </c>
-      <c r="E40" s="7" t="n">
-        <v>1099842</v>
-      </c>
-      <c r="F40" s="8">
-        <f>E40/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>39</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>斯洛伐克</t>
-        </is>
-      </c>
-      <c r="C41" t="n">
-        <v>703</v>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E41" s="7" t="n">
-        <v>1068939</v>
-      </c>
-      <c r="F41" s="8">
-        <f>E41/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>40</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>塞尔维亚</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>688</v>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E42" s="7" t="n">
-        <v>1057170</v>
-      </c>
-      <c r="F42" s="8">
-        <f>E42/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>41</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>马来西亚</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>458</v>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>亚太</t>
-        </is>
-      </c>
-      <c r="E43" s="7" t="n">
-        <v>996768</v>
-      </c>
-      <c r="F43" s="8">
-        <f>E43/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>42</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>斯洛文尼亚</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>705</v>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E44" s="7" t="n">
-        <v>951791</v>
-      </c>
-      <c r="F44" s="8">
-        <f>E44/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="n">
-        <v>43</v>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>肯尼亚</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>404</v>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>非洲</t>
-        </is>
-      </c>
-      <c r="E45" s="7" t="n">
-        <v>934046</v>
-      </c>
-      <c r="F45" s="8">
-        <f>E45/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="n">
-        <v>44</v>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>葡萄牙</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>620</v>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E46" s="7" t="n">
-        <v>927187</v>
-      </c>
-      <c r="F46" s="8">
-        <f>E46/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>45</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>克罗地亚</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>191</v>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E47" s="7" t="n">
-        <v>881827</v>
-      </c>
-      <c r="F47" s="8">
-        <f>E47/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>46</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>芬兰</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>246</v>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E48" s="7" t="n">
-        <v>843078</v>
-      </c>
-      <c r="F48" s="8">
-        <f>E48/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>47</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>乌兹别克斯坦</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
-        <v>860</v>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>独联体/中亚</t>
-        </is>
-      </c>
-      <c r="E49" s="7" t="n">
-        <v>802640</v>
-      </c>
-      <c r="F49" s="8">
-        <f>E49/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="n">
-        <v>48</v>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>沙特</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
-        <v>682</v>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>中东/土耳其</t>
-        </is>
-      </c>
-      <c r="E50" s="7" t="n">
-        <v>800914</v>
-      </c>
-      <c r="F50" s="8">
-        <f>E50/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="n">
-        <v>49</v>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>比利时</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>56</v>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E51" s="7" t="n">
-        <v>706207</v>
-      </c>
-      <c r="F51" s="8">
-        <f>E51/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="n">
-        <v>50</v>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>巴基斯坦</t>
-        </is>
-      </c>
-      <c r="C52" t="n">
-        <v>586</v>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>亚太</t>
-        </is>
-      </c>
-      <c r="E52" s="7" t="n">
-        <v>632718</v>
-      </c>
-      <c r="F52" s="8">
-        <f>E52/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>51</v>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>格鲁吉亚</t>
-        </is>
-      </c>
-      <c r="C53" t="n">
-        <v>268</v>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>独联体/中亚</t>
-        </is>
-      </c>
-      <c r="E53" s="7" t="n">
-        <v>612616</v>
-      </c>
-      <c r="F53" s="8">
-        <f>E53/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>52</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>中国台湾</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>490</v>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>亚太</t>
-        </is>
-      </c>
-      <c r="E54" s="7" t="n">
-        <v>601808</v>
-      </c>
-      <c r="F54" s="8">
-        <f>E54/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="n">
-        <v>53</v>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>阿尔巴尼亚</t>
-        </is>
-      </c>
-      <c r="C55" t="n">
-        <v>8</v>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E55" s="7" t="n">
-        <v>551402</v>
-      </c>
-      <c r="F55" s="8">
-        <f>E55/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="n">
-        <v>54</v>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>韩国</t>
-        </is>
-      </c>
-      <c r="C56" t="n">
-        <v>410</v>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>亚太</t>
-        </is>
-      </c>
-      <c r="E56" s="7" t="n">
-        <v>465113</v>
-      </c>
-      <c r="F56" s="8">
-        <f>E56/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="n">
-        <v>55</v>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>日本</t>
-        </is>
-      </c>
-      <c r="C57" t="n">
-        <v>392</v>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>亚太</t>
-        </is>
-      </c>
-      <c r="E57" s="7" t="n">
-        <v>430801</v>
-      </c>
-      <c r="F57" s="8">
-        <f>E57/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="n">
-        <v>56</v>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>菲律宾</t>
-        </is>
-      </c>
-      <c r="C58" t="n">
-        <v>608</v>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>亚太</t>
-        </is>
-      </c>
-      <c r="E58" s="7" t="n">
-        <v>381036</v>
-      </c>
-      <c r="F58" s="8">
-        <f>E58/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="n">
-        <v>57</v>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>爱尔兰</t>
-        </is>
-      </c>
-      <c r="C59" t="n">
-        <v>372</v>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E59" s="7" t="n">
-        <v>357037</v>
-      </c>
-      <c r="F59" s="8">
-        <f>E59/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="n">
-        <v>58</v>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>埃及</t>
-        </is>
-      </c>
-      <c r="C60" t="n">
-        <v>818</v>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>非洲</t>
-        </is>
-      </c>
-      <c r="E60" s="7" t="n">
-        <v>345877</v>
-      </c>
-      <c r="F60" s="8">
-        <f>E60/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="n">
-        <v>59</v>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>以色列</t>
-        </is>
-      </c>
-      <c r="C61" t="n">
-        <v>376</v>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>中东/土耳其</t>
-        </is>
-      </c>
-      <c r="E61" s="7" t="n">
-        <v>273731</v>
-      </c>
-      <c r="F61" s="8">
-        <f>E61/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="n">
-        <v>60</v>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>阿塞拜疆</t>
-        </is>
-      </c>
-      <c r="C62" t="n">
-        <v>31</v>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>独联体/中亚</t>
-        </is>
-      </c>
-      <c r="E62" s="7" t="n">
-        <v>273435</v>
-      </c>
-      <c r="F62" s="8">
-        <f>E62/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="n">
-        <v>61</v>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>尼日利亚</t>
-        </is>
-      </c>
-      <c r="C63" t="n">
-        <v>566</v>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>非洲</t>
-        </is>
-      </c>
-      <c r="E63" s="7" t="n">
-        <v>265052</v>
-      </c>
-      <c r="F63" s="8">
-        <f>E63/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="n">
-        <v>62</v>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>安哥拉</t>
-        </is>
-      </c>
-      <c r="C64" t="n">
-        <v>24</v>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>非洲</t>
-        </is>
-      </c>
-      <c r="E64" s="7" t="n">
-        <v>93579</v>
-      </c>
-      <c r="F64" s="8">
-        <f>E64/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="n">
-        <v>63</v>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>白俄罗斯</t>
-        </is>
-      </c>
-      <c r="C65" t="n">
-        <v>112</v>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>独联体/中亚</t>
-        </is>
-      </c>
-      <c r="E65" s="7" t="n">
-        <v>3144</v>
-      </c>
-      <c r="F65" s="8">
-        <f>E65/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66">
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>其他未查询国家（合计约 90 国）</t>
-        </is>
-      </c>
-      <c r="E66" s="7">
-        <f>422324814-SUM(E3:E65)</f>
-        <v/>
-      </c>
-      <c r="F66" s="8">
-        <f>E66/422324814</f>
-        <v/>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>余量</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="1" t="inlineStr"/>
-      <c r="B67" s="1" t="inlineStr">
-        <is>
-          <t>全球合计</t>
-        </is>
-      </c>
-      <c r="C67" s="1" t="inlineStr"/>
-      <c r="D67" s="1" t="inlineStr"/>
-      <c r="E67" s="9" t="n">
-        <v>422324814</v>
-      </c>
-      <c r="F67" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G67" s="1" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="1" t="inlineStr">
-        <is>
-          <t>区域汇总</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="1" t="inlineStr"/>
-      <c r="B70" s="1" t="inlineStr">
-        <is>
-          <t>区域</t>
-        </is>
-      </c>
-      <c r="C70" s="1" t="inlineStr"/>
-      <c r="D70" s="1" t="inlineStr"/>
-      <c r="E70" s="1" t="inlineStr">
-        <is>
-          <t>出口额 USD</t>
-        </is>
-      </c>
-      <c r="F70" s="1" t="inlineStr">
-        <is>
-          <t>占全球 %</t>
-        </is>
-      </c>
-      <c r="G70" s="1" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>欧洲</t>
-        </is>
-      </c>
-      <c r="E71" s="7">
-        <f>SUMIF(D3:D65,"欧洲",E3:E65)</f>
-        <v/>
-      </c>
-      <c r="F71" s="8">
-        <f>E71/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="72">
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>北美</t>
-        </is>
-      </c>
-      <c r="E72" s="7">
-        <f>SUMIF(D3:D65,"北美",E3:E65)</f>
-        <v/>
-      </c>
-      <c r="F72" s="8">
-        <f>E72/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73">
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>中东/土耳其</t>
-        </is>
-      </c>
-      <c r="E73" s="7">
-        <f>SUMIF(D3:D65,"中东/土耳其",E3:E65)</f>
-        <v/>
-      </c>
-      <c r="F73" s="8">
-        <f>E73/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74">
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>亚太</t>
-        </is>
-      </c>
-      <c r="E74" s="7">
-        <f>SUMIF(D3:D65,"亚太",E3:E65)</f>
-        <v/>
-      </c>
-      <c r="F74" s="8">
-        <f>E74/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75">
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>拉美</t>
-        </is>
-      </c>
-      <c r="E75" s="7">
-        <f>SUMIF(D3:D65,"拉美",E3:E65)</f>
-        <v/>
-      </c>
-      <c r="F75" s="8">
-        <f>E75/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76">
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>非洲</t>
-        </is>
-      </c>
-      <c r="E76" s="7">
-        <f>SUMIF(D3:D65,"非洲",E3:E65)</f>
-        <v/>
-      </c>
-      <c r="F76" s="8">
-        <f>E76/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77">
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>独联体/中亚</t>
-        </is>
-      </c>
-      <c r="E77" s="7">
-        <f>SUMIF(D3:D65,"独联体/中亚",E3:E65)</f>
-        <v/>
-      </c>
-      <c r="F77" s="8">
-        <f>E77/422324814</f>
-        <v/>
-      </c>
-    </row>
-    <row r="78">
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>其他未查询国家</t>
-        </is>
-      </c>
-      <c r="E78" s="7">
-        <f>422324814-SUM(E3:E65)</f>
-        <v/>
-      </c>
-      <c r="F78" s="8">
-        <f>E78/422324814</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add price rebuttal playbook and 28 new leads from ORing's European distributor locator
- 报价反击表_2026-09.md: four-step rebuttal framework, unit-cost tables
  (price per port, price per PoE watt, 5-year TCO) built from real street
  prices, per-model rebuttal cards (MikroTik CSS326/CRS326/CRS328, PLANET
  IGS-5225 series, Moxa EDS-405A/EDS-G308, ORing range, Teltonika TSW212,
  TP-Link Omada, Direktronik, StarTech, Zyxel), three near-price
  competitors, price-floor no-go zones, six pressure scenarios, anchoring
  moves, printable cheat sheet
- 28 new accounts with phone numbers from oringnet.com European distributor
  page (AT/BE/CZ/DK/FI/FR/DE/IE/IT/NL/NO/PL/PT/ES/RO/SE/CH/UA)
- 70 accounts total across 20 countries; CSV and workbook rebuilt
- Documented which brand locator pages work and which return 404/403

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,19 +11188,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q43"/>
+  <dimension ref="A1:Q71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
     <col width="32" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
     <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
     <col width="8" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
@@ -14200,6 +14200,1910 @@
       <c r="Q43" s="3" t="inlineStr">
         <is>
           <t>Amazon IT/DE</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Spectra GmbH (Niederlassung Österreich)</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>奥地利</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr"/>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>spectra-austria.at</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>ORing高价→同规格1/3价第二供应源</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>+43 (0) 7240 20190</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L44" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M44" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N44" s="3" t="inlineStr"/>
+      <c r="O44" s="3" t="inlineStr"/>
+      <c r="P44" s="3" t="inlineStr"/>
+      <c r="Q44" s="3" t="inlineStr">
+        <is>
+          <t>Spectra集团奥地利分支</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Koning &amp; Hartman B.V.</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>荷兰/比利时</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>koningenhartman.com</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Benelux 工业网络分销，第二供应源</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>+31-88-1818 666 / +32 2 257 02 00</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L45" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M45" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N45" s="3" t="inlineStr"/>
+      <c r="O45" s="3" t="inlineStr"/>
+      <c r="P45" s="3" t="inlineStr"/>
+      <c r="Q45" s="3" t="inlineStr">
+        <is>
+          <t>比荷卢全覆盖</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Tesla Networks</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>比利时</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr"/>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>teslanetworks.com</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>比利时工业网络分销</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>+32 (0)15 24 7007</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L46" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M46" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N46" s="3" t="inlineStr"/>
+      <c r="O46" s="3" t="inlineStr"/>
+      <c r="P46" s="3" t="inlineStr"/>
+      <c r="Q46" s="3" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Alternetivo s.r.o.</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>alternetivo.cz</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>捷克 T1，第二供应源</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>+420 221 771 881</t>
+        </is>
+      </c>
+      <c r="K47" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L47" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M47" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N47" s="3" t="inlineStr"/>
+      <c r="O47" s="3" t="inlineStr"/>
+      <c r="P47" s="3" t="inlineStr"/>
+      <c r="Q47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>TECON s.r.o.</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr"/>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>tecon.cz</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>捷克工业分销</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6320G-4GX16GT-D</t>
+        </is>
+      </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>+420 499 429 100</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L48" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M48" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N48" s="3" t="inlineStr"/>
+      <c r="O48" s="3" t="inlineStr"/>
+      <c r="P48" s="3" t="inlineStr"/>
+      <c r="Q48" s="3" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>LaboTest AB</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>瑞典/丹麦</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>labotest.se</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>北欧分销（同时覆盖丹麦）</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>+46 (0) 8 354360</t>
+        </is>
+      </c>
+      <c r="K49" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L49" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M49" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N49" s="3" t="inlineStr"/>
+      <c r="O49" s="3" t="inlineStr"/>
+      <c r="P49" s="3" t="inlineStr"/>
+      <c r="Q49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Data Monitor</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>芬兰</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr"/>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>datamonitor.fi</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>芬兰工业网络分销</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>+358 443 553 623</t>
+        </is>
+      </c>
+      <c r="K50" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L50" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M50" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N50" s="3" t="inlineStr"/>
+      <c r="O50" s="3" t="inlineStr"/>
+      <c r="P50" s="3" t="inlineStr"/>
+      <c r="Q50" s="3" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>LaboTest Oy</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>芬兰</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>labotest.fi</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>芬兰分销</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>+358 29 0039 600</t>
+        </is>
+      </c>
+      <c r="K51" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L51" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M51" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N51" s="3" t="inlineStr"/>
+      <c r="O51" s="3" t="inlineStr"/>
+      <c r="P51" s="3" t="inlineStr"/>
+      <c r="Q51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Phoebe IDF</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>法国</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr"/>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>distribution.phoebe.fr</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>法国分销（distribution 部门）</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>+33 1 30 67 69 15</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L52" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M52" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N52" s="3" t="inlineStr"/>
+      <c r="O52" s="3" t="inlineStr"/>
+      <c r="P52" s="3" t="inlineStr"/>
+      <c r="Q52" s="3" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>APLUS Systeme Automation</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>法国</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr"/>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>aplus-sa.com</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>法国工业自动化分销</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6320G-4GX16GT-D</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>+33 1 69884300</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L53" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M53" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N53" s="3" t="inlineStr"/>
+      <c r="O53" s="3" t="inlineStr"/>
+      <c r="P53" s="3" t="inlineStr"/>
+      <c r="Q53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Equipements Scientifiques</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>法国</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr"/>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>es-france.com</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>法国分销</t>
+        </is>
+      </c>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>+33 1 47 95 99 81</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L54" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M54" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N54" s="3" t="inlineStr"/>
+      <c r="O54" s="3" t="inlineStr"/>
+      <c r="P54" s="3" t="inlineStr"/>
+      <c r="Q54" s="3" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Acceed GmbH</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr"/>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>acceed.de</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>德国工业物联网/网络分销</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>+49 211 938898-0</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L55" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M55" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N55" s="3" t="inlineStr"/>
+      <c r="O55" s="3" t="inlineStr"/>
+      <c r="P55" s="3" t="inlineStr"/>
+      <c r="Q55" s="3" t="inlineStr">
+        <is>
+          <t>德国不冷邮件，走表单/电话</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>ALIDEX ITALIA</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr"/>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>alidex.it</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>意大利分销</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>+39 392 8499296</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L56" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M56" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N56" s="3" t="inlineStr"/>
+      <c r="O56" s="3" t="inlineStr"/>
+      <c r="P56" s="3" t="inlineStr"/>
+      <c r="Q56" s="3" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>GOMA ELETTRONICA SPA</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>都灵</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>goma.it</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>意大利电子分销</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>+39 011 7725024</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L57" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M57" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N57" s="3" t="inlineStr"/>
+      <c r="O57" s="3" t="inlineStr"/>
+      <c r="P57" s="3" t="inlineStr"/>
+      <c r="Q57" s="3" t="inlineStr">
+        <is>
+          <t>Strada Antica di Collegno 225</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>DIGIMAX S.r.l.</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr"/>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>digimax.it</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>意大利分销</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310GP-2GX8GT</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>+39 0444 574066</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L58" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M58" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N58" s="3" t="inlineStr"/>
+      <c r="O58" s="3" t="inlineStr"/>
+      <c r="P58" s="3" t="inlineStr"/>
+      <c r="Q58" s="3" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>DataLink Communications</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>爱尔兰/英国</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr"/>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>datalinkcom.net</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>爱尔兰 + 英国双覆盖</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>+353-91-840838 / UK +01214680041</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L59" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M59" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N59" s="3" t="inlineStr"/>
+      <c r="O59" s="3" t="inlineStr"/>
+      <c r="P59" s="3" t="inlineStr"/>
+      <c r="Q59" s="3" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>Lextron B.V.</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr"/>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>lextron.nl</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>荷兰工业网络分销</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>+31 162 220229</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L60" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M60" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N60" s="3" t="inlineStr"/>
+      <c r="O60" s="3" t="inlineStr"/>
+      <c r="P60" s="3" t="inlineStr"/>
+      <c r="Q60" s="3" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>SATEL NORGE AS</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>挪威</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr"/>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>satel.no</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>挪威工业无线通信分销</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>+47 69 27 70 40</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L61" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M61" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N61" s="3" t="inlineStr"/>
+      <c r="O61" s="3" t="inlineStr"/>
+      <c r="P61" s="3" t="inlineStr"/>
+      <c r="Q61" s="3" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>Fiberworks AS</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>挪威</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr"/>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>fiberworks.no</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>挪威光纤/网络分销</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J62" s="3" t="inlineStr">
+        <is>
+          <t>+47 23 03 53 30</t>
+        </is>
+      </c>
+      <c r="K62" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L62" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M62" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N62" s="3" t="inlineStr"/>
+      <c r="O62" s="3" t="inlineStr"/>
+      <c r="P62" s="3" t="inlineStr"/>
+      <c r="Q62" s="3" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>Atel Electronics</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr"/>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>atel.com.pl</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G63" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H63" s="3" t="inlineStr">
+        <is>
+          <t>波兰 T1，第二供应源</t>
+        </is>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>+48 77 455 60 76</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L63" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M63" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N63" s="3" t="inlineStr"/>
+      <c r="O63" s="3" t="inlineStr"/>
+      <c r="P63" s="3" t="inlineStr"/>
+      <c r="Q63" s="3" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>Maritex Leszek Łosin Sp.j.</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr"/>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>maritex.eu</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>波兰工业/电信分销</t>
+        </is>
+      </c>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6320G-4GX16GT-D</t>
+        </is>
+      </c>
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>+48 58 622 89 00</t>
+        </is>
+      </c>
+      <c r="K64" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L64" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M64" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N64" s="3" t="inlineStr"/>
+      <c r="O64" s="3" t="inlineStr"/>
+      <c r="P64" s="3" t="inlineStr"/>
+      <c r="Q64" s="3" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>Tempel Group</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>葡萄牙</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr"/>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>tempelgroup.pt</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H65" s="3" t="inlineStr">
+        <is>
+          <t>葡萄牙分销</t>
+        </is>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>+351 214220540</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L65" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M65" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N65" s="3" t="inlineStr"/>
+      <c r="O65" s="3" t="inlineStr"/>
+      <c r="P65" s="3" t="inlineStr"/>
+      <c r="Q65" s="3" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>ALIDEX IBERIA</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>西班牙/葡萄牙</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr"/>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>alidex.es</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>伊比利亚半岛分销</t>
+        </is>
+      </c>
+      <c r="I66" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t>+34 639 13 22 03</t>
+        </is>
+      </c>
+      <c r="K66" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L66" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M66" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N66" s="3" t="inlineStr"/>
+      <c r="O66" s="3" t="inlineStr"/>
+      <c r="P66" s="3" t="inlineStr"/>
+      <c r="Q66" s="3" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
+          <t>Tempel Group</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr"/>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>tempelgroup.com</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G67" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H67" s="3" t="inlineStr">
+        <is>
+          <t>西班牙分销（与葡萄牙同集团）</t>
+        </is>
+      </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>+34 936003600</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L67" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M67" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N67" s="3" t="inlineStr"/>
+      <c r="O67" s="3" t="inlineStr"/>
+      <c r="P67" s="3" t="inlineStr"/>
+      <c r="Q67" s="3" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>IMPERIAL ELECTRIC S.A.</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>罗马尼亚</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr"/>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>imperialelectric.ro</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>罗马尼亚电气/工业分销</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>+40 213240417</t>
+        </is>
+      </c>
+      <c r="K68" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L68" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M68" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N68" s="3" t="inlineStr"/>
+      <c r="O68" s="3" t="inlineStr"/>
+      <c r="P68" s="3" t="inlineStr"/>
+      <c r="Q68" s="3" t="inlineStr">
+        <is>
+          <t>中东欧增量市场</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>HighTech Nordic AB</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>瑞典</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr"/>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>hightechnordic.com</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H69" s="3" t="inlineStr">
+        <is>
+          <t>瑞典工业分销</t>
+        </is>
+      </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>+46 101775800</t>
+        </is>
+      </c>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L69" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M69" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N69" s="3" t="inlineStr"/>
+      <c r="O69" s="3" t="inlineStr"/>
+      <c r="P69" s="3" t="inlineStr"/>
+      <c r="Q69" s="3" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>MPI Technologies AG</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>瑞士</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr"/>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>mpi.ch</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>瑞士工业网络分销</t>
+        </is>
+      </c>
+      <c r="I70" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t>+41 564 83 34 44</t>
+        </is>
+      </c>
+      <c r="K70" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L70" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M70" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N70" s="3" t="inlineStr"/>
+      <c r="O70" s="3" t="inlineStr"/>
+      <c r="P70" s="3" t="inlineStr"/>
+      <c r="Q70" s="3" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>Alpha Metronik Ltd</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr"/>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>alfa-metronik.ua</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰分销（MikroTik 出货 T3 市场）</t>
+        </is>
+      </c>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>+380 (44) 501-96-01</t>
+        </is>
+      </c>
+      <c r="K71" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L71" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M71" s="3" t="inlineStr">
+        <is>
+          <t>ORing经销商名录/2026-09</t>
+        </is>
+      </c>
+      <c r="N71" s="3" t="inlineStr"/>
+      <c r="O71" s="3" t="inlineStr"/>
+      <c r="P71" s="3" t="inlineStr"/>
+      <c r="Q71" s="3" t="inlineStr">
+        <is>
+          <t>⚠️ 出货前做制裁与最终用途筛查</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mine Antaira, Westermo, ComNet and HMS partner directories: 62 new accounts, 132 total
Went through the brand directory list one by one. ORing (4 regions),
Antaira EU, Westermo (with gold/silver/bronze distributor tiers), ComNet
and HMS/Red Lion/N-Tron all yielded phone numbers and websites; PLANET,
Moxa, EtherWAN, CTC, Volktek, Lantech, Korenix, Perle, Teltonika and
Advantech B+B all dead-end in 404/403 or a bare contact form.

Adds 62 accounts across 20 more countries (incl. first US, South American
and Middle East entries), rebuilds the CSV and the 反向信号名单 sheet at
132 rows, and documents the directory scoreboard, the multi-brand
distributor insight and the next mining targets.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q71"/>
+  <dimension ref="A1:Q133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -16104,6 +16104,4332 @@
       <c r="Q71" s="3" t="inlineStr">
         <is>
           <t>⚠️ 出货前做制裁与最终用途筛查</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>CSI S.A.</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr"/>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>csi.pl</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>分销（Antaira 授权）</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>Antaira</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I72" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J72" s="3" t="inlineStr">
+        <is>
+          <t>+48 12 390 61 80 / kontakt@csi.pl</t>
+        </is>
+      </c>
+      <c r="K72" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L72" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M72" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N72" s="3" t="inlineStr"/>
+      <c r="O72" s="3" t="inlineStr"/>
+      <c r="P72" s="3" t="inlineStr"/>
+      <c r="Q72" s="3" t="inlineStr">
+        <is>
+          <t>克拉科夫，波兰工业网络分销</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>OEM AUTOMATIC Sp. z o.o.</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr"/>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>oemautomatic.pl</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>分销（Antaira 授权）</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr">
+        <is>
+          <t>Antaira</t>
+        </is>
+      </c>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I73" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>+48 22 863 27 22 / info@oemautomatic.pl</t>
+        </is>
+      </c>
+      <c r="K73" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L73" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M73" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N73" s="3" t="inlineStr"/>
+      <c r="O73" s="3" t="inlineStr"/>
+      <c r="P73" s="3" t="inlineStr"/>
+      <c r="Q73" s="3" t="inlineStr">
+        <is>
+          <t>华沙，自动化目录分销，SKU 量大</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>Industrial Personal Computer 2U GmbH (IPC2U)</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr"/>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>ipc2u.com</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>分销（Antaira + Korenix 授权）</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>Antaira, Korenix</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>同一家代理两个台湾品牌 → 典型多品牌分销</t>
+        </is>
+      </c>
+      <c r="I74" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J74" s="3" t="inlineStr">
+        <is>
+          <t>+49 511 807 259-0 / sales@ipc2u.de</t>
+        </is>
+      </c>
+      <c r="K74" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L74" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M74" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N74" s="3" t="inlineStr"/>
+      <c r="O74" s="3" t="inlineStr"/>
+      <c r="P74" s="3" t="inlineStr"/>
+      <c r="Q74" s="3" t="inlineStr">
+        <is>
+          <t>德/法/波/捷四国办公室，兼做系统集成</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>Alfa Systems</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>比利时/卢森堡</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr"/>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>alfasystems.be</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>分销（Antaira 授权）</t>
+        </is>
+      </c>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>Antaira</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I75" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>+32 15 45 11 60 / info@alfasys.be</t>
+        </is>
+      </c>
+      <c r="K75" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L75" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M75" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N75" s="3" t="inlineStr"/>
+      <c r="O75" s="3" t="inlineStr"/>
+      <c r="P75" s="3" t="inlineStr"/>
+      <c r="Q75" s="3" t="inlineStr">
+        <is>
+          <t>Hombeek，同时覆盖卢森堡</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>ATEsystem s.r.o.</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr"/>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>atesystem.cz</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>分销（Antaira 授权）</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>Antaira</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I76" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J76" s="3" t="inlineStr">
+        <is>
+          <t>+420 595 172 720 / atesystem@atesystem.cz</t>
+        </is>
+      </c>
+      <c r="K76" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L76" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M76" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N76" s="3" t="inlineStr"/>
+      <c r="O76" s="3" t="inlineStr"/>
+      <c r="P76" s="3" t="inlineStr"/>
+      <c r="Q76" s="3" t="inlineStr">
+        <is>
+          <t>俄斯特拉发，捷克 T1</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>Fiseg Oy</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>芬兰</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr"/>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>fiseg.fi</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>分销（Antaira 授权）</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr">
+        <is>
+          <t>Antaira</t>
+        </is>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I77" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>+358 50 5726 268 / myynti@fiseg.fi</t>
+        </is>
+      </c>
+      <c r="K77" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L77" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M77" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N77" s="3" t="inlineStr"/>
+      <c r="O77" s="3" t="inlineStr"/>
+      <c r="P77" s="3" t="inlineStr"/>
+      <c r="Q77" s="3" t="inlineStr">
+        <is>
+          <t>坦佩雷，北欧 T2</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>AXTEK line Kft.</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>匈牙利</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr"/>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>axtek.hu</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>分销（Antaira 授权）</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>Antaira</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I78" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J78" s="3" t="inlineStr">
+        <is>
+          <t>+36 1 700 42 70 / info@axtek.hu</t>
+        </is>
+      </c>
+      <c r="K78" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L78" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M78" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N78" s="3" t="inlineStr"/>
+      <c r="O78" s="3" t="inlineStr"/>
+      <c r="P78" s="3" t="inlineStr"/>
+      <c r="Q78" s="3" t="inlineStr">
+        <is>
+          <t>Pécel，中东欧增量市场</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>Automation Experts</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr"/>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>automationexperts.gr</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>分销（Antaira 授权）</t>
+        </is>
+      </c>
+      <c r="F79" s="3" t="inlineStr">
+        <is>
+          <t>Antaira</t>
+        </is>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H79" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I79" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J79" s="3" t="inlineStr">
+        <is>
+          <t>+30 210 28 15 988 / info@automationexperts.gr</t>
+        </is>
+      </c>
+      <c r="K79" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L79" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M79" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N79" s="3" t="inlineStr"/>
+      <c r="O79" s="3" t="inlineStr"/>
+      <c r="P79" s="3" t="inlineStr"/>
+      <c r="Q79" s="3" t="inlineStr">
+        <is>
+          <t>雅典</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>AGL Industrial Solutions</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>葡萄牙</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr"/>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>guedeslopes.pt</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>分销（Antaira 授权）</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>Antaira</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I80" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J80" s="3" t="inlineStr">
+        <is>
+          <t>+351 218 278 341 / geral@guedeslopes.pt</t>
+        </is>
+      </c>
+      <c r="K80" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L80" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M80" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N80" s="3" t="inlineStr"/>
+      <c r="O80" s="3" t="inlineStr"/>
+      <c r="P80" s="3" t="inlineStr"/>
+      <c r="Q80" s="3" t="inlineStr">
+        <is>
+          <t>Porto Salvo，伊比利亚工业方案商</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>System Devices UK Ltd</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr"/>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>systemdevices.co.uk</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>分销（Antaira 授权）</t>
+        </is>
+      </c>
+      <c r="F81" s="3" t="inlineStr">
+        <is>
+          <t>Antaira</t>
+        </is>
+      </c>
+      <c r="G81" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H81" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I81" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J81" s="3" t="inlineStr">
+        <is>
+          <t>+44 1928 571 977 / info@systemdevices.co.uk</t>
+        </is>
+      </c>
+      <c r="K81" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L81" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M81" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N81" s="3" t="inlineStr"/>
+      <c r="O81" s="3" t="inlineStr"/>
+      <c r="P81" s="3" t="inlineStr"/>
+      <c r="Q81" s="3" t="inlineStr">
+        <is>
+          <t>Runcorn，英国工业网络分销</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>Westercom</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>捷克/斯洛伐克</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr"/>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>westercom.eu</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Silver）</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>Westermo, B+B SmartWorx</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>同时代理 Westermo 与 B+B SmartWorx → 典型多品牌工业分销</t>
+        </is>
+      </c>
+      <c r="I82" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J82" s="3" t="inlineStr">
+        <is>
+          <t>+420 603 509 790</t>
+        </is>
+      </c>
+      <c r="K82" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L82" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M82" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N82" s="3" t="inlineStr"/>
+      <c r="O82" s="3" t="inlineStr"/>
+      <c r="P82" s="3" t="inlineStr"/>
+      <c r="Q82" s="3" t="inlineStr">
+        <is>
+          <t>已验证：站内还在卖 B+B SmartWorx 全线</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>Microstar</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>克罗地亚/斯洛文尼亚</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr"/>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>microstar.hr</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Bronze）</t>
+        </is>
+      </c>
+      <c r="F83" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H83" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I83" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J83" s="3" t="inlineStr">
+        <is>
+          <t>+385 1 364 78 49</t>
+        </is>
+      </c>
+      <c r="K83" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L83" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M83" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N83" s="3" t="inlineStr"/>
+      <c r="O83" s="3" t="inlineStr"/>
+      <c r="P83" s="3" t="inlineStr"/>
+      <c r="Q83" s="3" t="inlineStr">
+        <is>
+          <t>巴尔干，覆盖两国</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>Avtera BH</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>波黑</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr"/>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>avtera.ba</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Reseller）</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I84" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J84" s="3" t="inlineStr">
+        <is>
+          <t>+387 33 776 758</t>
+        </is>
+      </c>
+      <c r="K84" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L84" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M84" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N84" s="3" t="inlineStr"/>
+      <c r="O84" s="3" t="inlineStr"/>
+      <c r="P84" s="3" t="inlineStr"/>
+      <c r="Q84" s="3" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>Rittbul</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>保加利亚</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr"/>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>rittbul.bg</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Reseller）</t>
+        </is>
+      </c>
+      <c r="F85" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G85" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H85" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I85" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>+359 2 439 78 45</t>
+        </is>
+      </c>
+      <c r="K85" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L85" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M85" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N85" s="3" t="inlineStr"/>
+      <c r="O85" s="3" t="inlineStr"/>
+      <c r="P85" s="3" t="inlineStr"/>
+      <c r="Q85" s="3" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>Electrobit</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>爱沙尼亚</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr"/>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>electrobit.ee</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Reseller）</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H86" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I86" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J86" s="3" t="inlineStr">
+        <is>
+          <t>+372 6518 140</t>
+        </is>
+      </c>
+      <c r="K86" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L86" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M86" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N86" s="3" t="inlineStr"/>
+      <c r="O86" s="3" t="inlineStr"/>
+      <c r="P86" s="3" t="inlineStr"/>
+      <c r="Q86" s="3" t="inlineStr">
+        <is>
+          <t>波罗的海</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>NETAP</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr"/>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>netap.gr</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Reseller）</t>
+        </is>
+      </c>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H87" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I87" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J87" s="3" t="inlineStr">
+        <is>
+          <t>+30 210 243 33 83</t>
+        </is>
+      </c>
+      <c r="K87" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L87" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M87" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N87" s="3" t="inlineStr"/>
+      <c r="O87" s="3" t="inlineStr"/>
+      <c r="P87" s="3" t="inlineStr"/>
+      <c r="Q87" s="3" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>ATYS Co Controll Engineering</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>匈牙利</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr"/>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>atysco.hu</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Reseller）</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G88" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H88" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I88" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J88" s="3" t="inlineStr">
+        <is>
+          <t>+36 126 325 61</t>
+        </is>
+      </c>
+      <c r="K88" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L88" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M88" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N88" s="3" t="inlineStr"/>
+      <c r="O88" s="3" t="inlineStr"/>
+      <c r="P88" s="3" t="inlineStr"/>
+      <c r="Q88" s="3" t="inlineStr">
+        <is>
+          <t>另有罗马尼亚分公司</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>Mælibúnaður</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>冰岛</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr"/>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>maelibunadur.is</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Reseller）</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H89" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>+354 661 11 69</t>
+        </is>
+      </c>
+      <c r="K89" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L89" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M89" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N89" s="3" t="inlineStr"/>
+      <c r="O89" s="3" t="inlineStr"/>
+      <c r="P89" s="3" t="inlineStr"/>
+      <c r="Q89" s="3" t="inlineStr">
+        <is>
+          <t>北欧小市场，竞争小</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>El-Gev Electronics</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>以色列</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr"/>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>elgev.co.il</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Reseller）</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G90" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H90" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I90" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J90" s="3" t="inlineStr">
+        <is>
+          <t>+972 74-7190012</t>
+        </is>
+      </c>
+      <c r="K90" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L90" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M90" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N90" s="3" t="inlineStr"/>
+      <c r="O90" s="3" t="inlineStr"/>
+      <c r="P90" s="3" t="inlineStr"/>
+      <c r="Q90" s="3" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>Piero Bersanini</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr"/>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>pierobersanini.com</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Gold）</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G91" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H91" s="3" t="inlineStr">
+        <is>
+          <t>金牌分销 = 该品牌销量大 → 第二供应源首选</t>
+        </is>
+      </c>
+      <c r="I91" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6320G-4GX16GT-D</t>
+        </is>
+      </c>
+      <c r="J91" s="3" t="inlineStr">
+        <is>
+          <t>+39 02 268 531</t>
+        </is>
+      </c>
+      <c r="K91" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L91" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M91" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N91" s="3" t="inlineStr"/>
+      <c r="O91" s="3" t="inlineStr"/>
+      <c r="P91" s="3" t="inlineStr"/>
+      <c r="Q91" s="3" t="inlineStr">
+        <is>
+          <t>米兰</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>OAK INTEGRATOR</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>拉脱维亚</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr"/>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>oak-integrator.lv</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Reseller）</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G92" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H92" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I92" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J92" s="3" t="inlineStr">
+        <is>
+          <t>+371 67842280</t>
+        </is>
+      </c>
+      <c r="K92" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L92" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M92" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N92" s="3" t="inlineStr"/>
+      <c r="O92" s="3" t="inlineStr"/>
+      <c r="P92" s="3" t="inlineStr"/>
+      <c r="Q92" s="3" t="inlineStr">
+        <is>
+          <t>波罗的海</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>Automatikos centras, UAB</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>立陶宛</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr"/>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>automatikoscentras.lt</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Reseller）</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G93" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H93" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I93" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J93" s="3" t="inlineStr">
+        <is>
+          <t>+370 37 262707</t>
+        </is>
+      </c>
+      <c r="K93" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L93" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M93" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N93" s="3" t="inlineStr"/>
+      <c r="O93" s="3" t="inlineStr"/>
+      <c r="P93" s="3" t="inlineStr"/>
+      <c r="Q93" s="3" t="inlineStr">
+        <is>
+          <t>考纳斯</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>Aspect</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>北马其顿</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr"/>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>aspect.com.mk</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Reseller）</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H94" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I94" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J94" s="3" t="inlineStr">
+        <is>
+          <t>+389 2 32 33 777</t>
+        </is>
+      </c>
+      <c r="K94" s="3" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="L94" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M94" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N94" s="3" t="inlineStr"/>
+      <c r="O94" s="3" t="inlineStr"/>
+      <c r="P94" s="3" t="inlineStr"/>
+      <c r="Q94" s="3" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>Tektraco</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>马耳他</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr"/>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>tektraco.com</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Reseller）</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G95" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H95" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I95" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J95" s="3" t="inlineStr">
+        <is>
+          <t>+356 21 378 088</t>
+        </is>
+      </c>
+      <c r="K95" s="3" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="L95" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M95" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N95" s="3" t="inlineStr"/>
+      <c r="O95" s="3" t="inlineStr"/>
+      <c r="P95" s="3" t="inlineStr"/>
+      <c r="Q95" s="3" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>Modelec Data-Industrie</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr"/>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>modelec.nl</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Reseller）</t>
+        </is>
+      </c>
+      <c r="F96" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G96" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H96" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I96" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J96" s="3" t="inlineStr">
+        <is>
+          <t>+31 318 636 262</t>
+        </is>
+      </c>
+      <c r="K96" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L96" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M96" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N96" s="3" t="inlineStr"/>
+      <c r="O96" s="3" t="inlineStr"/>
+      <c r="P96" s="3" t="inlineStr"/>
+      <c r="Q96" s="3" t="inlineStr">
+        <is>
+          <t>荷兰工业数据通信分销</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>Last Mile Communication</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>挪威</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr"/>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>lastmile.no</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Gold）</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G97" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H97" s="3" t="inlineStr">
+        <is>
+          <t>金牌分销 = 销量大，第二供应源首选</t>
+        </is>
+      </c>
+      <c r="I97" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J97" s="3" t="inlineStr">
+        <is>
+          <t>+47 66 907 980</t>
+        </is>
+      </c>
+      <c r="K97" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L97" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M97" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N97" s="3" t="inlineStr"/>
+      <c r="O97" s="3" t="inlineStr"/>
+      <c r="P97" s="3" t="inlineStr"/>
+      <c r="Q97" s="3" t="inlineStr">
+        <is>
+          <t>挪威 T1</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>MVA - Electrotécnia</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>葡萄牙</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr"/>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>mva.pt</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Reseller）</t>
+        </is>
+      </c>
+      <c r="F98" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G98" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H98" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I98" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J98" s="3" t="inlineStr">
+        <is>
+          <t>+351 214 879 000</t>
+        </is>
+      </c>
+      <c r="K98" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L98" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M98" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N98" s="3" t="inlineStr"/>
+      <c r="O98" s="3" t="inlineStr"/>
+      <c r="P98" s="3" t="inlineStr"/>
+      <c r="Q98" s="3" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>Tekniska Polska</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr"/>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>tekniska.pl</t>
+        </is>
+      </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Gold）</t>
+        </is>
+      </c>
+      <c r="F99" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G99" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H99" s="3" t="inlineStr">
+        <is>
+          <t>金牌分销 + 波兰 T1，体量大</t>
+        </is>
+      </c>
+      <c r="I99" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6320G-4GX16GT-D</t>
+        </is>
+      </c>
+      <c r="J99" s="3" t="inlineStr">
+        <is>
+          <t>+48 32 331 110 608</t>
+        </is>
+      </c>
+      <c r="K99" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L99" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M99" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N99" s="3" t="inlineStr"/>
+      <c r="O99" s="3" t="inlineStr"/>
+      <c r="P99" s="3" t="inlineStr"/>
+      <c r="Q99" s="3" t="inlineStr">
+        <is>
+          <t>波兰 T1</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>ATYS-co Romania</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>罗马尼亚</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr"/>
+      <c r="D100" s="3" t="inlineStr">
+        <is>
+          <t>atysco.ro</t>
+        </is>
+      </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo）</t>
+        </is>
+      </c>
+      <c r="F100" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G100" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H100" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I100" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J100" s="3" t="inlineStr">
+        <is>
+          <t>+40 264 593 169</t>
+        </is>
+      </c>
+      <c r="K100" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L100" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M100" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N100" s="3" t="inlineStr"/>
+      <c r="O100" s="3" t="inlineStr"/>
+      <c r="P100" s="3" t="inlineStr"/>
+      <c r="Q100" s="3" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>NovaTel</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>塞尔维亚</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr"/>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>novatel.rs</t>
+        </is>
+      </c>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Reseller）</t>
+        </is>
+      </c>
+      <c r="F101" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G101" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H101" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I101" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J101" s="3" t="inlineStr">
+        <is>
+          <t>+381 11 4252012</t>
+        </is>
+      </c>
+      <c r="K101" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L101" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M101" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N101" s="3" t="inlineStr"/>
+      <c r="O101" s="3" t="inlineStr"/>
+      <c r="P101" s="3" t="inlineStr"/>
+      <c r="Q101" s="3" t="inlineStr">
+        <is>
+          <t>贝尔格莱德</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>Omron Electronics Iberia</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr"/>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>industrial.omron.es</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo Silver）</t>
+        </is>
+      </c>
+      <c r="F102" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G102" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H102" s="3" t="inlineStr">
+        <is>
+          <t>大集团自有渠道，宜先从其区域经销商切入</t>
+        </is>
+      </c>
+      <c r="I102" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6320G-4GX16GT-D</t>
+        </is>
+      </c>
+      <c r="J102" s="3" t="inlineStr">
+        <is>
+          <t>+34 913 777 900</t>
+        </is>
+      </c>
+      <c r="K102" s="3" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="L102" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M102" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N102" s="3" t="inlineStr"/>
+      <c r="O102" s="3" t="inlineStr"/>
+      <c r="P102" s="3" t="inlineStr"/>
+      <c r="Q102" s="3" t="inlineStr">
+        <is>
+          <t>体量大、流程长，优先级低</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
+          <t>Areskom İletişim Sistemleri</t>
+        </is>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>土耳其</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr"/>
+      <c r="D103" s="3" t="inlineStr">
+        <is>
+          <t>areskom.com.tr</t>
+        </is>
+      </c>
+      <c r="E103" s="3" t="inlineStr">
+        <is>
+          <t>分销（Westermo）</t>
+        </is>
+      </c>
+      <c r="F103" s="3" t="inlineStr">
+        <is>
+          <t>Westermo</t>
+        </is>
+      </c>
+      <c r="G103" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H103" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I103" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J103" s="3" t="inlineStr">
+        <is>
+          <t>+90 216 428 78 78</t>
+        </is>
+      </c>
+      <c r="K103" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L103" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M103" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N103" s="3" t="inlineStr"/>
+      <c r="O103" s="3" t="inlineStr"/>
+      <c r="P103" s="3" t="inlineStr"/>
+      <c r="Q103" s="3" t="inlineStr">
+        <is>
+          <t>伊斯坦布尔</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>SmartSD</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>荷兰/比利时/法国</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr"/>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>smartsd.com</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>分销（ComNet 授权）</t>
+        </is>
+      </c>
+      <c r="F104" s="3" t="inlineStr">
+        <is>
+          <t>ComNet</t>
+        </is>
+      </c>
+      <c r="G104" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H104" s="3" t="inlineStr">
+        <is>
+          <t>安防传输分销 → PoE 交换机是配套品类</t>
+        </is>
+      </c>
+      <c r="I104" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6320G-4GX16GT-D</t>
+        </is>
+      </c>
+      <c r="J104" s="3" t="inlineStr">
+        <is>
+          <t>smartsd.com</t>
+        </is>
+      </c>
+      <c r="K104" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L104" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M104" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N104" s="3" t="inlineStr"/>
+      <c r="O104" s="3" t="inlineStr"/>
+      <c r="P104" s="3" t="inlineStr"/>
+      <c r="Q104" s="3" t="inlineStr">
+        <is>
+          <t>ComNet 比荷卢+法国分销</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>Videor</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr"/>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>videor.com</t>
+        </is>
+      </c>
+      <c r="E105" s="3" t="inlineStr">
+        <is>
+          <t>分销（ComNet 授权）</t>
+        </is>
+      </c>
+      <c r="F105" s="3" t="inlineStr">
+        <is>
+          <t>ComNet</t>
+        </is>
+      </c>
+      <c r="G105" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H105" s="3" t="inlineStr">
+        <is>
+          <t>德国专业视频/安防分销，PoE 是刚需</t>
+        </is>
+      </c>
+      <c r="I105" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6320G-4GX16GT-D</t>
+        </is>
+      </c>
+      <c r="J105" s="3" t="inlineStr">
+        <is>
+          <t>videor.com</t>
+        </is>
+      </c>
+      <c r="K105" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L105" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M105" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N105" s="3" t="inlineStr"/>
+      <c r="O105" s="3" t="inlineStr"/>
+      <c r="P105" s="3" t="inlineStr"/>
+      <c r="Q105" s="3" t="inlineStr">
+        <is>
+          <t>德国安防分销主力之一</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>Transend</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr"/>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>transenduk.com</t>
+        </is>
+      </c>
+      <c r="E106" s="3" t="inlineStr">
+        <is>
+          <t>分销（ComNet 授权）</t>
+        </is>
+      </c>
+      <c r="F106" s="3" t="inlineStr">
+        <is>
+          <t>ComNet</t>
+        </is>
+      </c>
+      <c r="G106" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H106" s="3" t="inlineStr">
+        <is>
+          <t>CCTV/PoE 同规格第二供应源</t>
+        </is>
+      </c>
+      <c r="I106" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310GP-2GX8GT</t>
+        </is>
+      </c>
+      <c r="J106" s="3" t="inlineStr">
+        <is>
+          <t>transenduk.com</t>
+        </is>
+      </c>
+      <c r="K106" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L106" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M106" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N106" s="3" t="inlineStr"/>
+      <c r="O106" s="3" t="inlineStr"/>
+      <c r="P106" s="3" t="inlineStr"/>
+      <c r="Q106" s="3" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="inlineStr">
+        <is>
+          <t>Blue Helix</t>
+        </is>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr"/>
+      <c r="D107" s="3" t="inlineStr">
+        <is>
+          <t>bluehelix.co.uk</t>
+        </is>
+      </c>
+      <c r="E107" s="3" t="inlineStr">
+        <is>
+          <t>分销（ComNet 授权）</t>
+        </is>
+      </c>
+      <c r="F107" s="3" t="inlineStr">
+        <is>
+          <t>ComNet</t>
+        </is>
+      </c>
+      <c r="G107" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H107" s="3" t="inlineStr">
+        <is>
+          <t>CCTV/PoE 同规格第二供应源</t>
+        </is>
+      </c>
+      <c r="I107" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310GP-2GX8GT</t>
+        </is>
+      </c>
+      <c r="J107" s="3" t="inlineStr">
+        <is>
+          <t>bluehelix.co.uk</t>
+        </is>
+      </c>
+      <c r="K107" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L107" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M107" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N107" s="3" t="inlineStr"/>
+      <c r="O107" s="3" t="inlineStr"/>
+      <c r="P107" s="3" t="inlineStr"/>
+      <c r="Q107" s="3" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>Exertis Azenn</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>法国</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr"/>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>exertis.co.uk</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>分销（ComNet 授权）</t>
+        </is>
+      </c>
+      <c r="F108" s="3" t="inlineStr">
+        <is>
+          <t>ComNet</t>
+        </is>
+      </c>
+      <c r="G108" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H108" s="3" t="inlineStr">
+        <is>
+          <t>Exertis 集团法国分部，渠道体量大</t>
+        </is>
+      </c>
+      <c r="I108" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6320G-4GX16GT-D</t>
+        </is>
+      </c>
+      <c r="J108" s="3" t="inlineStr">
+        <is>
+          <t>exertis</t>
+        </is>
+      </c>
+      <c r="K108" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L108" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M108" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N108" s="3" t="inlineStr"/>
+      <c r="O108" s="3" t="inlineStr"/>
+      <c r="P108" s="3" t="inlineStr"/>
+      <c r="Q108" s="3" t="inlineStr">
+        <is>
+          <t>大分销，流程长</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>E.V.D.I.</t>
+        </is>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>法国</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr"/>
+      <c r="D109" s="3" t="inlineStr">
+        <is>
+          <t>evdi.fr</t>
+        </is>
+      </c>
+      <c r="E109" s="3" t="inlineStr">
+        <is>
+          <t>分销（ComNet 授权）</t>
+        </is>
+      </c>
+      <c r="F109" s="3" t="inlineStr">
+        <is>
+          <t>ComNet</t>
+        </is>
+      </c>
+      <c r="G109" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H109" s="3" t="inlineStr">
+        <is>
+          <t>CCTV/PoE 同规格第二供应源</t>
+        </is>
+      </c>
+      <c r="I109" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310GP-2GX8GT</t>
+        </is>
+      </c>
+      <c r="J109" s="3" t="inlineStr">
+        <is>
+          <t>evdi.fr</t>
+        </is>
+      </c>
+      <c r="K109" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L109" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M109" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N109" s="3" t="inlineStr"/>
+      <c r="O109" s="3" t="inlineStr"/>
+      <c r="P109" s="3" t="inlineStr"/>
+      <c r="Q109" s="3" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>Compass Distribution</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr"/>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>compass-distribution.it</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="inlineStr">
+        <is>
+          <t>分销（ComNet 授权）</t>
+        </is>
+      </c>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>ComNet</t>
+        </is>
+      </c>
+      <c r="G110" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H110" s="3" t="inlineStr">
+        <is>
+          <t>CCTV/PoE 同规格第二供应源</t>
+        </is>
+      </c>
+      <c r="I110" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310GP-2GX8GT</t>
+        </is>
+      </c>
+      <c r="J110" s="3" t="inlineStr">
+        <is>
+          <t>compass-distribution.it</t>
+        </is>
+      </c>
+      <c r="K110" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L110" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M110" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N110" s="3" t="inlineStr"/>
+      <c r="O110" s="3" t="inlineStr"/>
+      <c r="P110" s="3" t="inlineStr"/>
+      <c r="Q110" s="3" t="inlineStr">
+        <is>
+          <t>意大利安防分销</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="inlineStr">
+        <is>
+          <t>Aikom Technology</t>
+        </is>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr"/>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>aikomtech.com</t>
+        </is>
+      </c>
+      <c r="E111" s="3" t="inlineStr">
+        <is>
+          <t>分销（Teltonika Gold + ComNet 授权）</t>
+        </is>
+      </c>
+      <c r="F111" s="3" t="inlineStr">
+        <is>
+          <t>Teltonika, ComNet</t>
+        </is>
+      </c>
+      <c r="G111" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H111" s="3" t="inlineStr">
+        <is>
+          <t>同时是 Teltonika 金牌 + ComNet 分销 → 多品牌工业 IoT 分销</t>
+        </is>
+      </c>
+      <c r="I111" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J111" s="3" t="inlineStr">
+        <is>
+          <t>aikomtech.com</t>
+        </is>
+      </c>
+      <c r="K111" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L111" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M111" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N111" s="3" t="inlineStr"/>
+      <c r="O111" s="3" t="inlineStr"/>
+      <c r="P111" s="3" t="inlineStr"/>
+      <c r="Q111" s="3" t="inlineStr">
+        <is>
+          <t>意大利 T1，宜主攻</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>AIONA Automation GmbH</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>奥地利</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr"/>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>bestofautomation.at</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS：Red Lion / N-Tron）</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>Red Lion, N-Tron</t>
+        </is>
+      </c>
+      <c r="G112" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H112" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron 就是工业交换机品牌 → 直接同类替换</t>
+        </is>
+      </c>
+      <c r="I112" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J112" s="3" t="inlineStr">
+        <is>
+          <t>bestofautomation.at</t>
+        </is>
+      </c>
+      <c r="K112" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L112" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M112" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N112" s="3" t="inlineStr"/>
+      <c r="O112" s="3" t="inlineStr"/>
+      <c r="P112" s="3" t="inlineStr"/>
+      <c r="Q112" s="3" t="inlineStr">
+        <is>
+          <t>维也纳</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
+        <is>
+          <t>AiRiCOM</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>法国</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr"/>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>airicom.com</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS：Red Lion / N-Tron）</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>Red Lion, N-Tron</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H113" s="3" t="inlineStr">
+        <is>
+          <t>工业交换机同类替换</t>
+        </is>
+      </c>
+      <c r="I113" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J113" s="3" t="inlineStr">
+        <is>
+          <t>airicom.com</t>
+        </is>
+      </c>
+      <c r="K113" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L113" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M113" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N113" s="3" t="inlineStr"/>
+      <c r="O113" s="3" t="inlineStr"/>
+      <c r="P113" s="3" t="inlineStr"/>
+      <c r="Q113" s="3" t="inlineStr">
+        <is>
+          <t>Boufféré + 巴黎两处办公室</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="inlineStr">
+        <is>
+          <t>Adeptor AS</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>挪威</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr"/>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>adeptor.no</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS：Red Lion / N-Tron）</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>Red Lion, N-Tron</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H114" s="3" t="inlineStr">
+        <is>
+          <t>工业交换机同类替换</t>
+        </is>
+      </c>
+      <c r="I114" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J114" s="3" t="inlineStr">
+        <is>
+          <t>adeptor.no</t>
+        </is>
+      </c>
+      <c r="K114" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L114" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M114" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N114" s="3" t="inlineStr"/>
+      <c r="O114" s="3" t="inlineStr"/>
+      <c r="P114" s="3" t="inlineStr"/>
+      <c r="Q114" s="3" t="inlineStr">
+        <is>
+          <t>卑尔根</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="inlineStr">
+        <is>
+          <t>iComTech, Inc.</t>
+        </is>
+      </c>
+      <c r="B115" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C115" s="3" t="inlineStr"/>
+      <c r="D115" s="3" t="inlineStr">
+        <is>
+          <t>icomtechinc.com</t>
+        </is>
+      </c>
+      <c r="E115" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F115" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G115" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H115" s="3" t="inlineStr">
+        <is>
+          <t>官网设 ORing 专页 → 主推该品牌，第二供应源</t>
+        </is>
+      </c>
+      <c r="I115" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J115" s="3" t="inlineStr">
+        <is>
+          <t>+1 949 861-2550 / sales@icomtechinc.com</t>
+        </is>
+      </c>
+      <c r="K115" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L115" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M115" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N115" s="3" t="inlineStr"/>
+      <c r="O115" s="3" t="inlineStr"/>
+      <c r="P115" s="3" t="inlineStr"/>
+      <c r="Q115" s="3" t="inlineStr">
+        <is>
+          <t>加州</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="3" t="inlineStr">
+        <is>
+          <t>IEI Technology USA Corp.</t>
+        </is>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr"/>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>ieiworld.com</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F116" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G116" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H116" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I116" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J116" s="3" t="inlineStr">
+        <is>
+          <t>+1 909 595-2819 / sales@usa.ieiworld.com</t>
+        </is>
+      </c>
+      <c r="K116" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L116" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M116" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N116" s="3" t="inlineStr"/>
+      <c r="O116" s="3" t="inlineStr"/>
+      <c r="P116" s="3" t="inlineStr"/>
+      <c r="Q116" s="3" t="inlineStr">
+        <is>
+          <t>加州，台系工业电脑厂美国子公司</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="3" t="inlineStr">
+        <is>
+          <t>RUGGED SCIENCE</t>
+        </is>
+      </c>
+      <c r="B117" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C117" s="3" t="inlineStr"/>
+      <c r="D117" s="3" t="inlineStr">
+        <is>
+          <t>ruggedscience.com</t>
+        </is>
+      </c>
+      <c r="E117" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F117" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G117" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H117" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I117" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J117" s="3" t="inlineStr">
+        <is>
+          <t>+1 855 769-9747 / sales@ruggedscience.com</t>
+        </is>
+      </c>
+      <c r="K117" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L117" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M117" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N117" s="3" t="inlineStr"/>
+      <c r="O117" s="3" t="inlineStr"/>
+      <c r="P117" s="3" t="inlineStr"/>
+      <c r="Q117" s="3" t="inlineStr">
+        <is>
+          <t>加固计算机/军用方向</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>Mid Atlantic Rugged Systems</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr"/>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>midatlanticruggedsystems.com</t>
+        </is>
+      </c>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F118" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G118" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H118" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I118" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J118" s="3" t="inlineStr">
+        <is>
+          <t>+1 855 784-4334 / sales@marugged.com</t>
+        </is>
+      </c>
+      <c r="K118" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L118" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M118" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N118" s="3" t="inlineStr"/>
+      <c r="O118" s="3" t="inlineStr"/>
+      <c r="P118" s="3" t="inlineStr"/>
+      <c r="Q118" s="3" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>WAV, Inc.</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr"/>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>wavonline.com</t>
+        </is>
+      </c>
+      <c r="E119" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F119" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G119" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H119" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I119" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J119" s="3" t="inlineStr">
+        <is>
+          <t>+1 800 678-2419 / sales@wavonline.com</t>
+        </is>
+      </c>
+      <c r="K119" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L119" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M119" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N119" s="3" t="inlineStr"/>
+      <c r="O119" s="3" t="inlineStr"/>
+      <c r="P119" s="3" t="inlineStr"/>
+      <c r="Q119" s="3" t="inlineStr">
+        <is>
+          <t>伊利诺伊</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="inlineStr">
+        <is>
+          <t>TEMPEL GROUP ARGENTINA</t>
+        </is>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>阿根廷</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr"/>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>tempelgrouplatam.com</t>
+        </is>
+      </c>
+      <c r="E120" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F120" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G120" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H120" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I120" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J120" s="3" t="inlineStr">
+        <is>
+          <t>+54 11 4897-7184</t>
+        </is>
+      </c>
+      <c r="K120" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L120" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M120" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N120" s="3" t="inlineStr"/>
+      <c r="O120" s="3" t="inlineStr"/>
+      <c r="P120" s="3" t="inlineStr"/>
+      <c r="Q120" s="3" t="inlineStr">
+        <is>
+          <t>Tempel 集团拉美分支（另见西/葡 Tempel）</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>Above-Net Soluções Industriais</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>巴西</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr"/>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>abovenet.com.br</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F121" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G121" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H121" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I121" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J121" s="3" t="inlineStr">
+        <is>
+          <t>+55 21 2294-3931 / vendas@abovenet.com.br</t>
+        </is>
+      </c>
+      <c r="K121" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L121" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M121" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N121" s="3" t="inlineStr"/>
+      <c r="O121" s="3" t="inlineStr"/>
+      <c r="P121" s="3" t="inlineStr"/>
+      <c r="Q121" s="3" t="inlineStr">
+        <is>
+          <t>里约</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="3" t="inlineStr">
+        <is>
+          <t>All Tech Solutions (atsol)</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>巴西</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr"/>
+      <c r="D122" s="3" t="inlineStr">
+        <is>
+          <t>atsol.com.br</t>
+        </is>
+      </c>
+      <c r="E122" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F122" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G122" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H122" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I122" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J122" s="3" t="inlineStr">
+        <is>
+          <t>+55 11 99858-1492 / atendimento@atsol.com.br</t>
+        </is>
+      </c>
+      <c r="K122" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L122" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M122" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N122" s="3" t="inlineStr"/>
+      <c r="O122" s="3" t="inlineStr"/>
+      <c r="P122" s="3" t="inlineStr"/>
+      <c r="Q122" s="3" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="inlineStr">
+        <is>
+          <t>ICS Brasil</t>
+        </is>
+      </c>
+      <c r="B123" s="3" t="inlineStr">
+        <is>
+          <t>巴西</t>
+        </is>
+      </c>
+      <c r="C123" s="3" t="inlineStr"/>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>ics-brasil.com.br</t>
+        </is>
+      </c>
+      <c r="E123" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F123" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G123" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H123" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I123" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J123" s="3" t="inlineStr">
+        <is>
+          <t>+55 35 3623-5066</t>
+        </is>
+      </c>
+      <c r="K123" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L123" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M123" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N123" s="3" t="inlineStr"/>
+      <c r="O123" s="3" t="inlineStr"/>
+      <c r="P123" s="3" t="inlineStr"/>
+      <c r="Q123" s="3" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
+          <t>LRI AUTOMAÇÃO</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>巴西</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr"/>
+      <c r="D124" s="3" t="inlineStr">
+        <is>
+          <t>lri.com.br</t>
+        </is>
+      </c>
+      <c r="E124" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F124" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G124" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H124" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I124" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6320G-4GX16GT-D</t>
+        </is>
+      </c>
+      <c r="J124" s="3" t="inlineStr">
+        <is>
+          <t>+55 51 2129-3033 / vendas@lri.com.br</t>
+        </is>
+      </c>
+      <c r="K124" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L124" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M124" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N124" s="3" t="inlineStr"/>
+      <c r="O124" s="3" t="inlineStr"/>
+      <c r="P124" s="3" t="inlineStr"/>
+      <c r="Q124" s="3" t="inlineStr">
+        <is>
+          <t>巴西南部</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="3" t="inlineStr">
+        <is>
+          <t>TERABOX Soluciones Tecnológicas</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>智利</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr"/>
+      <c r="D125" s="3" t="inlineStr">
+        <is>
+          <t>terabox.cl</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F125" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G125" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H125" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I125" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J125" s="3" t="inlineStr">
+        <is>
+          <t>+56 9 8140 3392 / ventas@terabox.cl</t>
+        </is>
+      </c>
+      <c r="K125" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L125" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M125" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N125" s="3" t="inlineStr"/>
+      <c r="O125" s="3" t="inlineStr"/>
+      <c r="P125" s="3" t="inlineStr"/>
+      <c r="Q125" s="3" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="inlineStr">
+        <is>
+          <t>TEMPEL GROUP CHILE</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>智利</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr"/>
+      <c r="D126" s="3" t="inlineStr">
+        <is>
+          <t>tempelgroup.com</t>
+        </is>
+      </c>
+      <c r="E126" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F126" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G126" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H126" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I126" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J126" s="3" t="inlineStr">
+        <is>
+          <t>+56 2 2739 2829 / schile@tempelgroup.com</t>
+        </is>
+      </c>
+      <c r="K126" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L126" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M126" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N126" s="3" t="inlineStr"/>
+      <c r="O126" s="3" t="inlineStr"/>
+      <c r="P126" s="3" t="inlineStr"/>
+      <c r="Q126" s="3" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>EINS S.A.</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>厄瓜多尔</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr"/>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>einssa.com.ec</t>
+        </is>
+      </c>
+      <c r="E127" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F127" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G127" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H127" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I127" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J127" s="3" t="inlineStr">
+        <is>
+          <t>+593 99 695 1451 / comercial@einssa.com.ec</t>
+        </is>
+      </c>
+      <c r="K127" s="3" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="L127" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M127" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N127" s="3" t="inlineStr"/>
+      <c r="O127" s="3" t="inlineStr"/>
+      <c r="P127" s="3" t="inlineStr"/>
+      <c r="Q127" s="3" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="3" t="inlineStr">
+        <is>
+          <t>ValTekGroup</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>秘鲁</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr"/>
+      <c r="D128" s="3" t="inlineStr">
+        <is>
+          <t>valtek.com.pe</t>
+        </is>
+      </c>
+      <c r="E128" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F128" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G128" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H128" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I128" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J128" s="3" t="inlineStr">
+        <is>
+          <t>+51 1 4482249 / ventas@valtek.com.pe</t>
+        </is>
+      </c>
+      <c r="K128" s="3" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="L128" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M128" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N128" s="3" t="inlineStr"/>
+      <c r="O128" s="3" t="inlineStr"/>
+      <c r="P128" s="3" t="inlineStr"/>
+      <c r="Q128" s="3" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="3" t="inlineStr">
+        <is>
+          <t>IPNet Solutions LTD</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>以色列</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr"/>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t>ip-net.co.il</t>
+        </is>
+      </c>
+      <c r="E129" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F129" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G129" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H129" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I129" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J129" s="3" t="inlineStr">
+        <is>
+          <t>+972 52-7502200</t>
+        </is>
+      </c>
+      <c r="K129" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L129" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M129" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N129" s="3" t="inlineStr"/>
+      <c r="O129" s="3" t="inlineStr"/>
+      <c r="P129" s="3" t="inlineStr"/>
+      <c r="Q129" s="3" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
+          <t>Nokta Elektronik</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>土耳其</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr"/>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>noktaelektronik.net</t>
+        </is>
+      </c>
+      <c r="E130" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F130" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G130" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H130" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I130" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J130" s="3" t="inlineStr">
+        <is>
+          <t>+90 212 222 87 80 / nokta@noktaelektronik.net</t>
+        </is>
+      </c>
+      <c r="K130" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L130" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M130" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N130" s="3" t="inlineStr"/>
+      <c r="O130" s="3" t="inlineStr"/>
+      <c r="P130" s="3" t="inlineStr"/>
+      <c r="Q130" s="3" t="inlineStr">
+        <is>
+          <t>伊斯坦布尔</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr">
+        <is>
+          <t>I C T INTERNATIONAL L.L.C.</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>阿联酋</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr"/>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>ict-international.ae</t>
+        </is>
+      </c>
+      <c r="E131" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F131" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G131" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H131" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I131" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J131" s="3" t="inlineStr">
+        <is>
+          <t>+971 4 221 6756 / contact@ict-international.ae</t>
+        </is>
+      </c>
+      <c r="K131" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L131" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M131" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N131" s="3" t="inlineStr"/>
+      <c r="O131" s="3" t="inlineStr"/>
+      <c r="P131" s="3" t="inlineStr"/>
+      <c r="Q131" s="3" t="inlineStr">
+        <is>
+          <t>迪拜</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="3" t="inlineStr">
+        <is>
+          <t>Amplicon Middle East</t>
+        </is>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>阿联酋</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr"/>
+      <c r="D132" s="3" t="inlineStr">
+        <is>
+          <t>ampliconme.com</t>
+        </is>
+      </c>
+      <c r="E132" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F132" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G132" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H132" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I132" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J132" s="3" t="inlineStr">
+        <is>
+          <t>+971 4 3918897 / info@ampliconme.com</t>
+        </is>
+      </c>
+      <c r="K132" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L132" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M132" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N132" s="3" t="inlineStr"/>
+      <c r="O132" s="3" t="inlineStr"/>
+      <c r="P132" s="3" t="inlineStr"/>
+      <c r="Q132" s="3" t="inlineStr">
+        <is>
+          <t>Amplicon 集团中东分支</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>Shafaq Alforat General Trading</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>伊拉克</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr"/>
+      <c r="D133" s="3" t="inlineStr">
+        <is>
+          <t>shafaqalforat.com</t>
+        </is>
+      </c>
+      <c r="E133" s="3" t="inlineStr">
+        <is>
+          <t>分销（ORing 授权）</t>
+        </is>
+      </c>
+      <c r="F133" s="3" t="inlineStr">
+        <is>
+          <t>ORing</t>
+        </is>
+      </c>
+      <c r="G133" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H133" s="3" t="inlineStr">
+        <is>
+          <t>工业/轨道同规格 1/3 价第二供应源</t>
+        </is>
+      </c>
+      <c r="I133" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J133" s="3" t="inlineStr">
+        <is>
+          <t>+964 784 227 7262 / info@shafaqalforat.com</t>
+        </is>
+      </c>
+      <c r="K133" s="3" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="L133" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M133" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N133" s="3" t="inlineStr"/>
+      <c r="O133" s="3" t="inlineStr"/>
+      <c r="P133" s="3" t="inlineStr"/>
+      <c r="Q133" s="3" t="inlineStr">
+        <is>
+          <t>出库前做合规筛查</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sweep MikroTik distributors in 9 more countries: 265 accounts total
Adds the Netherlands (7), Czech Republic (13), Belgium (2), Austria (5),
Switzerland (5), Sweden (7), Norway (2), Denmark (6) and Finland (2).

Two more pan-European groups emerge: EET Group now spans 7 countries
(UK/NO/SE/DK/FI/NL/CZ) and Aurdel spans the Nordics (SE/DK/FI); ALLNET
now covers 4 (DE/FR/IT/DK). Several more single-brand-dependent targets
surfaced, e.g. Satellithuset (info@mikrotik.se), TRIOTRONIK
(mikrotik@triotronik.com) and Routershop.nl.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q217"/>
+  <dimension ref="A1:Q258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -26328,6 +26328,2917 @@
       <c r="O217" s="3" t="inlineStr"/>
       <c r="P217" s="3" t="inlineStr"/>
       <c r="Q217" s="3" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="3" t="inlineStr">
+        <is>
+          <t>Wimood（wimoodshop.nl）</t>
+        </is>
+      </c>
+      <c r="B218" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C218" s="3" t="inlineStr"/>
+      <c r="D218" s="3" t="inlineStr">
+        <is>
+          <t>wimoodshop.nl</t>
+        </is>
+      </c>
+      <c r="E218" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F218" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G218" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H218" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I218" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J218" s="3" t="inlineStr">
+        <is>
+          <t>+31 187 82 0204 / info@wimood.nl</t>
+        </is>
+      </c>
+      <c r="K218" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L218" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M218" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N218" s="3" t="inlineStr"/>
+      <c r="O218" s="3" t="inlineStr"/>
+      <c r="P218" s="3" t="inlineStr"/>
+      <c r="Q218" s="3" t="inlineStr">
+        <is>
+          <t>Goedereede</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="3" t="inlineStr">
+        <is>
+          <t>SDC Group</t>
+        </is>
+      </c>
+      <c r="B219" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C219" s="3" t="inlineStr"/>
+      <c r="D219" s="3" t="inlineStr">
+        <is>
+          <t>sdcgroup.nl</t>
+        </is>
+      </c>
+      <c r="E219" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F219" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G219" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H219" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I219" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT</t>
+        </is>
+      </c>
+      <c r="J219" s="3" t="inlineStr">
+        <is>
+          <t>+31 314 371 111 / verkoop@sdcgroup.nl</t>
+        </is>
+      </c>
+      <c r="K219" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L219" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M219" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N219" s="3" t="inlineStr"/>
+      <c r="O219" s="3" t="inlineStr"/>
+      <c r="P219" s="3" t="inlineStr"/>
+      <c r="Q219" s="3" t="inlineStr">
+        <is>
+          <t>Doetinchem</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="3" t="inlineStr">
+        <is>
+          <t>Routershop.nl</t>
+        </is>
+      </c>
+      <c r="B220" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C220" s="3" t="inlineStr"/>
+      <c r="D220" s="3" t="inlineStr">
+        <is>
+          <t>routershop.nl</t>
+        </is>
+      </c>
+      <c r="E220" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F220" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G220" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H220" s="3" t="inlineStr">
+        <is>
+          <t>域名就是 routershop → 单品牌依赖极高，最容易切第二品牌</t>
+        </is>
+      </c>
+      <c r="I220" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J220" s="3" t="inlineStr">
+        <is>
+          <t>030 669 14222 / info@routershop.nl</t>
+        </is>
+      </c>
+      <c r="K220" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L220" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M220" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N220" s="3" t="inlineStr"/>
+      <c r="O220" s="3" t="inlineStr"/>
+      <c r="P220" s="3" t="inlineStr"/>
+      <c r="Q220" s="3" t="inlineStr">
+        <is>
+          <t>Utrecht</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="3" t="inlineStr">
+        <is>
+          <t>Senetic B.V.</t>
+        </is>
+      </c>
+      <c r="B221" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C221" s="3" t="inlineStr"/>
+      <c r="D221" s="3" t="inlineStr">
+        <is>
+          <t>senetic.nl</t>
+        </is>
+      </c>
+      <c r="E221" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F221" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G221" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H221" s="3" t="inlineStr">
+        <is>
+          <t>Senetic 集团荷兰站</t>
+        </is>
+      </c>
+      <c r="I221" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J221" s="3" t="inlineStr">
+        <is>
+          <t>020 369 73 50 / info@senetic.nl</t>
+        </is>
+      </c>
+      <c r="K221" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L221" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M221" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N221" s="3" t="inlineStr"/>
+      <c r="O221" s="3" t="inlineStr"/>
+      <c r="P221" s="3" t="inlineStr"/>
+      <c r="Q221" s="3" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="3" t="inlineStr">
+        <is>
+          <t>Interstroom informatietechnologie b.v.</t>
+        </is>
+      </c>
+      <c r="B222" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C222" s="3" t="inlineStr"/>
+      <c r="D222" s="3" t="inlineStr">
+        <is>
+          <t>interstroom.nl</t>
+        </is>
+      </c>
+      <c r="E222" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F222" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G222" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H222" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I222" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J222" s="3" t="inlineStr">
+        <is>
+          <t>+31 74 245 20 50 / sales@interstroom.nl</t>
+        </is>
+      </c>
+      <c r="K222" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L222" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M222" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N222" s="3" t="inlineStr"/>
+      <c r="O222" s="3" t="inlineStr"/>
+      <c r="P222" s="3" t="inlineStr"/>
+      <c r="Q222" s="3" t="inlineStr">
+        <is>
+          <t>Hengelo</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="3" t="inlineStr">
+        <is>
+          <t>JPK Consulting</t>
+        </is>
+      </c>
+      <c r="B223" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C223" s="3" t="inlineStr"/>
+      <c r="D223" s="3" t="inlineStr">
+        <is>
+          <t>jpk-consulting.nl</t>
+        </is>
+      </c>
+      <c r="E223" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F223" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G223" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H223" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I223" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J223" s="3" t="inlineStr">
+        <is>
+          <t>038 234 0 333 / info@jpk-consulting.nl</t>
+        </is>
+      </c>
+      <c r="K223" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L223" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M223" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N223" s="3" t="inlineStr"/>
+      <c r="O223" s="3" t="inlineStr"/>
+      <c r="P223" s="3" t="inlineStr"/>
+      <c r="Q223" s="3" t="inlineStr">
+        <is>
+          <t>Zwolle</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="3" t="inlineStr">
+        <is>
+          <t>Discomp s.r.o.</t>
+        </is>
+      </c>
+      <c r="B224" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C224" s="3" t="inlineStr"/>
+      <c r="D224" s="3" t="inlineStr">
+        <is>
+          <t>discomp.cz</t>
+        </is>
+      </c>
+      <c r="E224" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F224" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD+WiFi6）</t>
+        </is>
+      </c>
+      <c r="G224" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H224" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I224" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J224" s="3" t="inlineStr">
+        <is>
+          <t>+420 377 221 177 / sales@discomp.cz</t>
+        </is>
+      </c>
+      <c r="K224" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L224" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M224" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N224" s="3" t="inlineStr"/>
+      <c r="O224" s="3" t="inlineStr"/>
+      <c r="P224" s="3" t="inlineStr"/>
+      <c r="Q224" s="3" t="inlineStr">
+        <is>
+          <t>Plzeň</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="3" t="inlineStr">
+        <is>
+          <t>AT Computers a.s.</t>
+        </is>
+      </c>
+      <c r="B225" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C225" s="3" t="inlineStr"/>
+      <c r="D225" s="3" t="inlineStr">
+        <is>
+          <t>atcmarket.cz</t>
+        </is>
+      </c>
+      <c r="E225" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F225" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G225" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H225" s="3" t="inlineStr">
+        <is>
+          <t>捷克三大 IT 分销之一</t>
+        </is>
+      </c>
+      <c r="I225" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT</t>
+        </is>
+      </c>
+      <c r="J225" s="3" t="inlineStr">
+        <is>
+          <t>+420 552 300 111 / obchod@atcomp.cz</t>
+        </is>
+      </c>
+      <c r="K225" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L225" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M225" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N225" s="3" t="inlineStr"/>
+      <c r="O225" s="3" t="inlineStr"/>
+      <c r="P225" s="3" t="inlineStr"/>
+      <c r="Q225" s="3" t="inlineStr">
+        <is>
+          <t>Ostrava/Praha/Brno</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="3" t="inlineStr">
+        <is>
+          <t>AxiLogi</t>
+        </is>
+      </c>
+      <c r="B226" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C226" s="3" t="inlineStr"/>
+      <c r="D226" s="3" t="inlineStr">
+        <is>
+          <t>axilogi.com</t>
+        </is>
+      </c>
+      <c r="E226" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F226" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G226" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H226" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I226" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J226" s="3" t="inlineStr">
+        <is>
+          <t>+420 777 103 488 / sales@axilogi.cz</t>
+        </is>
+      </c>
+      <c r="K226" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L226" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M226" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N226" s="3" t="inlineStr"/>
+      <c r="O226" s="3" t="inlineStr"/>
+      <c r="P226" s="3" t="inlineStr"/>
+      <c r="Q226" s="3" t="inlineStr">
+        <is>
+          <t>Pilsen</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="3" t="inlineStr">
+        <is>
+          <t>i4wifi a.s.</t>
+        </is>
+      </c>
+      <c r="B227" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C227" s="3" t="inlineStr"/>
+      <c r="D227" s="3" t="inlineStr">
+        <is>
+          <t>i4wifi.eu</t>
+        </is>
+      </c>
+      <c r="E227" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F227" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G227" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H227" s="3" t="inlineStr">
+        <is>
+          <t>有独立出口部门（export@）→ 能做跨国供货</t>
+        </is>
+      </c>
+      <c r="I227" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J227" s="3" t="inlineStr">
+        <is>
+          <t>+420 277 007 500 / export@i4wifi.eu</t>
+        </is>
+      </c>
+      <c r="K227" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L227" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M227" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N227" s="3" t="inlineStr"/>
+      <c r="O227" s="3" t="inlineStr"/>
+      <c r="P227" s="3" t="inlineStr"/>
+      <c r="Q227" s="3" t="inlineStr">
+        <is>
+          <t>Prague；有出口部</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="3" t="inlineStr">
+        <is>
+          <t>AIRCOM Praha s.r.o.</t>
+        </is>
+      </c>
+      <c r="B228" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C228" s="3" t="inlineStr"/>
+      <c r="D228" s="3" t="inlineStr">
+        <is>
+          <t>wifihw.cz</t>
+        </is>
+      </c>
+      <c r="E228" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F228" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G228" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H228" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I228" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J228" s="3" t="inlineStr">
+        <is>
+          <t>+420 241 400 304 / info@wifihw.cz</t>
+        </is>
+      </c>
+      <c r="K228" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L228" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M228" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N228" s="3" t="inlineStr"/>
+      <c r="O228" s="3" t="inlineStr"/>
+      <c r="P228" s="3" t="inlineStr"/>
+      <c r="Q228" s="3" t="inlineStr">
+        <is>
+          <t>Prague</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="3" t="inlineStr">
+        <is>
+          <t>eD's system Czech</t>
+        </is>
+      </c>
+      <c r="B229" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C229" s="3" t="inlineStr"/>
+      <c r="D229" s="3" t="inlineStr">
+        <is>
+          <t>edshop.edsystem.cz</t>
+        </is>
+      </c>
+      <c r="E229" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F229" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G229" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H229" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I229" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J229" s="3" t="inlineStr">
+        <is>
+          <t>+420 597 444 111 / info@edsystem.cz</t>
+        </is>
+      </c>
+      <c r="K229" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L229" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M229" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N229" s="3" t="inlineStr"/>
+      <c r="O229" s="3" t="inlineStr"/>
+      <c r="P229" s="3" t="inlineStr"/>
+      <c r="Q229" s="3" t="inlineStr">
+        <is>
+          <t>Ostrava</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="3" t="inlineStr">
+        <is>
+          <t>IPMEDIA</t>
+        </is>
+      </c>
+      <c r="B230" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C230" s="3" t="inlineStr"/>
+      <c r="D230" s="3" t="inlineStr">
+        <is>
+          <t>ipmedia.cz</t>
+        </is>
+      </c>
+      <c r="E230" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F230" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G230" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H230" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I230" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J230" s="3" t="inlineStr">
+        <is>
+          <t>+420 246 030 710 / info@ipmedia.cz</t>
+        </is>
+      </c>
+      <c r="K230" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L230" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M230" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N230" s="3" t="inlineStr"/>
+      <c r="O230" s="3" t="inlineStr"/>
+      <c r="P230" s="3" t="inlineStr"/>
+      <c r="Q230" s="3" t="inlineStr">
+        <is>
+          <t>Chomutov</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="3" t="inlineStr">
+        <is>
+          <t>PCV Computers, s.r.o.</t>
+        </is>
+      </c>
+      <c r="B231" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C231" s="3" t="inlineStr"/>
+      <c r="D231" s="3" t="inlineStr">
+        <is>
+          <t>pcvcomp.cz</t>
+        </is>
+      </c>
+      <c r="E231" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F231" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G231" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H231" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I231" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J231" s="3" t="inlineStr">
+        <is>
+          <t>+420 380 420 700 / obchod@pcvcomp.cz</t>
+        </is>
+      </c>
+      <c r="K231" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L231" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M231" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N231" s="3" t="inlineStr"/>
+      <c r="O231" s="3" t="inlineStr"/>
+      <c r="P231" s="3" t="inlineStr"/>
+      <c r="Q231" s="3" t="inlineStr">
+        <is>
+          <t>České Budějovice</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="3" t="inlineStr">
+        <is>
+          <t>VanCo.cz s.r.o.（wifi-shop.cz）</t>
+        </is>
+      </c>
+      <c r="B232" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C232" s="3" t="inlineStr"/>
+      <c r="D232" s="3" t="inlineStr">
+        <is>
+          <t>wifi-shop.cz</t>
+        </is>
+      </c>
+      <c r="E232" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F232" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G232" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H232" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I232" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J232" s="3" t="inlineStr">
+        <is>
+          <t>+420 246 035 451 / obchod@vanco.cz</t>
+        </is>
+      </c>
+      <c r="K232" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L232" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M232" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N232" s="3" t="inlineStr"/>
+      <c r="O232" s="3" t="inlineStr"/>
+      <c r="P232" s="3" t="inlineStr"/>
+      <c r="Q232" s="3" t="inlineStr">
+        <is>
+          <t>Praha 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="3" t="inlineStr">
+        <is>
+          <t>ABCtech s.r.o.</t>
+        </is>
+      </c>
+      <c r="B233" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C233" s="3" t="inlineStr"/>
+      <c r="D233" s="3" t="inlineStr">
+        <is>
+          <t>abctech.cz</t>
+        </is>
+      </c>
+      <c r="E233" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F233" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G233" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H233" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I233" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J233" s="3" t="inlineStr">
+        <is>
+          <t>+420 604 143 262 / obchod@abctech.cz</t>
+        </is>
+      </c>
+      <c r="K233" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L233" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M233" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N233" s="3" t="inlineStr"/>
+      <c r="O233" s="3" t="inlineStr"/>
+      <c r="P233" s="3" t="inlineStr"/>
+      <c r="Q233" s="3" t="inlineStr">
+        <is>
+          <t>Hradec Králové</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="3" t="inlineStr">
+        <is>
+          <t>WIFIPROFI.CZ</t>
+        </is>
+      </c>
+      <c r="B234" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C234" s="3" t="inlineStr"/>
+      <c r="D234" s="3" t="inlineStr">
+        <is>
+          <t>shop5.wifiprofi.cz</t>
+        </is>
+      </c>
+      <c r="E234" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F234" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G234" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H234" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I234" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J234" s="3" t="inlineStr">
+        <is>
+          <t>774 331 774 / klima@wifiprofi.cz</t>
+        </is>
+      </c>
+      <c r="K234" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L234" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M234" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N234" s="3" t="inlineStr"/>
+      <c r="O234" s="3" t="inlineStr"/>
+      <c r="P234" s="3" t="inlineStr"/>
+      <c r="Q234" s="3" t="inlineStr">
+        <is>
+          <t>Lety</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="3" t="inlineStr">
+        <is>
+          <t>Senetic s.r.o.</t>
+        </is>
+      </c>
+      <c r="B235" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C235" s="3" t="inlineStr"/>
+      <c r="D235" s="3" t="inlineStr">
+        <is>
+          <t>senetic.cz</t>
+        </is>
+      </c>
+      <c r="E235" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F235" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G235" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H235" s="3" t="inlineStr">
+        <is>
+          <t>Senetic 集团捷克站</t>
+        </is>
+      </c>
+      <c r="I235" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J235" s="3" t="inlineStr">
+        <is>
+          <t>+420 246 080 303 / info@senetic.cz</t>
+        </is>
+      </c>
+      <c r="K235" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L235" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M235" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N235" s="3" t="inlineStr"/>
+      <c r="O235" s="3" t="inlineStr"/>
+      <c r="P235" s="3" t="inlineStr"/>
+      <c r="Q235" s="3" t="inlineStr">
+        <is>
+          <t>Praha</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="3" t="inlineStr">
+        <is>
+          <t>SmartEye BV（wifistock.be）</t>
+        </is>
+      </c>
+      <c r="B236" s="3" t="inlineStr">
+        <is>
+          <t>比利时</t>
+        </is>
+      </c>
+      <c r="C236" s="3" t="inlineStr"/>
+      <c r="D236" s="3" t="inlineStr">
+        <is>
+          <t>wifistock.be</t>
+        </is>
+      </c>
+      <c r="E236" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F236" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G236" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H236" s="3" t="inlineStr">
+        <is>
+          <t>与英国 Wifi Stock 同名 → 疑似同集团，英比两国</t>
+        </is>
+      </c>
+      <c r="I236" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J236" s="3" t="inlineStr">
+        <is>
+          <t>+32 9 395 70 00 / sales@smarteye.eu</t>
+        </is>
+      </c>
+      <c r="K236" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L236" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M236" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N236" s="3" t="inlineStr"/>
+      <c r="O236" s="3" t="inlineStr"/>
+      <c r="P236" s="3" t="inlineStr"/>
+      <c r="Q236" s="3" t="inlineStr">
+        <is>
+          <t>Wilrijk</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="3" t="inlineStr">
+        <is>
+          <t>Foxconcept</t>
+        </is>
+      </c>
+      <c r="B237" s="3" t="inlineStr">
+        <is>
+          <t>比利时</t>
+        </is>
+      </c>
+      <c r="C237" s="3" t="inlineStr"/>
+      <c r="D237" s="3" t="inlineStr">
+        <is>
+          <t>foxconcept.be</t>
+        </is>
+      </c>
+      <c r="E237" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F237" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G237" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H237" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I237" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J237" s="3" t="inlineStr">
+        <is>
+          <t>+32 2 808 35 35 / info@foxconcept.be</t>
+        </is>
+      </c>
+      <c r="K237" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L237" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M237" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N237" s="3" t="inlineStr"/>
+      <c r="O237" s="3" t="inlineStr"/>
+      <c r="P237" s="3" t="inlineStr"/>
+      <c r="Q237" s="3" t="inlineStr">
+        <is>
+          <t>Tongrinne</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="3" t="inlineStr">
+        <is>
+          <t>NETZWARE</t>
+        </is>
+      </c>
+      <c r="B238" s="3" t="inlineStr">
+        <is>
+          <t>奥地利</t>
+        </is>
+      </c>
+      <c r="C238" s="3" t="inlineStr"/>
+      <c r="D238" s="3" t="inlineStr">
+        <is>
+          <t>netzware.at</t>
+        </is>
+      </c>
+      <c r="E238" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F238" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G238" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H238" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I238" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J238" s="3" t="inlineStr">
+        <is>
+          <t>+43 1 3577777 / office@netzware.at</t>
+        </is>
+      </c>
+      <c r="K238" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L238" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M238" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N238" s="3" t="inlineStr"/>
+      <c r="O238" s="3" t="inlineStr"/>
+      <c r="P238" s="3" t="inlineStr"/>
+      <c r="Q238" s="3" t="inlineStr">
+        <is>
+          <t>Wien</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="3" t="inlineStr">
+        <is>
+          <t>TRIOTRONIK</t>
+        </is>
+      </c>
+      <c r="B239" s="3" t="inlineStr">
+        <is>
+          <t>奥地利</t>
+        </is>
+      </c>
+      <c r="C239" s="3" t="inlineStr"/>
+      <c r="D239" s="3" t="inlineStr">
+        <is>
+          <t>triotronik.com</t>
+        </is>
+      </c>
+      <c r="E239" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F239" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G239" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H239" s="3" t="inlineStr">
+        <is>
+          <t>专属邮箱 mikrotik@triotronik.com + 站内 MikroTik 专页 → 单品牌依赖</t>
+        </is>
+      </c>
+      <c r="I239" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J239" s="3" t="inlineStr">
+        <is>
+          <t>+43 3172 42299 0 / mikrotik@triotronik.com</t>
+        </is>
+      </c>
+      <c r="K239" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L239" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M239" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N239" s="3" t="inlineStr"/>
+      <c r="O239" s="3" t="inlineStr"/>
+      <c r="P239" s="3" t="inlineStr"/>
+      <c r="Q239" s="3" t="inlineStr">
+        <is>
+          <t>Weiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="3" t="inlineStr">
+        <is>
+          <t>evoNET</t>
+        </is>
+      </c>
+      <c r="B240" s="3" t="inlineStr">
+        <is>
+          <t>奥地利</t>
+        </is>
+      </c>
+      <c r="C240" s="3" t="inlineStr"/>
+      <c r="D240" s="3" t="inlineStr">
+        <is>
+          <t>evonet.at</t>
+        </is>
+      </c>
+      <c r="E240" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F240" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G240" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H240" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I240" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J240" s="3" t="inlineStr">
+        <is>
+          <t>+43 5442 64381 / info@evonet.at</t>
+        </is>
+      </c>
+      <c r="K240" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L240" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M240" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N240" s="3" t="inlineStr"/>
+      <c r="O240" s="3" t="inlineStr"/>
+      <c r="P240" s="3" t="inlineStr"/>
+      <c r="Q240" s="3" t="inlineStr">
+        <is>
+          <t>Landeck</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="3" t="inlineStr">
+        <is>
+          <t>AlpenEDV</t>
+        </is>
+      </c>
+      <c r="B241" s="3" t="inlineStr">
+        <is>
+          <t>奥地利</t>
+        </is>
+      </c>
+      <c r="C241" s="3" t="inlineStr"/>
+      <c r="D241" s="3" t="inlineStr">
+        <is>
+          <t>alpenedv.at</t>
+        </is>
+      </c>
+      <c r="E241" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F241" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G241" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H241" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I241" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J241" s="3" t="inlineStr">
+        <is>
+          <t>0660 255 255 1 / office@alpenedv.at</t>
+        </is>
+      </c>
+      <c r="K241" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L241" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M241" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N241" s="3" t="inlineStr"/>
+      <c r="O241" s="3" t="inlineStr"/>
+      <c r="P241" s="3" t="inlineStr"/>
+      <c r="Q241" s="3" t="inlineStr">
+        <is>
+          <t>Hall in Tirol</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="3" t="inlineStr">
+        <is>
+          <t>QEDV IT-Lösungen（Raum4 GmbH）</t>
+        </is>
+      </c>
+      <c r="B242" s="3" t="inlineStr">
+        <is>
+          <t>奥地利</t>
+        </is>
+      </c>
+      <c r="C242" s="3" t="inlineStr"/>
+      <c r="D242" s="3" t="inlineStr">
+        <is>
+          <t>shop.qedv.at</t>
+        </is>
+      </c>
+      <c r="E242" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F242" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G242" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H242" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I242" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J242" s="3" t="inlineStr">
+        <is>
+          <t>+43 676 852 996 701 / office@qedv.at</t>
+        </is>
+      </c>
+      <c r="K242" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L242" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M242" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N242" s="3" t="inlineStr"/>
+      <c r="O242" s="3" t="inlineStr"/>
+      <c r="P242" s="3" t="inlineStr"/>
+      <c r="Q242" s="3" t="inlineStr">
+        <is>
+          <t>Hall in Tirol</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="3" t="inlineStr">
+        <is>
+          <t>Wifx SA</t>
+        </is>
+      </c>
+      <c r="B243" s="3" t="inlineStr">
+        <is>
+          <t>瑞士</t>
+        </is>
+      </c>
+      <c r="C243" s="3" t="inlineStr"/>
+      <c r="D243" s="3" t="inlineStr">
+        <is>
+          <t>shop.wifx.net</t>
+        </is>
+      </c>
+      <c r="E243" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F243" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G243" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H243" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I243" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J243" s="3" t="inlineStr">
+        <is>
+          <t>+41 24 550 01 70 / info@wifx.net</t>
+        </is>
+      </c>
+      <c r="K243" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L243" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M243" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N243" s="3" t="inlineStr"/>
+      <c r="O243" s="3" t="inlineStr"/>
+      <c r="P243" s="3" t="inlineStr"/>
+      <c r="Q243" s="3" t="inlineStr">
+        <is>
+          <t>Yverdon-les-Bains</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="3" t="inlineStr">
+        <is>
+          <t>ENGITECH S.A.</t>
+        </is>
+      </c>
+      <c r="B244" s="3" t="inlineStr">
+        <is>
+          <t>瑞士</t>
+        </is>
+      </c>
+      <c r="C244" s="3" t="inlineStr"/>
+      <c r="D244" s="3" t="inlineStr">
+        <is>
+          <t>engitech.ch</t>
+        </is>
+      </c>
+      <c r="E244" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F244" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G244" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H244" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I244" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J244" s="3" t="inlineStr">
+        <is>
+          <t>+41 76 326 40 00 / office@engitech.ch</t>
+        </is>
+      </c>
+      <c r="K244" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L244" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M244" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N244" s="3" t="inlineStr"/>
+      <c r="O244" s="3" t="inlineStr"/>
+      <c r="P244" s="3" t="inlineStr"/>
+      <c r="Q244" s="3" t="inlineStr">
+        <is>
+          <t>Genève</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="3" t="inlineStr">
+        <is>
+          <t>Senetic AG</t>
+        </is>
+      </c>
+      <c r="B245" s="3" t="inlineStr">
+        <is>
+          <t>瑞士</t>
+        </is>
+      </c>
+      <c r="C245" s="3" t="inlineStr"/>
+      <c r="D245" s="3" t="inlineStr">
+        <is>
+          <t>senetic.ch</t>
+        </is>
+      </c>
+      <c r="E245" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F245" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G245" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H245" s="3" t="inlineStr">
+        <is>
+          <t>Senetic 集团瑞士站</t>
+        </is>
+      </c>
+      <c r="I245" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J245" s="3" t="inlineStr">
+        <is>
+          <t>+41 43 210 52 00 / info@senetic.ch</t>
+        </is>
+      </c>
+      <c r="K245" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L245" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M245" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N245" s="3" t="inlineStr"/>
+      <c r="O245" s="3" t="inlineStr"/>
+      <c r="P245" s="3" t="inlineStr"/>
+      <c r="Q245" s="3" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="3" t="inlineStr">
+        <is>
+          <t>Alltron AG</t>
+        </is>
+      </c>
+      <c r="B246" s="3" t="inlineStr">
+        <is>
+          <t>瑞士</t>
+        </is>
+      </c>
+      <c r="C246" s="3" t="inlineStr"/>
+      <c r="D246" s="3" t="inlineStr">
+        <is>
+          <t>alltron.ch</t>
+        </is>
+      </c>
+      <c r="E246" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F246" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G246" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H246" s="3" t="inlineStr">
+        <is>
+          <t>瑞士本土大型 IT 分销</t>
+        </is>
+      </c>
+      <c r="I246" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT</t>
+        </is>
+      </c>
+      <c r="J246" s="3" t="inlineStr">
+        <is>
+          <t>062 889 88 88 / mail@alltron.ch</t>
+        </is>
+      </c>
+      <c r="K246" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L246" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M246" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N246" s="3" t="inlineStr"/>
+      <c r="O246" s="3" t="inlineStr"/>
+      <c r="P246" s="3" t="inlineStr"/>
+      <c r="Q246" s="3" t="inlineStr">
+        <is>
+          <t>Mägenwil</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="3" t="inlineStr">
+        <is>
+          <t>INOVIS Live Automation AG</t>
+        </is>
+      </c>
+      <c r="B247" s="3" t="inlineStr">
+        <is>
+          <t>瑞士</t>
+        </is>
+      </c>
+      <c r="C247" s="3" t="inlineStr"/>
+      <c r="D247" s="3" t="inlineStr">
+        <is>
+          <t>shop.inovis-group.com</t>
+        </is>
+      </c>
+      <c r="E247" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F247" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G247" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H247" s="3" t="inlineStr">
+        <is>
+          <t>工业自动化分销 → 最贴你的工业线</t>
+        </is>
+      </c>
+      <c r="I247" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J247" s="3" t="inlineStr">
+        <is>
+          <t>+41 55 253 44 88 / sales@inovis-group.com</t>
+        </is>
+      </c>
+      <c r="K247" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L247" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M247" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N247" s="3" t="inlineStr"/>
+      <c r="O247" s="3" t="inlineStr"/>
+      <c r="P247" s="3" t="inlineStr"/>
+      <c r="Q247" s="3" t="inlineStr">
+        <is>
+          <t>Bubikon/Zürich</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="3" t="inlineStr">
+        <is>
+          <t>Aurdel Sweden AB</t>
+        </is>
+      </c>
+      <c r="B248" s="3" t="inlineStr">
+        <is>
+          <t>瑞典</t>
+        </is>
+      </c>
+      <c r="C248" s="3" t="inlineStr"/>
+      <c r="D248" s="3" t="inlineStr">
+        <is>
+          <t>aurdel.com</t>
+        </is>
+      </c>
+      <c r="E248" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F248" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G248" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H248" s="3" t="inlineStr">
+        <is>
+          <t>Aurdel 集团北欧三国（瑞典/丹麦/芬兰）统一采购</t>
+        </is>
+      </c>
+      <c r="I248" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J248" s="3" t="inlineStr">
+        <is>
+          <t>+46 8 555 762 00 / Kundservice@deltaco.se</t>
+        </is>
+      </c>
+      <c r="K248" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L248" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M248" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N248" s="3" t="inlineStr"/>
+      <c r="O248" s="3" t="inlineStr"/>
+      <c r="P248" s="3" t="inlineStr"/>
+      <c r="Q248" s="3" t="inlineStr">
+        <is>
+          <t>Åkersberga；北欧集团总部</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="3" t="inlineStr">
+        <is>
+          <t>AxByte（netdist.se）</t>
+        </is>
+      </c>
+      <c r="B249" s="3" t="inlineStr">
+        <is>
+          <t>瑞典</t>
+        </is>
+      </c>
+      <c r="C249" s="3" t="inlineStr"/>
+      <c r="D249" s="3" t="inlineStr">
+        <is>
+          <t>netdist.se</t>
+        </is>
+      </c>
+      <c r="E249" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F249" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G249" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H249" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I249" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J249" s="3" t="inlineStr">
+        <is>
+          <t>08-586 195 00 / contact@axbyte.se</t>
+        </is>
+      </c>
+      <c r="K249" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L249" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M249" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N249" s="3" t="inlineStr"/>
+      <c r="O249" s="3" t="inlineStr"/>
+      <c r="P249" s="3" t="inlineStr"/>
+      <c r="Q249" s="3" t="inlineStr">
+        <is>
+          <t>Farsta</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="3" t="inlineStr">
+        <is>
+          <t>Satellithuset i Limmared AB（routerboard.se）</t>
+        </is>
+      </c>
+      <c r="B250" s="3" t="inlineStr">
+        <is>
+          <t>瑞典</t>
+        </is>
+      </c>
+      <c r="C250" s="3" t="inlineStr"/>
+      <c r="D250" s="3" t="inlineStr">
+        <is>
+          <t>routerboard.se</t>
+        </is>
+      </c>
+      <c r="E250" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F250" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G250" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H250" s="3" t="inlineStr">
+        <is>
+          <t>域名 mikrotik.se + routerboard.se → 单品牌依赖最高档</t>
+        </is>
+      </c>
+      <c r="I250" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J250" s="3" t="inlineStr">
+        <is>
+          <t>+46 325 660 650 / info@mikrotik.se</t>
+        </is>
+      </c>
+      <c r="K250" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L250" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M250" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N250" s="3" t="inlineStr"/>
+      <c r="O250" s="3" t="inlineStr"/>
+      <c r="P250" s="3" t="inlineStr"/>
+      <c r="Q250" s="3" t="inlineStr">
+        <is>
+          <t>Limmared</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="3" t="inlineStr">
+        <is>
+          <t>Senetic AB</t>
+        </is>
+      </c>
+      <c r="B251" s="3" t="inlineStr">
+        <is>
+          <t>瑞典</t>
+        </is>
+      </c>
+      <c r="C251" s="3" t="inlineStr"/>
+      <c r="D251" s="3" t="inlineStr">
+        <is>
+          <t>senetic.se</t>
+        </is>
+      </c>
+      <c r="E251" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F251" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G251" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H251" s="3" t="inlineStr">
+        <is>
+          <t>Senetic 集团瑞典站</t>
+        </is>
+      </c>
+      <c r="I251" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J251" s="3" t="inlineStr">
+        <is>
+          <t>+46 8 505 217 00 / info@senetic.se</t>
+        </is>
+      </c>
+      <c r="K251" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L251" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M251" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N251" s="3" t="inlineStr"/>
+      <c r="O251" s="3" t="inlineStr"/>
+      <c r="P251" s="3" t="inlineStr"/>
+      <c r="Q251" s="3" t="inlineStr">
+        <is>
+          <t>Stockholm</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="3" t="inlineStr">
+        <is>
+          <t>Dialect Skövde（evolvit.se）</t>
+        </is>
+      </c>
+      <c r="B252" s="3" t="inlineStr">
+        <is>
+          <t>瑞典</t>
+        </is>
+      </c>
+      <c r="C252" s="3" t="inlineStr"/>
+      <c r="D252" s="3" t="inlineStr">
+        <is>
+          <t>shop.evolvit.se</t>
+        </is>
+      </c>
+      <c r="E252" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F252" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G252" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H252" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I252" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J252" s="3" t="inlineStr">
+        <is>
+          <t>0500 105 300</t>
+        </is>
+      </c>
+      <c r="K252" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L252" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M252" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N252" s="3" t="inlineStr"/>
+      <c r="O252" s="3" t="inlineStr"/>
+      <c r="P252" s="3" t="inlineStr"/>
+      <c r="Q252" s="3" t="inlineStr">
+        <is>
+          <t>Skövde</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="3" t="inlineStr">
+        <is>
+          <t>Sanuk Systems AB</t>
+        </is>
+      </c>
+      <c r="B253" s="3" t="inlineStr">
+        <is>
+          <t>瑞典</t>
+        </is>
+      </c>
+      <c r="C253" s="3" t="inlineStr"/>
+      <c r="D253" s="3" t="inlineStr">
+        <is>
+          <t>sanuksystems.com</t>
+        </is>
+      </c>
+      <c r="E253" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F253" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G253" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H253" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I253" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J253" s="3" t="inlineStr">
+        <is>
+          <t>+46 70 696 66 60 / mail@sanuksystems.com</t>
+        </is>
+      </c>
+      <c r="K253" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L253" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M253" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N253" s="3" t="inlineStr"/>
+      <c r="O253" s="3" t="inlineStr"/>
+      <c r="P253" s="3" t="inlineStr"/>
+      <c r="Q253" s="3" t="inlineStr">
+        <is>
+          <t>Älvsjö</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="3" t="inlineStr">
+        <is>
+          <t>ALLNET Nordic A/S</t>
+        </is>
+      </c>
+      <c r="B254" s="3" t="inlineStr">
+        <is>
+          <t>丹麦</t>
+        </is>
+      </c>
+      <c r="C254" s="3" t="inlineStr"/>
+      <c r="D254" s="3" t="inlineStr">
+        <is>
+          <t>shop.allnet.dk</t>
+        </is>
+      </c>
+      <c r="E254" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F254" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G254" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H254" s="3" t="inlineStr">
+        <is>
+          <t>ALLNET 集团北欧站（德/法/意/丹 = 4 国）</t>
+        </is>
+      </c>
+      <c r="I254" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT</t>
+        </is>
+      </c>
+      <c r="J254" s="3" t="inlineStr">
+        <is>
+          <t>+45 69 96 00 00 / info@allnet.dk</t>
+        </is>
+      </c>
+      <c r="K254" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L254" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M254" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N254" s="3" t="inlineStr"/>
+      <c r="O254" s="3" t="inlineStr"/>
+      <c r="P254" s="3" t="inlineStr"/>
+      <c r="Q254" s="3" t="inlineStr">
+        <is>
+          <t>Ballerup</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="3" t="inlineStr">
+        <is>
+          <t>Dvisor IT ApS</t>
+        </is>
+      </c>
+      <c r="B255" s="3" t="inlineStr">
+        <is>
+          <t>丹麦</t>
+        </is>
+      </c>
+      <c r="C255" s="3" t="inlineStr"/>
+      <c r="D255" s="3" t="inlineStr">
+        <is>
+          <t>shop.dvisor.dk</t>
+        </is>
+      </c>
+      <c r="E255" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F255" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G255" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H255" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I255" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J255" s="3" t="inlineStr">
+        <is>
+          <t>+45 69 17 07 08 / info@dvisor.dk</t>
+        </is>
+      </c>
+      <c r="K255" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L255" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M255" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N255" s="3" t="inlineStr"/>
+      <c r="O255" s="3" t="inlineStr"/>
+      <c r="P255" s="3" t="inlineStr"/>
+      <c r="Q255" s="3" t="inlineStr">
+        <is>
+          <t>Rønde</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="3" t="inlineStr">
+        <is>
+          <t>Nextron AS</t>
+        </is>
+      </c>
+      <c r="B256" s="3" t="inlineStr">
+        <is>
+          <t>丹麦</t>
+        </is>
+      </c>
+      <c r="C256" s="3" t="inlineStr"/>
+      <c r="D256" s="3" t="inlineStr">
+        <is>
+          <t>nextron.dk</t>
+        </is>
+      </c>
+      <c r="E256" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F256" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G256" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H256" s="3" t="inlineStr">
+        <is>
+          <t>Nextron 北欧多国（丹/挪/芬/瑞典）</t>
+        </is>
+      </c>
+      <c r="I256" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J256" s="3" t="inlineStr">
+        <is>
+          <t>+45 70 10 37 00 / sales@nextron.dk</t>
+        </is>
+      </c>
+      <c r="K256" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L256" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M256" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N256" s="3" t="inlineStr"/>
+      <c r="O256" s="3" t="inlineStr"/>
+      <c r="P256" s="3" t="inlineStr"/>
+      <c r="Q256" s="3" t="inlineStr">
+        <is>
+          <t>Copenhagen</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="3" t="inlineStr">
+        <is>
+          <t>Puma Solutions ApS</t>
+        </is>
+      </c>
+      <c r="B257" s="3" t="inlineStr">
+        <is>
+          <t>丹麦</t>
+        </is>
+      </c>
+      <c r="C257" s="3" t="inlineStr"/>
+      <c r="D257" s="3" t="inlineStr">
+        <is>
+          <t>pumait.dk</t>
+        </is>
+      </c>
+      <c r="E257" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F257" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G257" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H257" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I257" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J257" s="3" t="inlineStr">
+        <is>
+          <t>+45 60 70 90 09 / rfi@pumait.dk</t>
+        </is>
+      </c>
+      <c r="K257" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L257" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M257" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N257" s="3" t="inlineStr"/>
+      <c r="O257" s="3" t="inlineStr"/>
+      <c r="P257" s="3" t="inlineStr"/>
+      <c r="Q257" s="3" t="inlineStr">
+        <is>
+          <t>Valby</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="3" t="inlineStr">
+        <is>
+          <t>LocalNet Finland</t>
+        </is>
+      </c>
+      <c r="B258" s="3" t="inlineStr">
+        <is>
+          <t>芬兰</t>
+        </is>
+      </c>
+      <c r="C258" s="3" t="inlineStr"/>
+      <c r="D258" s="3" t="inlineStr">
+        <is>
+          <t>localnet.fi</t>
+        </is>
+      </c>
+      <c r="E258" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F258" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G258" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H258" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I258" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J258" s="3" t="inlineStr">
+        <is>
+          <t>+358 9 4241 3260 / myynti@localnet.fi</t>
+        </is>
+      </c>
+      <c r="K258" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L258" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M258" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N258" s="3" t="inlineStr"/>
+      <c r="O258" s="3" t="inlineStr"/>
+      <c r="P258" s="3" t="inlineStr"/>
+      <c r="Q258" s="3" t="inlineStr">
+        <is>
+          <t>Espoo</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Sweep 7 more countries: Portugal, Romania, Hungary, Greece, Turkey, Ireland, Norway
40 more MikroTik official distributors with phone and email. Two more
pan-European groups surface: ALLNET now spans 5 countries (DE/FR/IT/DK/GR)
and ELKO Group (Baltic/CEE, 10+ countries) enters the list, alongside
ALSO, Dustin and Winncom as regional heavyweights.
Netter System (mikrotik.ro) joins the single-brand-dependent targets.
Running total: 292 accounts.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q258"/>
+  <dimension ref="A1:Q294"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -29237,6 +29237,2562 @@
       <c r="Q258" s="3" t="inlineStr">
         <is>
           <t>Espoo</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="3" t="inlineStr">
+        <is>
+          <t>Officelan</t>
+        </is>
+      </c>
+      <c r="B259" s="3" t="inlineStr">
+        <is>
+          <t>葡萄牙</t>
+        </is>
+      </c>
+      <c r="C259" s="3" t="inlineStr"/>
+      <c r="D259" s="3" t="inlineStr">
+        <is>
+          <t>shop.officelan.pt</t>
+        </is>
+      </c>
+      <c r="E259" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F259" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G259" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H259" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I259" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J259" s="3" t="inlineStr">
+        <is>
+          <t>+351 232 186 575 / comercial@officelan.pt</t>
+        </is>
+      </c>
+      <c r="K259" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L259" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M259" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N259" s="3" t="inlineStr"/>
+      <c r="O259" s="3" t="inlineStr"/>
+      <c r="P259" s="3" t="inlineStr"/>
+      <c r="Q259" s="3" t="inlineStr">
+        <is>
+          <t>Canas de Senhorim</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="3" t="inlineStr">
+        <is>
+          <t>TRUENET</t>
+        </is>
+      </c>
+      <c r="B260" s="3" t="inlineStr">
+        <is>
+          <t>葡萄牙</t>
+        </is>
+      </c>
+      <c r="C260" s="3" t="inlineStr"/>
+      <c r="D260" s="3" t="inlineStr">
+        <is>
+          <t>truenet.pt</t>
+        </is>
+      </c>
+      <c r="E260" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F260" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G260" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H260" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I260" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J260" s="3" t="inlineStr">
+        <is>
+          <t>+351 936 794 301 / comercial@truenet.pt</t>
+        </is>
+      </c>
+      <c r="K260" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L260" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M260" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N260" s="3" t="inlineStr"/>
+      <c r="O260" s="3" t="inlineStr"/>
+      <c r="P260" s="3" t="inlineStr"/>
+      <c r="Q260" s="3" t="inlineStr">
+        <is>
+          <t>Lisboa</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="3" t="inlineStr">
+        <is>
+          <t>Netter System SRL（mikrotik.ro）</t>
+        </is>
+      </c>
+      <c r="B261" s="3" t="inlineStr">
+        <is>
+          <t>罗马尼亚</t>
+        </is>
+      </c>
+      <c r="C261" s="3" t="inlineStr"/>
+      <c r="D261" s="3" t="inlineStr">
+        <is>
+          <t>mikrotik.ro</t>
+        </is>
+      </c>
+      <c r="E261" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F261" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G261" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H261" s="3" t="inlineStr">
+        <is>
+          <t>域名就是 mikrotik.ro → 单品牌依赖最高档</t>
+        </is>
+      </c>
+      <c r="I261" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J261" s="3" t="inlineStr">
+        <is>
+          <t>+40 744 334 260 / office@mikrotik.ro</t>
+        </is>
+      </c>
+      <c r="K261" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L261" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M261" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N261" s="3" t="inlineStr"/>
+      <c r="O261" s="3" t="inlineStr"/>
+      <c r="P261" s="3" t="inlineStr"/>
+      <c r="Q261" s="3" t="inlineStr">
+        <is>
+          <t>Cristuru Secuiesc</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="3" t="inlineStr">
+        <is>
+          <t>TELESYSTEM</t>
+        </is>
+      </c>
+      <c r="B262" s="3" t="inlineStr">
+        <is>
+          <t>罗马尼亚</t>
+        </is>
+      </c>
+      <c r="C262" s="3" t="inlineStr"/>
+      <c r="D262" s="3" t="inlineStr">
+        <is>
+          <t>telesystem.ro</t>
+        </is>
+      </c>
+      <c r="E262" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F262" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G262" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H262" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I262" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J262" s="3" t="inlineStr">
+        <is>
+          <t>+40 31 101 99 09 / comenzi@telesystem.ro</t>
+        </is>
+      </c>
+      <c r="K262" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L262" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M262" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N262" s="3" t="inlineStr"/>
+      <c r="O262" s="3" t="inlineStr"/>
+      <c r="P262" s="3" t="inlineStr"/>
+      <c r="Q262" s="3" t="inlineStr">
+        <is>
+          <t>Bacău / București / Iași</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="3" t="inlineStr">
+        <is>
+          <t>Wifimag.ro</t>
+        </is>
+      </c>
+      <c r="B263" s="3" t="inlineStr">
+        <is>
+          <t>罗马尼亚</t>
+        </is>
+      </c>
+      <c r="C263" s="3" t="inlineStr"/>
+      <c r="D263" s="3" t="inlineStr">
+        <is>
+          <t>wifimag.ro</t>
+        </is>
+      </c>
+      <c r="E263" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F263" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G263" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H263" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I263" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J263" s="3" t="inlineStr">
+        <is>
+          <t>+40 748 113 178 / mikrotik@wifimag.ro</t>
+        </is>
+      </c>
+      <c r="K263" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L263" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M263" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N263" s="3" t="inlineStr"/>
+      <c r="O263" s="3" t="inlineStr"/>
+      <c r="P263" s="3" t="inlineStr"/>
+      <c r="Q263" s="3" t="inlineStr">
+        <is>
+          <t>Tulcea</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="3" t="inlineStr">
+        <is>
+          <t>Dipol Connect SRL</t>
+        </is>
+      </c>
+      <c r="B264" s="3" t="inlineStr">
+        <is>
+          <t>罗马尼亚</t>
+        </is>
+      </c>
+      <c r="C264" s="3" t="inlineStr"/>
+      <c r="D264" s="3" t="inlineStr">
+        <is>
+          <t>dipolnet.ro</t>
+        </is>
+      </c>
+      <c r="E264" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F264" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G264" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H264" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I264" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J264" s="3" t="inlineStr">
+        <is>
+          <t>+40 742 145 758 / office@dipolnet.ro</t>
+        </is>
+      </c>
+      <c r="K264" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L264" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M264" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N264" s="3" t="inlineStr"/>
+      <c r="O264" s="3" t="inlineStr"/>
+      <c r="P264" s="3" t="inlineStr"/>
+      <c r="Q264" s="3" t="inlineStr">
+        <is>
+          <t>București</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="3" t="inlineStr">
+        <is>
+          <t>Senetic Romania SRL</t>
+        </is>
+      </c>
+      <c r="B265" s="3" t="inlineStr">
+        <is>
+          <t>罗马尼亚</t>
+        </is>
+      </c>
+      <c r="C265" s="3" t="inlineStr"/>
+      <c r="D265" s="3" t="inlineStr">
+        <is>
+          <t>senetic.ro</t>
+        </is>
+      </c>
+      <c r="E265" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F265" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G265" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H265" s="3" t="inlineStr">
+        <is>
+          <t>Senetic 集团罗马尼亚站</t>
+        </is>
+      </c>
+      <c r="I265" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J265" s="3" t="inlineStr">
+        <is>
+          <t>+40 21 555 71 00 / info@senetic.ro</t>
+        </is>
+      </c>
+      <c r="K265" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L265" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M265" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N265" s="3" t="inlineStr"/>
+      <c r="O265" s="3" t="inlineStr"/>
+      <c r="P265" s="3" t="inlineStr"/>
+      <c r="Q265" s="3" t="inlineStr">
+        <is>
+          <t>București</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="3" t="inlineStr">
+        <is>
+          <t>Elko Romania</t>
+        </is>
+      </c>
+      <c r="B266" s="3" t="inlineStr">
+        <is>
+          <t>罗马尼亚</t>
+        </is>
+      </c>
+      <c r="C266" s="3" t="inlineStr"/>
+      <c r="D266" s="3" t="inlineStr">
+        <is>
+          <t>elko.ro</t>
+        </is>
+      </c>
+      <c r="E266" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F266" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G266" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H266" s="3" t="inlineStr">
+        <is>
+          <t>ELKO 集团 = 波罗的海/中东欧最大 IT 分销（拉脱维亚总部，覆盖 10+ 国）</t>
+        </is>
+      </c>
+      <c r="I266" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT</t>
+        </is>
+      </c>
+      <c r="J266" s="3" t="inlineStr">
+        <is>
+          <t>+40 21 224 60 94 / sales@elko.ro</t>
+        </is>
+      </c>
+      <c r="K266" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L266" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M266" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N266" s="3" t="inlineStr"/>
+      <c r="O266" s="3" t="inlineStr"/>
+      <c r="P266" s="3" t="inlineStr"/>
+      <c r="Q266" s="3" t="inlineStr">
+        <is>
+          <t>București；跨国集团</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="3" t="inlineStr">
+        <is>
+          <t>Compmarket Hungary Zrt.</t>
+        </is>
+      </c>
+      <c r="B267" s="3" t="inlineStr">
+        <is>
+          <t>匈牙利</t>
+        </is>
+      </c>
+      <c r="C267" s="3" t="inlineStr"/>
+      <c r="D267" s="3" t="inlineStr">
+        <is>
+          <t>compmarket.hu</t>
+        </is>
+      </c>
+      <c r="E267" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F267" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G267" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H267" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I267" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J267" s="3" t="inlineStr">
+        <is>
+          <t>+36 1 222 6403 / rakos.zoltan@compmarket.hu</t>
+        </is>
+      </c>
+      <c r="K267" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L267" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M267" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N267" s="3" t="inlineStr"/>
+      <c r="O267" s="3" t="inlineStr"/>
+      <c r="P267" s="3" t="inlineStr"/>
+      <c r="Q267" s="3" t="inlineStr">
+        <is>
+          <t>Budapest</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="3" t="inlineStr">
+        <is>
+          <t>Expert Zrt.</t>
+        </is>
+      </c>
+      <c r="B268" s="3" t="inlineStr">
+        <is>
+          <t>匈牙利</t>
+        </is>
+      </c>
+      <c r="C268" s="3" t="inlineStr"/>
+      <c r="D268" s="3" t="inlineStr">
+        <is>
+          <t>expert.hu</t>
+        </is>
+      </c>
+      <c r="E268" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F268" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G268" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H268" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I268" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT</t>
+        </is>
+      </c>
+      <c r="J268" s="3" t="inlineStr">
+        <is>
+          <t>+36 30 906 3854 / network@expert.hu</t>
+        </is>
+      </c>
+      <c r="K268" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L268" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M268" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N268" s="3" t="inlineStr"/>
+      <c r="O268" s="3" t="inlineStr"/>
+      <c r="P268" s="3" t="inlineStr"/>
+      <c r="Q268" s="3" t="inlineStr">
+        <is>
+          <t>Budapest</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="3" t="inlineStr">
+        <is>
+          <t>AccessPoint Kft.</t>
+        </is>
+      </c>
+      <c r="B269" s="3" t="inlineStr">
+        <is>
+          <t>匈牙利</t>
+        </is>
+      </c>
+      <c r="C269" s="3" t="inlineStr"/>
+      <c r="D269" s="3" t="inlineStr">
+        <is>
+          <t>accesspoint.hu</t>
+        </is>
+      </c>
+      <c r="E269" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F269" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G269" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H269" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I269" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J269" s="3" t="inlineStr">
+        <is>
+          <t>+36 1 219 5345 / info@accesspoint.hu</t>
+        </is>
+      </c>
+      <c r="K269" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L269" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M269" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N269" s="3" t="inlineStr"/>
+      <c r="O269" s="3" t="inlineStr"/>
+      <c r="P269" s="3" t="inlineStr"/>
+      <c r="Q269" s="3" t="inlineStr">
+        <is>
+          <t>Budapest</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="3" t="inlineStr">
+        <is>
+          <t>ALSO Hungary（Ramiris）</t>
+        </is>
+      </c>
+      <c r="B270" s="3" t="inlineStr">
+        <is>
+          <t>匈牙利</t>
+        </is>
+      </c>
+      <c r="C270" s="3" t="inlineStr"/>
+      <c r="D270" s="3" t="inlineStr">
+        <is>
+          <t>also.com</t>
+        </is>
+      </c>
+      <c r="E270" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F270" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G270" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H270" s="3" t="inlineStr">
+        <is>
+          <t>ALSO 集团 = 欧洲三大 IT 分销之一（德/瑞/奥/匈等）</t>
+        </is>
+      </c>
+      <c r="I270" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J270" s="3" t="inlineStr">
+        <is>
+          <t>+36 1 888 3200 / info@ramiris.eu</t>
+        </is>
+      </c>
+      <c r="K270" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L270" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M270" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N270" s="3" t="inlineStr"/>
+      <c r="O270" s="3" t="inlineStr"/>
+      <c r="P270" s="3" t="inlineStr"/>
+      <c r="Q270" s="3" t="inlineStr">
+        <is>
+          <t>Budapest；泛欧大分销</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="3" t="inlineStr">
+        <is>
+          <t>Wireless-Bolt</t>
+        </is>
+      </c>
+      <c r="B271" s="3" t="inlineStr">
+        <is>
+          <t>匈牙利</t>
+        </is>
+      </c>
+      <c r="C271" s="3" t="inlineStr"/>
+      <c r="D271" s="3" t="inlineStr">
+        <is>
+          <t>wireless-bolt.hu</t>
+        </is>
+      </c>
+      <c r="E271" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F271" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G271" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H271" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I271" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J271" s="3" t="inlineStr">
+        <is>
+          <t>+36 20 927 2662 / info@wireless-bolt.hu</t>
+        </is>
+      </c>
+      <c r="K271" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L271" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M271" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N271" s="3" t="inlineStr"/>
+      <c r="O271" s="3" t="inlineStr"/>
+      <c r="P271" s="3" t="inlineStr"/>
+      <c r="Q271" s="3" t="inlineStr">
+        <is>
+          <t>Albertirsa</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="3" t="inlineStr">
+        <is>
+          <t>AbsolCom Kft.</t>
+        </is>
+      </c>
+      <c r="B272" s="3" t="inlineStr">
+        <is>
+          <t>匈牙利</t>
+        </is>
+      </c>
+      <c r="C272" s="3" t="inlineStr"/>
+      <c r="D272" s="3" t="inlineStr">
+        <is>
+          <t>absolcom.hu</t>
+        </is>
+      </c>
+      <c r="E272" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F272" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G272" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H272" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I272" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J272" s="3" t="inlineStr">
+        <is>
+          <t>+36 1 431 0116 / info@absolcom.hu</t>
+        </is>
+      </c>
+      <c r="K272" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L272" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M272" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N272" s="3" t="inlineStr"/>
+      <c r="O272" s="3" t="inlineStr"/>
+      <c r="P272" s="3" t="inlineStr"/>
+      <c r="Q272" s="3" t="inlineStr">
+        <is>
+          <t>Budapest</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="3" t="inlineStr">
+        <is>
+          <t>Senetic Magyarország Kft.</t>
+        </is>
+      </c>
+      <c r="B273" s="3" t="inlineStr">
+        <is>
+          <t>匈牙利</t>
+        </is>
+      </c>
+      <c r="C273" s="3" t="inlineStr"/>
+      <c r="D273" s="3" t="inlineStr">
+        <is>
+          <t>senetic.hu</t>
+        </is>
+      </c>
+      <c r="E273" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F273" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G273" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H273" s="3" t="inlineStr">
+        <is>
+          <t>Senetic 集团匈牙利站</t>
+        </is>
+      </c>
+      <c r="I273" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J273" s="3" t="inlineStr">
+        <is>
+          <t>+36 1 700 8371 / info@senetic.hu</t>
+        </is>
+      </c>
+      <c r="K273" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L273" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M273" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N273" s="3" t="inlineStr"/>
+      <c r="O273" s="3" t="inlineStr"/>
+      <c r="P273" s="3" t="inlineStr"/>
+      <c r="Q273" s="3" t="inlineStr">
+        <is>
+          <t>Budapest</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="3" t="inlineStr">
+        <is>
+          <t>XPATIT S.A.</t>
+        </is>
+      </c>
+      <c r="B274" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C274" s="3" t="inlineStr"/>
+      <c r="D274" s="3" t="inlineStr">
+        <is>
+          <t>xpatit.gr</t>
+        </is>
+      </c>
+      <c r="E274" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F274" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G274" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H274" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I274" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J274" s="3" t="inlineStr">
+        <is>
+          <t>+30 211 800 0313 / info@xpatit.gr</t>
+        </is>
+      </c>
+      <c r="K274" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L274" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M274" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N274" s="3" t="inlineStr"/>
+      <c r="O274" s="3" t="inlineStr"/>
+      <c r="P274" s="3" t="inlineStr"/>
+      <c r="Q274" s="3" t="inlineStr">
+        <is>
+          <t>Attika</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="3" t="inlineStr">
+        <is>
+          <t>HellasCom L.t.d.</t>
+        </is>
+      </c>
+      <c r="B275" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C275" s="3" t="inlineStr"/>
+      <c r="D275" s="3" t="inlineStr">
+        <is>
+          <t>hellascom.gr</t>
+        </is>
+      </c>
+      <c r="E275" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F275" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G275" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H275" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I275" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J275" s="3" t="inlineStr">
+        <is>
+          <t>+30 210 4523890 / sales@hellascom.gr</t>
+        </is>
+      </c>
+      <c r="K275" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L275" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M275" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N275" s="3" t="inlineStr"/>
+      <c r="O275" s="3" t="inlineStr"/>
+      <c r="P275" s="3" t="inlineStr"/>
+      <c r="Q275" s="3" t="inlineStr">
+        <is>
+          <t>Piraeus</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="3" t="inlineStr">
+        <is>
+          <t>Hellas Digital</t>
+        </is>
+      </c>
+      <c r="B276" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C276" s="3" t="inlineStr"/>
+      <c r="D276" s="3" t="inlineStr">
+        <is>
+          <t>hellasdigital.gr</t>
+        </is>
+      </c>
+      <c r="E276" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F276" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G276" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H276" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I276" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J276" s="3" t="inlineStr">
+        <is>
+          <t>+30 210 96 111 69 / info@hellasdigital.gr</t>
+        </is>
+      </c>
+      <c r="K276" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L276" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M276" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N276" s="3" t="inlineStr"/>
+      <c r="O276" s="3" t="inlineStr"/>
+      <c r="P276" s="3" t="inlineStr"/>
+      <c r="Q276" s="3" t="inlineStr">
+        <is>
+          <t>Athens</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="3" t="inlineStr">
+        <is>
+          <t>E-WIRELESS</t>
+        </is>
+      </c>
+      <c r="B277" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C277" s="3" t="inlineStr"/>
+      <c r="D277" s="3" t="inlineStr">
+        <is>
+          <t>e-wireless.gr</t>
+        </is>
+      </c>
+      <c r="E277" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F277" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G277" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H277" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I277" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J277" s="3" t="inlineStr">
+        <is>
+          <t>+30 211 850 2484 / info@e-wireless.gr</t>
+        </is>
+      </c>
+      <c r="K277" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L277" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M277" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N277" s="3" t="inlineStr"/>
+      <c r="O277" s="3" t="inlineStr"/>
+      <c r="P277" s="3" t="inlineStr"/>
+      <c r="Q277" s="3" t="inlineStr">
+        <is>
+          <t>Argyroupoli</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="3" t="inlineStr">
+        <is>
+          <t>Allnet.Greece</t>
+        </is>
+      </c>
+      <c r="B278" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C278" s="3" t="inlineStr"/>
+      <c r="D278" s="3" t="inlineStr">
+        <is>
+          <t>allnet-italia.it</t>
+        </is>
+      </c>
+      <c r="E278" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F278" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G278" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H278" s="3" t="inlineStr">
+        <is>
+          <t>ALLNET 集团希腊站（德/法/意/丹/希 = 5 国）</t>
+        </is>
+      </c>
+      <c r="I278" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT</t>
+        </is>
+      </c>
+      <c r="J278" s="3" t="inlineStr">
+        <is>
+          <t>+30 697 552 0100 / ioanna@allnet-italia.it</t>
+        </is>
+      </c>
+      <c r="K278" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L278" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M278" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N278" s="3" t="inlineStr"/>
+      <c r="O278" s="3" t="inlineStr"/>
+      <c r="P278" s="3" t="inlineStr"/>
+      <c r="Q278" s="3" t="inlineStr">
+        <is>
+          <t>Argyroupoli</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="3" t="inlineStr">
+        <is>
+          <t>wirelesslan.gr - Teledata e.e.</t>
+        </is>
+      </c>
+      <c r="B279" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C279" s="3" t="inlineStr"/>
+      <c r="D279" s="3" t="inlineStr">
+        <is>
+          <t>wirelesslan.gr</t>
+        </is>
+      </c>
+      <c r="E279" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F279" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G279" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H279" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I279" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J279" s="3" t="inlineStr">
+        <is>
+          <t>+30 2310 510030 / info@wirelesslan.gr</t>
+        </is>
+      </c>
+      <c r="K279" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L279" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M279" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N279" s="3" t="inlineStr"/>
+      <c r="O279" s="3" t="inlineStr"/>
+      <c r="P279" s="3" t="inlineStr"/>
+      <c r="Q279" s="3" t="inlineStr">
+        <is>
+          <t>Thessaloniki</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="3" t="inlineStr">
+        <is>
+          <t>MARAC Electronics S.A.</t>
+        </is>
+      </c>
+      <c r="B280" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C280" s="3" t="inlineStr"/>
+      <c r="D280" s="3" t="inlineStr">
+        <is>
+          <t>marac.gr</t>
+        </is>
+      </c>
+      <c r="E280" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F280" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G280" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H280" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I280" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J280" s="3" t="inlineStr">
+        <is>
+          <t>+30 210 431 4361 / pipitsoulis.c@marac.gr</t>
+        </is>
+      </c>
+      <c r="K280" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L280" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M280" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N280" s="3" t="inlineStr"/>
+      <c r="O280" s="3" t="inlineStr"/>
+      <c r="P280" s="3" t="inlineStr"/>
+      <c r="Q280" s="3" t="inlineStr">
+        <is>
+          <t>Perama</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="3" t="inlineStr">
+        <is>
+          <t>CABLEWORKS</t>
+        </is>
+      </c>
+      <c r="B281" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C281" s="3" t="inlineStr"/>
+      <c r="D281" s="3" t="inlineStr">
+        <is>
+          <t>cableworks.gr</t>
+        </is>
+      </c>
+      <c r="E281" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F281" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G281" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H281" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I281" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J281" s="3" t="inlineStr">
+        <is>
+          <t>+30 211 850 2484 / info@cableworks.gr</t>
+        </is>
+      </c>
+      <c r="K281" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L281" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M281" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N281" s="3" t="inlineStr"/>
+      <c r="O281" s="3" t="inlineStr"/>
+      <c r="P281" s="3" t="inlineStr"/>
+      <c r="Q281" s="3" t="inlineStr">
+        <is>
+          <t>Argyroupoli</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="3" t="inlineStr">
+        <is>
+          <t>NODENET GLOBAL</t>
+        </is>
+      </c>
+      <c r="B282" s="3" t="inlineStr">
+        <is>
+          <t>土耳其</t>
+        </is>
+      </c>
+      <c r="C282" s="3" t="inlineStr"/>
+      <c r="D282" s="3" t="inlineStr">
+        <is>
+          <t>nodenetglobal.com</t>
+        </is>
+      </c>
+      <c r="E282" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F282" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G282" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H282" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I282" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J282" s="3" t="inlineStr">
+        <is>
+          <t>+90 533 391 2232 / sales@nodenetglobal.com</t>
+        </is>
+      </c>
+      <c r="K282" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L282" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M282" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N282" s="3" t="inlineStr"/>
+      <c r="O282" s="3" t="inlineStr"/>
+      <c r="P282" s="3" t="inlineStr"/>
+      <c r="Q282" s="3" t="inlineStr">
+        <is>
+          <t>Istanbul</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="3" t="inlineStr">
+        <is>
+          <t>Poyraz Network</t>
+        </is>
+      </c>
+      <c r="B283" s="3" t="inlineStr">
+        <is>
+          <t>土耳其</t>
+        </is>
+      </c>
+      <c r="C283" s="3" t="inlineStr"/>
+      <c r="D283" s="3" t="inlineStr">
+        <is>
+          <t>poyraznetwork.com</t>
+        </is>
+      </c>
+      <c r="E283" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F283" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G283" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H283" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I283" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J283" s="3" t="inlineStr">
+        <is>
+          <t>+90 850 346 93 63 / sales@poyraznetwork.com</t>
+        </is>
+      </c>
+      <c r="K283" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L283" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M283" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N283" s="3" t="inlineStr"/>
+      <c r="O283" s="3" t="inlineStr"/>
+      <c r="P283" s="3" t="inlineStr"/>
+      <c r="Q283" s="3" t="inlineStr">
+        <is>
+          <t>Kocaeli</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="3" t="inlineStr">
+        <is>
+          <t>Sis Bil tek（wifianten.com）</t>
+        </is>
+      </c>
+      <c r="B284" s="3" t="inlineStr">
+        <is>
+          <t>土耳其</t>
+        </is>
+      </c>
+      <c r="C284" s="3" t="inlineStr"/>
+      <c r="D284" s="3" t="inlineStr">
+        <is>
+          <t>wifianten.com</t>
+        </is>
+      </c>
+      <c r="E284" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F284" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G284" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H284" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I284" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J284" s="3" t="inlineStr">
+        <is>
+          <t>+90 850 277 5959 / bilgi@wifianten.com</t>
+        </is>
+      </c>
+      <c r="K284" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L284" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M284" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N284" s="3" t="inlineStr"/>
+      <c r="O284" s="3" t="inlineStr"/>
+      <c r="P284" s="3" t="inlineStr"/>
+      <c r="Q284" s="3" t="inlineStr">
+        <is>
+          <t>Corlu / Tekirdağ</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="3" t="inlineStr">
+        <is>
+          <t>Internetten Ltd.（wi.com.tr）</t>
+        </is>
+      </c>
+      <c r="B285" s="3" t="inlineStr">
+        <is>
+          <t>土耳其</t>
+        </is>
+      </c>
+      <c r="C285" s="3" t="inlineStr"/>
+      <c r="D285" s="3" t="inlineStr">
+        <is>
+          <t>wi.com.tr</t>
+        </is>
+      </c>
+      <c r="E285" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F285" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G285" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H285" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I285" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J285" s="3" t="inlineStr">
+        <is>
+          <t>+90 262 644 66 63 / satis@wi.com.tr</t>
+        </is>
+      </c>
+      <c r="K285" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L285" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M285" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N285" s="3" t="inlineStr"/>
+      <c r="O285" s="3" t="inlineStr"/>
+      <c r="P285" s="3" t="inlineStr"/>
+      <c r="Q285" s="3" t="inlineStr">
+        <is>
+          <t>Gebze / Kocaeli</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="3" t="inlineStr">
+        <is>
+          <t>COOLTECH TRADING</t>
+        </is>
+      </c>
+      <c r="B286" s="3" t="inlineStr">
+        <is>
+          <t>土耳其</t>
+        </is>
+      </c>
+      <c r="C286" s="3" t="inlineStr"/>
+      <c r="D286" s="3" t="inlineStr">
+        <is>
+          <t>cooltechtrading.com</t>
+        </is>
+      </c>
+      <c r="E286" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F286" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G286" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H286" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I286" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J286" s="3" t="inlineStr">
+        <is>
+          <t>+90 542 883 1111 / info@cooltechtrading.com</t>
+        </is>
+      </c>
+      <c r="K286" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L286" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M286" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N286" s="3" t="inlineStr"/>
+      <c r="O286" s="3" t="inlineStr"/>
+      <c r="P286" s="3" t="inlineStr"/>
+      <c r="Q286" s="3" t="inlineStr">
+        <is>
+          <t>Istanbul</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="3" t="inlineStr">
+        <is>
+          <t>C TECH BILISIM（enucuzmikrotik.com）</t>
+        </is>
+      </c>
+      <c r="B287" s="3" t="inlineStr">
+        <is>
+          <t>土耳其</t>
+        </is>
+      </c>
+      <c r="C287" s="3" t="inlineStr"/>
+      <c r="D287" s="3" t="inlineStr">
+        <is>
+          <t>bilisimyol.com</t>
+        </is>
+      </c>
+      <c r="E287" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F287" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G287" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H287" s="3" t="inlineStr">
+        <is>
+          <t>域名 = "最便宜的 MikroTik" → 价格导向，最看重成本</t>
+        </is>
+      </c>
+      <c r="I287" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J287" s="3" t="inlineStr">
+        <is>
+          <t>+90 850 480 44 74 / info@enucuzmikrotik.com</t>
+        </is>
+      </c>
+      <c r="K287" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L287" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M287" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N287" s="3" t="inlineStr"/>
+      <c r="O287" s="3" t="inlineStr"/>
+      <c r="P287" s="3" t="inlineStr"/>
+      <c r="Q287" s="3" t="inlineStr">
+        <is>
+          <t>Fatih；价格敏感型</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="3" t="inlineStr">
+        <is>
+          <t>Net Vizyon（4mimo.com）</t>
+        </is>
+      </c>
+      <c r="B288" s="3" t="inlineStr">
+        <is>
+          <t>土耳其</t>
+        </is>
+      </c>
+      <c r="C288" s="3" t="inlineStr"/>
+      <c r="D288" s="3" t="inlineStr">
+        <is>
+          <t>4mimo.com</t>
+        </is>
+      </c>
+      <c r="E288" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F288" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G288" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H288" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I288" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J288" s="3" t="inlineStr">
+        <is>
+          <t>+90 212 354 90 00 / satis@netvizyon.net</t>
+        </is>
+      </c>
+      <c r="K288" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L288" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M288" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N288" s="3" t="inlineStr"/>
+      <c r="O288" s="3" t="inlineStr"/>
+      <c r="P288" s="3" t="inlineStr"/>
+      <c r="Q288" s="3" t="inlineStr">
+        <is>
+          <t>Istanbul</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="3" t="inlineStr">
+        <is>
+          <t>Sekuritim Bilisim</t>
+        </is>
+      </c>
+      <c r="B289" s="3" t="inlineStr">
+        <is>
+          <t>土耳其</t>
+        </is>
+      </c>
+      <c r="C289" s="3" t="inlineStr"/>
+      <c r="D289" s="3" t="inlineStr">
+        <is>
+          <t>sekuritim.com</t>
+        </is>
+      </c>
+      <c r="E289" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F289" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G289" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H289" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I289" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J289" s="3" t="inlineStr">
+        <is>
+          <t>+90 216 302 22 21 / info@sekuritim.com</t>
+        </is>
+      </c>
+      <c r="K289" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L289" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M289" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N289" s="3" t="inlineStr"/>
+      <c r="O289" s="3" t="inlineStr"/>
+      <c r="P289" s="3" t="inlineStr"/>
+      <c r="Q289" s="3" t="inlineStr">
+        <is>
+          <t>Istanbul；安全/监控方向</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="3" t="inlineStr">
+        <is>
+          <t>Merpa Bilişim（merpazar.com）</t>
+        </is>
+      </c>
+      <c r="B290" s="3" t="inlineStr">
+        <is>
+          <t>土耳其</t>
+        </is>
+      </c>
+      <c r="C290" s="3" t="inlineStr"/>
+      <c r="D290" s="3" t="inlineStr">
+        <is>
+          <t>merpazar.com</t>
+        </is>
+      </c>
+      <c r="E290" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F290" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G290" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H290" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I290" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J290" s="3" t="inlineStr">
+        <is>
+          <t>+90 212 213 3873 / alinail@merpazar.com</t>
+        </is>
+      </c>
+      <c r="K290" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L290" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M290" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N290" s="3" t="inlineStr"/>
+      <c r="O290" s="3" t="inlineStr"/>
+      <c r="P290" s="3" t="inlineStr"/>
+      <c r="Q290" s="3" t="inlineStr">
+        <is>
+          <t>Istanbul</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="3" t="inlineStr">
+        <is>
+          <t>Winncom Technologies（Dublin）</t>
+        </is>
+      </c>
+      <c r="B291" s="3" t="inlineStr">
+        <is>
+          <t>爱尔兰</t>
+        </is>
+      </c>
+      <c r="C291" s="3" t="inlineStr"/>
+      <c r="D291" s="3" t="inlineStr">
+        <is>
+          <t>winncom.com</t>
+        </is>
+      </c>
+      <c r="E291" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F291" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G291" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H291" s="3" t="inlineStr">
+        <is>
+          <t>Winncom 是跨国无线分销集团（美/欧/独联体）</t>
+        </is>
+      </c>
+      <c r="I291" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J291" s="3" t="inlineStr">
+        <is>
+          <t>+44 203 002 8410 / sales.emea@winncom.com</t>
+        </is>
+      </c>
+      <c r="K291" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L291" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M291" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N291" s="3" t="inlineStr"/>
+      <c r="O291" s="3" t="inlineStr"/>
+      <c r="P291" s="3" t="inlineStr"/>
+      <c r="Q291" s="3" t="inlineStr">
+        <is>
+          <t>Dublin；EMEA 总部</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="3" t="inlineStr">
+        <is>
+          <t>Irish Wireless</t>
+        </is>
+      </c>
+      <c r="B292" s="3" t="inlineStr">
+        <is>
+          <t>爱尔兰</t>
+        </is>
+      </c>
+      <c r="C292" s="3" t="inlineStr"/>
+      <c r="D292" s="3" t="inlineStr">
+        <is>
+          <t>irishwireless.net</t>
+        </is>
+      </c>
+      <c r="E292" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F292" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G292" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H292" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I292" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J292" s="3" t="inlineStr">
+        <is>
+          <t>+353 61 514444 / sales@irishwireless.net</t>
+        </is>
+      </c>
+      <c r="K292" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L292" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M292" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N292" s="3" t="inlineStr"/>
+      <c r="O292" s="3" t="inlineStr"/>
+      <c r="P292" s="3" t="inlineStr"/>
+      <c r="Q292" s="3" t="inlineStr">
+        <is>
+          <t>Co. Clare</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="3" t="inlineStr">
+        <is>
+          <t>gCnTech Limited</t>
+        </is>
+      </c>
+      <c r="B293" s="3" t="inlineStr">
+        <is>
+          <t>爱尔兰</t>
+        </is>
+      </c>
+      <c r="C293" s="3" t="inlineStr"/>
+      <c r="D293" s="3" t="inlineStr">
+        <is>
+          <t>gcntech.ie</t>
+        </is>
+      </c>
+      <c r="E293" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F293" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G293" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H293" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I293" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J293" s="3" t="inlineStr">
+        <is>
+          <t>+353 1 282 0458 / greg@gcntech.ie</t>
+        </is>
+      </c>
+      <c r="K293" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L293" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M293" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N293" s="3" t="inlineStr"/>
+      <c r="O293" s="3" t="inlineStr"/>
+      <c r="P293" s="3" t="inlineStr"/>
+      <c r="Q293" s="3" t="inlineStr">
+        <is>
+          <t>Dublin</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="3" t="inlineStr">
+        <is>
+          <t>Dustin Norway</t>
+        </is>
+      </c>
+      <c r="B294" s="3" t="inlineStr">
+        <is>
+          <t>挪威</t>
+        </is>
+      </c>
+      <c r="C294" s="3" t="inlineStr"/>
+      <c r="D294" s="3" t="inlineStr">
+        <is>
+          <t>dustin.no</t>
+        </is>
+      </c>
+      <c r="E294" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F294" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G294" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H294" s="3" t="inlineStr">
+        <is>
+          <t>Dustin 集团 = 北欧大型 IT 分销（瑞典/挪威/丹麦/芬兰/荷兰/比利时）</t>
+        </is>
+      </c>
+      <c r="I294" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT</t>
+        </is>
+      </c>
+      <c r="J294" s="3" t="inlineStr">
+        <is>
+          <t>+47 21 04 40 40 / ordre@dustin.no</t>
+        </is>
+      </c>
+      <c r="K294" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L294" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M294" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N294" s="3" t="inlineStr"/>
+      <c r="O294" s="3" t="inlineStr"/>
+      <c r="P294" s="3" t="inlineStr"/>
+      <c r="Q294" s="3" t="inlineStr">
+        <is>
+          <t>Moss；泛欧大分销</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Finish the European sweep: Baltics, Ukraine, Balkans, Caucasus, Israel, Malta, Iceland
72 more MikroTik official distributors closes out Europe - 38 countries
scanned in total. Ukraine alone yielded 18. Two more regional groups
confirmed: ELKO now spans Estonia/Lithuania/Ukraine/Romania, and ACC
Distribution spans Estonia/Lithuania, alongside ASBIS (Slovakia, 30+
countries EMEA). New single-brand finds: MTBG (mikrotikbg.shop), WinTik,
RIM2000 and Setevuha. Running total: 365 accounts.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q294"/>
+  <dimension ref="A1:Q363"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -31793,6 +31793,4901 @@
       <c r="Q294" s="3" t="inlineStr">
         <is>
           <t>Moss；泛欧大分销</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="3" t="inlineStr">
+        <is>
+          <t>SPX, SIA（router.lv）</t>
+        </is>
+      </c>
+      <c r="B295" s="3" t="inlineStr">
+        <is>
+          <t>拉脱维亚</t>
+        </is>
+      </c>
+      <c r="C295" s="3" t="inlineStr"/>
+      <c r="D295" s="3" t="inlineStr">
+        <is>
+          <t>router.lv</t>
+        </is>
+      </c>
+      <c r="E295" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F295" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G295" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H295" s="3" t="inlineStr">
+        <is>
+          <t>域名 router.lv → 网络设备专业户</t>
+        </is>
+      </c>
+      <c r="I295" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J295" s="3" t="inlineStr">
+        <is>
+          <t>+371 6772 4000 / sales@router.lv</t>
+        </is>
+      </c>
+      <c r="K295" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L295" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M295" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N295" s="3" t="inlineStr"/>
+      <c r="O295" s="3" t="inlineStr"/>
+      <c r="P295" s="3" t="inlineStr"/>
+      <c r="Q295" s="3" t="inlineStr">
+        <is>
+          <t>Riga</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="3" t="inlineStr">
+        <is>
+          <t>NetPro SIA（nasstore.eu）</t>
+        </is>
+      </c>
+      <c r="B296" s="3" t="inlineStr">
+        <is>
+          <t>拉脱维亚</t>
+        </is>
+      </c>
+      <c r="C296" s="3" t="inlineStr"/>
+      <c r="D296" s="3" t="inlineStr">
+        <is>
+          <t>nasstore.eu</t>
+        </is>
+      </c>
+      <c r="E296" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F296" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G296" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H296" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I296" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J296" s="3" t="inlineStr">
+        <is>
+          <t>+371 2786 6444 / info@netpro.lv</t>
+        </is>
+      </c>
+      <c r="K296" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L296" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M296" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N296" s="3" t="inlineStr"/>
+      <c r="O296" s="3" t="inlineStr"/>
+      <c r="P296" s="3" t="inlineStr"/>
+      <c r="Q296" s="3" t="inlineStr">
+        <is>
+          <t>Riga</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="3" t="inlineStr">
+        <is>
+          <t>GOODSTORE</t>
+        </is>
+      </c>
+      <c r="B297" s="3" t="inlineStr">
+        <is>
+          <t>拉脱维亚</t>
+        </is>
+      </c>
+      <c r="C297" s="3" t="inlineStr"/>
+      <c r="D297" s="3" t="inlineStr">
+        <is>
+          <t>goodstore.lv</t>
+        </is>
+      </c>
+      <c r="E297" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F297" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G297" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H297" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I297" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J297" s="3" t="inlineStr">
+        <is>
+          <t>+371 2701 7034 / info@goodstore.lv</t>
+        </is>
+      </c>
+      <c r="K297" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L297" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M297" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N297" s="3" t="inlineStr"/>
+      <c r="O297" s="3" t="inlineStr"/>
+      <c r="P297" s="3" t="inlineStr"/>
+      <c r="Q297" s="3" t="inlineStr">
+        <is>
+          <t>Daugavpils</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="3" t="inlineStr">
+        <is>
+          <t>WiFi-Stock.com（JSC Katalita）</t>
+        </is>
+      </c>
+      <c r="B298" s="3" t="inlineStr">
+        <is>
+          <t>立陶宛</t>
+        </is>
+      </c>
+      <c r="C298" s="3" t="inlineStr"/>
+      <c r="D298" s="3" t="inlineStr">
+        <is>
+          <t>wifi-stock.com</t>
+        </is>
+      </c>
+      <c r="E298" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F298" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G298" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H298" s="3" t="inlineStr">
+        <is>
+          <t>与英国 Wifi Stock、比利时 SmartEye 同名 → 疑似同一网络体系</t>
+        </is>
+      </c>
+      <c r="I298" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J298" s="3" t="inlineStr">
+        <is>
+          <t>+370 615 85560 / sales@wifi-stock.com</t>
+        </is>
+      </c>
+      <c r="K298" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L298" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M298" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N298" s="3" t="inlineStr"/>
+      <c r="O298" s="3" t="inlineStr"/>
+      <c r="P298" s="3" t="inlineStr"/>
+      <c r="Q298" s="3" t="inlineStr">
+        <is>
+          <t>Kaunas</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="3" t="inlineStr">
+        <is>
+          <t>ACC Distribution UAB</t>
+        </is>
+      </c>
+      <c r="B299" s="3" t="inlineStr">
+        <is>
+          <t>立陶宛</t>
+        </is>
+      </c>
+      <c r="C299" s="3" t="inlineStr"/>
+      <c r="D299" s="3" t="inlineStr">
+        <is>
+          <t>accdistribution.eu</t>
+        </is>
+      </c>
+      <c r="E299" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F299" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G299" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H299" s="3" t="inlineStr">
+        <is>
+          <t>ACC Distribution 波罗的海集团（爱沙尼亚+立陶宛）</t>
+        </is>
+      </c>
+      <c r="I299" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J299" s="3" t="inlineStr">
+        <is>
+          <t>+370 37 33 39 33 / info@accdistribution.lt</t>
+        </is>
+      </c>
+      <c r="K299" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L299" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M299" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N299" s="3" t="inlineStr"/>
+      <c r="O299" s="3" t="inlineStr"/>
+      <c r="P299" s="3" t="inlineStr"/>
+      <c r="Q299" s="3" t="inlineStr">
+        <is>
+          <t>Kaunas</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="3" t="inlineStr">
+        <is>
+          <t>UAB ELKO Lietuva</t>
+        </is>
+      </c>
+      <c r="B300" s="3" t="inlineStr">
+        <is>
+          <t>立陶宛</t>
+        </is>
+      </c>
+      <c r="C300" s="3" t="inlineStr"/>
+      <c r="D300" s="3" t="inlineStr">
+        <is>
+          <t>elko.lt</t>
+        </is>
+      </c>
+      <c r="E300" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F300" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G300" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H300" s="3" t="inlineStr">
+        <is>
+          <t>ELKO 集团立陶宛站（集团总部在拉脱维亚，覆盖 5+ 国）</t>
+        </is>
+      </c>
+      <c r="I300" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT</t>
+        </is>
+      </c>
+      <c r="J300" s="3" t="inlineStr">
+        <is>
+          <t>+370 37 302 450 / info@elko.lt</t>
+        </is>
+      </c>
+      <c r="K300" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L300" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M300" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N300" s="3" t="inlineStr"/>
+      <c r="O300" s="3" t="inlineStr"/>
+      <c r="P300" s="3" t="inlineStr"/>
+      <c r="Q300" s="3" t="inlineStr">
+        <is>
+          <t>Kaunas</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="3" t="inlineStr">
+        <is>
+          <t>Frineta UAB</t>
+        </is>
+      </c>
+      <c r="B301" s="3" t="inlineStr">
+        <is>
+          <t>立陶宛</t>
+        </is>
+      </c>
+      <c r="C301" s="3" t="inlineStr"/>
+      <c r="D301" s="3" t="inlineStr">
+        <is>
+          <t>frineta.lt</t>
+        </is>
+      </c>
+      <c r="E301" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F301" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G301" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H301" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I301" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J301" s="3" t="inlineStr">
+        <is>
+          <t>+370 3730 0807</t>
+        </is>
+      </c>
+      <c r="K301" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L301" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M301" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N301" s="3" t="inlineStr"/>
+      <c r="O301" s="3" t="inlineStr"/>
+      <c r="P301" s="3" t="inlineStr"/>
+      <c r="Q301" s="3" t="inlineStr">
+        <is>
+          <t>Kaunas</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="3" t="inlineStr">
+        <is>
+          <t>ELKO Eesti OÜ</t>
+        </is>
+      </c>
+      <c r="B302" s="3" t="inlineStr">
+        <is>
+          <t>爱沙尼亚</t>
+        </is>
+      </c>
+      <c r="C302" s="3" t="inlineStr"/>
+      <c r="D302" s="3" t="inlineStr">
+        <is>
+          <t>elko.ee</t>
+        </is>
+      </c>
+      <c r="E302" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F302" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G302" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H302" s="3" t="inlineStr">
+        <is>
+          <t>ELKO 集团爱沙尼亚站</t>
+        </is>
+      </c>
+      <c r="I302" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT</t>
+        </is>
+      </c>
+      <c r="J302" s="3" t="inlineStr">
+        <is>
+          <t>+372 658 1378 / info@elko.ee</t>
+        </is>
+      </c>
+      <c r="K302" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L302" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M302" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N302" s="3" t="inlineStr"/>
+      <c r="O302" s="3" t="inlineStr"/>
+      <c r="P302" s="3" t="inlineStr"/>
+      <c r="Q302" s="3" t="inlineStr">
+        <is>
+          <t>Tallinn</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="3" t="inlineStr">
+        <is>
+          <t>Sonictest OÜ</t>
+        </is>
+      </c>
+      <c r="B303" s="3" t="inlineStr">
+        <is>
+          <t>爱沙尼亚</t>
+        </is>
+      </c>
+      <c r="C303" s="3" t="inlineStr"/>
+      <c r="D303" s="3" t="inlineStr">
+        <is>
+          <t>sonictest.ee</t>
+        </is>
+      </c>
+      <c r="E303" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F303" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G303" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H303" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I303" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J303" s="3" t="inlineStr">
+        <is>
+          <t>+372 505 5961 / imre@sonictest.ee</t>
+        </is>
+      </c>
+      <c r="K303" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L303" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M303" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N303" s="3" t="inlineStr"/>
+      <c r="O303" s="3" t="inlineStr"/>
+      <c r="P303" s="3" t="inlineStr"/>
+      <c r="Q303" s="3" t="inlineStr">
+        <is>
+          <t>Tartu</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="3" t="inlineStr">
+        <is>
+          <t>Kernel AS</t>
+        </is>
+      </c>
+      <c r="B304" s="3" t="inlineStr">
+        <is>
+          <t>爱沙尼亚</t>
+        </is>
+      </c>
+      <c r="C304" s="3" t="inlineStr"/>
+      <c r="D304" s="3" t="inlineStr">
+        <is>
+          <t>kernel.ee</t>
+        </is>
+      </c>
+      <c r="E304" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F304" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G304" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H304" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I304" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J304" s="3" t="inlineStr">
+        <is>
+          <t>+372 7 420 234 / info@kernel.ee</t>
+        </is>
+      </c>
+      <c r="K304" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L304" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M304" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N304" s="3" t="inlineStr"/>
+      <c r="O304" s="3" t="inlineStr"/>
+      <c r="P304" s="3" t="inlineStr"/>
+      <c r="Q304" s="3" t="inlineStr">
+        <is>
+          <t>Tartu</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="3" t="inlineStr">
+        <is>
+          <t>DEPS</t>
+        </is>
+      </c>
+      <c r="B305" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C305" s="3" t="inlineStr"/>
+      <c r="D305" s="3" t="inlineStr">
+        <is>
+          <t>deps.ua</t>
+        </is>
+      </c>
+      <c r="E305" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F305" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G305" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H305" s="3" t="inlineStr">
+        <is>
+          <t>四城分部（基辅/利沃夫/哈尔科夫/敖德萨）</t>
+        </is>
+      </c>
+      <c r="I305" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J305" s="3" t="inlineStr">
+        <is>
+          <t>+380 44 323 88 88 / Oleg.Smaliychuk@deps.ua</t>
+        </is>
+      </c>
+      <c r="K305" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L305" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M305" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N305" s="3" t="inlineStr"/>
+      <c r="O305" s="3" t="inlineStr"/>
+      <c r="P305" s="3" t="inlineStr"/>
+      <c r="Q305" s="3" t="inlineStr">
+        <is>
+          <t>Kyiv 等 4 城</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="3" t="inlineStr">
+        <is>
+          <t>ERC</t>
+        </is>
+      </c>
+      <c r="B306" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C306" s="3" t="inlineStr"/>
+      <c r="D306" s="3" t="inlineStr">
+        <is>
+          <t>erc.ua</t>
+        </is>
+      </c>
+      <c r="E306" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F306" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G306" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H306" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I306" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J306" s="3" t="inlineStr">
+        <is>
+          <t>+380 44 230 3474 / Network_SOHO@erc.ua</t>
+        </is>
+      </c>
+      <c r="K306" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L306" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M306" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N306" s="3" t="inlineStr"/>
+      <c r="O306" s="3" t="inlineStr"/>
+      <c r="P306" s="3" t="inlineStr"/>
+      <c r="Q306" s="3" t="inlineStr">
+        <is>
+          <t>Kyiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="3" t="inlineStr">
+        <is>
+          <t>Viatec</t>
+        </is>
+      </c>
+      <c r="B307" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C307" s="3" t="inlineStr"/>
+      <c r="D307" s="3" t="inlineStr">
+        <is>
+          <t>viatec.ua</t>
+        </is>
+      </c>
+      <c r="E307" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F307" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G307" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H307" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I307" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J307" s="3" t="inlineStr">
+        <is>
+          <t>+380 44 364 77 20 / viatec@viatec.ua</t>
+        </is>
+      </c>
+      <c r="K307" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L307" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M307" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N307" s="3" t="inlineStr"/>
+      <c r="O307" s="3" t="inlineStr"/>
+      <c r="P307" s="3" t="inlineStr"/>
+      <c r="Q307" s="3" t="inlineStr">
+        <is>
+          <t>Kyiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="3" t="inlineStr">
+        <is>
+          <t>MTI</t>
+        </is>
+      </c>
+      <c r="B308" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C308" s="3" t="inlineStr"/>
+      <c r="D308" s="3" t="inlineStr">
+        <is>
+          <t>products.mti.ua</t>
+        </is>
+      </c>
+      <c r="E308" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F308" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G308" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H308" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰大型 IT 分销</t>
+        </is>
+      </c>
+      <c r="I308" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT</t>
+        </is>
+      </c>
+      <c r="J308" s="3" t="inlineStr">
+        <is>
+          <t>+380 44 207 40 61 / itdistri@mti.ua</t>
+        </is>
+      </c>
+      <c r="K308" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L308" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M308" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N308" s="3" t="inlineStr"/>
+      <c r="O308" s="3" t="inlineStr"/>
+      <c r="P308" s="3" t="inlineStr"/>
+      <c r="Q308" s="3" t="inlineStr">
+        <is>
+          <t>Kyiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="3" t="inlineStr">
+        <is>
+          <t>ELKO Ukraine</t>
+        </is>
+      </c>
+      <c r="B309" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C309" s="3" t="inlineStr"/>
+      <c r="D309" s="3" t="inlineStr">
+        <is>
+          <t>elko.ua</t>
+        </is>
+      </c>
+      <c r="E309" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F309" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G309" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H309" s="3" t="inlineStr">
+        <is>
+          <t>ELKO 集团乌克兰站</t>
+        </is>
+      </c>
+      <c r="I309" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J309" s="3" t="inlineStr">
+        <is>
+          <t>+380 44 461 9670 / elko@elko.ua</t>
+        </is>
+      </c>
+      <c r="K309" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L309" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M309" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N309" s="3" t="inlineStr"/>
+      <c r="O309" s="3" t="inlineStr"/>
+      <c r="P309" s="3" t="inlineStr"/>
+      <c r="Q309" s="3" t="inlineStr">
+        <is>
+          <t>Kyiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="3" t="inlineStr">
+        <is>
+          <t>Romsat</t>
+        </is>
+      </c>
+      <c r="B310" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C310" s="3" t="inlineStr"/>
+      <c r="D310" s="3" t="inlineStr">
+        <is>
+          <t>romsat.ua</t>
+        </is>
+      </c>
+      <c r="E310" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F310" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G310" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H310" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I310" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J310" s="3" t="inlineStr">
+        <is>
+          <t>+380 44 225 5454 / info@romsat.ua</t>
+        </is>
+      </c>
+      <c r="K310" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L310" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M310" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N310" s="3" t="inlineStr"/>
+      <c r="O310" s="3" t="inlineStr"/>
+      <c r="P310" s="3" t="inlineStr"/>
+      <c r="Q310" s="3" t="inlineStr">
+        <is>
+          <t>Kyiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="3" t="inlineStr">
+        <is>
+          <t>RIM2000</t>
+        </is>
+      </c>
+      <c r="B311" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C311" s="3" t="inlineStr"/>
+      <c r="D311" s="3" t="inlineStr">
+        <is>
+          <t>rim2000.ua</t>
+        </is>
+      </c>
+      <c r="E311" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F311" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G311" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H311" s="3" t="inlineStr">
+        <is>
+          <t>专属邮箱 mikrotik@rim2000.com；四城分部</t>
+        </is>
+      </c>
+      <c r="I311" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J311" s="3" t="inlineStr">
+        <is>
+          <t>+380 562 360 300 / mikrotik@rim2000.com</t>
+        </is>
+      </c>
+      <c r="K311" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L311" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M311" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N311" s="3" t="inlineStr"/>
+      <c r="O311" s="3" t="inlineStr"/>
+      <c r="P311" s="3" t="inlineStr"/>
+      <c r="Q311" s="3" t="inlineStr">
+        <is>
+          <t>Dnipro 等 4 城</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="3" t="inlineStr">
+        <is>
+          <t>Setevuha</t>
+        </is>
+      </c>
+      <c r="B312" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C312" s="3" t="inlineStr"/>
+      <c r="D312" s="3" t="inlineStr">
+        <is>
+          <t>setevuha.com.ua</t>
+        </is>
+      </c>
+      <c r="E312" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F312" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G312" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H312" s="3" t="inlineStr">
+        <is>
+          <t>专属邮箱 mikrotik@setevuha.ua</t>
+        </is>
+      </c>
+      <c r="I312" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J312" s="3" t="inlineStr">
+        <is>
+          <t>+380 44 384 02 29 / mikrotik@setevuha.ua</t>
+        </is>
+      </c>
+      <c r="K312" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L312" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M312" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N312" s="3" t="inlineStr"/>
+      <c r="O312" s="3" t="inlineStr"/>
+      <c r="P312" s="3" t="inlineStr"/>
+      <c r="Q312" s="3" t="inlineStr">
+        <is>
+          <t>Kyiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="3" t="inlineStr">
+        <is>
+          <t>WinTik</t>
+        </is>
+      </c>
+      <c r="B313" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C313" s="3" t="inlineStr"/>
+      <c r="D313" s="3" t="inlineStr">
+        <is>
+          <t>wintik.com.ua</t>
+        </is>
+      </c>
+      <c r="E313" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F313" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G313" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H313" s="3" t="inlineStr">
+        <is>
+          <t>域名含 Tik → 单品牌店</t>
+        </is>
+      </c>
+      <c r="I313" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J313" s="3" t="inlineStr">
+        <is>
+          <t>+380 68 810 46 29 / sale@wintik.com.ua</t>
+        </is>
+      </c>
+      <c r="K313" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L313" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M313" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N313" s="3" t="inlineStr"/>
+      <c r="O313" s="3" t="inlineStr"/>
+      <c r="P313" s="3" t="inlineStr"/>
+      <c r="Q313" s="3" t="inlineStr">
+        <is>
+          <t>Kharkiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="3" t="inlineStr">
+        <is>
+          <t>Gazik Store</t>
+        </is>
+      </c>
+      <c r="B314" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C314" s="3" t="inlineStr"/>
+      <c r="D314" s="3" t="inlineStr">
+        <is>
+          <t>gazik.ua</t>
+        </is>
+      </c>
+      <c r="E314" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F314" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G314" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H314" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I314" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J314" s="3" t="inlineStr">
+        <is>
+          <t>+380 67 323 17 30 / orest@gazik.in</t>
+        </is>
+      </c>
+      <c r="K314" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L314" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M314" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N314" s="3" t="inlineStr"/>
+      <c r="O314" s="3" t="inlineStr"/>
+      <c r="P314" s="3" t="inlineStr"/>
+      <c r="Q314" s="3" t="inlineStr">
+        <is>
+          <t>Lviv</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="3" t="inlineStr">
+        <is>
+          <t>Lanbox</t>
+        </is>
+      </c>
+      <c r="B315" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C315" s="3" t="inlineStr"/>
+      <c r="D315" s="3" t="inlineStr">
+        <is>
+          <t>lanbox.com.ua</t>
+        </is>
+      </c>
+      <c r="E315" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F315" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G315" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H315" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I315" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J315" s="3" t="inlineStr">
+        <is>
+          <t>+380 44 384 02 29 / sale@lanbox.com.ua</t>
+        </is>
+      </c>
+      <c r="K315" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L315" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M315" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N315" s="3" t="inlineStr"/>
+      <c r="O315" s="3" t="inlineStr"/>
+      <c r="P315" s="3" t="inlineStr"/>
+      <c r="Q315" s="3" t="inlineStr">
+        <is>
+          <t>Lviv</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="3" t="inlineStr">
+        <is>
+          <t>Technotrade LLC</t>
+        </is>
+      </c>
+      <c r="B316" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C316" s="3" t="inlineStr"/>
+      <c r="D316" s="3" t="inlineStr">
+        <is>
+          <t>technotrade.com.ua</t>
+        </is>
+      </c>
+      <c r="E316" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F316" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G316" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H316" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I316" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J316" s="3" t="inlineStr">
+        <is>
+          <t>+380 57 764 02 54 / molya@technotrade.com.ua</t>
+        </is>
+      </c>
+      <c r="K316" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L316" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M316" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N316" s="3" t="inlineStr"/>
+      <c r="O316" s="3" t="inlineStr"/>
+      <c r="P316" s="3" t="inlineStr"/>
+      <c r="Q316" s="3" t="inlineStr">
+        <is>
+          <t>Kharkiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="3" t="inlineStr">
+        <is>
+          <t>Omnilink</t>
+        </is>
+      </c>
+      <c r="B317" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C317" s="3" t="inlineStr"/>
+      <c r="D317" s="3" t="inlineStr">
+        <is>
+          <t>omnilink.ua</t>
+        </is>
+      </c>
+      <c r="E317" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F317" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G317" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H317" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I317" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J317" s="3" t="inlineStr">
+        <is>
+          <t>+380 44 359 0770 / sale@omnilink.com.ua</t>
+        </is>
+      </c>
+      <c r="K317" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L317" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M317" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N317" s="3" t="inlineStr"/>
+      <c r="O317" s="3" t="inlineStr"/>
+      <c r="P317" s="3" t="inlineStr"/>
+      <c r="Q317" s="3" t="inlineStr">
+        <is>
+          <t>Kyiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="3" t="inlineStr">
+        <is>
+          <t>Lanmarket</t>
+        </is>
+      </c>
+      <c r="B318" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C318" s="3" t="inlineStr"/>
+      <c r="D318" s="3" t="inlineStr">
+        <is>
+          <t>lanmarket.ua</t>
+        </is>
+      </c>
+      <c r="E318" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F318" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G318" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H318" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I318" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J318" s="3" t="inlineStr">
+        <is>
+          <t>+380 50 666 78 58 / sale@lanmarket.net</t>
+        </is>
+      </c>
+      <c r="K318" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L318" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M318" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N318" s="3" t="inlineStr"/>
+      <c r="O318" s="3" t="inlineStr"/>
+      <c r="P318" s="3" t="inlineStr"/>
+      <c r="Q318" s="3" t="inlineStr">
+        <is>
+          <t>Chernivtsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="3" t="inlineStr">
+        <is>
+          <t>Lantorg</t>
+        </is>
+      </c>
+      <c r="B319" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C319" s="3" t="inlineStr"/>
+      <c r="D319" s="3" t="inlineStr">
+        <is>
+          <t>lantorg.com</t>
+        </is>
+      </c>
+      <c r="E319" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F319" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G319" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H319" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I319" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J319" s="3" t="inlineStr">
+        <is>
+          <t>+380 57 780 40 63 / 238100@lantorg.com</t>
+        </is>
+      </c>
+      <c r="K319" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L319" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M319" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N319" s="3" t="inlineStr"/>
+      <c r="O319" s="3" t="inlineStr"/>
+      <c r="P319" s="3" t="inlineStr"/>
+      <c r="Q319" s="3" t="inlineStr">
+        <is>
+          <t>Kharkiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="3" t="inlineStr">
+        <is>
+          <t>SHOP-GSM.NET</t>
+        </is>
+      </c>
+      <c r="B320" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C320" s="3" t="inlineStr"/>
+      <c r="D320" s="3" t="inlineStr">
+        <is>
+          <t>shop-gsm.ua</t>
+        </is>
+      </c>
+      <c r="E320" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F320" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G320" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H320" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I320" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J320" s="3" t="inlineStr">
+        <is>
+          <t>+380 44 361 13 34 / info@shop-gsm.net</t>
+        </is>
+      </c>
+      <c r="K320" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L320" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M320" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N320" s="3" t="inlineStr"/>
+      <c r="O320" s="3" t="inlineStr"/>
+      <c r="P320" s="3" t="inlineStr"/>
+      <c r="Q320" s="3" t="inlineStr">
+        <is>
+          <t>Kyiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="3" t="inlineStr">
+        <is>
+          <t>Network Discount</t>
+        </is>
+      </c>
+      <c r="B321" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C321" s="3" t="inlineStr"/>
+      <c r="D321" s="3" t="inlineStr">
+        <is>
+          <t>networkdiscount.com.ua</t>
+        </is>
+      </c>
+      <c r="E321" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F321" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G321" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H321" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I321" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J321" s="3" t="inlineStr">
+        <is>
+          <t>+380 44 392 28 30 / sales@networkdiscount.com.ua</t>
+        </is>
+      </c>
+      <c r="K321" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L321" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M321" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N321" s="3" t="inlineStr"/>
+      <c r="O321" s="3" t="inlineStr"/>
+      <c r="P321" s="3" t="inlineStr"/>
+      <c r="Q321" s="3" t="inlineStr">
+        <is>
+          <t>Kyiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="3" t="inlineStr">
+        <is>
+          <t>Lux-Mobil</t>
+        </is>
+      </c>
+      <c r="B322" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C322" s="3" t="inlineStr"/>
+      <c r="D322" s="3" t="inlineStr">
+        <is>
+          <t>lux-mobil.com.ua</t>
+        </is>
+      </c>
+      <c r="E322" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F322" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G322" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H322" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I322" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J322" s="3" t="inlineStr">
+        <is>
+          <t>+380 98 152 09 27 / info@lux-mobil.com.ua</t>
+        </is>
+      </c>
+      <c r="K322" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L322" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M322" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N322" s="3" t="inlineStr"/>
+      <c r="O322" s="3" t="inlineStr"/>
+      <c r="P322" s="3" t="inlineStr"/>
+      <c r="Q322" s="3" t="inlineStr">
+        <is>
+          <t>Kyiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="3" t="inlineStr">
+        <is>
+          <t>ASBIS SK</t>
+        </is>
+      </c>
+      <c r="B323" s="3" t="inlineStr">
+        <is>
+          <t>斯洛伐克</t>
+        </is>
+      </c>
+      <c r="C323" s="3" t="inlineStr"/>
+      <c r="D323" s="3" t="inlineStr">
+        <is>
+          <t>online.asbis.sk</t>
+        </is>
+      </c>
+      <c r="E323" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F323" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G323" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H323" s="3" t="inlineStr">
+        <is>
+          <t>ASBIS 集团 = EMEA 最大 IT 分销之一（覆盖 30+ 国）</t>
+        </is>
+      </c>
+      <c r="I323" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J323" s="3" t="inlineStr">
+        <is>
+          <t>+421 2 321 65 111 / sales@asbis.sk</t>
+        </is>
+      </c>
+      <c r="K323" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L323" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M323" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N323" s="3" t="inlineStr"/>
+      <c r="O323" s="3" t="inlineStr"/>
+      <c r="P323" s="3" t="inlineStr"/>
+      <c r="Q323" s="3" t="inlineStr">
+        <is>
+          <t>Bratislava；泛欧大分销</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="3" t="inlineStr">
+        <is>
+          <t>WESTech, spol. s r.o.</t>
+        </is>
+      </c>
+      <c r="B324" s="3" t="inlineStr">
+        <is>
+          <t>斯洛伐克</t>
+        </is>
+      </c>
+      <c r="C324" s="3" t="inlineStr"/>
+      <c r="D324" s="3" t="inlineStr">
+        <is>
+          <t>online.westech.sk</t>
+        </is>
+      </c>
+      <c r="E324" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F324" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G324" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H324" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I324" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J324" s="3" t="inlineStr">
+        <is>
+          <t>+421 2 4445 4090 / obchodba@westech.sk</t>
+        </is>
+      </c>
+      <c r="K324" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L324" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M324" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N324" s="3" t="inlineStr"/>
+      <c r="O324" s="3" t="inlineStr"/>
+      <c r="P324" s="3" t="inlineStr"/>
+      <c r="Q324" s="3" t="inlineStr">
+        <is>
+          <t>Bratislava</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="3" t="inlineStr">
+        <is>
+          <t>TIMES NETWORKS（lancentrum）</t>
+        </is>
+      </c>
+      <c r="B325" s="3" t="inlineStr">
+        <is>
+          <t>斯洛伐克</t>
+        </is>
+      </c>
+      <c r="C325" s="3" t="inlineStr"/>
+      <c r="D325" s="3" t="inlineStr">
+        <is>
+          <t>lancentrum.eu</t>
+        </is>
+      </c>
+      <c r="E325" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F325" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G325" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H325" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I325" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J325" s="3" t="inlineStr">
+        <is>
+          <t>+421 46 542 7050 / info@lancentrum.sk</t>
+        </is>
+      </c>
+      <c r="K325" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L325" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M325" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N325" s="3" t="inlineStr"/>
+      <c r="O325" s="3" t="inlineStr"/>
+      <c r="P325" s="3" t="inlineStr"/>
+      <c r="Q325" s="3" t="inlineStr">
+        <is>
+          <t>Prievidza</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="3" t="inlineStr">
+        <is>
+          <t>PC H.AND d.o.o.</t>
+        </is>
+      </c>
+      <c r="B326" s="3" t="inlineStr">
+        <is>
+          <t>斯洛文尼亚</t>
+        </is>
+      </c>
+      <c r="C326" s="3" t="inlineStr"/>
+      <c r="D326" s="3" t="inlineStr">
+        <is>
+          <t>pchand.si</t>
+        </is>
+      </c>
+      <c r="E326" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F326" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G326" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H326" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I326" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J326" s="3" t="inlineStr">
+        <is>
+          <t>+386 1 530 08 00 / info@pchand.si</t>
+        </is>
+      </c>
+      <c r="K326" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L326" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M326" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N326" s="3" t="inlineStr"/>
+      <c r="O326" s="3" t="inlineStr"/>
+      <c r="P326" s="3" t="inlineStr"/>
+      <c r="Q326" s="3" t="inlineStr">
+        <is>
+          <t>Trzin</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="3" t="inlineStr">
+        <is>
+          <t>PEC SISTEMI d.o.o.（tehnox.si）</t>
+        </is>
+      </c>
+      <c r="B327" s="3" t="inlineStr">
+        <is>
+          <t>斯洛文尼亚</t>
+        </is>
+      </c>
+      <c r="C327" s="3" t="inlineStr"/>
+      <c r="D327" s="3" t="inlineStr">
+        <is>
+          <t>tehnox.si</t>
+        </is>
+      </c>
+      <c r="E327" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F327" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G327" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H327" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I327" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J327" s="3" t="inlineStr">
+        <is>
+          <t>+386 2 250 2235 / info@pec-sistemi.si</t>
+        </is>
+      </c>
+      <c r="K327" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L327" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M327" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N327" s="3" t="inlineStr"/>
+      <c r="O327" s="3" t="inlineStr"/>
+      <c r="P327" s="3" t="inlineStr"/>
+      <c r="Q327" s="3" t="inlineStr">
+        <is>
+          <t>Maribor</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="3" t="inlineStr">
+        <is>
+          <t>Elkotex d.o.o.</t>
+        </is>
+      </c>
+      <c r="B328" s="3" t="inlineStr">
+        <is>
+          <t>斯洛文尼亚</t>
+        </is>
+      </c>
+      <c r="C328" s="3" t="inlineStr"/>
+      <c r="D328" s="3" t="inlineStr">
+        <is>
+          <t>b2b.elkotex.si</t>
+        </is>
+      </c>
+      <c r="E328" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F328" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G328" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H328" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I328" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J328" s="3" t="inlineStr">
+        <is>
+          <t>+386 1 583 79 10</t>
+        </is>
+      </c>
+      <c r="K328" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L328" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M328" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N328" s="3" t="inlineStr"/>
+      <c r="O328" s="3" t="inlineStr"/>
+      <c r="P328" s="3" t="inlineStr"/>
+      <c r="Q328" s="3" t="inlineStr">
+        <is>
+          <t>Ljubljana</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="3" t="inlineStr">
+        <is>
+          <t>LOST d.o.o.</t>
+        </is>
+      </c>
+      <c r="B329" s="3" t="inlineStr">
+        <is>
+          <t>克罗地亚</t>
+        </is>
+      </c>
+      <c r="C329" s="3" t="inlineStr"/>
+      <c r="D329" s="3" t="inlineStr">
+        <is>
+          <t>lost.hr</t>
+        </is>
+      </c>
+      <c r="E329" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F329" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G329" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H329" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I329" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J329" s="3" t="inlineStr">
+        <is>
+          <t>+385 1 3027 163 / lost@lost.hr</t>
+        </is>
+      </c>
+      <c r="K329" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L329" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M329" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N329" s="3" t="inlineStr"/>
+      <c r="O329" s="3" t="inlineStr"/>
+      <c r="P329" s="3" t="inlineStr"/>
+      <c r="Q329" s="3" t="inlineStr">
+        <is>
+          <t>Zagreb</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="3" t="inlineStr">
+        <is>
+          <t>EZY Infotech d.o.o.</t>
+        </is>
+      </c>
+      <c r="B330" s="3" t="inlineStr">
+        <is>
+          <t>克罗地亚</t>
+        </is>
+      </c>
+      <c r="C330" s="3" t="inlineStr"/>
+      <c r="D330" s="3" t="inlineStr">
+        <is>
+          <t>ezy.hr</t>
+        </is>
+      </c>
+      <c r="E330" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F330" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G330" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H330" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I330" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J330" s="3" t="inlineStr">
+        <is>
+          <t>+385 40 363 888 / prodaja@ezy.hr</t>
+        </is>
+      </c>
+      <c r="K330" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L330" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M330" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N330" s="3" t="inlineStr"/>
+      <c r="O330" s="3" t="inlineStr"/>
+      <c r="P330" s="3" t="inlineStr"/>
+      <c r="Q330" s="3" t="inlineStr">
+        <is>
+          <t>Čakovec</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="3" t="inlineStr">
+        <is>
+          <t>Pondi d.o.o.</t>
+        </is>
+      </c>
+      <c r="B331" s="3" t="inlineStr">
+        <is>
+          <t>克罗地亚</t>
+        </is>
+      </c>
+      <c r="C331" s="3" t="inlineStr"/>
+      <c r="D331" s="3" t="inlineStr">
+        <is>
+          <t>pondi.hr</t>
+        </is>
+      </c>
+      <c r="E331" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F331" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G331" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H331" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I331" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J331" s="3" t="inlineStr">
+        <is>
+          <t>+385 21 494 000</t>
+        </is>
+      </c>
+      <c r="K331" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L331" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M331" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N331" s="3" t="inlineStr"/>
+      <c r="O331" s="3" t="inlineStr"/>
+      <c r="P331" s="3" t="inlineStr"/>
+      <c r="Q331" s="3" t="inlineStr">
+        <is>
+          <t>Split</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="3" t="inlineStr">
+        <is>
+          <t>3NET</t>
+        </is>
+      </c>
+      <c r="B332" s="3" t="inlineStr">
+        <is>
+          <t>塞尔维亚</t>
+        </is>
+      </c>
+      <c r="C332" s="3" t="inlineStr"/>
+      <c r="D332" s="3" t="inlineStr">
+        <is>
+          <t>3net.rs</t>
+        </is>
+      </c>
+      <c r="E332" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F332" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G332" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H332" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I332" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J332" s="3" t="inlineStr">
+        <is>
+          <t>+381 65 678 2201 / contact@3net.rs</t>
+        </is>
+      </c>
+      <c r="K332" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L332" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M332" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N332" s="3" t="inlineStr"/>
+      <c r="O332" s="3" t="inlineStr"/>
+      <c r="P332" s="3" t="inlineStr"/>
+      <c r="Q332" s="3" t="inlineStr">
+        <is>
+          <t>Vranje</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="3" t="inlineStr">
+        <is>
+          <t>Pixel Network LLC</t>
+        </is>
+      </c>
+      <c r="B333" s="3" t="inlineStr">
+        <is>
+          <t>塞尔维亚</t>
+        </is>
+      </c>
+      <c r="C333" s="3" t="inlineStr"/>
+      <c r="D333" s="3" t="inlineStr">
+        <is>
+          <t>pixelnetwork.rs</t>
+        </is>
+      </c>
+      <c r="E333" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F333" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G333" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H333" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I333" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J333" s="3" t="inlineStr">
+        <is>
+          <t>+381 21 271 85 04 / office@pixelnetwork.rs</t>
+        </is>
+      </c>
+      <c r="K333" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L333" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M333" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N333" s="3" t="inlineStr"/>
+      <c r="O333" s="3" t="inlineStr"/>
+      <c r="P333" s="3" t="inlineStr"/>
+      <c r="Q333" s="3" t="inlineStr">
+        <is>
+          <t>Novi Sad</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="3" t="inlineStr">
+        <is>
+          <t>Riva.Ltd</t>
+        </is>
+      </c>
+      <c r="B334" s="3" t="inlineStr">
+        <is>
+          <t>保加利亚</t>
+        </is>
+      </c>
+      <c r="C334" s="3" t="inlineStr"/>
+      <c r="D334" s="3" t="inlineStr">
+        <is>
+          <t>riva.bg</t>
+        </is>
+      </c>
+      <c r="E334" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F334" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G334" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H334" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I334" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT</t>
+        </is>
+      </c>
+      <c r="J334" s="3" t="inlineStr">
+        <is>
+          <t>+359 56 84 23 23 / riva@riva.bg</t>
+        </is>
+      </c>
+      <c r="K334" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L334" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M334" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N334" s="3" t="inlineStr"/>
+      <c r="O334" s="3" t="inlineStr"/>
+      <c r="P334" s="3" t="inlineStr"/>
+      <c r="Q334" s="3" t="inlineStr">
+        <is>
+          <t>Burgas</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="3" t="inlineStr">
+        <is>
+          <t>MTBG OOD（mikrotikbg.shop）</t>
+        </is>
+      </c>
+      <c r="B335" s="3" t="inlineStr">
+        <is>
+          <t>保加利亚</t>
+        </is>
+      </c>
+      <c r="C335" s="3" t="inlineStr"/>
+      <c r="D335" s="3" t="inlineStr">
+        <is>
+          <t>mikrotikbg.shop</t>
+        </is>
+      </c>
+      <c r="E335" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F335" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G335" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H335" s="3" t="inlineStr">
+        <is>
+          <t>域名就是 mikrotikbg.shop → 单品牌依赖最高档</t>
+        </is>
+      </c>
+      <c r="I335" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J335" s="3" t="inlineStr">
+        <is>
+          <t>+359 2 45 125 25 / info@mikrotikbg.shop</t>
+        </is>
+      </c>
+      <c r="K335" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L335" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M335" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N335" s="3" t="inlineStr"/>
+      <c r="O335" s="3" t="inlineStr"/>
+      <c r="P335" s="3" t="inlineStr"/>
+      <c r="Q335" s="3" t="inlineStr">
+        <is>
+          <t>Burgas</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="3" t="inlineStr">
+        <is>
+          <t>Rootelsat, Ltd.（vesuviustreamline.com）</t>
+        </is>
+      </c>
+      <c r="B336" s="3" t="inlineStr">
+        <is>
+          <t>保加利亚</t>
+        </is>
+      </c>
+      <c r="C336" s="3" t="inlineStr"/>
+      <c r="D336" s="3" t="inlineStr">
+        <is>
+          <t>vesuviustreamline.com</t>
+        </is>
+      </c>
+      <c r="E336" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F336" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G336" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H336" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I336" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J336" s="3" t="inlineStr">
+        <is>
+          <t>+359 54 862 991 / office@vesuviustreamline.com</t>
+        </is>
+      </c>
+      <c r="K336" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L336" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M336" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N336" s="3" t="inlineStr"/>
+      <c r="O336" s="3" t="inlineStr"/>
+      <c r="P336" s="3" t="inlineStr"/>
+      <c r="Q336" s="3" t="inlineStr">
+        <is>
+          <t>Shumen</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="3" t="inlineStr">
+        <is>
+          <t>Senetic Bulgaria LTD</t>
+        </is>
+      </c>
+      <c r="B337" s="3" t="inlineStr">
+        <is>
+          <t>保加利亚</t>
+        </is>
+      </c>
+      <c r="C337" s="3" t="inlineStr"/>
+      <c r="D337" s="3" t="inlineStr">
+        <is>
+          <t>senetic.bg</t>
+        </is>
+      </c>
+      <c r="E337" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F337" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G337" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H337" s="3" t="inlineStr">
+        <is>
+          <t>Senetic 集团保加利亚站</t>
+        </is>
+      </c>
+      <c r="I337" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J337" s="3" t="inlineStr">
+        <is>
+          <t>+359 2 448 6700 / info@senetic.bg</t>
+        </is>
+      </c>
+      <c r="K337" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L337" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M337" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N337" s="3" t="inlineStr"/>
+      <c r="O337" s="3" t="inlineStr"/>
+      <c r="P337" s="3" t="inlineStr"/>
+      <c r="Q337" s="3" t="inlineStr">
+        <is>
+          <t>Sofia</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="3" t="inlineStr">
+        <is>
+          <t>Computer Market</t>
+        </is>
+      </c>
+      <c r="B338" s="3" t="inlineStr">
+        <is>
+          <t>保加利亚</t>
+        </is>
+      </c>
+      <c r="C338" s="3" t="inlineStr"/>
+      <c r="D338" s="3" t="inlineStr">
+        <is>
+          <t>computermarket.bg</t>
+        </is>
+      </c>
+      <c r="E338" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F338" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G338" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H338" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I338" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J338" s="3" t="inlineStr">
+        <is>
+          <t>+359 700 200 02 / sales@computermarket.bg</t>
+        </is>
+      </c>
+      <c r="K338" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L338" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M338" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N338" s="3" t="inlineStr"/>
+      <c r="O338" s="3" t="inlineStr"/>
+      <c r="P338" s="3" t="inlineStr"/>
+      <c r="Q338" s="3" t="inlineStr">
+        <is>
+          <t>Burgas</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="3" t="inlineStr">
+        <is>
+          <t>PCLife LTD.</t>
+        </is>
+      </c>
+      <c r="B339" s="3" t="inlineStr">
+        <is>
+          <t>保加利亚</t>
+        </is>
+      </c>
+      <c r="C339" s="3" t="inlineStr"/>
+      <c r="D339" s="3" t="inlineStr">
+        <is>
+          <t>pclife.bg</t>
+        </is>
+      </c>
+      <c r="E339" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F339" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G339" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H339" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I339" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J339" s="3" t="inlineStr">
+        <is>
+          <t>+359 88 762 4895 / orders@pclife.bg</t>
+        </is>
+      </c>
+      <c r="K339" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L339" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M339" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N339" s="3" t="inlineStr"/>
+      <c r="O339" s="3" t="inlineStr"/>
+      <c r="P339" s="3" t="inlineStr"/>
+      <c r="Q339" s="3" t="inlineStr">
+        <is>
+          <t>Plovdiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="3" t="inlineStr">
+        <is>
+          <t>ASAP</t>
+        </is>
+      </c>
+      <c r="B340" s="3" t="inlineStr">
+        <is>
+          <t>保加利亚</t>
+        </is>
+      </c>
+      <c r="C340" s="3" t="inlineStr"/>
+      <c r="D340" s="3" t="inlineStr">
+        <is>
+          <t>asap.bg</t>
+        </is>
+      </c>
+      <c r="E340" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F340" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G340" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H340" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I340" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J340" s="3" t="inlineStr">
+        <is>
+          <t>+359 2 4475 100 / sales@asap.bg</t>
+        </is>
+      </c>
+      <c r="K340" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L340" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M340" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N340" s="3" t="inlineStr"/>
+      <c r="O340" s="3" t="inlineStr"/>
+      <c r="P340" s="3" t="inlineStr"/>
+      <c r="Q340" s="3" t="inlineStr">
+        <is>
+          <t>Sofia</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="3" t="inlineStr">
+        <is>
+          <t>Voicenter LTD</t>
+        </is>
+      </c>
+      <c r="B341" s="3" t="inlineStr">
+        <is>
+          <t>以色列</t>
+        </is>
+      </c>
+      <c r="C341" s="3" t="inlineStr"/>
+      <c r="D341" s="3" t="inlineStr">
+        <is>
+          <t>voicenter.co.il</t>
+        </is>
+      </c>
+      <c r="E341" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F341" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G341" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H341" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I341" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J341" s="3" t="inlineStr">
+        <is>
+          <t>+972 72 2776 771 / info@voicenter.co.il</t>
+        </is>
+      </c>
+      <c r="K341" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L341" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M341" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N341" s="3" t="inlineStr"/>
+      <c r="O341" s="3" t="inlineStr"/>
+      <c r="P341" s="3" t="inlineStr"/>
+      <c r="Q341" s="3" t="inlineStr">
+        <is>
+          <t>Tel Aviv</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="3" t="inlineStr">
+        <is>
+          <t>Dipole Wireless Communication</t>
+        </is>
+      </c>
+      <c r="B342" s="3" t="inlineStr">
+        <is>
+          <t>以色列</t>
+        </is>
+      </c>
+      <c r="C342" s="3" t="inlineStr"/>
+      <c r="D342" s="3" t="inlineStr">
+        <is>
+          <t>dipole.co.il</t>
+        </is>
+      </c>
+      <c r="E342" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F342" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G342" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H342" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I342" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J342" s="3" t="inlineStr">
+        <is>
+          <t>+972 3 573 2221 / sales@dipole-ltd.com</t>
+        </is>
+      </c>
+      <c r="K342" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L342" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M342" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N342" s="3" t="inlineStr"/>
+      <c r="O342" s="3" t="inlineStr"/>
+      <c r="P342" s="3" t="inlineStr"/>
+      <c r="Q342" s="3" t="inlineStr">
+        <is>
+          <t>Givatayim</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="3" t="inlineStr">
+        <is>
+          <t>Senetic Israel</t>
+        </is>
+      </c>
+      <c r="B343" s="3" t="inlineStr">
+        <is>
+          <t>以色列</t>
+        </is>
+      </c>
+      <c r="C343" s="3" t="inlineStr"/>
+      <c r="D343" s="3" t="inlineStr">
+        <is>
+          <t>senetic.co.il</t>
+        </is>
+      </c>
+      <c r="E343" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F343" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G343" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H343" s="3" t="inlineStr">
+        <is>
+          <t>Senetic 集团以色列站</t>
+        </is>
+      </c>
+      <c r="I343" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J343" s="3" t="inlineStr">
+        <is>
+          <t>+972 37 207 326 / info@senetic.co.il</t>
+        </is>
+      </c>
+      <c r="K343" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L343" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M343" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N343" s="3" t="inlineStr"/>
+      <c r="O343" s="3" t="inlineStr"/>
+      <c r="P343" s="3" t="inlineStr"/>
+      <c r="Q343" s="3" t="inlineStr">
+        <is>
+          <t>Tel Aviv</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="3" t="inlineStr">
+        <is>
+          <t>Ronitek</t>
+        </is>
+      </c>
+      <c r="B344" s="3" t="inlineStr">
+        <is>
+          <t>以色列</t>
+        </is>
+      </c>
+      <c r="C344" s="3" t="inlineStr"/>
+      <c r="D344" s="3" t="inlineStr">
+        <is>
+          <t>ronitek.co.il</t>
+        </is>
+      </c>
+      <c r="E344" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F344" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G344" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H344" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I344" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J344" s="3" t="inlineStr">
+        <is>
+          <t>+972 77 249 5881 / Info@ronitek.co.il</t>
+        </is>
+      </c>
+      <c r="K344" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L344" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M344" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N344" s="3" t="inlineStr"/>
+      <c r="O344" s="3" t="inlineStr"/>
+      <c r="P344" s="3" t="inlineStr"/>
+      <c r="Q344" s="3" t="inlineStr">
+        <is>
+          <t>Tel Aviv</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="3" t="inlineStr">
+        <is>
+          <t>Triple core</t>
+        </is>
+      </c>
+      <c r="B345" s="3" t="inlineStr">
+        <is>
+          <t>以色列</t>
+        </is>
+      </c>
+      <c r="C345" s="3" t="inlineStr"/>
+      <c r="D345" s="3" t="inlineStr">
+        <is>
+          <t>triple-core.com</t>
+        </is>
+      </c>
+      <c r="E345" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F345" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G345" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H345" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I345" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J345" s="3" t="inlineStr">
+        <is>
+          <t>+972 2 372 2666 / info@triple-core.com</t>
+        </is>
+      </c>
+      <c r="K345" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L345" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M345" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N345" s="3" t="inlineStr"/>
+      <c r="O345" s="3" t="inlineStr"/>
+      <c r="P345" s="3" t="inlineStr"/>
+      <c r="Q345" s="3" t="inlineStr">
+        <is>
+          <t>Jerusalem</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="3" t="inlineStr">
+        <is>
+          <t>Öruggt Net ehf（Secure Net）</t>
+        </is>
+      </c>
+      <c r="B346" s="3" t="inlineStr">
+        <is>
+          <t>冰岛</t>
+        </is>
+      </c>
+      <c r="C346" s="3" t="inlineStr"/>
+      <c r="D346" s="3" t="inlineStr">
+        <is>
+          <t>securenet.is</t>
+        </is>
+      </c>
+      <c r="E346" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F346" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G346" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H346" s="3" t="inlineStr">
+        <is>
+          <t>冰岛唯一 Master 分销 → 无竞争</t>
+        </is>
+      </c>
+      <c r="I346" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J346" s="3" t="inlineStr">
+        <is>
+          <t>+354 551 5120 / sales@securenet.is</t>
+        </is>
+      </c>
+      <c r="K346" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L346" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M346" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N346" s="3" t="inlineStr"/>
+      <c r="O346" s="3" t="inlineStr"/>
+      <c r="P346" s="3" t="inlineStr"/>
+      <c r="Q346" s="3" t="inlineStr">
+        <is>
+          <t>Reykjavik</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="3" t="inlineStr">
+        <is>
+          <t>Accreda Ltd</t>
+        </is>
+      </c>
+      <c r="B347" s="3" t="inlineStr">
+        <is>
+          <t>马耳他</t>
+        </is>
+      </c>
+      <c r="C347" s="3" t="inlineStr"/>
+      <c r="D347" s="3" t="inlineStr">
+        <is>
+          <t>accreda.eu</t>
+        </is>
+      </c>
+      <c r="E347" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F347" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G347" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H347" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I347" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J347" s="3" t="inlineStr">
+        <is>
+          <t>+356 2205 6847 / sales@accreda.eu</t>
+        </is>
+      </c>
+      <c r="K347" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L347" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M347" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N347" s="3" t="inlineStr"/>
+      <c r="O347" s="3" t="inlineStr"/>
+      <c r="P347" s="3" t="inlineStr"/>
+      <c r="Q347" s="3" t="inlineStr">
+        <is>
+          <t>Valletta</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="3" t="inlineStr">
+        <is>
+          <t>Nexus Networks</t>
+        </is>
+      </c>
+      <c r="B348" s="3" t="inlineStr">
+        <is>
+          <t>马耳他</t>
+        </is>
+      </c>
+      <c r="C348" s="3" t="inlineStr"/>
+      <c r="D348" s="3" t="inlineStr">
+        <is>
+          <t>nexus.com.mt</t>
+        </is>
+      </c>
+      <c r="E348" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F348" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G348" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H348" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I348" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J348" s="3" t="inlineStr">
+        <is>
+          <t>+356 7946 1720 / hello@nexus.com.mt</t>
+        </is>
+      </c>
+      <c r="K348" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L348" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M348" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N348" s="3" t="inlineStr"/>
+      <c r="O348" s="3" t="inlineStr"/>
+      <c r="P348" s="3" t="inlineStr"/>
+      <c r="Q348" s="3" t="inlineStr">
+        <is>
+          <t>Mgarr</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="3" t="inlineStr">
+        <is>
+          <t>WST Systems Ltd</t>
+        </is>
+      </c>
+      <c r="B349" s="3" t="inlineStr">
+        <is>
+          <t>马耳他</t>
+        </is>
+      </c>
+      <c r="C349" s="3" t="inlineStr"/>
+      <c r="D349" s="3" t="inlineStr">
+        <is>
+          <t>wstsystems.com</t>
+        </is>
+      </c>
+      <c r="E349" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F349" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G349" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H349" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I349" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J349" s="3" t="inlineStr">
+        <is>
+          <t>+356 2144 7003 / nz@wstsystems.com</t>
+        </is>
+      </c>
+      <c r="K349" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L349" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M349" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N349" s="3" t="inlineStr"/>
+      <c r="O349" s="3" t="inlineStr"/>
+      <c r="P349" s="3" t="inlineStr"/>
+      <c r="Q349" s="3" t="inlineStr">
+        <is>
+          <t>Birkirkara</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="3" t="inlineStr">
+        <is>
+          <t>MS Electronics LTD</t>
+        </is>
+      </c>
+      <c r="B350" s="3" t="inlineStr">
+        <is>
+          <t>塞浦路斯</t>
+        </is>
+      </c>
+      <c r="C350" s="3" t="inlineStr"/>
+      <c r="D350" s="3" t="inlineStr">
+        <is>
+          <t>mstronics.com</t>
+        </is>
+      </c>
+      <c r="E350" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F350" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G350" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H350" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I350" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J350" s="3" t="inlineStr">
+        <is>
+          <t>+357 25 580 611 / pieris@mstronics.com</t>
+        </is>
+      </c>
+      <c r="K350" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L350" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M350" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N350" s="3" t="inlineStr"/>
+      <c r="O350" s="3" t="inlineStr"/>
+      <c r="P350" s="3" t="inlineStr"/>
+      <c r="Q350" s="3" t="inlineStr">
+        <is>
+          <t>Limassol</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="3" t="inlineStr">
+        <is>
+          <t>Cy-Wireless（art2soft）</t>
+        </is>
+      </c>
+      <c r="B351" s="3" t="inlineStr">
+        <is>
+          <t>塞浦路斯</t>
+        </is>
+      </c>
+      <c r="C351" s="3" t="inlineStr"/>
+      <c r="D351" s="3" t="inlineStr">
+        <is>
+          <t>prod.cy-wireless.com</t>
+        </is>
+      </c>
+      <c r="E351" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F351" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G351" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H351" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I351" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J351" s="3" t="inlineStr">
+        <is>
+          <t>+357 22 814 244 / thomas.thoma@art2soft.com</t>
+        </is>
+      </c>
+      <c r="K351" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L351" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M351" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N351" s="3" t="inlineStr"/>
+      <c r="O351" s="3" t="inlineStr"/>
+      <c r="P351" s="3" t="inlineStr"/>
+      <c r="Q351" s="3" t="inlineStr"/>
+    </row>
+    <row r="352">
+      <c r="A352" s="3" t="inlineStr">
+        <is>
+          <t>Netmont DOO</t>
+        </is>
+      </c>
+      <c r="B352" s="3" t="inlineStr">
+        <is>
+          <t>黑山</t>
+        </is>
+      </c>
+      <c r="C352" s="3" t="inlineStr"/>
+      <c r="D352" s="3" t="inlineStr">
+        <is>
+          <t>netmont.me</t>
+        </is>
+      </c>
+      <c r="E352" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F352" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G352" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H352" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I352" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J352" s="3" t="inlineStr">
+        <is>
+          <t>+382 67 244 376 / info@setehnica.com</t>
+        </is>
+      </c>
+      <c r="K352" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L352" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M352" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N352" s="3" t="inlineStr"/>
+      <c r="O352" s="3" t="inlineStr"/>
+      <c r="P352" s="3" t="inlineStr"/>
+      <c r="Q352" s="3" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="3" t="inlineStr">
+        <is>
+          <t>RIDMONT D.O.O.</t>
+        </is>
+      </c>
+      <c r="B353" s="3" t="inlineStr">
+        <is>
+          <t>黑山</t>
+        </is>
+      </c>
+      <c r="C353" s="3" t="inlineStr"/>
+      <c r="D353" s="3" t="inlineStr">
+        <is>
+          <t>ridmont.me</t>
+        </is>
+      </c>
+      <c r="E353" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F353" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G353" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H353" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I353" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J353" s="3" t="inlineStr">
+        <is>
+          <t>+382 67 335 148 / info@ridmont.me</t>
+        </is>
+      </c>
+      <c r="K353" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L353" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M353" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N353" s="3" t="inlineStr"/>
+      <c r="O353" s="3" t="inlineStr"/>
+      <c r="P353" s="3" t="inlineStr"/>
+      <c r="Q353" s="3" t="inlineStr">
+        <is>
+          <t>Podgorica</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="3" t="inlineStr">
+        <is>
+          <t>ALL4NET DOOEL</t>
+        </is>
+      </c>
+      <c r="B354" s="3" t="inlineStr">
+        <is>
+          <t>北马其顿</t>
+        </is>
+      </c>
+      <c r="C354" s="3" t="inlineStr"/>
+      <c r="D354" s="3" t="inlineStr">
+        <is>
+          <t>toten.com.mk</t>
+        </is>
+      </c>
+      <c r="E354" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F354" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G354" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H354" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I354" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J354" s="3" t="inlineStr">
+        <is>
+          <t>+389 2 321 77 99 / dejan.dudeski@overnet.com.mk</t>
+        </is>
+      </c>
+      <c r="K354" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L354" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M354" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N354" s="3" t="inlineStr"/>
+      <c r="O354" s="3" t="inlineStr"/>
+      <c r="P354" s="3" t="inlineStr"/>
+      <c r="Q354" s="3" t="inlineStr">
+        <is>
+          <t>Skopje</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="3" t="inlineStr">
+        <is>
+          <t>Treco</t>
+        </is>
+      </c>
+      <c r="B355" s="3" t="inlineStr">
+        <is>
+          <t>北马其顿</t>
+        </is>
+      </c>
+      <c r="C355" s="3" t="inlineStr"/>
+      <c r="D355" s="3" t="inlineStr">
+        <is>
+          <t>treco.mk</t>
+        </is>
+      </c>
+      <c r="E355" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F355" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G355" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H355" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I355" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J355" s="3" t="inlineStr">
+        <is>
+          <t>+389 70 411 415 / info@treco.mk</t>
+        </is>
+      </c>
+      <c r="K355" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L355" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M355" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N355" s="3" t="inlineStr"/>
+      <c r="O355" s="3" t="inlineStr"/>
+      <c r="P355" s="3" t="inlineStr"/>
+      <c r="Q355" s="3" t="inlineStr">
+        <is>
+          <t>Skopje</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="3" t="inlineStr">
+        <is>
+          <t>Pride</t>
+        </is>
+      </c>
+      <c r="B356" s="3" t="inlineStr">
+        <is>
+          <t>摩尔多瓦</t>
+        </is>
+      </c>
+      <c r="C356" s="3" t="inlineStr"/>
+      <c r="D356" s="3" t="inlineStr">
+        <is>
+          <t>pride.md</t>
+        </is>
+      </c>
+      <c r="E356" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F356" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G356" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H356" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I356" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J356" s="3" t="inlineStr">
+        <is>
+          <t>sales@pride.md</t>
+        </is>
+      </c>
+      <c r="K356" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L356" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M356" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N356" s="3" t="inlineStr"/>
+      <c r="O356" s="3" t="inlineStr"/>
+      <c r="P356" s="3" t="inlineStr"/>
+      <c r="Q356" s="3" t="inlineStr">
+        <is>
+          <t>Chișinău</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="3" t="inlineStr">
+        <is>
+          <t>Star Net</t>
+        </is>
+      </c>
+      <c r="B357" s="3" t="inlineStr">
+        <is>
+          <t>摩尔多瓦</t>
+        </is>
+      </c>
+      <c r="C357" s="3" t="inlineStr"/>
+      <c r="D357" s="3" t="inlineStr">
+        <is>
+          <t>starnet.md</t>
+        </is>
+      </c>
+      <c r="E357" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F357" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G357" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H357" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I357" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J357" s="3" t="inlineStr">
+        <is>
+          <t>022 844 444</t>
+        </is>
+      </c>
+      <c r="K357" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L357" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M357" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N357" s="3" t="inlineStr"/>
+      <c r="O357" s="3" t="inlineStr"/>
+      <c r="P357" s="3" t="inlineStr"/>
+      <c r="Q357" s="3" t="inlineStr">
+        <is>
+          <t>Chișinău</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="3" t="inlineStr">
+        <is>
+          <t>Comitek（doxyterra.md）</t>
+        </is>
+      </c>
+      <c r="B358" s="3" t="inlineStr">
+        <is>
+          <t>摩尔多瓦</t>
+        </is>
+      </c>
+      <c r="C358" s="3" t="inlineStr"/>
+      <c r="D358" s="3" t="inlineStr">
+        <is>
+          <t>doxyterra.md</t>
+        </is>
+      </c>
+      <c r="E358" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F358" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G358" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H358" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I358" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J358" s="3" t="inlineStr">
+        <is>
+          <t>+373 533 74848 / info@doxyterra.md</t>
+        </is>
+      </c>
+      <c r="K358" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L358" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M358" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N358" s="3" t="inlineStr"/>
+      <c r="O358" s="3" t="inlineStr"/>
+      <c r="P358" s="3" t="inlineStr"/>
+      <c r="Q358" s="3" t="inlineStr">
+        <is>
+          <t>Chișinău</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="3" t="inlineStr">
+        <is>
+          <t>KosProd</t>
+        </is>
+      </c>
+      <c r="B359" s="3" t="inlineStr">
+        <is>
+          <t>科索沃</t>
+        </is>
+      </c>
+      <c r="C359" s="3" t="inlineStr"/>
+      <c r="D359" s="3" t="inlineStr">
+        <is>
+          <t>kosprod.com</t>
+        </is>
+      </c>
+      <c r="E359" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F359" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G359" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H359" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I359" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J359" s="3" t="inlineStr">
+        <is>
+          <t>+377 45 607 000 / order@kosprod.com</t>
+        </is>
+      </c>
+      <c r="K359" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L359" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M359" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N359" s="3" t="inlineStr"/>
+      <c r="O359" s="3" t="inlineStr"/>
+      <c r="P359" s="3" t="inlineStr"/>
+      <c r="Q359" s="3" t="inlineStr">
+        <is>
+          <t>Fushë Kosovë</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="3" t="inlineStr">
+        <is>
+          <t>H2 HOLDING LLC（fortshpejt.com）</t>
+        </is>
+      </c>
+      <c r="B360" s="3" t="inlineStr">
+        <is>
+          <t>科索沃</t>
+        </is>
+      </c>
+      <c r="C360" s="3" t="inlineStr"/>
+      <c r="D360" s="3" t="inlineStr">
+        <is>
+          <t>fortshpejt.com</t>
+        </is>
+      </c>
+      <c r="E360" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F360" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G360" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H360" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I360" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J360" s="3" t="inlineStr">
+        <is>
+          <t>+383 46 150 051 / info@fortshpejt.com</t>
+        </is>
+      </c>
+      <c r="K360" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L360" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M360" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N360" s="3" t="inlineStr"/>
+      <c r="O360" s="3" t="inlineStr"/>
+      <c r="P360" s="3" t="inlineStr"/>
+      <c r="Q360" s="3" t="inlineStr">
+        <is>
+          <t>Prishtina</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="3" t="inlineStr">
+        <is>
+          <t>Intellcom Group Ltd</t>
+        </is>
+      </c>
+      <c r="B361" s="3" t="inlineStr">
+        <is>
+          <t>格鲁吉亚</t>
+        </is>
+      </c>
+      <c r="C361" s="3" t="inlineStr"/>
+      <c r="D361" s="3" t="inlineStr">
+        <is>
+          <t>intellcom.net</t>
+        </is>
+      </c>
+      <c r="E361" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F361" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G361" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H361" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I361" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J361" s="3" t="inlineStr">
+        <is>
+          <t>+995 32 298 98 49 / sale@intellcom.net</t>
+        </is>
+      </c>
+      <c r="K361" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L361" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M361" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N361" s="3" t="inlineStr"/>
+      <c r="O361" s="3" t="inlineStr"/>
+      <c r="P361" s="3" t="inlineStr"/>
+      <c r="Q361" s="3" t="inlineStr">
+        <is>
+          <t>Tbilisi</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="3" t="inlineStr">
+        <is>
+          <t>TAKOPI GEORGIA（smart-network.ge）</t>
+        </is>
+      </c>
+      <c r="B362" s="3" t="inlineStr">
+        <is>
+          <t>格鲁吉亚</t>
+        </is>
+      </c>
+      <c r="C362" s="3" t="inlineStr"/>
+      <c r="D362" s="3" t="inlineStr">
+        <is>
+          <t>smart-network.ge</t>
+        </is>
+      </c>
+      <c r="E362" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F362" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G362" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H362" s="3" t="inlineStr">
+        <is>
+          <t>专设 smart-network.ge 项目站做 MikroTik</t>
+        </is>
+      </c>
+      <c r="I362" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J362" s="3" t="inlineStr">
+        <is>
+          <t>+995 505 05 05 60 / info@takopi.ge</t>
+        </is>
+      </c>
+      <c r="K362" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L362" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M362" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N362" s="3" t="inlineStr"/>
+      <c r="O362" s="3" t="inlineStr"/>
+      <c r="P362" s="3" t="inlineStr"/>
+      <c r="Q362" s="3" t="inlineStr">
+        <is>
+          <t>Tbilisi</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="3" t="inlineStr">
+        <is>
+          <t>GCOM</t>
+        </is>
+      </c>
+      <c r="B363" s="3" t="inlineStr">
+        <is>
+          <t>格鲁吉亚</t>
+        </is>
+      </c>
+      <c r="C363" s="3" t="inlineStr"/>
+      <c r="D363" s="3" t="inlineStr">
+        <is>
+          <t>gcom.ge</t>
+        </is>
+      </c>
+      <c r="E363" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F363" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G363" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H363" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I363" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J363" s="3" t="inlineStr">
+        <is>
+          <t>+995 322 420 449 / info@gcom.ge</t>
+        </is>
+      </c>
+      <c r="K363" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L363" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M363" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N363" s="3" t="inlineStr"/>
+      <c r="O363" s="3" t="inlineStr"/>
+      <c r="P363" s="3" t="inlineStr"/>
+      <c r="Q363" s="3" t="inlineStr">
+        <is>
+          <t>Tbilisi</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sweep USA (27) and Canada (7): 396 accounts total
Completes North America from the MikroTik official distributor directory.
Winncom's global HQ in Solon OH links the US, Irish, Lithuanian and
Latvian entities under one negotiation; WAV/MBSI WAV/ISP Supplies is one
group across both countries. Miami clusters 7 more Latin America-facing
distributors. US entries carry the TAA/NDAA caveat: China-origin gear
cannot serve government or utility projects, commercial channel only.
Europe (38 countries) and North America are now fully covered.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q363"/>
+  <dimension ref="A1:Q396"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -36688,6 +36688,2477 @@
       <c r="Q363" s="3" t="inlineStr">
         <is>
           <t>Tbilisi</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="3" t="inlineStr">
+        <is>
+          <t>Streakwave</t>
+        </is>
+      </c>
+      <c r="B364" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C364" s="3" t="inlineStr">
+        <is>
+          <t>CA（另有 UT、OH）</t>
+        </is>
+      </c>
+      <c r="D364" s="3" t="inlineStr">
+        <is>
+          <t>streakwave.com</t>
+        </is>
+      </c>
+      <c r="E364" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F364" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G364" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H364" s="3" t="inlineStr">
+        <is>
+          <t>美国西部最大无线/网络分销之一，三州仓库</t>
+        </is>
+      </c>
+      <c r="I364" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J364" s="3" t="inlineStr">
+        <is>
+          <t>+1 888 604 5234 / contact@streakwave.com</t>
+        </is>
+      </c>
+      <c r="K364" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L364" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M364" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N364" s="3" t="inlineStr"/>
+      <c r="O364" s="3" t="inlineStr"/>
+      <c r="P364" s="3" t="inlineStr"/>
+      <c r="Q364" s="3" t="inlineStr">
+        <is>
+          <t>USSan Jose, CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="3" t="inlineStr">
+        <is>
+          <t>Baltic Network</t>
+        </is>
+      </c>
+      <c r="B365" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C365" s="3" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="D365" s="3" t="inlineStr">
+        <is>
+          <t>balticnetworks.com</t>
+        </is>
+      </c>
+      <c r="E365" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F365" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G365" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H365" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I365" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J365" s="3" t="inlineStr">
+        <is>
+          <t>+1 630 929 3610 / hello@balticnetworks.com</t>
+        </is>
+      </c>
+      <c r="K365" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L365" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M365" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N365" s="3" t="inlineStr"/>
+      <c r="O365" s="3" t="inlineStr"/>
+      <c r="P365" s="3" t="inlineStr"/>
+      <c r="Q365" s="3" t="inlineStr">
+        <is>
+          <t>USChicago</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="3" t="inlineStr">
+        <is>
+          <t>Digicomm International</t>
+        </is>
+      </c>
+      <c r="B366" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C366" s="3" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="D366" s="3" t="inlineStr">
+        <is>
+          <t>digicomm.com</t>
+        </is>
+      </c>
+      <c r="E366" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F366" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G366" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H366" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I366" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J366" s="3" t="inlineStr">
+        <is>
+          <t>+1 303 799 3444 / sales@digicomm.com</t>
+        </is>
+      </c>
+      <c r="K366" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L366" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M366" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N366" s="3" t="inlineStr"/>
+      <c r="O366" s="3" t="inlineStr"/>
+      <c r="P366" s="3" t="inlineStr"/>
+      <c r="Q366" s="3" t="inlineStr">
+        <is>
+          <t>USEnglewood</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="3" t="inlineStr">
+        <is>
+          <t>Flytec Computers</t>
+        </is>
+      </c>
+      <c r="B367" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C367" s="3" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="D367" s="3" t="inlineStr">
+        <is>
+          <t>flyteccomputers.com</t>
+        </is>
+      </c>
+      <c r="E367" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F367" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G367" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H367" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I367" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J367" s="3" t="inlineStr">
+        <is>
+          <t>+1 305 471 5142 / sales@flyteccomputers.com</t>
+        </is>
+      </c>
+      <c r="K367" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L367" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M367" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N367" s="3" t="inlineStr"/>
+      <c r="O367" s="3" t="inlineStr"/>
+      <c r="P367" s="3" t="inlineStr"/>
+      <c r="Q367" s="3" t="inlineStr">
+        <is>
+          <t>USMiami；拉美渠道强</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="3" t="inlineStr">
+        <is>
+          <t>4Net Networking, Corp.</t>
+        </is>
+      </c>
+      <c r="B368" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C368" s="3" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="D368" s="3" t="inlineStr">
+        <is>
+          <t>4netonline.com</t>
+        </is>
+      </c>
+      <c r="E368" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F368" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G368" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H368" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I368" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J368" s="3" t="inlineStr">
+        <is>
+          <t>+1 305 599 0086 / sales@4netonline.com</t>
+        </is>
+      </c>
+      <c r="K368" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L368" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M368" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N368" s="3" t="inlineStr"/>
+      <c r="O368" s="3" t="inlineStr"/>
+      <c r="P368" s="3" t="inlineStr"/>
+      <c r="Q368" s="3" t="inlineStr">
+        <is>
+          <t>USMiami</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="3" t="inlineStr">
+        <is>
+          <t>Pace International</t>
+        </is>
+      </c>
+      <c r="B369" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C369" s="3" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="D369" s="3" t="inlineStr">
+        <is>
+          <t>paceintl.com</t>
+        </is>
+      </c>
+      <c r="E369" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F369" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G369" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H369" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I369" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J369" s="3" t="inlineStr">
+        <is>
+          <t>+1 800 444 7223 / sales@paceintl.com</t>
+        </is>
+      </c>
+      <c r="K369" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L369" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M369" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N369" s="3" t="inlineStr"/>
+      <c r="O369" s="3" t="inlineStr"/>
+      <c r="P369" s="3" t="inlineStr"/>
+      <c r="Q369" s="3" t="inlineStr">
+        <is>
+          <t>USRochester</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="3" t="inlineStr">
+        <is>
+          <t>ROC-NOC</t>
+        </is>
+      </c>
+      <c r="B370" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C370" s="3" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="D370" s="3" t="inlineStr">
+        <is>
+          <t>roc-noc.com</t>
+        </is>
+      </c>
+      <c r="E370" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F370" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G370" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H370" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I370" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J370" s="3" t="inlineStr">
+        <is>
+          <t>+1 815 209 2224 / sales@roc-noc.com</t>
+        </is>
+      </c>
+      <c r="K370" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L370" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M370" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N370" s="3" t="inlineStr"/>
+      <c r="O370" s="3" t="inlineStr"/>
+      <c r="P370" s="3" t="inlineStr"/>
+      <c r="Q370" s="3" t="inlineStr">
+        <is>
+          <t>USRockford</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="3" t="inlineStr">
+        <is>
+          <t>Microcom Technologies</t>
+        </is>
+      </c>
+      <c r="B371" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C371" s="3" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="D371" s="3" t="inlineStr">
+        <is>
+          <t>microcom.us</t>
+        </is>
+      </c>
+      <c r="E371" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F371" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G371" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H371" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I371" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J371" s="3" t="inlineStr">
+        <is>
+          <t>+1 818 880 8008 / sales@microcomtec.com</t>
+        </is>
+      </c>
+      <c r="K371" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L371" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M371" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N371" s="3" t="inlineStr"/>
+      <c r="O371" s="3" t="inlineStr"/>
+      <c r="P371" s="3" t="inlineStr"/>
+      <c r="Q371" s="3" t="inlineStr">
+        <is>
+          <t>USCalabasas</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="3" t="inlineStr">
+        <is>
+          <t>Link Technologies, Inc.</t>
+        </is>
+      </c>
+      <c r="B372" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C372" s="3" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="D372" s="3" t="inlineStr">
+        <is>
+          <t>linktechs.net</t>
+        </is>
+      </c>
+      <c r="E372" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F372" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G372" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H372" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I372" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J372" s="3" t="inlineStr">
+        <is>
+          <t>+1 314 735 0270 / support@linktechs.net</t>
+        </is>
+      </c>
+      <c r="K372" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L372" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M372" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N372" s="3" t="inlineStr"/>
+      <c r="O372" s="3" t="inlineStr"/>
+      <c r="P372" s="3" t="inlineStr"/>
+      <c r="Q372" s="3" t="inlineStr">
+        <is>
+          <t>USDittmer</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="3" t="inlineStr">
+        <is>
+          <t>Multilink Solutions</t>
+        </is>
+      </c>
+      <c r="B373" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C373" s="3" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="D373" s="3" t="inlineStr">
+        <is>
+          <t>multilink.us</t>
+        </is>
+      </c>
+      <c r="E373" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F373" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G373" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H373" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I373" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J373" s="3" t="inlineStr">
+        <is>
+          <t>+1 513 501 8006 / info@multilink.us</t>
+        </is>
+      </c>
+      <c r="K373" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L373" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M373" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N373" s="3" t="inlineStr"/>
+      <c r="O373" s="3" t="inlineStr"/>
+      <c r="P373" s="3" t="inlineStr"/>
+      <c r="Q373" s="3" t="inlineStr">
+        <is>
+          <t>USCincinnati</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="3" t="inlineStr">
+        <is>
+          <t>Solution Box LLC</t>
+        </is>
+      </c>
+      <c r="B374" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C374" s="3" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="D374" s="3" t="inlineStr">
+        <is>
+          <t>solutionboxusa.com</t>
+        </is>
+      </c>
+      <c r="E374" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F374" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G374" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H374" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I374" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J374" s="3" t="inlineStr">
+        <is>
+          <t>+1 305 722 3826 / contact@solutionboxusa.com</t>
+        </is>
+      </c>
+      <c r="K374" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L374" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M374" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N374" s="3" t="inlineStr"/>
+      <c r="O374" s="3" t="inlineStr"/>
+      <c r="P374" s="3" t="inlineStr"/>
+      <c r="Q374" s="3" t="inlineStr">
+        <is>
+          <t>USDoral</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="3" t="inlineStr">
+        <is>
+          <t>Vodanet Systems LLC</t>
+        </is>
+      </c>
+      <c r="B375" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C375" s="3" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="D375" s="3" t="inlineStr">
+        <is>
+          <t>vodanetsystems.com</t>
+        </is>
+      </c>
+      <c r="E375" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F375" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G375" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H375" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I375" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J375" s="3" t="inlineStr">
+        <is>
+          <t>+1 862 274 9010 / info@vodanetsystems.com</t>
+        </is>
+      </c>
+      <c r="K375" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L375" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M375" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N375" s="3" t="inlineStr"/>
+      <c r="O375" s="3" t="inlineStr"/>
+      <c r="P375" s="3" t="inlineStr"/>
+      <c r="Q375" s="3" t="inlineStr">
+        <is>
+          <t>USPompton Plains</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="3" t="inlineStr">
+        <is>
+          <t>NACE Inc（North American Cable）</t>
+        </is>
+      </c>
+      <c r="B376" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C376" s="3" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="D376" s="3" t="inlineStr">
+        <is>
+          <t>products.nace.tv</t>
+        </is>
+      </c>
+      <c r="E376" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F376" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master）</t>
+        </is>
+      </c>
+      <c r="G376" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H376" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I376" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT</t>
+        </is>
+      </c>
+      <c r="J376" s="3" t="inlineStr">
+        <is>
+          <t>+1 800 688 9282 / sales@northamericancable.com</t>
+        </is>
+      </c>
+      <c r="K376" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L376" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M376" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N376" s="3" t="inlineStr"/>
+      <c r="O376" s="3" t="inlineStr"/>
+      <c r="P376" s="3" t="inlineStr"/>
+      <c r="Q376" s="3" t="inlineStr">
+        <is>
+          <t>USWest Chester</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="3" t="inlineStr">
+        <is>
+          <t>ISP Supplies（powered by WAV）</t>
+        </is>
+      </c>
+      <c r="B377" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C377" s="3" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="D377" s="3" t="inlineStr">
+        <is>
+          <t>ispsupplies.com</t>
+        </is>
+      </c>
+      <c r="E377" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F377" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G377" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H377" s="3" t="inlineStr">
+        <is>
+          <t>WAV 集团旗下；另有加拿大站</t>
+        </is>
+      </c>
+      <c r="I377" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J377" s="3" t="inlineStr">
+        <is>
+          <t>+1 855 947 7776 / sales@ispsupplies.com</t>
+        </is>
+      </c>
+      <c r="K377" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L377" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M377" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N377" s="3" t="inlineStr"/>
+      <c r="O377" s="3" t="inlineStr"/>
+      <c r="P377" s="3" t="inlineStr"/>
+      <c r="Q377" s="3" t="inlineStr">
+        <is>
+          <t>USCollege Station</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="3" t="inlineStr">
+        <is>
+          <t>DoubleRadius, Inc.</t>
+        </is>
+      </c>
+      <c r="B378" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C378" s="3" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="D378" s="3" t="inlineStr">
+        <is>
+          <t>doubleradius.com</t>
+        </is>
+      </c>
+      <c r="E378" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F378" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G378" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H378" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I378" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J378" s="3" t="inlineStr">
+        <is>
+          <t>+1 704 927 6100 / salesteam@doubleradius.com</t>
+        </is>
+      </c>
+      <c r="K378" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L378" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M378" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N378" s="3" t="inlineStr"/>
+      <c r="O378" s="3" t="inlineStr"/>
+      <c r="P378" s="3" t="inlineStr"/>
+      <c r="Q378" s="3" t="inlineStr">
+        <is>
+          <t>USIndian Trail；WISP 方案商</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="3" t="inlineStr">
+        <is>
+          <t>EPCOM</t>
+        </is>
+      </c>
+      <c r="B379" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C379" s="3" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="D379" s="3" t="inlineStr">
+        <is>
+          <t>epcom.net</t>
+        </is>
+      </c>
+      <c r="E379" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F379" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G379" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H379" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I379" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J379" s="3" t="inlineStr">
+        <is>
+          <t>+1 915 533 5119 / sales@epcom.net</t>
+        </is>
+      </c>
+      <c r="K379" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L379" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M379" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N379" s="3" t="inlineStr"/>
+      <c r="O379" s="3" t="inlineStr"/>
+      <c r="P379" s="3" t="inlineStr"/>
+      <c r="Q379" s="3" t="inlineStr">
+        <is>
+          <t>USDoral；拉美渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="3" t="inlineStr">
+        <is>
+          <t>CTIconnect LLC</t>
+        </is>
+      </c>
+      <c r="B380" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C380" s="3" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="D380" s="3" t="inlineStr">
+        <is>
+          <t>cticonnect.com</t>
+        </is>
+      </c>
+      <c r="E380" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F380" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G380" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H380" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I380" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J380" s="3" t="inlineStr">
+        <is>
+          <t>+1 561 295 7899 / sales@cticonnect.com</t>
+        </is>
+      </c>
+      <c r="K380" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L380" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M380" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N380" s="3" t="inlineStr"/>
+      <c r="O380" s="3" t="inlineStr"/>
+      <c r="P380" s="3" t="inlineStr"/>
+      <c r="Q380" s="3" t="inlineStr">
+        <is>
+          <t>USRiviera Beach</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="3" t="inlineStr">
+        <is>
+          <t>Leverify LLC</t>
+        </is>
+      </c>
+      <c r="B381" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C381" s="3" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="D381" s="3" t="inlineStr">
+        <is>
+          <t>leverify.com</t>
+        </is>
+      </c>
+      <c r="E381" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F381" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G381" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H381" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I381" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J381" s="3" t="inlineStr">
+        <is>
+          <t>+1 425 654 0681 / brands@leverify.com</t>
+        </is>
+      </c>
+      <c r="K381" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L381" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M381" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N381" s="3" t="inlineStr"/>
+      <c r="O381" s="3" t="inlineStr"/>
+      <c r="P381" s="3" t="inlineStr"/>
+      <c r="Q381" s="3" t="inlineStr">
+        <is>
+          <t>USBellevue</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="3" t="inlineStr">
+        <is>
+          <t>Altanet Corporation</t>
+        </is>
+      </c>
+      <c r="B382" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C382" s="3" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="D382" s="3" t="inlineStr">
+        <is>
+          <t>altanet-corp.com</t>
+        </is>
+      </c>
+      <c r="E382" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F382" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G382" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H382" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I382" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J382" s="3" t="inlineStr">
+        <is>
+          <t>+1 786 228 5758 / aeal@altanet-corp.com</t>
+        </is>
+      </c>
+      <c r="K382" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L382" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M382" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N382" s="3" t="inlineStr"/>
+      <c r="O382" s="3" t="inlineStr"/>
+      <c r="P382" s="3" t="inlineStr"/>
+      <c r="Q382" s="3" t="inlineStr">
+        <is>
+          <t>USMiami</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="3" t="inlineStr">
+        <is>
+          <t>Interamerican Tech Corp.</t>
+        </is>
+      </c>
+      <c r="B383" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C383" s="3" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="D383" s="3" t="inlineStr">
+        <is>
+          <t>itamtech.com</t>
+        </is>
+      </c>
+      <c r="E383" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F383" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G383" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H383" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I383" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J383" s="3" t="inlineStr">
+        <is>
+          <t>+1 305 639 2524 / sales@itamtech.com</t>
+        </is>
+      </c>
+      <c r="K383" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L383" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M383" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N383" s="3" t="inlineStr"/>
+      <c r="O383" s="3" t="inlineStr"/>
+      <c r="P383" s="3" t="inlineStr"/>
+      <c r="Q383" s="3" t="inlineStr">
+        <is>
+          <t>USMiami</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="3" t="inlineStr">
+        <is>
+          <t>BIBAOnline</t>
+        </is>
+      </c>
+      <c r="B384" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C384" s="3" t="inlineStr">
+        <is>
+          <t>VA</t>
+        </is>
+      </c>
+      <c r="D384" s="3" t="inlineStr">
+        <is>
+          <t>bibaonline.com</t>
+        </is>
+      </c>
+      <c r="E384" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F384" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G384" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H384" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I384" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J384" s="3" t="inlineStr">
+        <is>
+          <t>+1 571 249 2422 / info@biballc.com</t>
+        </is>
+      </c>
+      <c r="K384" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L384" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M384" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N384" s="3" t="inlineStr"/>
+      <c r="O384" s="3" t="inlineStr"/>
+      <c r="P384" s="3" t="inlineStr"/>
+      <c r="Q384" s="3" t="inlineStr">
+        <is>
+          <t>USCentreville</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="3" t="inlineStr">
+        <is>
+          <t>Business Systems Connection, Inc.</t>
+        </is>
+      </c>
+      <c r="B385" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C385" s="3" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="D385" s="3" t="inlineStr">
+        <is>
+          <t>shop.bizsyscon.com</t>
+        </is>
+      </c>
+      <c r="E385" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F385" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G385" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H385" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I385" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J385" s="3" t="inlineStr">
+        <is>
+          <t>+1 636 600 1400 / sales@bizsyscon.com</t>
+        </is>
+      </c>
+      <c r="K385" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L385" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M385" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N385" s="3" t="inlineStr"/>
+      <c r="O385" s="3" t="inlineStr"/>
+      <c r="P385" s="3" t="inlineStr"/>
+      <c r="Q385" s="3" t="inlineStr">
+        <is>
+          <t>USFenton</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="3" t="inlineStr">
+        <is>
+          <t>Hexstar</t>
+        </is>
+      </c>
+      <c r="B386" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C386" s="3" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="D386" s="3" t="inlineStr">
+        <is>
+          <t>hexstar.com</t>
+        </is>
+      </c>
+      <c r="E386" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F386" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G386" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H386" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I386" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J386" s="3" t="inlineStr">
+        <is>
+          <t>+1 888 NETFIX8 / info@hexstar.com</t>
+        </is>
+      </c>
+      <c r="K386" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L386" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M386" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N386" s="3" t="inlineStr"/>
+      <c r="O386" s="3" t="inlineStr"/>
+      <c r="P386" s="3" t="inlineStr"/>
+      <c r="Q386" s="3" t="inlineStr">
+        <is>
+          <t>USDallas</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="3" t="inlineStr">
+        <is>
+          <t>Makro Wisp</t>
+        </is>
+      </c>
+      <c r="B387" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C387" s="3" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="D387" s="3" t="inlineStr">
+        <is>
+          <t>makrowisp.com</t>
+        </is>
+      </c>
+      <c r="E387" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F387" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G387" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H387" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I387" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J387" s="3" t="inlineStr">
+        <is>
+          <t>+1 980 441 1125 / Sales@makrowisp.com</t>
+        </is>
+      </c>
+      <c r="K387" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L387" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M387" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N387" s="3" t="inlineStr"/>
+      <c r="O387" s="3" t="inlineStr"/>
+      <c r="P387" s="3" t="inlineStr"/>
+      <c r="Q387" s="3" t="inlineStr">
+        <is>
+          <t>USMonroe；WISP 渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="3" t="inlineStr">
+        <is>
+          <t>Itshopp.com</t>
+        </is>
+      </c>
+      <c r="B388" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C388" s="3" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="D388" s="3" t="inlineStr">
+        <is>
+          <t>itshopp.com</t>
+        </is>
+      </c>
+      <c r="E388" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F388" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G388" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H388" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I388" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J388" s="3" t="inlineStr">
+        <is>
+          <t>+1 786 495 0313 / eddy@itshopp.com</t>
+        </is>
+      </c>
+      <c r="K388" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L388" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M388" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N388" s="3" t="inlineStr"/>
+      <c r="O388" s="3" t="inlineStr"/>
+      <c r="P388" s="3" t="inlineStr"/>
+      <c r="Q388" s="3" t="inlineStr">
+        <is>
+          <t>USMiami</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="3" t="inlineStr">
+        <is>
+          <t>Distrigo Inc.</t>
+        </is>
+      </c>
+      <c r="B389" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C389" s="3" t="inlineStr">
+        <is>
+          <t>FL</t>
+        </is>
+      </c>
+      <c r="D389" s="3" t="inlineStr">
+        <is>
+          <t>distrigoinc.com</t>
+        </is>
+      </c>
+      <c r="E389" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F389" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G389" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H389" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I389" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J389" s="3" t="inlineStr">
+        <is>
+          <t>+1 203 883 9169 / sales@distrigoinc.com</t>
+        </is>
+      </c>
+      <c r="K389" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L389" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M389" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N389" s="3" t="inlineStr"/>
+      <c r="O389" s="3" t="inlineStr"/>
+      <c r="P389" s="3" t="inlineStr"/>
+      <c r="Q389" s="3" t="inlineStr">
+        <is>
+          <t>USNorth Miami</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="3" t="inlineStr">
+        <is>
+          <t>MBSI WAV</t>
+        </is>
+      </c>
+      <c r="B390" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C390" s="3" t="inlineStr">
+        <is>
+          <t>Alberta</t>
+        </is>
+      </c>
+      <c r="D390" s="3" t="inlineStr">
+        <is>
+          <t>mbsiwav.com</t>
+        </is>
+      </c>
+      <c r="E390" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F390" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G390" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H390" s="3" t="inlineStr">
+        <is>
+          <t>WAV 集团加拿大主体（美加一体）</t>
+        </is>
+      </c>
+      <c r="I390" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J390" s="3" t="inlineStr">
+        <is>
+          <t>+1 866 597 6274 / sales@mbsiwav.com</t>
+        </is>
+      </c>
+      <c r="K390" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L390" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M390" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N390" s="3" t="inlineStr"/>
+      <c r="O390" s="3" t="inlineStr"/>
+      <c r="P390" s="3" t="inlineStr"/>
+      <c r="Q390" s="3" t="inlineStr">
+        <is>
+          <t>Medicine Hat</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="3" t="inlineStr">
+        <is>
+          <t>Wireless Netware</t>
+        </is>
+      </c>
+      <c r="B391" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C391" s="3" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="D391" s="3" t="inlineStr">
+        <is>
+          <t>wirelessnetware.ca</t>
+        </is>
+      </c>
+      <c r="E391" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F391" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G391" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H391" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I391" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J391" s="3" t="inlineStr">
+        <is>
+          <t>+1 647 477 0163 / info@wirelessnetware.ca</t>
+        </is>
+      </c>
+      <c r="K391" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L391" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M391" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N391" s="3" t="inlineStr"/>
+      <c r="O391" s="3" t="inlineStr"/>
+      <c r="P391" s="3" t="inlineStr"/>
+      <c r="Q391" s="3" t="inlineStr">
+        <is>
+          <t>Markham</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="3" t="inlineStr">
+        <is>
+          <t>JRS Global Technologies Ltd</t>
+        </is>
+      </c>
+      <c r="B392" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C392" s="3" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="D392" s="3" t="inlineStr">
+        <is>
+          <t>jrsglcanada.com</t>
+        </is>
+      </c>
+      <c r="E392" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F392" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G392" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H392" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 官方分销，商用线可直接比价，工业线为零 → 新品类增量</t>
+        </is>
+      </c>
+      <c r="I392" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS8GT-S</t>
+        </is>
+      </c>
+      <c r="J392" s="3" t="inlineStr">
+        <is>
+          <t>+1 905 805 6660 / Sales@jrsgl.com</t>
+        </is>
+      </c>
+      <c r="K392" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L392" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M392" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N392" s="3" t="inlineStr"/>
+      <c r="O392" s="3" t="inlineStr"/>
+      <c r="P392" s="3" t="inlineStr"/>
+      <c r="Q392" s="3" t="inlineStr">
+        <is>
+          <t>Oakville</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="3" t="inlineStr">
+        <is>
+          <t>Solimedia Technology Inc</t>
+        </is>
+      </c>
+      <c r="B393" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C393" s="3" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="D393" s="3" t="inlineStr">
+        <is>
+          <t>solimedia.net</t>
+        </is>
+      </c>
+      <c r="E393" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F393" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Master+VAD）</t>
+        </is>
+      </c>
+      <c r="G393" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H393" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I393" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J393" s="3" t="inlineStr">
+        <is>
+          <t>+1 604 568 9797 / sales@solimedia.net</t>
+        </is>
+      </c>
+      <c r="K393" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L393" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M393" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N393" s="3" t="inlineStr"/>
+      <c r="O393" s="3" t="inlineStr"/>
+      <c r="P393" s="3" t="inlineStr"/>
+      <c r="Q393" s="3" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="3" t="inlineStr">
+        <is>
+          <t>Optitera Global Networks Inc.</t>
+        </is>
+      </c>
+      <c r="B394" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C394" s="3" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="D394" s="3" t="inlineStr">
+        <is>
+          <t>optiteraglobal.ca</t>
+        </is>
+      </c>
+      <c r="E394" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F394" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G394" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H394" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I394" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J394" s="3" t="inlineStr">
+        <is>
+          <t>+1 437 424 4024 / sales@optiteraglobal.ca</t>
+        </is>
+      </c>
+      <c r="K394" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L394" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M394" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N394" s="3" t="inlineStr"/>
+      <c r="O394" s="3" t="inlineStr"/>
+      <c r="P394" s="3" t="inlineStr"/>
+      <c r="Q394" s="3" t="inlineStr"/>
+    </row>
+    <row r="395">
+      <c r="A395" s="3" t="inlineStr">
+        <is>
+          <t>ISP Supplies Canada（MBSI WAV）</t>
+        </is>
+      </c>
+      <c r="B395" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C395" s="3" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="D395" s="3" t="inlineStr">
+        <is>
+          <t>ispsupplies.ca</t>
+        </is>
+      </c>
+      <c r="E395" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F395" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G395" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H395" s="3" t="inlineStr">
+        <is>
+          <t>WAV 集团加拿大站</t>
+        </is>
+      </c>
+      <c r="I395" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J395" s="3" t="inlineStr">
+        <is>
+          <t>+1 866 242 9853 / sales@ispsupplies.com</t>
+        </is>
+      </c>
+      <c r="K395" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L395" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M395" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N395" s="3" t="inlineStr"/>
+      <c r="O395" s="3" t="inlineStr"/>
+      <c r="P395" s="3" t="inlineStr"/>
+      <c r="Q395" s="3" t="inlineStr">
+        <is>
+          <t>Ottawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="3" t="inlineStr">
+        <is>
+          <t>Mahkesis Group Inc.</t>
+        </is>
+      </c>
+      <c r="B396" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C396" s="3" t="inlineStr">
+        <is>
+          <t>Manitoba</t>
+        </is>
+      </c>
+      <c r="D396" s="3" t="inlineStr">
+        <is>
+          <t>shop.mahkesis.com</t>
+        </is>
+      </c>
+      <c r="E396" s="3" t="inlineStr">
+        <is>
+          <t>分销（MikroTik 官方）</t>
+        </is>
+      </c>
+      <c r="F396" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik（Reseller）</t>
+        </is>
+      </c>
+      <c r="G396" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H396" s="3" t="inlineStr">
+        <is>
+          <t>卖 MikroTik 但缺工业/ERPS/PoE++ → 用同价位工业线补他的产品缺口</t>
+        </is>
+      </c>
+      <c r="I396" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J396" s="3" t="inlineStr">
+        <is>
+          <t>+1 204 949 4012 / admin@mahkesis.com</t>
+        </is>
+      </c>
+      <c r="K396" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L396" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M396" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N396" s="3" t="inlineStr"/>
+      <c r="O396" s="3" t="inlineStr"/>
+      <c r="P396" s="3" t="inlineStr"/>
+      <c r="Q396" s="3" t="inlineStr">
+        <is>
+          <t>Winnipeg</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
HMS N-Tron/Red Lion channel: UK, Ireland, Canada, NL, DE, SE, BE (+30)
Mines the HMS Networks partner directory filtered to the N-Tron and Red
Lion brands, the industrial Ethernet switch line and therefore the
closest match to the SmartByte industrial range. The angle is a second
source rather than a MikroTik-style gap: N-Tron list prices run several
times the SmartByte equivalent at the same port count.
Franklin Empire (5 Canadian branches) and EB Horsman (3) are stored as
one account each since the directory lists branches separately.
OEM Automatic AB is flagged as the strongest OEM candidate in the batch.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q396"/>
+  <dimension ref="A1:Q426"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -39159,6 +39159,2220 @@
       <c r="Q396" s="3" t="inlineStr">
         <is>
           <t>Winnipeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="3" t="inlineStr">
+        <is>
+          <t>AA Jones Electric Ltd</t>
+        </is>
+      </c>
+      <c r="B397" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C397" s="3" t="inlineStr">
+        <is>
+          <t>Hull / East Yorkshire</t>
+        </is>
+      </c>
+      <c r="D397" s="3" t="inlineStr">
+        <is>
+          <t>aajones.co.uk</t>
+        </is>
+      </c>
+      <c r="E397" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F397" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ixxat</t>
+        </is>
+      </c>
+      <c r="G397" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H397" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I397" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G / LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J397" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K397" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L397" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M397" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N397" s="3" t="inlineStr"/>
+      <c r="O397" s="3" t="inlineStr"/>
+      <c r="P397" s="3" t="inlineStr"/>
+      <c r="Q397" s="3" t="inlineStr">
+        <is>
+          <t>Hull 工业电气分销，有售前+售后支持</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="3" t="inlineStr">
+        <is>
+          <t>Control Technologies UK Ltd</t>
+        </is>
+      </c>
+      <c r="B398" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C398" s="3" t="inlineStr">
+        <is>
+          <t>Sharnbrook</t>
+        </is>
+      </c>
+      <c r="D398" s="3" t="inlineStr">
+        <is>
+          <t>controltech.uk.com</t>
+        </is>
+      </c>
+      <c r="E398" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F398" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G398" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H398" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I398" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J398" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K398" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L398" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M398" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N398" s="3" t="inlineStr"/>
+      <c r="O398" s="3" t="inlineStr"/>
+      <c r="P398" s="3" t="inlineStr"/>
+      <c r="Q398" s="3" t="inlineStr">
+        <is>
+          <t>同时覆盖爱尔兰</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="3" t="inlineStr">
+        <is>
+          <t>Digital Controls</t>
+        </is>
+      </c>
+      <c r="B399" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C399" s="3" t="inlineStr">
+        <is>
+          <t>Peterborough</t>
+        </is>
+      </c>
+      <c r="D399" s="3" t="inlineStr">
+        <is>
+          <t>digitalcontrols.biz</t>
+        </is>
+      </c>
+      <c r="E399" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F399" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G399" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H399" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I399" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J399" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K399" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L399" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M399" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N399" s="3" t="inlineStr"/>
+      <c r="O399" s="3" t="inlineStr"/>
+      <c r="P399" s="3" t="inlineStr"/>
+      <c r="Q399" s="3" t="inlineStr"/>
+    </row>
+    <row r="400">
+      <c r="A400" s="3" t="inlineStr">
+        <is>
+          <t>IVORY EGG (UK) LIMITED</t>
+        </is>
+      </c>
+      <c r="B400" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C400" s="3" t="inlineStr">
+        <is>
+          <t>Nottingham</t>
+        </is>
+      </c>
+      <c r="D400" s="3" t="inlineStr">
+        <is>
+          <t>ivoryegg.co.uk</t>
+        </is>
+      </c>
+      <c r="E400" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F400" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G400" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H400" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I400" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J400" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K400" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L400" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M400" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N400" s="3" t="inlineStr"/>
+      <c r="O400" s="3" t="inlineStr"/>
+      <c r="P400" s="3" t="inlineStr"/>
+      <c r="Q400" s="3" t="inlineStr"/>
+    </row>
+    <row r="401">
+      <c r="A401" s="3" t="inlineStr">
+        <is>
+          <t>LC Automation Ltd</t>
+        </is>
+      </c>
+      <c r="B401" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C401" s="3" t="inlineStr">
+        <is>
+          <t>Blackburn</t>
+        </is>
+      </c>
+      <c r="D401" s="3" t="inlineStr">
+        <is>
+          <t>lcautomation.com</t>
+        </is>
+      </c>
+      <c r="E401" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F401" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G401" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H401" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I401" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J401" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K401" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L401" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M401" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N401" s="3" t="inlineStr"/>
+      <c r="O401" s="3" t="inlineStr"/>
+      <c r="P401" s="3" t="inlineStr"/>
+      <c r="Q401" s="3" t="inlineStr">
+        <is>
+          <t>官网有 HMS 供应商专页 → 主力线</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="3" t="inlineStr">
+        <is>
+          <t>MAC Solutions UK Ltd</t>
+        </is>
+      </c>
+      <c r="B402" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C402" s="3" t="inlineStr">
+        <is>
+          <t>Redditch</t>
+        </is>
+      </c>
+      <c r="D402" s="3" t="inlineStr">
+        <is>
+          <t>mac-solutions.net</t>
+        </is>
+      </c>
+      <c r="E402" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F402" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G402" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H402" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I402" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J402" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K402" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L402" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M402" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N402" s="3" t="inlineStr"/>
+      <c r="O402" s="3" t="inlineStr"/>
+      <c r="P402" s="3" t="inlineStr"/>
+      <c r="Q402" s="3" t="inlineStr"/>
+    </row>
+    <row r="403">
+      <c r="A403" s="3" t="inlineStr">
+        <is>
+          <t>MCC Controls Ltd T/A PES Ireland</t>
+        </is>
+      </c>
+      <c r="B403" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C403" s="3" t="inlineStr">
+        <is>
+          <t>Dublin（爱尔兰）</t>
+        </is>
+      </c>
+      <c r="D403" s="3" t="inlineStr">
+        <is>
+          <t>parkelect.com</t>
+        </is>
+      </c>
+      <c r="E403" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F403" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon + Intesis</t>
+        </is>
+      </c>
+      <c r="G403" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H403" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I403" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J403" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K403" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L403" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M403" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N403" s="3" t="inlineStr"/>
+      <c r="O403" s="3" t="inlineStr"/>
+      <c r="P403" s="3" t="inlineStr"/>
+      <c r="Q403" s="3" t="inlineStr">
+        <is>
+          <t>Park Electrical 集团爱尔兰分部</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="3" t="inlineStr">
+        <is>
+          <t>Park Electrical Services</t>
+        </is>
+      </c>
+      <c r="B404" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C404" s="3" t="inlineStr">
+        <is>
+          <t>Belfast（北爱）</t>
+        </is>
+      </c>
+      <c r="D404" s="3" t="inlineStr">
+        <is>
+          <t>parkelect.co.uk</t>
+        </is>
+      </c>
+      <c r="E404" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F404" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon + Ixxat</t>
+        </is>
+      </c>
+      <c r="G404" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H404" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I404" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J404" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K404" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L404" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M404" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N404" s="3" t="inlineStr"/>
+      <c r="O404" s="3" t="inlineStr"/>
+      <c r="P404" s="3" t="inlineStr"/>
+      <c r="Q404" s="3" t="inlineStr">
+        <is>
+          <t>Park Electrical 集团总部</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="3" t="inlineStr">
+        <is>
+          <t>Parmley Graham Ltd</t>
+        </is>
+      </c>
+      <c r="B405" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C405" s="3" t="inlineStr">
+        <is>
+          <t>Gateshead</t>
+        </is>
+      </c>
+      <c r="D405" s="3" t="inlineStr">
+        <is>
+          <t>parmley-graham.co.uk</t>
+        </is>
+      </c>
+      <c r="E405" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F405" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G405" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H405" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I405" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J405" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K405" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L405" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M405" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N405" s="3" t="inlineStr"/>
+      <c r="O405" s="3" t="inlineStr"/>
+      <c r="P405" s="3" t="inlineStr"/>
+      <c r="Q405" s="3" t="inlineStr">
+        <is>
+          <t>英国老牌工业自动化分销</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="3" t="inlineStr">
+        <is>
+          <t>Routeco Limited</t>
+        </is>
+      </c>
+      <c r="B406" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C406" s="3" t="inlineStr">
+        <is>
+          <t>Milton Keynes</t>
+        </is>
+      </c>
+      <c r="D406" s="3" t="inlineStr">
+        <is>
+          <t>routeco.com</t>
+        </is>
+      </c>
+      <c r="E406" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F406" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon + Ixxat</t>
+        </is>
+      </c>
+      <c r="G406" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H406" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I406" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J406" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K406" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L406" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M406" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N406" s="3" t="inlineStr"/>
+      <c r="O406" s="3" t="inlineStr"/>
+      <c r="P406" s="3" t="inlineStr"/>
+      <c r="Q406" s="3" t="inlineStr">
+        <is>
+          <t>英国工业自动化大分销</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="3" t="inlineStr">
+        <is>
+          <t>Diamond Technologies Inc</t>
+        </is>
+      </c>
+      <c r="B407" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C407" s="3" t="inlineStr">
+        <is>
+          <t>Hudson, MA（美国总部）</t>
+        </is>
+      </c>
+      <c r="D407" s="3" t="inlineStr">
+        <is>
+          <t>diamondt.com</t>
+        </is>
+      </c>
+      <c r="E407" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F407" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G407" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H407" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I407" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J407" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K407" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L407" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M407" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N407" s="3" t="inlineStr"/>
+      <c r="O407" s="3" t="inlineStr"/>
+      <c r="P407" s="3" t="inlineStr"/>
+      <c r="Q407" s="3" t="inlineStr">
+        <is>
+          <t>英美两地，覆盖美国 9 个州</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="3" t="inlineStr">
+        <is>
+          <t>Consyst Limited</t>
+        </is>
+      </c>
+      <c r="B408" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C408" s="3" t="inlineStr">
+        <is>
+          <t>London / Edgware</t>
+        </is>
+      </c>
+      <c r="D408" s="3" t="inlineStr">
+        <is>
+          <t>consyst-int.com</t>
+        </is>
+      </c>
+      <c r="E408" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F408" s="3" t="inlineStr">
+        <is>
+          <t>Ixxat + 其他</t>
+        </is>
+      </c>
+      <c r="G408" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H408" s="3" t="inlineStr">
+        <is>
+          <t>HMS 渠道工业自动化分销，做 Intesis/Ewon 楼宇与远程运维 → 项目里需要交换机，做配套增量</t>
+        </is>
+      </c>
+      <c r="I408" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J408" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K408" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L408" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M408" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N408" s="3" t="inlineStr"/>
+      <c r="O408" s="3" t="inlineStr"/>
+      <c r="P408" s="3" t="inlineStr"/>
+      <c r="Q408" s="3" t="inlineStr">
+        <is>
+          <t>CAN/工业总线方向</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="3" t="inlineStr">
+        <is>
+          <t>Automation24 GmbH</t>
+        </is>
+      </c>
+      <c r="B409" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C409" s="3" t="inlineStr">
+        <is>
+          <t>Essen</t>
+        </is>
+      </c>
+      <c r="D409" s="3" t="inlineStr">
+        <is>
+          <t>automation24.de</t>
+        </is>
+      </c>
+      <c r="E409" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F409" s="3" t="inlineStr">
+        <is>
+          <t>Intesis（覆盖 10 国）</t>
+        </is>
+      </c>
+      <c r="G409" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H409" s="3" t="inlineStr">
+        <is>
+          <t>HMS 渠道工业自动化分销，做 Intesis/Ewon 楼宇与远程运维 → 项目里需要交换机，做配套增量</t>
+        </is>
+      </c>
+      <c r="I409" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J409" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K409" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L409" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M409" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N409" s="3" t="inlineStr"/>
+      <c r="O409" s="3" t="inlineStr"/>
+      <c r="P409" s="3" t="inlineStr"/>
+      <c r="Q409" s="3" t="inlineStr">
+        <is>
+          <t>德/奥/比/法/意/荷/波/西/瑞/英 10 国电商渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="3" t="inlineStr">
+        <is>
+          <t>Distec Ltd</t>
+        </is>
+      </c>
+      <c r="B410" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C410" s="3" t="inlineStr">
+        <is>
+          <t>Manchester</t>
+        </is>
+      </c>
+      <c r="D410" s="3" t="inlineStr">
+        <is>
+          <t>distec.co.uk</t>
+        </is>
+      </c>
+      <c r="E410" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F410" s="3" t="inlineStr">
+        <is>
+          <t>Ewon + Intesis</t>
+        </is>
+      </c>
+      <c r="G410" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H410" s="3" t="inlineStr">
+        <is>
+          <t>HMS 渠道工业自动化分销，做 Intesis/Ewon 楼宇与远程运维 → 项目里需要交换机，做配套增量</t>
+        </is>
+      </c>
+      <c r="I410" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J410" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K410" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L410" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M410" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N410" s="3" t="inlineStr"/>
+      <c r="O410" s="3" t="inlineStr"/>
+      <c r="P410" s="3" t="inlineStr"/>
+      <c r="Q410" s="3" t="inlineStr"/>
+    </row>
+    <row r="411">
+      <c r="A411" s="3" t="inlineStr">
+        <is>
+          <t>Clanrye Electrical Supplies Ltd</t>
+        </is>
+      </c>
+      <c r="B411" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C411" s="3" t="inlineStr">
+        <is>
+          <t>Newry（北爱）</t>
+        </is>
+      </c>
+      <c r="D411" s="3" t="inlineStr">
+        <is>
+          <t>knxireland.com</t>
+        </is>
+      </c>
+      <c r="E411" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F411" s="3" t="inlineStr">
+        <is>
+          <t>Intesis</t>
+        </is>
+      </c>
+      <c r="G411" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H411" s="3" t="inlineStr">
+        <is>
+          <t>HMS 渠道工业自动化分销，做 Intesis/Ewon 楼宇与远程运维 → 项目里需要交换机，做配套增量</t>
+        </is>
+      </c>
+      <c r="I411" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J411" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K411" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L411" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M411" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N411" s="3" t="inlineStr"/>
+      <c r="O411" s="3" t="inlineStr"/>
+      <c r="P411" s="3" t="inlineStr"/>
+      <c r="Q411" s="3" t="inlineStr">
+        <is>
+          <t>KNX 楼宇方向</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="3" t="inlineStr">
+        <is>
+          <t>Future Focus Energy Ltd</t>
+        </is>
+      </c>
+      <c r="B412" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C412" s="3" t="inlineStr">
+        <is>
+          <t>Blackpool</t>
+        </is>
+      </c>
+      <c r="D412" s="3" t="inlineStr">
+        <is>
+          <t>futurefocusenergy.co.uk</t>
+        </is>
+      </c>
+      <c r="E412" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F412" s="3" t="inlineStr">
+        <is>
+          <t>Intesis</t>
+        </is>
+      </c>
+      <c r="G412" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H412" s="3" t="inlineStr">
+        <is>
+          <t>HMS 渠道工业自动化分销，做 Intesis/Ewon 楼宇与远程运维 → 项目里需要交换机，做配套增量</t>
+        </is>
+      </c>
+      <c r="I412" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J412" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K412" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L412" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M412" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N412" s="3" t="inlineStr"/>
+      <c r="O412" s="3" t="inlineStr"/>
+      <c r="P412" s="3" t="inlineStr"/>
+      <c r="Q412" s="3" t="inlineStr"/>
+    </row>
+    <row r="413">
+      <c r="A413" s="3" t="inlineStr">
+        <is>
+          <t>ATC Automation（L.E.D. Lighting &amp; Electrical Distribution）</t>
+        </is>
+      </c>
+      <c r="B413" s="3" t="inlineStr">
+        <is>
+          <t>爱尔兰</t>
+        </is>
+      </c>
+      <c r="C413" s="3" t="inlineStr">
+        <is>
+          <t>Dublin 12</t>
+        </is>
+      </c>
+      <c r="D413" s="3" t="inlineStr">
+        <is>
+          <t>atcautomation.ie</t>
+        </is>
+      </c>
+      <c r="E413" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F413" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G413" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H413" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I413" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J413" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K413" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L413" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M413" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N413" s="3" t="inlineStr"/>
+      <c r="O413" s="3" t="inlineStr"/>
+      <c r="P413" s="3" t="inlineStr"/>
+      <c r="Q413" s="3" t="inlineStr">
+        <is>
+          <t>英爱两地</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="3" t="inlineStr">
+        <is>
+          <t>RS Components GmbH</t>
+        </is>
+      </c>
+      <c r="B414" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C414" s="3" t="inlineStr">
+        <is>
+          <t>Frankfurt am Main</t>
+        </is>
+      </c>
+      <c r="D414" s="3" t="inlineStr">
+        <is>
+          <t>rs-online.com</t>
+        </is>
+      </c>
+      <c r="E414" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F414" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion（覆盖 60+ 国）</t>
+        </is>
+      </c>
+      <c r="G414" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H414" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I414" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J414" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K414" s="3" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="L414" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M414" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N414" s="3" t="inlineStr"/>
+      <c r="O414" s="3" t="inlineStr"/>
+      <c r="P414" s="3" t="inlineStr"/>
+      <c r="Q414" s="3" t="inlineStr">
+        <is>
+          <t>目录巨头，只做线上寄售，不宜主攻</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="3" t="inlineStr">
+        <is>
+          <t>Franklin Empire</t>
+        </is>
+      </c>
+      <c r="B415" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C415" s="3" t="inlineStr">
+        <is>
+          <t>Saint-Laurent QC（另 Sherbrooke/Toronto/Newmarket/Scarborough）</t>
+        </is>
+      </c>
+      <c r="D415" s="3" t="inlineStr">
+        <is>
+          <t>franklinempire.com</t>
+        </is>
+      </c>
+      <c r="E415" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F415" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus</t>
+        </is>
+      </c>
+      <c r="G415" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H415" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I415" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G / LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J415" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K415" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L415" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M415" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N415" s="3" t="inlineStr"/>
+      <c r="O415" s="3" t="inlineStr"/>
+      <c r="P415" s="3" t="inlineStr"/>
+      <c r="Q415" s="3" t="inlineStr">
+        <is>
+          <t>5 个仓库覆盖 ON/QC/AB/MB/SK</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="3" t="inlineStr">
+        <is>
+          <t>EB Horsman &amp; Son</t>
+        </is>
+      </c>
+      <c r="B416" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C416" s="3" t="inlineStr">
+        <is>
+          <t>Surrey BC（另 Calgary / Edmonton AB）</t>
+        </is>
+      </c>
+      <c r="D416" s="3" t="inlineStr">
+        <is>
+          <t>ebhorsman.com</t>
+        </is>
+      </c>
+      <c r="E416" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F416" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G416" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H416" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I416" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J416" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K416" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L416" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M416" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N416" s="3" t="inlineStr"/>
+      <c r="O416" s="3" t="inlineStr"/>
+      <c r="P416" s="3" t="inlineStr"/>
+      <c r="Q416" s="3" t="inlineStr">
+        <is>
+          <t>加拿大西部电气分销，3 家分公司</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="3" t="inlineStr">
+        <is>
+          <t>Graybar Canada</t>
+        </is>
+      </c>
+      <c r="B417" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C417" s="3" t="inlineStr">
+        <is>
+          <t>Dartmouth NS</t>
+        </is>
+      </c>
+      <c r="D417" s="3" t="inlineStr">
+        <is>
+          <t>graybarcanada.com</t>
+        </is>
+      </c>
+      <c r="E417" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F417" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon + Intesis</t>
+        </is>
+      </c>
+      <c r="G417" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H417" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I417" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J417" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K417" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L417" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M417" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N417" s="3" t="inlineStr"/>
+      <c r="O417" s="3" t="inlineStr"/>
+      <c r="P417" s="3" t="inlineStr"/>
+      <c r="Q417" s="3" t="inlineStr">
+        <is>
+          <t>Graybar 集团，北美最大电气分销之一</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="3" t="inlineStr">
+        <is>
+          <t>Industrial Solutions Inc</t>
+        </is>
+      </c>
+      <c r="B418" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C418" s="3" t="inlineStr">
+        <is>
+          <t>Sherwood Park AB</t>
+        </is>
+      </c>
+      <c r="D418" s="3" t="inlineStr">
+        <is>
+          <t>indsol.com</t>
+        </is>
+      </c>
+      <c r="E418" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F418" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G418" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H418" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I418" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J418" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K418" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L418" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M418" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N418" s="3" t="inlineStr"/>
+      <c r="O418" s="3" t="inlineStr"/>
+      <c r="P418" s="3" t="inlineStr"/>
+      <c r="Q418" s="3" t="inlineStr">
+        <is>
+          <t>阿尔伯塔工业自动化</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="3" t="inlineStr">
+        <is>
+          <t>Cesco Electrical Supply Ltd</t>
+        </is>
+      </c>
+      <c r="B419" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C419" s="3" t="inlineStr">
+        <is>
+          <t>Port Coquitlam BC</t>
+        </is>
+      </c>
+      <c r="D419" s="3" t="inlineStr">
+        <is>
+          <t>cescoelectrical.com</t>
+        </is>
+      </c>
+      <c r="E419" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F419" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G419" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H419" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I419" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J419" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K419" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L419" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M419" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N419" s="3" t="inlineStr"/>
+      <c r="O419" s="3" t="inlineStr"/>
+      <c r="P419" s="3" t="inlineStr"/>
+      <c r="Q419" s="3" t="inlineStr"/>
+    </row>
+    <row r="420">
+      <c r="A420" s="3" t="inlineStr">
+        <is>
+          <t>OEM Automatic AB</t>
+        </is>
+      </c>
+      <c r="B420" s="3" t="inlineStr">
+        <is>
+          <t>瑞典</t>
+        </is>
+      </c>
+      <c r="C420" s="3" t="inlineStr">
+        <is>
+          <t>Tranås</t>
+        </is>
+      </c>
+      <c r="D420" s="3" t="inlineStr">
+        <is>
+          <t>oemautomatic.se</t>
+        </is>
+      </c>
+      <c r="E420" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F420" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G420" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H420" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍；北欧工业零部件大分销、自有品牌 → OEM 最优先</t>
+        </is>
+      </c>
+      <c r="I420" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J420" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K420" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L420" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M420" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N420" s="3" t="inlineStr"/>
+      <c r="O420" s="3" t="inlineStr"/>
+      <c r="P420" s="3" t="inlineStr"/>
+      <c r="Q420" s="3" t="inlineStr">
+        <is>
+          <t>本批 OEM 第一优先</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="3" t="inlineStr">
+        <is>
+          <t>EG Electronics AB</t>
+        </is>
+      </c>
+      <c r="B421" s="3" t="inlineStr">
+        <is>
+          <t>瑞典</t>
+        </is>
+      </c>
+      <c r="C421" s="3" t="inlineStr">
+        <is>
+          <t>Spånga (Stockholm)</t>
+        </is>
+      </c>
+      <c r="D421" s="3" t="inlineStr">
+        <is>
+          <t>egelectronics.com</t>
+        </is>
+      </c>
+      <c r="E421" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F421" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus</t>
+        </is>
+      </c>
+      <c r="G421" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H421" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I421" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J421" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K421" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L421" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M421" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N421" s="3" t="inlineStr"/>
+      <c r="O421" s="3" t="inlineStr"/>
+      <c r="P421" s="3" t="inlineStr"/>
+      <c r="Q421" s="3" t="inlineStr"/>
+    </row>
+    <row r="422">
+      <c r="A422" s="3" t="inlineStr">
+        <is>
+          <t>ATEG Automation GmbH</t>
+        </is>
+      </c>
+      <c r="B422" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C422" s="3" t="inlineStr">
+        <is>
+          <t>Remscheid</t>
+        </is>
+      </c>
+      <c r="D422" s="3" t="inlineStr">
+        <is>
+          <t>ateg.de</t>
+        </is>
+      </c>
+      <c r="E422" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F422" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G422" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H422" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I422" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J422" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K422" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L422" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M422" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N422" s="3" t="inlineStr"/>
+      <c r="O422" s="3" t="inlineStr"/>
+      <c r="P422" s="3" t="inlineStr"/>
+      <c r="Q422" s="3" t="inlineStr"/>
+    </row>
+    <row r="423">
+      <c r="A423" s="3" t="inlineStr">
+        <is>
+          <t>PRIMATION Systemtechnik GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B423" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C423" s="3" t="inlineStr">
+        <is>
+          <t>Grasbrunn (München)</t>
+        </is>
+      </c>
+      <c r="D423" s="3" t="inlineStr">
+        <is>
+          <t>primation.de</t>
+        </is>
+      </c>
+      <c r="E423" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F423" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon + Ixxat</t>
+        </is>
+      </c>
+      <c r="G423" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H423" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I423" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J423" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K423" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L423" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M423" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N423" s="3" t="inlineStr"/>
+      <c r="O423" s="3" t="inlineStr"/>
+      <c r="P423" s="3" t="inlineStr"/>
+      <c r="Q423" s="3" t="inlineStr">
+        <is>
+          <t>HMS 全品牌 → 技术能力强</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="3" t="inlineStr">
+        <is>
+          <t>Computer Products Professional Benelux B.V.</t>
+        </is>
+      </c>
+      <c r="B424" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C424" s="3" t="inlineStr">
+        <is>
+          <t>Puttershoek（比荷卢）</t>
+        </is>
+      </c>
+      <c r="D424" s="3" t="inlineStr">
+        <is>
+          <t>cppb.nl</t>
+        </is>
+      </c>
+      <c r="E424" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F424" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon + Ixxat + Intesis</t>
+        </is>
+      </c>
+      <c r="G424" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H424" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I424" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J424" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K424" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L424" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M424" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N424" s="3" t="inlineStr"/>
+      <c r="O424" s="3" t="inlineStr"/>
+      <c r="P424" s="3" t="inlineStr"/>
+      <c r="Q424" s="3" t="inlineStr">
+        <is>
+          <t>HMS 全品牌 → 比荷卢主力代理</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="3" t="inlineStr">
+        <is>
+          <t>CimPro Holding NV</t>
+        </is>
+      </c>
+      <c r="B425" s="3" t="inlineStr">
+        <is>
+          <t>比利时</t>
+        </is>
+      </c>
+      <c r="C425" s="3" t="inlineStr">
+        <is>
+          <t>Sint Niklaas（覆盖荷）</t>
+        </is>
+      </c>
+      <c r="D425" s="3" t="inlineStr"/>
+      <c r="E425" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F425" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus</t>
+        </is>
+      </c>
+      <c r="G425" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H425" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I425" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J425" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K425" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L425" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M425" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N425" s="3" t="inlineStr"/>
+      <c r="O425" s="3" t="inlineStr"/>
+      <c r="P425" s="3" t="inlineStr"/>
+      <c r="Q425" s="3" t="inlineStr">
+        <is>
+          <t>无公开网址，需 LinkedIn 找人</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="3" t="inlineStr">
+        <is>
+          <t>Digi-Key Corporation</t>
+        </is>
+      </c>
+      <c r="B426" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C426" s="3" t="inlineStr">
+        <is>
+          <t>Thief River Falls, MN</t>
+        </is>
+      </c>
+      <c r="D426" s="3" t="inlineStr">
+        <is>
+          <t>digikey.com</t>
+        </is>
+      </c>
+      <c r="E426" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F426" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G426" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H426" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商/替换，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I426" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J426" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K426" s="3" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="L426" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M426" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N426" s="3" t="inlineStr"/>
+      <c r="O426" s="3" t="inlineStr"/>
+      <c r="P426" s="3" t="inlineStr"/>
+      <c r="Q426" s="3" t="inlineStr">
+        <is>
+          <t>全球目录分销，可谈线上寄售，不宜主攻</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
HMS Europe batch 2: FR, ES, IT, NO, PL, PT, RO, GR, HU, CZ, AT, FI, IE, SI (+21)
Completes the western, southern and central European N-Tron channel.
Proelektronika in Zagreb alone covers eight Balkan countries and is the
single best entry point for that region. OEM Automatic now appears in
three countries (SE, PL, CZ) under one group, so one negotiation covers
all three. Balkan coverage is largely handled by Proelektronika and
RBT Technologies rather than by separate national distributors.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q426"/>
+  <dimension ref="A1:Q444"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -41373,6 +41373,1336 @@
       <c r="Q426" s="3" t="inlineStr">
         <is>
           <t>全球目录分销，可谈线上寄售，不宜主攻</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="3" t="inlineStr">
+        <is>
+          <t>Audin</t>
+        </is>
+      </c>
+      <c r="B427" s="3" t="inlineStr">
+        <is>
+          <t>法国</t>
+        </is>
+      </c>
+      <c r="C427" s="3" t="inlineStr">
+        <is>
+          <t>St Brice Courcelles (Reims)</t>
+        </is>
+      </c>
+      <c r="D427" s="3" t="inlineStr">
+        <is>
+          <t>shop-audin.fr</t>
+        </is>
+      </c>
+      <c r="E427" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F427" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G427" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H427" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I427" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J427" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K427" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L427" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M427" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N427" s="3" t="inlineStr"/>
+      <c r="O427" s="3" t="inlineStr"/>
+      <c r="P427" s="3" t="inlineStr"/>
+      <c r="Q427" s="3" t="inlineStr">
+        <is>
+          <t>自有电商站 shop-audin.fr，可谈线上</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="3" t="inlineStr">
+        <is>
+          <t>Cir Toulouse</t>
+        </is>
+      </c>
+      <c r="B428" s="3" t="inlineStr">
+        <is>
+          <t>法国</t>
+        </is>
+      </c>
+      <c r="C428" s="3" t="inlineStr">
+        <is>
+          <t>Toulouse</t>
+        </is>
+      </c>
+      <c r="D428" s="3" t="inlineStr">
+        <is>
+          <t>cir.fr</t>
+        </is>
+      </c>
+      <c r="E428" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F428" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G428" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H428" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I428" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J428" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K428" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L428" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M428" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N428" s="3" t="inlineStr"/>
+      <c r="O428" s="3" t="inlineStr"/>
+      <c r="P428" s="3" t="inlineStr"/>
+      <c r="Q428" s="3" t="inlineStr">
+        <is>
+          <t>法国南部工业分销</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="3" t="inlineStr">
+        <is>
+          <t>FGET International</t>
+        </is>
+      </c>
+      <c r="B429" s="3" t="inlineStr">
+        <is>
+          <t>法国</t>
+        </is>
+      </c>
+      <c r="C429" s="3" t="inlineStr">
+        <is>
+          <t>Genas (Lyon)</t>
+        </is>
+      </c>
+      <c r="D429" s="3" t="inlineStr">
+        <is>
+          <t>fget.fr</t>
+        </is>
+      </c>
+      <c r="E429" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F429" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G429" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H429" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I429" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J429" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K429" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L429" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M429" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N429" s="3" t="inlineStr"/>
+      <c r="O429" s="3" t="inlineStr"/>
+      <c r="P429" s="3" t="inlineStr"/>
+      <c r="Q429" s="3" t="inlineStr"/>
+    </row>
+    <row r="430">
+      <c r="A430" s="3" t="inlineStr">
+        <is>
+          <t>HD Technology</t>
+        </is>
+      </c>
+      <c r="B430" s="3" t="inlineStr">
+        <is>
+          <t>法国</t>
+        </is>
+      </c>
+      <c r="C430" s="3" t="inlineStr">
+        <is>
+          <t>Bron (Lyon)</t>
+        </is>
+      </c>
+      <c r="D430" s="3" t="inlineStr">
+        <is>
+          <t>hdtechnology.com</t>
+        </is>
+      </c>
+      <c r="E430" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F430" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G430" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H430" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I430" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J430" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K430" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L430" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M430" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N430" s="3" t="inlineStr"/>
+      <c r="O430" s="3" t="inlineStr"/>
+      <c r="P430" s="3" t="inlineStr"/>
+      <c r="Q430" s="3" t="inlineStr"/>
+    </row>
+    <row r="431">
+      <c r="A431" s="3" t="inlineStr">
+        <is>
+          <t>QL3D</t>
+        </is>
+      </c>
+      <c r="B431" s="3" t="inlineStr">
+        <is>
+          <t>法国</t>
+        </is>
+      </c>
+      <c r="C431" s="3" t="inlineStr">
+        <is>
+          <t>Bazainville (Yvelines)</t>
+        </is>
+      </c>
+      <c r="D431" s="3" t="inlineStr">
+        <is>
+          <t>ql3d.fr</t>
+        </is>
+      </c>
+      <c r="E431" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F431" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon + Ixxat</t>
+        </is>
+      </c>
+      <c r="G431" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H431" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I431" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J431" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K431" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L431" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M431" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N431" s="3" t="inlineStr"/>
+      <c r="O431" s="3" t="inlineStr"/>
+      <c r="P431" s="3" t="inlineStr"/>
+      <c r="Q431" s="3" t="inlineStr">
+        <is>
+          <t>HMS 全品牌</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="3" t="inlineStr">
+        <is>
+          <t>Garma Electronica</t>
+        </is>
+      </c>
+      <c r="B432" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C432" s="3" t="inlineStr">
+        <is>
+          <t>San Sebastián</t>
+        </is>
+      </c>
+      <c r="D432" s="3" t="inlineStr">
+        <is>
+          <t>garmasl.com</t>
+        </is>
+      </c>
+      <c r="E432" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F432" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G432" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H432" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I432" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J432" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K432" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L432" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M432" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N432" s="3" t="inlineStr"/>
+      <c r="O432" s="3" t="inlineStr"/>
+      <c r="P432" s="3" t="inlineStr"/>
+      <c r="Q432" s="3" t="inlineStr">
+        <is>
+          <t>西班牙北部</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="3" t="inlineStr">
+        <is>
+          <t>Leadernet Sistemas Telec</t>
+        </is>
+      </c>
+      <c r="B433" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C433" s="3" t="inlineStr">
+        <is>
+          <t>Oricáin (Navarra)</t>
+        </is>
+      </c>
+      <c r="D433" s="3" t="inlineStr">
+        <is>
+          <t>leadernet.es</t>
+        </is>
+      </c>
+      <c r="E433" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F433" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G433" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H433" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I433" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J433" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K433" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L433" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M433" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N433" s="3" t="inlineStr"/>
+      <c r="O433" s="3" t="inlineStr"/>
+      <c r="P433" s="3" t="inlineStr"/>
+      <c r="Q433" s="3" t="inlineStr"/>
+    </row>
+    <row r="434">
+      <c r="A434" s="3" t="inlineStr">
+        <is>
+          <t>Efa Automazione S.p.A.</t>
+        </is>
+      </c>
+      <c r="B434" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C434" s="3" t="inlineStr">
+        <is>
+          <t>Cernusco Sul Naviglio (MI)</t>
+        </is>
+      </c>
+      <c r="D434" s="3" t="inlineStr">
+        <is>
+          <t>efa.it</t>
+        </is>
+      </c>
+      <c r="E434" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F434" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G434" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H434" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I434" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J434" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K434" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L434" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M434" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N434" s="3" t="inlineStr"/>
+      <c r="O434" s="3" t="inlineStr"/>
+      <c r="P434" s="3" t="inlineStr"/>
+      <c r="Q434" s="3" t="inlineStr">
+        <is>
+          <t>米兰工业区</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="3" t="inlineStr">
+        <is>
+          <t>Autic System AS</t>
+        </is>
+      </c>
+      <c r="B435" s="3" t="inlineStr">
+        <is>
+          <t>挪威</t>
+        </is>
+      </c>
+      <c r="C435" s="3" t="inlineStr">
+        <is>
+          <t>Tønsberg</t>
+        </is>
+      </c>
+      <c r="D435" s="3" t="inlineStr">
+        <is>
+          <t>autic.no</t>
+        </is>
+      </c>
+      <c r="E435" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F435" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G435" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H435" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I435" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J435" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K435" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L435" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M435" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N435" s="3" t="inlineStr"/>
+      <c r="O435" s="3" t="inlineStr"/>
+      <c r="P435" s="3" t="inlineStr"/>
+      <c r="Q435" s="3" t="inlineStr">
+        <is>
+          <t>挪威 N-Tron 主力</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="3" t="inlineStr">
+        <is>
+          <t>F.Fonseca S.A</t>
+        </is>
+      </c>
+      <c r="B436" s="3" t="inlineStr">
+        <is>
+          <t>葡萄牙</t>
+        </is>
+      </c>
+      <c r="C436" s="3" t="inlineStr">
+        <is>
+          <t>Aveiro</t>
+        </is>
+      </c>
+      <c r="D436" s="3" t="inlineStr">
+        <is>
+          <t>ffonseca.com</t>
+        </is>
+      </c>
+      <c r="E436" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F436" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G436" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H436" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I436" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J436" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K436" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L436" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M436" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N436" s="3" t="inlineStr"/>
+      <c r="O436" s="3" t="inlineStr"/>
+      <c r="P436" s="3" t="inlineStr"/>
+      <c r="Q436" s="3" t="inlineStr">
+        <is>
+          <t>葡萄牙工业自动化老牌分销</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="3" t="inlineStr">
+        <is>
+          <t>Eltrec Power Srl</t>
+        </is>
+      </c>
+      <c r="B437" s="3" t="inlineStr">
+        <is>
+          <t>罗马尼亚</t>
+        </is>
+      </c>
+      <c r="C437" s="3" t="inlineStr">
+        <is>
+          <t>Bucharest（覆盖摩尔多瓦）</t>
+        </is>
+      </c>
+      <c r="D437" s="3" t="inlineStr">
+        <is>
+          <t>eltrec.ro</t>
+        </is>
+      </c>
+      <c r="E437" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F437" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon + Ixxat + Intesis</t>
+        </is>
+      </c>
+      <c r="G437" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H437" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I437" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J437" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K437" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L437" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M437" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N437" s="3" t="inlineStr"/>
+      <c r="O437" s="3" t="inlineStr"/>
+      <c r="P437" s="3" t="inlineStr"/>
+      <c r="Q437" s="3" t="inlineStr">
+        <is>
+          <t>HMS 全品牌 → 罗马尼亚+摩尔多瓦</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="3" t="inlineStr">
+        <is>
+          <t>Alpha Motion S.A.</t>
+        </is>
+      </c>
+      <c r="B438" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C438" s="3" t="inlineStr">
+        <is>
+          <t>Pikermi (Attica)</t>
+        </is>
+      </c>
+      <c r="D438" s="3" t="inlineStr">
+        <is>
+          <t>alpha-motion.gr</t>
+        </is>
+      </c>
+      <c r="E438" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F438" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G438" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H438" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I438" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J438" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K438" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L438" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M438" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N438" s="3" t="inlineStr"/>
+      <c r="O438" s="3" t="inlineStr"/>
+      <c r="P438" s="3" t="inlineStr"/>
+      <c r="Q438" s="3" t="inlineStr"/>
+    </row>
+    <row r="439">
+      <c r="A439" s="3" t="inlineStr">
+        <is>
+          <t>Controsys Control Engineering Ltd.</t>
+        </is>
+      </c>
+      <c r="B439" s="3" t="inlineStr">
+        <is>
+          <t>匈牙利</t>
+        </is>
+      </c>
+      <c r="C439" s="3" t="inlineStr">
+        <is>
+          <t>Budapest</t>
+        </is>
+      </c>
+      <c r="D439" s="3" t="inlineStr">
+        <is>
+          <t>controsys.hu</t>
+        </is>
+      </c>
+      <c r="E439" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F439" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G439" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H439" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I439" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J439" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K439" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L439" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M439" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N439" s="3" t="inlineStr"/>
+      <c r="O439" s="3" t="inlineStr"/>
+      <c r="P439" s="3" t="inlineStr"/>
+      <c r="Q439" s="3" t="inlineStr"/>
+    </row>
+    <row r="440">
+      <c r="A440" s="3" t="inlineStr">
+        <is>
+          <t>OEM Automatic spol. s r.o.</t>
+        </is>
+      </c>
+      <c r="B440" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C440" s="3" t="inlineStr">
+        <is>
+          <t>Zdiby (Praha)</t>
+        </is>
+      </c>
+      <c r="D440" s="3" t="inlineStr">
+        <is>
+          <t>oemautomatic.cz</t>
+        </is>
+      </c>
+      <c r="E440" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F440" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G440" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H440" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍；OEM Automatic 集团捷克分公司 → 一次谈 SE/PL/CZ 三国</t>
+        </is>
+      </c>
+      <c r="I440" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J440" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K440" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L440" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M440" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N440" s="3" t="inlineStr"/>
+      <c r="O440" s="3" t="inlineStr"/>
+      <c r="P440" s="3" t="inlineStr"/>
+      <c r="Q440" s="3" t="inlineStr">
+        <is>
+          <t>与瑞典 OEM Automatic AB 同集团</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="3" t="inlineStr">
+        <is>
+          <t>Sarlin Oy Ab</t>
+        </is>
+      </c>
+      <c r="B441" s="3" t="inlineStr">
+        <is>
+          <t>芬兰</t>
+        </is>
+      </c>
+      <c r="C441" s="3" t="inlineStr">
+        <is>
+          <t>Vantaa (Helsinki)</t>
+        </is>
+      </c>
+      <c r="D441" s="3" t="inlineStr">
+        <is>
+          <t>sarlin.com</t>
+        </is>
+      </c>
+      <c r="E441" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F441" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G441" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H441" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I441" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J441" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K441" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L441" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M441" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N441" s="3" t="inlineStr"/>
+      <c r="O441" s="3" t="inlineStr"/>
+      <c r="P441" s="3" t="inlineStr"/>
+      <c r="Q441" s="3" t="inlineStr">
+        <is>
+          <t>芬兰工业分销</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="3" t="inlineStr">
+        <is>
+          <t>Profibus Ireland Ltd</t>
+        </is>
+      </c>
+      <c r="B442" s="3" t="inlineStr">
+        <is>
+          <t>爱尔兰</t>
+        </is>
+      </c>
+      <c r="C442" s="3" t="inlineStr">
+        <is>
+          <t>Limerick</t>
+        </is>
+      </c>
+      <c r="D442" s="3" t="inlineStr">
+        <is>
+          <t>profibus.ie</t>
+        </is>
+      </c>
+      <c r="E442" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F442" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon + Ixxat + Intesis</t>
+        </is>
+      </c>
+      <c r="G442" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H442" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I442" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J442" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K442" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L442" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M442" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N442" s="3" t="inlineStr"/>
+      <c r="O442" s="3" t="inlineStr"/>
+      <c r="P442" s="3" t="inlineStr"/>
+      <c r="Q442" s="3" t="inlineStr">
+        <is>
+          <t>HMS 全品牌 → 爱尔兰现场总线专业户</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="3" t="inlineStr">
+        <is>
+          <t>RBT Technologies d.o.o.</t>
+        </is>
+      </c>
+      <c r="B443" s="3" t="inlineStr">
+        <is>
+          <t>斯洛文尼亚</t>
+        </is>
+      </c>
+      <c r="C443" s="3" t="inlineStr">
+        <is>
+          <t>Ljubljana</t>
+        </is>
+      </c>
+      <c r="D443" s="3" t="inlineStr">
+        <is>
+          <t>rbt-technologies.si</t>
+        </is>
+      </c>
+      <c r="E443" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F443" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon + Ixxat</t>
+        </is>
+      </c>
+      <c r="G443" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H443" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I443" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J443" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K443" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L443" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M443" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N443" s="3" t="inlineStr"/>
+      <c r="O443" s="3" t="inlineStr"/>
+      <c r="P443" s="3" t="inlineStr"/>
+      <c r="Q443" s="3" t="inlineStr">
+        <is>
+          <t>覆盖斯洛文尼亚+阿尔巴尼亚+波黑+科索沃+北马其顿+黑山 6 国</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="3" t="inlineStr">
+        <is>
+          <t>Proelektronika</t>
+        </is>
+      </c>
+      <c r="B444" s="3" t="inlineStr">
+        <is>
+          <t>克罗地亚</t>
+        </is>
+      </c>
+      <c r="C444" s="3" t="inlineStr">
+        <is>
+          <t>Zagreb</t>
+        </is>
+      </c>
+      <c r="D444" s="3" t="inlineStr">
+        <is>
+          <t>proelektronika.hr</t>
+        </is>
+      </c>
+      <c r="E444" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F444" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G444" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H444" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I444" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J444" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K444" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L444" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M444" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N444" s="3" t="inlineStr"/>
+      <c r="O444" s="3" t="inlineStr"/>
+      <c r="P444" s="3" t="inlineStr"/>
+      <c r="Q444" s="3" t="inlineStr">
+        <is>
+          <t>★ 一家覆盖 8 国：克/塞/黑山/波黑/阿尔巴尼亚/科索沃/北马其顿/斯洛文尼亚 → 巴尔干最优入口</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Finish HMS Europe: Balkans, Nordics, Israel, Baltics (+6)
Closes out the European N-Tron channel. The Balkans turn out to have
only six partners in total, with Proelektronika and RBT Technologies
covering most countries between them rather than national distributors.
Denmark, Iceland, Bulgaria and Israel each have exactly one local
distributor outside the RS catalogue, which makes them uncontested.
Estonia, Latvia, Lithuania, Slovakia, Switzerland, Turkey and Cyprus
have no local N-Tron partner at all and are served only by RS.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q444"/>
+  <dimension ref="A1:Q448"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -16245,7 +16245,7 @@
       <c r="P73" s="3" t="inlineStr"/>
       <c r="Q73" s="3" t="inlineStr">
         <is>
-          <t>华沙，自动化目录分销，SKU 量大</t>
+          <t>华沙，自动化目录分销，SKU 量大；OEM Automatic 集团：瑞典 oemautomatic.se（自有品牌，OEM 优先）+ 捷克 oemautomatic.cz，一单谈三国</t>
         </is>
       </c>
     </row>
@@ -40934,7 +40934,7 @@
       <c r="P420" s="3" t="inlineStr"/>
       <c r="Q420" s="3" t="inlineStr">
         <is>
-          <t>本批 OEM 第一优先</t>
+          <t>波兰分公司已在名单第73行，有真实联系人：+48 22 863 27 22 / info@oemautomatic.pl（Antaira 授权）→ 从华沙打进去一次覆盖 SE/PL/CZ</t>
         </is>
       </c>
     </row>
@@ -42402,7 +42402,7 @@
       <c r="P440" s="3" t="inlineStr"/>
       <c r="Q440" s="3" t="inlineStr">
         <is>
-          <t>与瑞典 OEM Automatic AB 同集团</t>
+          <t>波兰分公司已在名单第73行，有真实联系人：+48 22 863 27 22 / info@oemautomatic.pl（Antaira 授权）→ 从华沙打进去一次覆盖 SE/PL/CZ</t>
         </is>
       </c>
     </row>
@@ -42627,7 +42627,7 @@
       <c r="P443" s="3" t="inlineStr"/>
       <c r="Q443" s="3" t="inlineStr">
         <is>
-          <t>覆盖斯洛文尼亚+阿尔巴尼亚+波黑+科索沃+北马其顿+黑山 6 国</t>
+          <t>RBT 集团总部（斯洛文尼亚）；另有塞尔维亚 rbt-technologies.rs、克罗地亚 rbt-technologies.hr → 一单覆盖 SI/HR/RS 三国，且都覆盖阿尔巴尼亚/波黑/科索沃/北马其顿/黑山</t>
         </is>
       </c>
     </row>
@@ -42702,7 +42702,307 @@
       <c r="P444" s="3" t="inlineStr"/>
       <c r="Q444" s="3" t="inlineStr">
         <is>
-          <t>★ 一家覆盖 8 国：克/塞/黑山/波黑/阿尔巴尼亚/科索沃/北马其顿/斯洛文尼亚 → 巴尔干最优入口</t>
+          <t>★ 巴尔干最优入口：一家覆盖 8 国（克/塞/黑山/波黑/阿尔巴尼亚/科索沃/北马其顿/斯洛文尼亚）；HMS 全品牌授权</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="3" t="inlineStr">
+        <is>
+          <t>Comicon Ltd.</t>
+        </is>
+      </c>
+      <c r="B445" s="3" t="inlineStr">
+        <is>
+          <t>保加利亚</t>
+        </is>
+      </c>
+      <c r="C445" s="3" t="inlineStr">
+        <is>
+          <t>Sofia</t>
+        </is>
+      </c>
+      <c r="D445" s="3" t="inlineStr">
+        <is>
+          <t>comicon.bg</t>
+        </is>
+      </c>
+      <c r="E445" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F445" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G445" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H445" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I445" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J445" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K445" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L445" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M445" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N445" s="3" t="inlineStr"/>
+      <c r="O445" s="3" t="inlineStr"/>
+      <c r="P445" s="3" t="inlineStr"/>
+      <c r="Q445" s="3" t="inlineStr">
+        <is>
+          <t>保加利亚唯一本地 N-Tron 代理（除 RS）</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="3" t="inlineStr">
+        <is>
+          <t>Bross Engineering Aps</t>
+        </is>
+      </c>
+      <c r="B446" s="3" t="inlineStr">
+        <is>
+          <t>丹麦</t>
+        </is>
+      </c>
+      <c r="C446" s="3" t="inlineStr">
+        <is>
+          <t>Ballerup (København)</t>
+        </is>
+      </c>
+      <c r="D446" s="3" t="inlineStr">
+        <is>
+          <t>bross.dk</t>
+        </is>
+      </c>
+      <c r="E446" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F446" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon + Ixxat</t>
+        </is>
+      </c>
+      <c r="G446" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H446" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I446" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J446" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K446" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L446" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M446" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N446" s="3" t="inlineStr"/>
+      <c r="O446" s="3" t="inlineStr"/>
+      <c r="P446" s="3" t="inlineStr"/>
+      <c r="Q446" s="3" t="inlineStr">
+        <is>
+          <t>丹麦唯一本地 N-Tron 代理（除 RS）</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="3" t="inlineStr">
+        <is>
+          <t>Fálkinn Ísmar ehf.</t>
+        </is>
+      </c>
+      <c r="B447" s="3" t="inlineStr">
+        <is>
+          <t>冰岛</t>
+        </is>
+      </c>
+      <c r="C447" s="3" t="inlineStr">
+        <is>
+          <t>Kopavogur</t>
+        </is>
+      </c>
+      <c r="D447" s="3" t="inlineStr">
+        <is>
+          <t>falkinnismar.is</t>
+        </is>
+      </c>
+      <c r="E447" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F447" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G447" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H447" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I447" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J447" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K447" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L447" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M447" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N447" s="3" t="inlineStr"/>
+      <c r="O447" s="3" t="inlineStr"/>
+      <c r="P447" s="3" t="inlineStr"/>
+      <c r="Q447" s="3" t="inlineStr">
+        <is>
+          <t>冰岛唯一本地 N-Tron 代理（除 RS）→ 无竞争</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="3" t="inlineStr">
+        <is>
+          <t>Galoz Electronics Ltd</t>
+        </is>
+      </c>
+      <c r="B448" s="3" t="inlineStr">
+        <is>
+          <t>以色列</t>
+        </is>
+      </c>
+      <c r="C448" s="3" t="inlineStr">
+        <is>
+          <t>Rosh Ha Ayin</t>
+        </is>
+      </c>
+      <c r="D448" s="3" t="inlineStr">
+        <is>
+          <t>galoz.co.il</t>
+        </is>
+      </c>
+      <c r="E448" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F448" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon + Ixxat</t>
+        </is>
+      </c>
+      <c r="G448" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H448" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I448" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J448" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K448" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L448" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M448" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N448" s="3" t="inlineStr"/>
+      <c r="O448" s="3" t="inlineStr"/>
+      <c r="P448" s="3" t="inlineStr"/>
+      <c r="Q448" s="3" t="inlineStr">
+        <is>
+          <t>以色列 N-Tron 主力</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add the Serbian and Croatian RBT Technologies branches
Both were dropped in the previous commit because the dedupe key strips
non-ASCII characters, so the parenthesised country suffix collapsed all
three RBT entities onto one name. Renaming with the local-language
country word keeps them distinct.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q448"/>
+  <dimension ref="A1:Q450"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -43003,6 +43003,156 @@
       <c r="Q448" s="3" t="inlineStr">
         <is>
           <t>以色列 N-Tron 主力</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="3" t="inlineStr">
+        <is>
+          <t>RBT Technologies Srbija d.o.o.</t>
+        </is>
+      </c>
+      <c r="B449" s="3" t="inlineStr">
+        <is>
+          <t>塞尔维亚</t>
+        </is>
+      </c>
+      <c r="C449" s="3" t="inlineStr">
+        <is>
+          <t>Zemun / Beograd</t>
+        </is>
+      </c>
+      <c r="D449" s="3" t="inlineStr">
+        <is>
+          <t>rbt-technologies.rs</t>
+        </is>
+      </c>
+      <c r="E449" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F449" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon + Ixxat + Intesis</t>
+        </is>
+      </c>
+      <c r="G449" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H449" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I449" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J449" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K449" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L449" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M449" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N449" s="3" t="inlineStr"/>
+      <c r="O449" s="3" t="inlineStr"/>
+      <c r="P449" s="3" t="inlineStr"/>
+      <c r="Q449" s="3" t="inlineStr">
+        <is>
+          <t>RBT 集团塞尔维亚分部；集团另有斯洛文尼亚 rbt-technologies.si、克罗地亚 rbt-technologies.hr → 一单覆盖 SI/HR/RS</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="3" t="inlineStr">
+        <is>
+          <t>RBT Technologies Hrvatska d.o.o.</t>
+        </is>
+      </c>
+      <c r="B450" s="3" t="inlineStr">
+        <is>
+          <t>克罗地亚</t>
+        </is>
+      </c>
+      <c r="C450" s="3" t="inlineStr">
+        <is>
+          <t>Zagreb</t>
+        </is>
+      </c>
+      <c r="D450" s="3" t="inlineStr">
+        <is>
+          <t>rbt-technologies.hr</t>
+        </is>
+      </c>
+      <c r="E450" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F450" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon + Ixxat</t>
+        </is>
+      </c>
+      <c r="G450" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H450" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口非网管约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I450" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J450" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K450" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L450" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M450" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N450" s="3" t="inlineStr"/>
+      <c r="O450" s="3" t="inlineStr"/>
+      <c r="P450" s="3" t="inlineStr"/>
+      <c r="Q450" s="3" t="inlineStr">
+        <is>
+          <t>RBT 集团克罗地亚分部；集团另有斯洛文尼亚 rbt-technologies.si、塞尔维亚 rbt-technologies.rs → 一单覆盖 SI/HR/RS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
HMS USA page 1 of 8: 12 accounts from 20 directory entries
Opens the US N-Tron channel. Branch listings run about half the
directory, so 20 entries collapse to 12 companies: AWC alone has seven
branches across the south and CBT Company three in Ohio. Every US row
carries the TAA caveat since China-origin gear cannot serve government
or utility projects.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q450"/>
+  <dimension ref="A1:Q462"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -43153,6 +43153,898 @@
       <c r="Q450" s="3" t="inlineStr">
         <is>
           <t>RBT 集团克罗地亚分部；集团另有斯洛文尼亚 rbt-technologies.si、塞尔维亚 rbt-technologies.rs → 一单覆盖 SI/HR/RS</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="3" t="inlineStr">
+        <is>
+          <t>A A Electric</t>
+        </is>
+      </c>
+      <c r="B451" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C451" s="3" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="D451" s="3" t="inlineStr">
+        <is>
+          <t>a-aelectric.com</t>
+        </is>
+      </c>
+      <c r="E451" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F451" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G451" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H451" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I451" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J451" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K451" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L451" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M451" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N451" s="3" t="inlineStr"/>
+      <c r="O451" s="3" t="inlineStr"/>
+      <c r="P451" s="3" t="inlineStr"/>
+      <c r="Q451" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 40+ 州的全国电气分销；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="3" t="inlineStr">
+        <is>
+          <t>ACD（Automation Components Distributor）</t>
+        </is>
+      </c>
+      <c r="B452" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C452" s="3" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="D452" s="3" t="inlineStr">
+        <is>
+          <t>acdist.com</t>
+        </is>
+      </c>
+      <c r="E452" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F452" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G452" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H452" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I452" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J452" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K452" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L452" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M452" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N452" s="3" t="inlineStr"/>
+      <c r="O452" s="3" t="inlineStr"/>
+      <c r="P452" s="3" t="inlineStr"/>
+      <c r="Q452" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 40+ 州；有售前+售后支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="3" t="inlineStr">
+        <is>
+          <t>Adcon Engineering（ACD/Adcon）</t>
+        </is>
+      </c>
+      <c r="B453" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C453" s="3" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="D453" s="3" t="inlineStr">
+        <is>
+          <t>adconengineering.com</t>
+        </is>
+      </c>
+      <c r="E453" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F453" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Ewon</t>
+        </is>
+      </c>
+      <c r="G453" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H453" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I453" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J453" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K453" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L453" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M453" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N453" s="3" t="inlineStr"/>
+      <c r="O453" s="3" t="inlineStr"/>
+      <c r="P453" s="3" t="inlineStr"/>
+      <c r="Q453" s="3" t="inlineStr">
+        <is>
+          <t>只覆盖俄亥俄州；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="3" t="inlineStr">
+        <is>
+          <t>Agilix Solutions LLC</t>
+        </is>
+      </c>
+      <c r="B454" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C454" s="3" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="D454" s="3" t="inlineStr"/>
+      <c r="E454" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F454" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G454" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H454" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I454" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J454" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K454" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L454" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M454" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N454" s="3" t="inlineStr"/>
+      <c r="O454" s="3" t="inlineStr"/>
+      <c r="P454" s="3" t="inlineStr"/>
+      <c r="Q454" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 KS/MO；无公开网址，需 LinkedIn 找人；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="3" t="inlineStr">
+        <is>
+          <t>Applied Automation Controls Inc</t>
+        </is>
+      </c>
+      <c r="B455" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C455" s="3" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="D455" s="3" t="inlineStr">
+        <is>
+          <t>appliedautomation.com</t>
+        </is>
+      </c>
+      <c r="E455" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F455" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G455" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H455" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I455" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J455" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K455" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L455" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M455" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N455" s="3" t="inlineStr"/>
+      <c r="O455" s="3" t="inlineStr"/>
+      <c r="P455" s="3" t="inlineStr"/>
+      <c r="Q455" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 40+ 州；有售前+售后支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="3" t="inlineStr">
+        <is>
+          <t>Applied Industrial Controls</t>
+        </is>
+      </c>
+      <c r="B456" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C456" s="3" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="D456" s="3" t="inlineStr">
+        <is>
+          <t>aic-controls.com</t>
+        </is>
+      </c>
+      <c r="E456" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F456" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G456" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H456" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I456" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J456" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K456" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L456" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M456" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N456" s="3" t="inlineStr"/>
+      <c r="O456" s="3" t="inlineStr"/>
+      <c r="P456" s="3" t="inlineStr"/>
+      <c r="Q456" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 40+ 州；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="3" t="inlineStr">
+        <is>
+          <t>AWC, Inc.</t>
+        </is>
+      </c>
+      <c r="B457" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C457" s="3" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="D457" s="3" t="inlineStr">
+        <is>
+          <t>awc-inc.com</t>
+        </is>
+      </c>
+      <c r="E457" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F457" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G457" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H457" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I457" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J457" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K457" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L457" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M457" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N457" s="3" t="inlineStr"/>
+      <c r="O457" s="3" t="inlineStr"/>
+      <c r="P457" s="3" t="inlineStr"/>
+      <c r="Q457" s="3" t="inlineStr">
+        <is>
+          <t>★ 7 个分部：LA Baton Rouge / GA Conyers / FL Jacksonville / FL Tampa / TX Houston / OK OKC / AL Mobile → 美国南部最大工业分销之一；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="3" t="inlineStr">
+        <is>
+          <t>B&amp;K Electric Wholesale Co</t>
+        </is>
+      </c>
+      <c r="B458" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C458" s="3" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="D458" s="3" t="inlineStr">
+        <is>
+          <t>bk-electric.com</t>
+        </is>
+      </c>
+      <c r="E458" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F458" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G458" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H458" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I458" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J458" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K458" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L458" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M458" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N458" s="3" t="inlineStr"/>
+      <c r="O458" s="3" t="inlineStr"/>
+      <c r="P458" s="3" t="inlineStr"/>
+      <c r="Q458" s="3" t="inlineStr">
+        <is>
+          <t>加州；有售前+售后支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="3" t="inlineStr">
+        <is>
+          <t>Branom Instrument Co</t>
+        </is>
+      </c>
+      <c r="B459" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C459" s="3" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="D459" s="3" t="inlineStr">
+        <is>
+          <t>branom.com</t>
+        </is>
+      </c>
+      <c r="E459" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F459" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G459" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H459" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I459" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J459" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K459" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L459" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M459" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N459" s="3" t="inlineStr"/>
+      <c r="O459" s="3" t="inlineStr"/>
+      <c r="P459" s="3" t="inlineStr"/>
+      <c r="Q459" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 AK/ID/OR/WA 西北四州；仪表+自动化；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="3" t="inlineStr">
+        <is>
+          <t>Brenner Industrial Sales and Supply</t>
+        </is>
+      </c>
+      <c r="B460" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C460" s="3" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="D460" s="3" t="inlineStr">
+        <is>
+          <t>brenner-industrial.com</t>
+        </is>
+      </c>
+      <c r="E460" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F460" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G460" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H460" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I460" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J460" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K460" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L460" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M460" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N460" s="3" t="inlineStr"/>
+      <c r="O460" s="3" t="inlineStr"/>
+      <c r="P460" s="3" t="inlineStr"/>
+      <c r="Q460" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 OH/PA；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="3" t="inlineStr">
+        <is>
+          <t>C&amp;E Advanced Technologies</t>
+        </is>
+      </c>
+      <c r="B461" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C461" s="3" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="D461" s="3" t="inlineStr"/>
+      <c r="E461" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F461" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G461" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H461" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I461" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J461" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K461" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L461" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M461" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N461" s="3" t="inlineStr"/>
+      <c r="O461" s="3" t="inlineStr"/>
+      <c r="P461" s="3" t="inlineStr"/>
+      <c r="Q461" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 IN/OH/TN；无公开网址；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="3" t="inlineStr">
+        <is>
+          <t>CBT Company</t>
+        </is>
+      </c>
+      <c r="B462" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C462" s="3" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="D462" s="3" t="inlineStr">
+        <is>
+          <t>cbtcompany.com</t>
+        </is>
+      </c>
+      <c r="E462" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F462" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G462" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H462" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I462" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J462" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K462" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L462" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M462" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N462" s="3" t="inlineStr"/>
+      <c r="O462" s="3" t="inlineStr"/>
+      <c r="P462" s="3" t="inlineStr"/>
+      <c r="Q462" s="3" t="inlineStr">
+        <is>
+          <t>俄亥俄 3 个点，动力传动+自动化分销；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
HMS USA page 2 of 8: 4 accounts, mostly multi-branch groups
Crawford Electric (8 branches across the southeast) and Crescent
Electric Supply (9 across the midwest) are the finds here. Two separate
companies trade as Clayton Engineering under different domains, which
needs verifying before either is approached.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q462"/>
+  <dimension ref="A1:Q466"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -44045,6 +44045,306 @@
       <c r="Q462" s="3" t="inlineStr">
         <is>
           <t>俄亥俄 3 个点，动力传动+自动化分销；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="3" t="inlineStr">
+        <is>
+          <t>Clayton Engineering Company</t>
+        </is>
+      </c>
+      <c r="B463" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C463" s="3" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="D463" s="3" t="inlineStr">
+        <is>
+          <t>claytonengineering.com</t>
+        </is>
+      </c>
+      <c r="E463" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F463" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G463" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H463" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I463" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J463" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K463" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L463" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M463" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N463" s="3" t="inlineStr"/>
+      <c r="O463" s="3" t="inlineStr"/>
+      <c r="P463" s="3" t="inlineStr"/>
+      <c r="Q463" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 PA/OH/WV；有售前+售后支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="3" t="inlineStr">
+        <is>
+          <t>Clayton Engineering（Ohio）</t>
+        </is>
+      </c>
+      <c r="B464" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C464" s="3" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="D464" s="3" t="inlineStr">
+        <is>
+          <t>clayeng.net</t>
+        </is>
+      </c>
+      <c r="E464" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F464" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G464" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H464" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I464" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J464" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K464" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L464" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M464" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N464" s="3" t="inlineStr"/>
+      <c r="O464" s="3" t="inlineStr"/>
+      <c r="P464" s="3" t="inlineStr"/>
+      <c r="Q464" s="3" t="inlineStr">
+        <is>
+          <t>独立域名 clayeng.net，覆盖 40+ 州；与 PA 的 Clayton Engineering Company 同名不同站，需核实是否同集团；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="3" t="inlineStr">
+        <is>
+          <t>Crawford Electric Supply</t>
+        </is>
+      </c>
+      <c r="B465" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C465" s="3" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="D465" s="3" t="inlineStr">
+        <is>
+          <t>crawfordelectricsupply.com</t>
+        </is>
+      </c>
+      <c r="E465" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F465" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon + Intesis</t>
+        </is>
+      </c>
+      <c r="G465" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H465" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I465" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J465" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K465" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L465" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M465" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N465" s="3" t="inlineStr"/>
+      <c r="O465" s="3" t="inlineStr"/>
+      <c r="P465" s="3" t="inlineStr"/>
+      <c r="Q465" s="3" t="inlineStr">
+        <is>
+          <t>★ 8 个分部：MS Hattiesburg/Tupelo/Jackson、TN Cookeville/Jackson/La Vergne、FL Pensacola、AL Decatur → 美国东南部；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="3" t="inlineStr">
+        <is>
+          <t>Crescent Electric Supply</t>
+        </is>
+      </c>
+      <c r="B466" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C466" s="3" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="D466" s="3" t="inlineStr">
+        <is>
+          <t>crescentelectric.com</t>
+        </is>
+      </c>
+      <c r="E466" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F466" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G466" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H466" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I466" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J466" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K466" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L466" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M466" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N466" s="3" t="inlineStr"/>
+      <c r="O466" s="3" t="inlineStr"/>
+      <c r="P466" s="3" t="inlineStr"/>
+      <c r="Q466" s="3" t="inlineStr">
+        <is>
+          <t>★ 美国大型电气分销；9 个点：WI/OH Defiance·Perrysburg·Columbus·West Chester·Valley View/PA Warrendale/AZ Phoenix/IN Jeffersonville；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
HMS USA page 3 of 8: 12 accounts including Gexpro and Graybar Electric
Graybar Electric links to the Graybar Canada row already in the list,
and Kendall Electric turns out to sit under the CBT Company group since
its Montgomery branch carries that domain. Industrial Networking
Solutions is the closest name match in the whole directory.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q466"/>
+  <dimension ref="A1:Q478"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -44345,6 +44345,898 @@
       <c r="Q466" s="3" t="inlineStr">
         <is>
           <t>★ 美国大型电气分销；9 个点：WI/OH Defiance·Perrysburg·Columbus·West Chester·Valley View/PA Warrendale/AZ Phoenix/IN Jeffersonville；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="3" t="inlineStr">
+        <is>
+          <t>E &amp; M Electric</t>
+        </is>
+      </c>
+      <c r="B467" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C467" s="3" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="D467" s="3" t="inlineStr">
+        <is>
+          <t>eandm.com</t>
+        </is>
+      </c>
+      <c r="E467" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F467" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G467" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H467" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I467" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J467" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K467" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L467" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M467" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N467" s="3" t="inlineStr"/>
+      <c r="O467" s="3" t="inlineStr"/>
+      <c r="P467" s="3" t="inlineStr"/>
+      <c r="Q467" s="3" t="inlineStr">
+        <is>
+          <t>加州北部；有售前+售后支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="3" t="inlineStr">
+        <is>
+          <t>EESCO（Englewood Electric Supply）</t>
+        </is>
+      </c>
+      <c r="B468" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C468" s="3" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="D468" s="3" t="inlineStr">
+        <is>
+          <t>buy.eescodist.com</t>
+        </is>
+      </c>
+      <c r="E468" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F468" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G468" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H468" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I468" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J468" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K468" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L468" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M468" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N468" s="3" t="inlineStr"/>
+      <c r="O468" s="3" t="inlineStr"/>
+      <c r="P468" s="3" t="inlineStr"/>
+      <c r="Q468" s="3" t="inlineStr">
+        <is>
+          <t>★ 5 个分部：IL Woodridge / MN New Brighton / SC West Columbia·Florence / GA Augusta；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="3" t="inlineStr">
+        <is>
+          <t>Electric Motor Shop and Supply Co</t>
+        </is>
+      </c>
+      <c r="B469" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C469" s="3" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="D469" s="3" t="inlineStr">
+        <is>
+          <t>electricmotorshop.com</t>
+        </is>
+      </c>
+      <c r="E469" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F469" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G469" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H469" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I469" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J469" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K469" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L469" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M469" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N469" s="3" t="inlineStr"/>
+      <c r="O469" s="3" t="inlineStr"/>
+      <c r="P469" s="3" t="inlineStr"/>
+      <c r="Q469" s="3" t="inlineStr">
+        <is>
+          <t>加州中部；电机+自动化；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="3" t="inlineStr">
+        <is>
+          <t>Electric Supply &amp; Equipment</t>
+        </is>
+      </c>
+      <c r="B470" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C470" s="3" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="D470" s="3" t="inlineStr"/>
+      <c r="E470" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F470" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G470" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H470" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I470" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J470" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K470" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L470" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M470" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N470" s="3" t="inlineStr"/>
+      <c r="O470" s="3" t="inlineStr"/>
+      <c r="P470" s="3" t="inlineStr"/>
+      <c r="Q470" s="3" t="inlineStr">
+        <is>
+          <t>北卡；无公开网址；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="3" t="inlineStr">
+        <is>
+          <t>ErieTec, Inc</t>
+        </is>
+      </c>
+      <c r="B471" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C471" s="3" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="D471" s="3" t="inlineStr">
+        <is>
+          <t>erietecinc.com</t>
+        </is>
+      </c>
+      <c r="E471" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F471" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G471" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H471" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I471" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J471" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K471" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L471" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M471" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N471" s="3" t="inlineStr"/>
+      <c r="O471" s="3" t="inlineStr"/>
+      <c r="P471" s="3" t="inlineStr"/>
+      <c r="Q471" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 OH/PA；有售前+售后支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="3" t="inlineStr">
+        <is>
+          <t>Gexpro</t>
+        </is>
+      </c>
+      <c r="B472" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C472" s="3" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="D472" s="3" t="inlineStr">
+        <is>
+          <t>gexpro.com</t>
+        </is>
+      </c>
+      <c r="E472" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F472" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G472" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H472" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I472" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J472" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K472" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L472" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M472" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N472" s="3" t="inlineStr"/>
+      <c r="O472" s="3" t="inlineStr"/>
+      <c r="P472" s="3" t="inlineStr"/>
+      <c r="Q472" s="3" t="inlineStr">
+        <is>
+          <t>美国大型工业/电气分销（原 GE Supply）；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="3" t="inlineStr">
+        <is>
+          <t>Graybar Electric</t>
+        </is>
+      </c>
+      <c r="B473" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C473" s="3" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="D473" s="3" t="inlineStr">
+        <is>
+          <t>graybar.com</t>
+        </is>
+      </c>
+      <c r="E473" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F473" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G473" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H473" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I473" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J473" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K473" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L473" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M473" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N473" s="3" t="inlineStr"/>
+      <c r="O473" s="3" t="inlineStr"/>
+      <c r="P473" s="3" t="inlineStr"/>
+      <c r="Q473" s="3" t="inlineStr">
+        <is>
+          <t>★ 北美最大电气分销之一；与名单里的 Graybar Canada 同集团；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="3" t="inlineStr">
+        <is>
+          <t>Hannan Supply Company</t>
+        </is>
+      </c>
+      <c r="B474" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C474" s="3" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="D474" s="3" t="inlineStr">
+        <is>
+          <t>hannansupply.com</t>
+        </is>
+      </c>
+      <c r="E474" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F474" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon + Ixxat</t>
+        </is>
+      </c>
+      <c r="G474" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H474" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I474" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J474" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K474" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L474" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M474" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N474" s="3" t="inlineStr"/>
+      <c r="O474" s="3" t="inlineStr"/>
+      <c r="P474" s="3" t="inlineStr"/>
+      <c r="Q474" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 40+ 州；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="3" t="inlineStr">
+        <is>
+          <t>Industrial Electronic Supply</t>
+        </is>
+      </c>
+      <c r="B475" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C475" s="3" t="inlineStr">
+        <is>
+          <t>LA</t>
+        </is>
+      </c>
+      <c r="D475" s="3" t="inlineStr"/>
+      <c r="E475" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F475" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G475" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H475" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I475" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J475" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K475" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L475" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M475" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N475" s="3" t="inlineStr"/>
+      <c r="O475" s="3" t="inlineStr"/>
+      <c r="P475" s="3" t="inlineStr"/>
+      <c r="Q475" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 40+ 州；无公开网址；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="3" t="inlineStr">
+        <is>
+          <t>Industrial Networking Solutions</t>
+        </is>
+      </c>
+      <c r="B476" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C476" s="3" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="D476" s="3" t="inlineStr">
+        <is>
+          <t>industrialnetworking.com</t>
+        </is>
+      </c>
+      <c r="E476" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F476" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G476" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H476" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I476" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J476" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K476" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L476" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M476" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N476" s="3" t="inlineStr"/>
+      <c r="O476" s="3" t="inlineStr"/>
+      <c r="P476" s="3" t="inlineStr"/>
+      <c r="Q476" s="3" t="inlineStr">
+        <is>
+          <t>★ 公司名就是工业网络，最对口；覆盖 40+ 州；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="3" t="inlineStr">
+        <is>
+          <t>J A Shomer Company</t>
+        </is>
+      </c>
+      <c r="B477" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C477" s="3" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="D477" s="3" t="inlineStr">
+        <is>
+          <t>jashomer.com</t>
+        </is>
+      </c>
+      <c r="E477" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F477" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G477" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H477" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I477" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J477" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K477" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L477" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M477" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N477" s="3" t="inlineStr"/>
+      <c r="O477" s="3" t="inlineStr"/>
+      <c r="P477" s="3" t="inlineStr"/>
+      <c r="Q477" s="3" t="inlineStr">
+        <is>
+          <t>俄亥俄工业分销；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="3" t="inlineStr">
+        <is>
+          <t>Kendall Electric</t>
+        </is>
+      </c>
+      <c r="B478" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C478" s="3" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D478" s="3" t="inlineStr">
+        <is>
+          <t>kendallelectric.com</t>
+        </is>
+      </c>
+      <c r="E478" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F478" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G478" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H478" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I478" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J478" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K478" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L478" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M478" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N478" s="3" t="inlineStr"/>
+      <c r="O478" s="3" t="inlineStr"/>
+      <c r="P478" s="3" t="inlineStr"/>
+      <c r="Q478" s="3" t="inlineStr">
+        <is>
+          <t>与名单里的 CBT Company 同集团（Montgomery 分部挂 cbtcompany.com）；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
HMS USA page 4 of 8: Lakeland Engineering plus Kendall's full branch list
Nineteen of the twenty entries on this page are branches of Kendall
Electric and Lakeland Engineering, which is why it yields only one new
account. Kendall's branch count is corrected to seventeen.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q478"/>
+  <dimension ref="A1:Q479"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -45236,7 +45236,82 @@
       <c r="P478" s="3" t="inlineStr"/>
       <c r="Q478" s="3" t="inlineStr">
         <is>
-          <t>与名单里的 CBT Company 同集团（Montgomery 分部挂 cbtcompany.com）；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+          <t>★ 17 个分部（MI Traverse City/Benton Harbor/Wyoming/Lansing/Portage/Saginaw、IN Elkhart/Fort Wayne/Greensburg、AL Montgomery/Irondale、GA Tallapoosa、OH Sidney/Columbus、PA Conshohocken、TN Jackson/Chattanooga/Knoxville/Cleveland）；与 CBT Company 同集团；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="3" t="inlineStr">
+        <is>
+          <t>Lakeland Engineering</t>
+        </is>
+      </c>
+      <c r="B479" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C479" s="3" t="inlineStr">
+        <is>
+          <t>NE</t>
+        </is>
+      </c>
+      <c r="D479" s="3" t="inlineStr">
+        <is>
+          <t>lakelandengineering.com</t>
+        </is>
+      </c>
+      <c r="E479" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F479" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G479" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H479" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I479" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J479" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K479" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L479" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M479" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N479" s="3" t="inlineStr"/>
+      <c r="O479" s="3" t="inlineStr"/>
+      <c r="P479" s="3" t="inlineStr"/>
+      <c r="Q479" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 NE/MN/IA/KS；有售前+售后支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
HMS USA page 5 of 8: 11 accounts including Rexel USA
Rexel appears as nine branches under one domain. The rest are midwest
and southeast industrial automation distributors, most with both
pre-sales and after-sales support, which means they have the technical
staff to evaluate a second source on spec.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q479"/>
+  <dimension ref="A1:Q490"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -45312,6 +45312,827 @@
       <c r="Q479" s="3" t="inlineStr">
         <is>
           <t>覆盖 NE/MN/IA/KS；有售前+售后支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="3" t="inlineStr">
+        <is>
+          <t>Logic Inc</t>
+        </is>
+      </c>
+      <c r="B480" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C480" s="3" t="inlineStr">
+        <is>
+          <t>KS</t>
+        </is>
+      </c>
+      <c r="D480" s="3" t="inlineStr">
+        <is>
+          <t>logic-control.com</t>
+        </is>
+      </c>
+      <c r="E480" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F480" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G480" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H480" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I480" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J480" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K480" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L480" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M480" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N480" s="3" t="inlineStr"/>
+      <c r="O480" s="3" t="inlineStr"/>
+      <c r="P480" s="3" t="inlineStr"/>
+      <c r="Q480" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 KS/MO；有售前+售后支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="3" t="inlineStr">
+        <is>
+          <t>Power Drives</t>
+        </is>
+      </c>
+      <c r="B481" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C481" s="3" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="D481" s="3" t="inlineStr">
+        <is>
+          <t>power-drives.com</t>
+        </is>
+      </c>
+      <c r="E481" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F481" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G481" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H481" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I481" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J481" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K481" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L481" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M481" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N481" s="3" t="inlineStr"/>
+      <c r="O481" s="3" t="inlineStr"/>
+      <c r="P481" s="3" t="inlineStr"/>
+      <c r="Q481" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 40+ 州；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="3" t="inlineStr">
+        <is>
+          <t>Power Motion</t>
+        </is>
+      </c>
+      <c r="B482" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C482" s="3" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="D482" s="3" t="inlineStr">
+        <is>
+          <t>powermotionsales.com</t>
+        </is>
+      </c>
+      <c r="E482" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F482" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G482" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H482" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I482" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J482" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K482" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L482" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M482" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N482" s="3" t="inlineStr"/>
+      <c r="O482" s="3" t="inlineStr"/>
+      <c r="P482" s="3" t="inlineStr"/>
+      <c r="Q482" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 AR/IL/KS/MO；有售前+售后支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" s="3" t="inlineStr">
+        <is>
+          <t>Power Mation</t>
+        </is>
+      </c>
+      <c r="B483" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C483" s="3" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="D483" s="3" t="inlineStr">
+        <is>
+          <t>powermation.com</t>
+        </is>
+      </c>
+      <c r="E483" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F483" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G483" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H483" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I483" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J483" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K483" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L483" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M483" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N483" s="3" t="inlineStr"/>
+      <c r="O483" s="3" t="inlineStr"/>
+      <c r="P483" s="3" t="inlineStr"/>
+      <c r="Q483" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 IA/MN/WI；有售前+售后支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="3" t="inlineStr">
+        <is>
+          <t>Prime Industrial Components, Inc</t>
+        </is>
+      </c>
+      <c r="B484" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C484" s="3" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="D484" s="3" t="inlineStr">
+        <is>
+          <t>prime-industrial.com</t>
+        </is>
+      </c>
+      <c r="E484" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F484" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus</t>
+        </is>
+      </c>
+      <c r="G484" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H484" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I484" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J484" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K484" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L484" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M484" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N484" s="3" t="inlineStr"/>
+      <c r="O484" s="3" t="inlineStr"/>
+      <c r="P484" s="3" t="inlineStr"/>
+      <c r="Q484" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 40+ 州；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="3" t="inlineStr">
+        <is>
+          <t>Process Technology, Inc. (PTI)</t>
+        </is>
+      </c>
+      <c r="B485" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C485" s="3" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="D485" s="3" t="inlineStr">
+        <is>
+          <t>process-tech.com</t>
+        </is>
+      </c>
+      <c r="E485" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F485" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G485" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H485" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I485" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J485" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K485" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L485" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M485" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N485" s="3" t="inlineStr"/>
+      <c r="O485" s="3" t="inlineStr"/>
+      <c r="P485" s="3" t="inlineStr"/>
+      <c r="Q485" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 AZ/CO/ID/UT；有售前支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="3" t="inlineStr">
+        <is>
+          <t>PTS Precision Tools Service, Inc.</t>
+        </is>
+      </c>
+      <c r="B486" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C486" s="3" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D486" s="3" t="inlineStr">
+        <is>
+          <t>ptservice.com</t>
+        </is>
+      </c>
+      <c r="E486" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F486" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G486" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H486" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I486" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J486" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K486" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L486" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M486" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N486" s="3" t="inlineStr"/>
+      <c r="O486" s="3" t="inlineStr"/>
+      <c r="P486" s="3" t="inlineStr"/>
+      <c r="Q486" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 40+ 州；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="3" t="inlineStr">
+        <is>
+          <t>Purvis Industries LLC</t>
+        </is>
+      </c>
+      <c r="B487" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C487" s="3" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="D487" s="3" t="inlineStr"/>
+      <c r="E487" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F487" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G487" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H487" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I487" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J487" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K487" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L487" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M487" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N487" s="3" t="inlineStr"/>
+      <c r="O487" s="3" t="inlineStr"/>
+      <c r="P487" s="3" t="inlineStr"/>
+      <c r="Q487" s="3" t="inlineStr">
+        <is>
+          <t>密苏里；无公开网址；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="3" t="inlineStr">
+        <is>
+          <t>Queen City Supply Co.（MQ Automation 分部）</t>
+        </is>
+      </c>
+      <c r="B488" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C488" s="3" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="D488" s="3" t="inlineStr">
+        <is>
+          <t>mqautomation.com</t>
+        </is>
+      </c>
+      <c r="E488" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F488" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G488" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H488" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I488" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J488" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K488" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L488" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M488" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N488" s="3" t="inlineStr"/>
+      <c r="O488" s="3" t="inlineStr"/>
+      <c r="P488" s="3" t="inlineStr"/>
+      <c r="Q488" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 40+ 州；母公司 MQ Automation；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="3" t="inlineStr">
+        <is>
+          <t>Ramco Innovations</t>
+        </is>
+      </c>
+      <c r="B489" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C489" s="3" t="inlineStr">
+        <is>
+          <t>IA</t>
+        </is>
+      </c>
+      <c r="D489" s="3" t="inlineStr">
+        <is>
+          <t>ramcoi.com</t>
+        </is>
+      </c>
+      <c r="E489" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F489" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G489" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H489" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I489" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J489" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K489" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L489" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M489" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N489" s="3" t="inlineStr"/>
+      <c r="O489" s="3" t="inlineStr"/>
+      <c r="P489" s="3" t="inlineStr"/>
+      <c r="Q489" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 40+ 州；工业自动化专业分销；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="3" t="inlineStr">
+        <is>
+          <t>Rexel USA</t>
+        </is>
+      </c>
+      <c r="B490" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C490" s="3" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="D490" s="3" t="inlineStr">
+        <is>
+          <t>rexelusa.com</t>
+        </is>
+      </c>
+      <c r="E490" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F490" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G490" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H490" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I490" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J490" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K490" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L490" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M490" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N490" s="3" t="inlineStr"/>
+      <c r="O490" s="3" t="inlineStr"/>
+      <c r="P490" s="3" t="inlineStr"/>
+      <c r="Q490" s="3" t="inlineStr">
+        <is>
+          <t>★ 全球电气分销巨头；9 个点：TX Missouri City·Carrollton / FL Pinellas Park·Orlando·Ocala·Ft Lauderdale·Miami·Sarasota / OH Solon；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
HMS USA page 6 of 8: 4 accounts, Rexel branch count corrected to 18
Another nine Rexel branches push its total to eighteen, the largest
branch network in the US directory. Standard Electric Supply carries
all six HMS brands across seven midwest branches.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q490"/>
+  <dimension ref="A1:Q494"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -46132,7 +46132,303 @@
       <c r="P490" s="3" t="inlineStr"/>
       <c r="Q490" s="3" t="inlineStr">
         <is>
-          <t>★ 全球电气分销巨头；9 个点：TX Missouri City·Carrollton / FL Pinellas Park·Orlando·Ocala·Ft Lauderdale·Miami·Sarasota / OH Solon；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+          <t>★ 全球电气分销巨头；目录里 18 个分部：TX Missouri City·Carrollton / FL Pinellas Park·Orlando·Ocala·Ft Lauderdale·Miami·Sarasota·Tampa·Lakeland·Melbourne·Daytona Beach / OH Solon / CA Santa Clara / NC Hickory·Asheville / MD Sparks·Capitol Heights；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="3" t="inlineStr">
+        <is>
+          <t>RS Americas（RS Components 美国）</t>
+        </is>
+      </c>
+      <c r="B491" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C491" s="3" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="D491" s="3" t="inlineStr">
+        <is>
+          <t>us.rs-online.com</t>
+        </is>
+      </c>
+      <c r="E491" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F491" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G491" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H491" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I491" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J491" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K491" s="3" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="L491" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M491" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N491" s="3" t="inlineStr"/>
+      <c r="O491" s="3" t="inlineStr"/>
+      <c r="P491" s="3" t="inlineStr"/>
+      <c r="Q491" s="3" t="inlineStr">
+        <is>
+          <t>目录分销；与欧洲 RS Components 同集团，只谈线上寄售；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="3" t="inlineStr">
+        <is>
+          <t>Seltrol</t>
+        </is>
+      </c>
+      <c r="B492" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C492" s="3" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="D492" s="3" t="inlineStr"/>
+      <c r="E492" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F492" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G492" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H492" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I492" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J492" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K492" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L492" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M492" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N492" s="3" t="inlineStr"/>
+      <c r="O492" s="3" t="inlineStr"/>
+      <c r="P492" s="3" t="inlineStr"/>
+      <c r="Q492" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 40+ 州；无公开网址，需 LinkedIn 找人；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" s="3" t="inlineStr">
+        <is>
+          <t>Shingle &amp; Gibb</t>
+        </is>
+      </c>
+      <c r="B493" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C493" s="3" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="D493" s="3" t="inlineStr">
+        <is>
+          <t>shingle.com</t>
+        </is>
+      </c>
+      <c r="E493" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F493" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon + Intesis</t>
+        </is>
+      </c>
+      <c r="G493" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H493" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I493" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J493" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K493" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L493" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M493" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N493" s="3" t="inlineStr"/>
+      <c r="O493" s="3" t="inlineStr"/>
+      <c r="P493" s="3" t="inlineStr"/>
+      <c r="Q493" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 NJ/PA/FL；自动化分销；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="3" t="inlineStr">
+        <is>
+          <t>Standard Electric Supply</t>
+        </is>
+      </c>
+      <c r="B494" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C494" s="3" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="D494" s="3" t="inlineStr">
+        <is>
+          <t>standardelectricsupply.com</t>
+        </is>
+      </c>
+      <c r="E494" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F494" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon + Ixxat + Intesis</t>
+        </is>
+      </c>
+      <c r="G494" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H494" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I494" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J494" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K494" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L494" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M494" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N494" s="3" t="inlineStr"/>
+      <c r="O494" s="3" t="inlineStr"/>
+      <c r="P494" s="3" t="inlineStr"/>
+      <c r="Q494" s="3" t="inlineStr">
+        <is>
+          <t>★ 7 个分部：IL Tinley Park·Champaign / IN Indianapolis·Warsaw / WI Stevens Point·Verona·Sheboygan；HMS 全品牌；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
HMS USA page 7 of 8: 12 accounts including Wesco
Wesco is the second North American electrical distribution giant on the
list after Graybar. The page is otherwise midwest and mountain-state
industrial distributors, most with both pre-sales and after-sales
support.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q494"/>
+  <dimension ref="A1:Q506"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -46429,6 +46429,902 @@
       <c r="Q494" s="3" t="inlineStr">
         <is>
           <t>★ 7 个分部：IL Tinley Park·Champaign / IN Indianapolis·Warsaw / WI Stevens Point·Verona·Sheboygan；HMS 全品牌；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="3" t="inlineStr">
+        <is>
+          <t>Stoneway Electric Supply Co</t>
+        </is>
+      </c>
+      <c r="B495" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C495" s="3" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="D495" s="3" t="inlineStr">
+        <is>
+          <t>stoneway.com</t>
+        </is>
+      </c>
+      <c r="E495" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F495" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G495" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H495" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I495" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J495" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K495" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L495" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M495" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N495" s="3" t="inlineStr"/>
+      <c r="O495" s="3" t="inlineStr"/>
+      <c r="P495" s="3" t="inlineStr"/>
+      <c r="Q495" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 WA/ID；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="3" t="inlineStr">
+        <is>
+          <t>Sure Controls Inc</t>
+        </is>
+      </c>
+      <c r="B496" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C496" s="3" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="D496" s="3" t="inlineStr">
+        <is>
+          <t>surecontrols.com</t>
+        </is>
+      </c>
+      <c r="E496" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F496" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G496" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H496" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I496" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J496" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K496" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L496" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M496" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N496" s="3" t="inlineStr"/>
+      <c r="O496" s="3" t="inlineStr"/>
+      <c r="P496" s="3" t="inlineStr"/>
+      <c r="Q496" s="3" t="inlineStr">
+        <is>
+          <t>威斯康星；有售前+售后支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" s="3" t="inlineStr">
+        <is>
+          <t>TCIC（Total Control &amp; Instrumentation）</t>
+        </is>
+      </c>
+      <c r="B497" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C497" s="3" t="inlineStr">
+        <is>
+          <t>MN</t>
+        </is>
+      </c>
+      <c r="D497" s="3" t="inlineStr">
+        <is>
+          <t>tcicinc.com</t>
+        </is>
+      </c>
+      <c r="E497" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F497" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Anybus + Ewon + Ixxat</t>
+        </is>
+      </c>
+      <c r="G497" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H497" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I497" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J497" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K497" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L497" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M497" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N497" s="3" t="inlineStr"/>
+      <c r="O497" s="3" t="inlineStr"/>
+      <c r="P497" s="3" t="inlineStr"/>
+      <c r="Q497" s="3" t="inlineStr">
+        <is>
+          <t>明尼苏达；有售前+售后支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="3" t="inlineStr">
+        <is>
+          <t>The Reynolds Company</t>
+        </is>
+      </c>
+      <c r="B498" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C498" s="3" t="inlineStr">
+        <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="D498" s="3" t="inlineStr">
+        <is>
+          <t>reynoldsonline.com</t>
+        </is>
+      </c>
+      <c r="E498" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F498" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G498" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H498" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I498" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J498" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K498" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L498" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M498" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N498" s="3" t="inlineStr"/>
+      <c r="O498" s="3" t="inlineStr"/>
+      <c r="P498" s="3" t="inlineStr"/>
+      <c r="Q498" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 40+ 州；德州工业分销；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="3" t="inlineStr">
+        <is>
+          <t>Thorp Controls</t>
+        </is>
+      </c>
+      <c r="B499" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C499" s="3" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="D499" s="3" t="inlineStr">
+        <is>
+          <t>tcas.com</t>
+        </is>
+      </c>
+      <c r="E499" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F499" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G499" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H499" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I499" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J499" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K499" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L499" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M499" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N499" s="3" t="inlineStr"/>
+      <c r="O499" s="3" t="inlineStr"/>
+      <c r="P499" s="3" t="inlineStr"/>
+      <c r="Q499" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 CO/KS/MO；有售前+售后支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="3" t="inlineStr">
+        <is>
+          <t>TMMI, LLC</t>
+        </is>
+      </c>
+      <c r="B500" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C500" s="3" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="D500" s="3" t="inlineStr">
+        <is>
+          <t>tmmi.com</t>
+        </is>
+      </c>
+      <c r="E500" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F500" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G500" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H500" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I500" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J500" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K500" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L500" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M500" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N500" s="3" t="inlineStr"/>
+      <c r="O500" s="3" t="inlineStr"/>
+      <c r="P500" s="3" t="inlineStr"/>
+      <c r="Q500" s="3" t="inlineStr">
+        <is>
+          <t>科罗拉多；有售前+售后支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" s="3" t="inlineStr">
+        <is>
+          <t>Torpey Denver Inc</t>
+        </is>
+      </c>
+      <c r="B501" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C501" s="3" t="inlineStr">
+        <is>
+          <t>CO</t>
+        </is>
+      </c>
+      <c r="D501" s="3" t="inlineStr"/>
+      <c r="E501" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F501" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G501" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H501" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I501" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J501" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K501" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L501" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M501" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N501" s="3" t="inlineStr"/>
+      <c r="O501" s="3" t="inlineStr"/>
+      <c r="P501" s="3" t="inlineStr"/>
+      <c r="Q501" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 40+ 州；无公开网址；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" s="3" t="inlineStr">
+        <is>
+          <t>Tri-Power MPT/OTP Industrial Solutions</t>
+        </is>
+      </c>
+      <c r="B502" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C502" s="3" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="D502" s="3" t="inlineStr">
+        <is>
+          <t>otcindustrial.com</t>
+        </is>
+      </c>
+      <c r="E502" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F502" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G502" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H502" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I502" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J502" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K502" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L502" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M502" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N502" s="3" t="inlineStr"/>
+      <c r="O502" s="3" t="inlineStr"/>
+      <c r="P502" s="3" t="inlineStr"/>
+      <c r="Q502" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 40+ 州；有售前+售后支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="3" t="inlineStr">
+        <is>
+          <t>TRI-Phase</t>
+        </is>
+      </c>
+      <c r="B503" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C503" s="3" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="D503" s="3" t="inlineStr">
+        <is>
+          <t>tri-phase.com</t>
+        </is>
+      </c>
+      <c r="E503" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F503" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G503" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H503" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I503" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J503" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K503" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L503" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M503" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N503" s="3" t="inlineStr"/>
+      <c r="O503" s="3" t="inlineStr"/>
+      <c r="P503" s="3" t="inlineStr"/>
+      <c r="Q503" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 40+ 州；有售前+售后支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="3" t="inlineStr">
+        <is>
+          <t>Van Meter Inc.</t>
+        </is>
+      </c>
+      <c r="B504" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C504" s="3" t="inlineStr">
+        <is>
+          <t>IA</t>
+        </is>
+      </c>
+      <c r="D504" s="3" t="inlineStr">
+        <is>
+          <t>vanmeterinc.com</t>
+        </is>
+      </c>
+      <c r="E504" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F504" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G504" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H504" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I504" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J504" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K504" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L504" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M504" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N504" s="3" t="inlineStr"/>
+      <c r="O504" s="3" t="inlineStr"/>
+      <c r="P504" s="3" t="inlineStr"/>
+      <c r="Q504" s="3" t="inlineStr">
+        <is>
+          <t>中西部电气分销，3 个点；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="3" t="inlineStr">
+        <is>
+          <t>Werner Electric</t>
+        </is>
+      </c>
+      <c r="B505" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C505" s="3" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="D505" s="3" t="inlineStr">
+        <is>
+          <t>wernerelectric.com</t>
+        </is>
+      </c>
+      <c r="E505" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F505" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon + Ixxat</t>
+        </is>
+      </c>
+      <c r="G505" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H505" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I505" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J505" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K505" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L505" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M505" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N505" s="3" t="inlineStr"/>
+      <c r="O505" s="3" t="inlineStr"/>
+      <c r="P505" s="3" t="inlineStr"/>
+      <c r="Q505" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 40+ 州；威斯康星工业分销；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="3" t="inlineStr">
+        <is>
+          <t>Wesco</t>
+        </is>
+      </c>
+      <c r="B506" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C506" s="3" t="inlineStr">
+        <is>
+          <t>NC</t>
+        </is>
+      </c>
+      <c r="D506" s="3" t="inlineStr">
+        <is>
+          <t>wesco.com</t>
+        </is>
+      </c>
+      <c r="E506" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F506" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G506" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H506" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I506" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J506" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K506" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L506" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M506" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N506" s="3" t="inlineStr"/>
+      <c r="O506" s="3" t="inlineStr"/>
+      <c r="P506" s="3" t="inlineStr"/>
+      <c r="Q506" s="3" t="inlineStr">
+        <is>
+          <t>★ 北美最大电气分销之一（原 Anixter），目录里还有更多分部；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
HMS USA page 8 of 8: completes the US N-Tron channel
All 149 US directory entries are now covered. They resolve to 68
distinct companies, since branch listings make up more than half the
directory. Wesco's branch count is corrected to nine.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q506"/>
+  <dimension ref="A1:Q508"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -47324,7 +47324,157 @@
       <c r="P506" s="3" t="inlineStr"/>
       <c r="Q506" s="3" t="inlineStr">
         <is>
-          <t>★ 北美最大电气分销之一（原 Anixter），目录里还有更多分部；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+          <t>★ 北美最大电气分销之一（原 Anixter）；目录里 9 个分部：NC Charlotte·Raleigh / SC Greenville / VA Chesapeake·Midlothian·Lynchburg·Norfolk·Roanoke·Hampton；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="3" t="inlineStr">
+        <is>
+          <t>Wille Electric Supply Co</t>
+        </is>
+      </c>
+      <c r="B507" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C507" s="3" t="inlineStr">
+        <is>
+          <t>CA</t>
+        </is>
+      </c>
+      <c r="D507" s="3" t="inlineStr">
+        <is>
+          <t>willeelectric.com</t>
+        </is>
+      </c>
+      <c r="E507" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F507" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion</t>
+        </is>
+      </c>
+      <c r="G507" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H507" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I507" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6310G</t>
+        </is>
+      </c>
+      <c r="J507" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K507" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L507" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M507" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N507" s="3" t="inlineStr"/>
+      <c r="O507" s="3" t="inlineStr"/>
+      <c r="P507" s="3" t="inlineStr"/>
+      <c r="Q507" s="3" t="inlineStr">
+        <is>
+          <t>加州；电气分销；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="3" t="inlineStr">
+        <is>
+          <t>Zesco Inc</t>
+        </is>
+      </c>
+      <c r="B508" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C508" s="3" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="D508" s="3" t="inlineStr">
+        <is>
+          <t>zescoinc.com</t>
+        </is>
+      </c>
+      <c r="E508" s="3" t="inlineStr">
+        <is>
+          <t>分销（HMS/N-Tron·Red Lion 渠道）</t>
+        </is>
+      </c>
+      <c r="F508" s="3" t="inlineStr">
+        <is>
+          <t>N-Tron + Red Lion + Anybus + Ewon</t>
+        </is>
+      </c>
+      <c r="G508" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H508" s="3" t="inlineStr">
+        <is>
+          <t>卖 N-Tron/Red Lion 工业交换机（8口约 $500+）→ 中性货同规格 LT-IS6310G 约 $91，做第二供应商，价差 5 倍</t>
+        </is>
+      </c>
+      <c r="I508" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XG-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J508" s="3" t="inlineStr">
+        <is>
+          <t>官网联系页（HMS 名录只公开地址与网址）</t>
+        </is>
+      </c>
+      <c r="K508" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L508" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M508" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N508" s="3" t="inlineStr"/>
+      <c r="O508" s="3" t="inlineStr"/>
+      <c r="P508" s="3" t="inlineStr"/>
+      <c r="Q508" s="3" t="inlineStr">
+        <is>
+          <t>覆盖 OH/PA；有售前+售后支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Open the MikroTik consultant directory: first 6 German consultants
The consultants directory is a different kind of source from the
distributor directory: entries carry a named person, direct phone,
personal email, city, certification list and a written skills profile
rather than just a company website. These are the technical buyers most
likely to evaluate a switch on ERPS, IGMP and CLI behaviour.
Germany's first page yields SKYTRON (a WISP operating its own backbone)
and FMS Web, where three consultants share one company.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q508"/>
+  <dimension ref="A1:Q512"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -47475,6 +47475,306 @@
       <c r="Q508" s="3" t="inlineStr">
         <is>
           <t>覆盖 OH/PA；有售前+售后支持；⚠️ 中国产地不能做 TAA/NDAA 政府/电力项目，只谈商业渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="3" t="inlineStr">
+        <is>
+          <t>Kehrlein（MikroTik 认证顾问）</t>
+        </is>
+      </c>
+      <c r="B509" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C509" s="3" t="inlineStr">
+        <is>
+          <t>München</t>
+        </is>
+      </c>
+      <c r="D509" s="3" t="inlineStr">
+        <is>
+          <t>kehrlein.de</t>
+        </is>
+      </c>
+      <c r="E509" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F509" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCRE 等</t>
+        </is>
+      </c>
+      <c r="G509" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H509" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维，会自己采购设备 → 用 ERPS/IGMP/VLAN/CLI 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I509" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J509" s="3" t="inlineStr">
+        <is>
+          <t>+49 89 69387111 / info@kehrlein.de</t>
+        </is>
+      </c>
+      <c r="K509" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L509" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M509" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N509" s="3" t="inlineStr"/>
+      <c r="O509" s="3" t="inlineStr"/>
+      <c r="P509" s="3" t="inlineStr"/>
+      <c r="Q509" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> München；技能含 VPN/IPsec/L2TP/OpenVPN/PPPoE/IPv6/无线/CAPsMAN/QoS/HA/负载均衡/数据中心</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="3" t="inlineStr">
+        <is>
+          <t>Michael Gisbers / Linux-Schmie.de</t>
+        </is>
+      </c>
+      <c r="B510" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C510" s="3" t="inlineStr">
+        <is>
+          <t>Oberhausen</t>
+        </is>
+      </c>
+      <c r="D510" s="3" t="inlineStr">
+        <is>
+          <t>linux-schmie.de</t>
+        </is>
+      </c>
+      <c r="E510" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F510" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCTCE+MTCUME+MTCINE+MTCIPv6E+MTCSE+MTCSWE+MTCEWE（10 证，全证）</t>
+        </is>
+      </c>
+      <c r="G510" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H510" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维，会自己采购设备 → 用 ERPS/IGMP/VLAN/CLI 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I510" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J510" s="3" t="inlineStr">
+        <is>
+          <t>+49 173 5106822 / m.gisbers@linux-schmie.de</t>
+        </is>
+      </c>
+      <c r="K510" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L510" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M510" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N510" s="3" t="inlineStr"/>
+      <c r="O510" s="3" t="inlineStr"/>
+      <c r="P510" s="3" t="inlineStr"/>
+      <c r="Q510" s="3" t="inlineStr">
+        <is>
+          <t>10 项认证全拿 → 技术能力最强档；做 RouterOS 咨询/运维/培训，含 Linux 与云集成</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" s="3" t="inlineStr">
+        <is>
+          <t>Holger Witt / SKYTRON Communications GmbH &amp; Co. KG</t>
+        </is>
+      </c>
+      <c r="B511" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C511" s="3" t="inlineStr">
+        <is>
+          <t>Karlsbad</t>
+        </is>
+      </c>
+      <c r="D511" s="3" t="inlineStr">
+        <is>
+          <t>skytron.business</t>
+        </is>
+      </c>
+      <c r="E511" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F511" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCTCE+MTCUME+MTCINE+MTCIPv6E+MTCSE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G511" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H511" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维，会自己采购设备 → 用 ERPS/IGMP/VLAN/CLI 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I511" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J511" s="3" t="inlineStr">
+        <is>
+          <t>+49 7248 4528-130 / h.witt@skytron.de</t>
+        </is>
+      </c>
+      <c r="K511" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L511" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M511" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N511" s="3" t="inlineStr"/>
+      <c r="O511" s="3" t="inlineStr"/>
+      <c r="P511" s="3" t="inlineStr"/>
+      <c r="Q511" s="3" t="inlineStr">
+        <is>
+          <t>WISP/运营商：自建骨干网、BGP/OSPF/MPLS-VPLS、光纤与微波回传、公共 WiFi、IPv6/IoT/LoRaWAN → 最对口</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="3" t="inlineStr">
+        <is>
+          <t>Sebastian Inacker / FMS Web（fmsweb.de）</t>
+        </is>
+      </c>
+      <c r="B512" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C512" s="3" t="inlineStr">
+        <is>
+          <t>Umkirch (Freiburg)</t>
+        </is>
+      </c>
+      <c r="D512" s="3" t="inlineStr">
+        <is>
+          <t>fmsweb.de</t>
+        </is>
+      </c>
+      <c r="E512" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F512" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCTCE+MTCIPv6E</t>
+        </is>
+      </c>
+      <c r="G512" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H512" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维，会自己采购设备 → 用 ERPS/IGMP/VLAN/CLI 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I512" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J512" s="3" t="inlineStr">
+        <is>
+          <t>+49 761 2926500 / inacker@fmsweb.de</t>
+        </is>
+      </c>
+      <c r="K512" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L512" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M512" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N512" s="3" t="inlineStr"/>
+      <c r="O512" s="3" t="inlineStr"/>
+      <c r="P512" s="3" t="inlineStr"/>
+      <c r="Q512" s="3" t="inlineStr">
+        <is>
+          <t>WISP 方向：无线、Hotspot、User Manager、PPPoE、防火墙、QoS、WISP 安全审计</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Polish MikroTik consultants, first page: 11 named contacts
Ryszard Labus works on BMS and industrial automation networks and
Jacek Rokicki lists CRS switching and L2 work directly in his profile,
which makes them the most natural switch conversations in the batch.
Ihor Hreskiv is a certified trainer with 300 sessions delivered, so he
reaches further than his own projects.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q512"/>
+  <dimension ref="A1:Q523"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -47774,7 +47774,824 @@
       <c r="P512" s="3" t="inlineStr"/>
       <c r="Q512" s="3" t="inlineStr">
         <is>
-          <t>WISP 方向：无线、Hotspot、User Manager、PPPoE、防火墙、QoS、WISP 安全审计</t>
+          <t>同公司还有 2 位 MikroTik 认证顾问（同一电话 +49 761 2926500）：Henrik Brinkmann（brinkmann@fmsweb.de，MTCNA+MTCRE+MTCTCE+MTCIPv6E，做企业/ISP/运营商网、HA、MPLS-VPLS、公共 WiFi、3G-LTE M2M 与监控）；Patrik Schaub（MTCNA+MTCRE+MTCTCE+MTCIPv6E，无线/PtMP/MESH）。一家公司 3 个顾问，谈一次覆盖三人项目</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" s="3" t="inlineStr">
+        <is>
+          <t>Piotr Wasyk / MWTC</t>
+        </is>
+      </c>
+      <c r="B513" s="3" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C513" s="3" t="inlineStr">
+        <is>
+          <t>Warszawa</t>
+        </is>
+      </c>
+      <c r="D513" s="3" t="inlineStr">
+        <is>
+          <t>mwtc.pl</t>
+        </is>
+      </c>
+      <c r="E513" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F513" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 10 证全拿</t>
+        </is>
+      </c>
+      <c r="G513" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H513" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I513" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J513" s="3" t="inlineStr">
+        <is>
+          <t>+48 513 322 115 / piotr@mwtc.pl（总机 +48 796 171 971 / info@mwtc.pl）</t>
+        </is>
+      </c>
+      <c r="K513" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L513" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M513" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N513" s="3" t="inlineStr"/>
+      <c r="O513" s="3" t="inlineStr"/>
+      <c r="P513" s="3" t="inlineStr"/>
+      <c r="Q513" s="3" t="inlineStr">
+        <is>
+          <t>网络架构师 12+ 年，中大型 IP 基础设施；动态路由/流量整形/负载均衡/HA/VPN/安全；同公司另有 info@mwtc.pl</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="3" t="inlineStr">
+        <is>
+          <t>Ihor Hreskiv / mtik.pl</t>
+        </is>
+      </c>
+      <c r="B514" s="3" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C514" s="3" t="inlineStr">
+        <is>
+          <t>Kraków</t>
+        </is>
+      </c>
+      <c r="D514" s="3" t="inlineStr">
+        <is>
+          <t>mtik.pl</t>
+        </is>
+      </c>
+      <c r="E514" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F514" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 10 证全拿</t>
+        </is>
+      </c>
+      <c r="G514" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H514" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I514" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J514" s="3" t="inlineStr">
+        <is>
+          <t>+48 512 438 083 / biuro@mtik.pl</t>
+        </is>
+      </c>
+      <c r="K514" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L514" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M514" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N514" s="3" t="inlineStr"/>
+      <c r="O514" s="3" t="inlineStr"/>
+      <c r="P514" s="3" t="inlineStr"/>
+      <c r="Q514" s="3" t="inlineStr">
+        <is>
+          <t>★ MikroTik 认证讲师，已授课 300+ 场；20+ 年经验，ISP 咨询、动态路由、交换、WiFi/CAPsMAN；英/波/乌三语</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="3" t="inlineStr">
+        <is>
+          <t>Paweł Wandas / SAFES</t>
+        </is>
+      </c>
+      <c r="B515" s="3" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C515" s="3" t="inlineStr">
+        <is>
+          <t>Kraków</t>
+        </is>
+      </c>
+      <c r="D515" s="3" t="inlineStr">
+        <is>
+          <t>safes.pl</t>
+        </is>
+      </c>
+      <c r="E515" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F515" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCTCE+MTCINE+MTCIPv6E+MTCSE+MTCSWE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G515" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H515" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I515" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J515" s="3" t="inlineStr">
+        <is>
+          <t>+48 412 412 324 / biuro@safes.pl</t>
+        </is>
+      </c>
+      <c r="K515" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L515" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M515" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N515" s="3" t="inlineStr"/>
+      <c r="O515" s="3" t="inlineStr"/>
+      <c r="P515" s="3" t="inlineStr"/>
+      <c r="Q515" s="3" t="inlineStr">
+        <is>
+          <t>防火墙/VPN/隧道/负载均衡/故障切换/QoS/高级路由/无线；熟 The Dude 网管 → 对 SNMP/MIB/NMS 集成有感觉</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="3" t="inlineStr">
+        <is>
+          <t>Wojciech Mańka / Mikrotikon</t>
+        </is>
+      </c>
+      <c r="B516" s="3" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C516" s="3" t="inlineStr">
+        <is>
+          <t>Czerwionka-Leszczyny</t>
+        </is>
+      </c>
+      <c r="D516" s="3" t="inlineStr">
+        <is>
+          <t>mikrotikon.pl</t>
+        </is>
+      </c>
+      <c r="E516" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F516" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCTCE+MTCINE+MTCIPv6E+MTCSE+MTCSWE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G516" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H516" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I516" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J516" s="3" t="inlineStr">
+        <is>
+          <t>+48 791 560 569 / kontakt@mikrotechnology.pl</t>
+        </is>
+      </c>
+      <c r="K516" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L516" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M516" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N516" s="3" t="inlineStr"/>
+      <c r="O516" s="3" t="inlineStr"/>
+      <c r="P516" s="3" t="inlineStr"/>
+      <c r="Q516" s="3" t="inlineStr">
+        <is>
+          <t>VPN/无线/防火墙/网络安全；小企业到运营商级方案</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="3" t="inlineStr">
+        <is>
+          <t>Jacek Rokicki / C3NET</t>
+        </is>
+      </c>
+      <c r="B517" s="3" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C517" s="3" t="inlineStr">
+        <is>
+          <t>Falenty Nowe</t>
+        </is>
+      </c>
+      <c r="D517" s="3" t="inlineStr">
+        <is>
+          <t>c3net.pl</t>
+        </is>
+      </c>
+      <c r="E517" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F517" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCTCE+MTCINE+MTCSE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G517" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H517" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I517" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J517" s="3" t="inlineStr">
+        <is>
+          <t>+48 506 457 447 / mt-support@c3net.pl</t>
+        </is>
+      </c>
+      <c r="K517" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L517" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M517" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N517" s="3" t="inlineStr"/>
+      <c r="O517" s="3" t="inlineStr"/>
+      <c r="P517" s="3" t="inlineStr"/>
+      <c r="Q517" s="3" t="inlineStr">
+        <is>
+          <t>★ 自述技能直接写「CRS switches and many L2 topics」+ BGP/OSPF/CAPsMAN/队列与策略路由 → 交换机话题现成</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="3" t="inlineStr">
+        <is>
+          <t>Ryszard Labus / SINUX</t>
+        </is>
+      </c>
+      <c r="B518" s="3" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C518" s="3" t="inlineStr">
+        <is>
+          <t>Warszawa</t>
+        </is>
+      </c>
+      <c r="D518" s="3" t="inlineStr">
+        <is>
+          <t>sinux.pl</t>
+        </is>
+      </c>
+      <c r="E518" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F518" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCSE+MTCSWE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G518" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H518" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I518" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J518" s="3" t="inlineStr">
+        <is>
+          <t>+48 666 385 002 / r.labus@sinux.pl</t>
+        </is>
+      </c>
+      <c r="K518" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L518" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M518" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N518" s="3" t="inlineStr"/>
+      <c r="O518" s="3" t="inlineStr"/>
+      <c r="P518" s="3" t="inlineStr"/>
+      <c r="Q518" s="3" t="inlineStr">
+        <is>
+          <t>★ 专注 BMS / 工业 / 楼宇自动化网络，含 VLAN、VPN、跨网互联、与自动化系统集成 → 工业线最对口</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" s="3" t="inlineStr">
+        <is>
+          <t>Bartłomiej Maliszewski</t>
+        </is>
+      </c>
+      <c r="B519" s="3" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C519" s="3" t="inlineStr">
+        <is>
+          <t>Maciejów</t>
+        </is>
+      </c>
+      <c r="D519" s="3" t="inlineStr">
+        <is>
+          <t>maliszewski.pro</t>
+        </is>
+      </c>
+      <c r="E519" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F519" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCSE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G519" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H519" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I519" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J519" s="3" t="inlineStr">
+        <is>
+          <t>+48 881 447 860 / bartlomiej@maliszewski.pro</t>
+        </is>
+      </c>
+      <c r="K519" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L519" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M519" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N519" s="3" t="inlineStr"/>
+      <c r="O519" s="3" t="inlineStr"/>
+      <c r="P519" s="3" t="inlineStr"/>
+      <c r="Q519" s="3" t="inlineStr">
+        <is>
+          <t>8 年网络经验，其中 5 年在 ISP；为服务商和企业搭建 RouterOS 环境</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="3" t="inlineStr">
+        <is>
+          <t>Piotr Poniatowski</t>
+        </is>
+      </c>
+      <c r="B520" s="3" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C520" s="3" t="inlineStr">
+        <is>
+          <t>Miedzyrzec Podlaski</t>
+        </is>
+      </c>
+      <c r="D520" s="3" t="inlineStr">
+        <is>
+          <t>poniatowski.pl</t>
+        </is>
+      </c>
+      <c r="E520" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F520" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCUME+MTCSWE</t>
+        </is>
+      </c>
+      <c r="G520" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H520" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I520" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J520" s="3" t="inlineStr">
+        <is>
+          <t>+48 501 337 777 / piotr@poniatowski.pl</t>
+        </is>
+      </c>
+      <c r="K520" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L520" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M520" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N520" s="3" t="inlineStr"/>
+      <c r="O520" s="3" t="inlineStr"/>
+      <c r="P520" s="3" t="inlineStr"/>
+      <c r="Q520" s="3" t="inlineStr">
+        <is>
+          <t>含 MTCUME（用户管理）→ Hotspot/PPPoE 方向</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" s="3" t="inlineStr">
+        <is>
+          <t>Piotr Maślak</t>
+        </is>
+      </c>
+      <c r="B521" s="3" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C521" s="3" t="inlineStr">
+        <is>
+          <t>Warszawa</t>
+        </is>
+      </c>
+      <c r="D521" s="3" t="inlineStr">
+        <is>
+          <t>maslak.waw.pl</t>
+        </is>
+      </c>
+      <c r="E521" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F521" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCINE</t>
+        </is>
+      </c>
+      <c r="G521" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H521" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I521" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J521" s="3" t="inlineStr">
+        <is>
+          <t>+48 606 225 270 / piotr@maslak.waw.pl</t>
+        </is>
+      </c>
+      <c r="K521" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L521" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M521" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N521" s="3" t="inlineStr"/>
+      <c r="O521" s="3" t="inlineStr"/>
+      <c r="P521" s="3" t="inlineStr"/>
+      <c r="Q521" s="3" t="inlineStr">
+        <is>
+          <t>含 MTCINE（ISP 互联）→ 运营商方向</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="3" t="inlineStr">
+        <is>
+          <t>Grzegorz Śliwiński</t>
+        </is>
+      </c>
+      <c r="B522" s="3" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C522" s="3" t="inlineStr">
+        <is>
+          <t>Szczecin</t>
+        </is>
+      </c>
+      <c r="D522" s="3" t="inlineStr"/>
+      <c r="E522" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F522" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G522" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H522" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I522" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J522" s="3" t="inlineStr">
+        <is>
+          <t>（见 MikroTik 顾问名录）</t>
+        </is>
+      </c>
+      <c r="K522" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L522" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M522" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N522" s="3" t="inlineStr"/>
+      <c r="O522" s="3" t="inlineStr"/>
+      <c r="P522" s="3" t="inlineStr"/>
+      <c r="Q522" s="3" t="inlineStr">
+        <is>
+          <t>26 年网络经验 + 讲师，带过数千学生 → 影响力型，可发展成渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" s="3" t="inlineStr">
+        <is>
+          <t>Kacper Kisielewski</t>
+        </is>
+      </c>
+      <c r="B523" s="3" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C523" s="3" t="inlineStr">
+        <is>
+          <t>Nałęczów</t>
+        </is>
+      </c>
+      <c r="D523" s="3" t="inlineStr"/>
+      <c r="E523" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F523" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G523" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H523" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I523" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J523" s="3" t="inlineStr">
+        <is>
+          <t>+48 669 271 768 / kacperxawer.123@gmail.com</t>
+        </is>
+      </c>
+      <c r="K523" s="3" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="L523" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M523" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N523" s="3" t="inlineStr"/>
+      <c r="O523" s="3" t="inlineStr"/>
+      <c r="P523" s="3" t="inlineStr"/>
+      <c r="Q523" s="3" t="inlineStr">
+        <is>
+          <t>个人邮箱（gmail），可能是个人兼职 → 低优先</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Finish the Polish consultant list: 15 consultants in total
Adds the last two and fills in the university email for Grzegorz
Sliwinski, who runs a MikroTik Academy and teaches MTCNA.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q523"/>
+  <dimension ref="A1:Q525"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -48497,7 +48497,7 @@
       </c>
       <c r="J522" s="3" t="inlineStr">
         <is>
-          <t>（见 MikroTik 顾问名录）</t>
+          <t>gsliwinski@zut.edu.pl（西波美拉尼亚理工大学）</t>
         </is>
       </c>
       <c r="K522" s="3" t="inlineStr">
@@ -48520,7 +48520,7 @@
       <c r="P522" s="3" t="inlineStr"/>
       <c r="Q522" s="3" t="inlineStr">
         <is>
-          <t>26 年网络经验 + 讲师，带过数千学生 → 影响力型，可发展成渠道</t>
+          <t>26 年网络经验 + 高校教师，带过数千学生；运营 MikroTik Academy，做 MTCNA 培训 → 影响力型，可发展成渠道/讲师合作</t>
         </is>
       </c>
     </row>
@@ -48592,6 +48592,156 @@
       <c r="Q523" s="3" t="inlineStr">
         <is>
           <t>个人邮箱（gmail），可能是个人兼职 → 低优先</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="3" t="inlineStr">
+        <is>
+          <t>Maciej Ziółkowski</t>
+        </is>
+      </c>
+      <c r="B524" s="3" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C524" s="3" t="inlineStr">
+        <is>
+          <t>Włocławek / Poznań</t>
+        </is>
+      </c>
+      <c r="D524" s="3" t="inlineStr">
+        <is>
+          <t>mziolkowski.pl</t>
+        </is>
+      </c>
+      <c r="E524" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F524" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G524" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H524" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I524" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J524" s="3" t="inlineStr">
+        <is>
+          <t>kontakt@mziolkowski.pl</t>
+        </is>
+      </c>
+      <c r="K524" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L524" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M524" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N524" s="3" t="inlineStr"/>
+      <c r="O524" s="3" t="inlineStr"/>
+      <c r="P524" s="3" t="inlineStr"/>
+      <c r="Q524" s="3" t="inlineStr">
+        <is>
+          <t>10+ 年；VPN/路由/防火墙/安全/**交换**/脚本/MikroTik API → 自述含 switching 与 API，做自动化集成</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="3" t="inlineStr">
+        <is>
+          <t>Krzysztof Dudek / Innored</t>
+        </is>
+      </c>
+      <c r="B525" s="3" t="inlineStr">
+        <is>
+          <t>波兰</t>
+        </is>
+      </c>
+      <c r="C525" s="3" t="inlineStr">
+        <is>
+          <t>Jelcz-Laskowice</t>
+        </is>
+      </c>
+      <c r="D525" s="3" t="inlineStr">
+        <is>
+          <t>innored.pl</t>
+        </is>
+      </c>
+      <c r="E525" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F525" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSE</t>
+        </is>
+      </c>
+      <c r="G525" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H525" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I525" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J525" s="3" t="inlineStr">
+        <is>
+          <t>+48 533 376 662 / krzysztof.d@adar.net.pl</t>
+        </is>
+      </c>
+      <c r="K525" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L525" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M525" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N525" s="3" t="inlineStr"/>
+      <c r="O525" s="3" t="inlineStr"/>
+      <c r="P525" s="3" t="inlineStr"/>
+      <c r="Q525" s="3" t="inlineStr">
+        <is>
+          <t>含 MTCSE（安全）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Finish the German consultant list: 9 consultants in total
Alexej Sokolow holds MTCSWE, the switching certificate, so switching is
a declared specialism rather than an aside. Dinko Ivanov works at a
fibre ISP where FTTH rollouts need access-layer switches. Also records
Patrik Schaub's direct email on the FMS Web row.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q525"/>
+  <dimension ref="A1:Q528"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -47774,7 +47774,7 @@
       <c r="P512" s="3" t="inlineStr"/>
       <c r="Q512" s="3" t="inlineStr">
         <is>
-          <t>同公司还有 2 位 MikroTik 认证顾问（同一电话 +49 761 2926500）：Henrik Brinkmann（brinkmann@fmsweb.de，MTCNA+MTCRE+MTCTCE+MTCIPv6E，做企业/ISP/运营商网、HA、MPLS-VPLS、公共 WiFi、3G-LTE M2M 与监控）；Patrik Schaub（MTCNA+MTCRE+MTCTCE+MTCIPv6E，无线/PtMP/MESH）。一家公司 3 个顾问，谈一次覆盖三人项目</t>
+          <t>同公司共 3 位 MikroTik 认证顾问（同一电话 +49 761 2926500）：Henrik Brinkmann（brinkmann@fmsweb.de，企业/ISP/运营商、MPLS-VPLS、公共 WiFi、3G-LTE M2M 与监控）；Patrik Schaub（schaub@fmsweb.de，无线/PtP·PtMP/MESH）。谈一次覆盖三人项目</t>
         </is>
       </c>
     </row>
@@ -48742,6 +48742,231 @@
       <c r="Q525" s="3" t="inlineStr">
         <is>
           <t>含 MTCSE（安全）</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="3" t="inlineStr">
+        <is>
+          <t>Alexej Sokolow / DECOIT</t>
+        </is>
+      </c>
+      <c r="B526" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C526" s="3" t="inlineStr">
+        <is>
+          <t>Bremen</t>
+        </is>
+      </c>
+      <c r="D526" s="3" t="inlineStr">
+        <is>
+          <t>decoit.de</t>
+        </is>
+      </c>
+      <c r="E526" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F526" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCSWE</t>
+        </is>
+      </c>
+      <c r="G526" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H526" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I526" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J526" s="3" t="inlineStr">
+        <is>
+          <t>+49 421 5960640 / sokolow@decoit.de</t>
+        </is>
+      </c>
+      <c r="K526" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L526" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M526" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N526" s="3" t="inlineStr"/>
+      <c r="O526" s="3" t="inlineStr"/>
+      <c r="P526" s="3" t="inlineStr"/>
+      <c r="Q526" s="3" t="inlineStr">
+        <is>
+          <t>★ 持 MTCSWE（交换认证）→ 交换机是正式专长，不是顺带；DECOIT 是不来梅 IT 安全/网络公司</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" s="3" t="inlineStr">
+        <is>
+          <t>Manuel Kuhn / EBC Marburg</t>
+        </is>
+      </c>
+      <c r="B527" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C527" s="3" t="inlineStr">
+        <is>
+          <t>Marburg</t>
+        </is>
+      </c>
+      <c r="D527" s="3" t="inlineStr">
+        <is>
+          <t>ebc-marburg.de</t>
+        </is>
+      </c>
+      <c r="E527" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F527" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCSE</t>
+        </is>
+      </c>
+      <c r="G527" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H527" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I527" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J527" s="3" t="inlineStr">
+        <is>
+          <t>+49 6421 9792437 / manuel.kuhn@ebc-marburg.de</t>
+        </is>
+      </c>
+      <c r="K527" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L527" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M527" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N527" s="3" t="inlineStr"/>
+      <c r="O527" s="3" t="inlineStr"/>
+      <c r="P527" s="3" t="inlineStr"/>
+      <c r="Q527" s="3" t="inlineStr">
+        <is>
+          <t>含 MTCSE（安全）</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="3" t="inlineStr">
+        <is>
+          <t>Dinko Ivanov / MBN Glasfaser</t>
+        </is>
+      </c>
+      <c r="B528" s="3" t="inlineStr">
+        <is>
+          <t>德国</t>
+        </is>
+      </c>
+      <c r="C528" s="3" t="inlineStr">
+        <is>
+          <t>Westhofen</t>
+        </is>
+      </c>
+      <c r="D528" s="3" t="inlineStr">
+        <is>
+          <t>mbn-glasfaser.de</t>
+        </is>
+      </c>
+      <c r="E528" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F528" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSE</t>
+        </is>
+      </c>
+      <c r="G528" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H528" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I528" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J528" s="3" t="inlineStr">
+        <is>
+          <t>+49 6344 9442084 / dinko.ivanov@mbn-glasfaser.de</t>
+        </is>
+      </c>
+      <c r="K528" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L528" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M528" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N528" s="3" t="inlineStr"/>
+      <c r="O528" s="3" t="inlineStr"/>
+      <c r="P528" s="3" t="inlineStr"/>
+      <c r="Q528" s="3" t="inlineStr">
+        <is>
+          <t>★ 光纤接入 ISP（公司名带 Glasfaser）→ FTTH 项目需要接入层交换机</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Czech consultants: 5 including a product manager at 100MEGA
Michal Stepanek is a product manager at i4wifi 100MEGA Distribution,
one of the largest Czech network distributors, which is exactly the
category-manager entry route rather than a cold approach to a CPO.
Martin Pina holds both the switching and ISP interconnection
certificates.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q528"/>
+  <dimension ref="A1:Q532"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -48967,6 +48967,306 @@
       <c r="Q528" s="3" t="inlineStr">
         <is>
           <t>★ 光纤接入 ISP（公司名带 Glasfaser）→ FTTH 项目需要接入层交换机</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" s="3" t="inlineStr">
+        <is>
+          <t>Michal Stepanek / i4wifi 100MEGA Distribution s.r.o.</t>
+        </is>
+      </c>
+      <c r="B529" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C529" s="3" t="inlineStr">
+        <is>
+          <t>Neratovice</t>
+        </is>
+      </c>
+      <c r="D529" s="3" t="inlineStr">
+        <is>
+          <t>100mega.cz</t>
+        </is>
+      </c>
+      <c r="E529" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F529" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCTCE+MTCSE</t>
+        </is>
+      </c>
+      <c r="G529" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H529" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I529" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J529" s="3" t="inlineStr">
+        <is>
+          <t>+420 774 198 272 / mikrotikpodpora@gmail.com</t>
+        </is>
+      </c>
+      <c r="K529" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L529" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M529" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N529" s="3" t="inlineStr"/>
+      <c r="O529" s="3" t="inlineStr"/>
+      <c r="P529" s="3" t="inlineStr"/>
+      <c r="Q529" s="3" t="inlineStr">
+        <is>
+          <t>★ 100MEGA（i4wifi）是捷克最大 MikroTik/网络设备分销之一，此人是**产品经理** → 正是「找品类经理不找 CPO」那条路；他还在 skoleni.100mega.cz 讲课、办 mtpc.world 大会</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" s="3" t="inlineStr">
+        <is>
+          <t>Martin Pina</t>
+        </is>
+      </c>
+      <c r="B530" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C530" s="3" t="inlineStr">
+        <is>
+          <t>Olomouc</t>
+        </is>
+      </c>
+      <c r="D530" s="3" t="inlineStr">
+        <is>
+          <t>hanacke.net</t>
+        </is>
+      </c>
+      <c r="E530" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F530" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCINE+MTCIPv6E+MTCSE+MTCSWE</t>
+        </is>
+      </c>
+      <c r="G530" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H530" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I530" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J530" s="3" t="inlineStr">
+        <is>
+          <t>+420 732 712 317 / martin.pina@hanacke.net</t>
+        </is>
+      </c>
+      <c r="K530" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L530" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M530" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N530" s="3" t="inlineStr"/>
+      <c r="O530" s="3" t="inlineStr"/>
+      <c r="P530" s="3" t="inlineStr"/>
+      <c r="Q530" s="3" t="inlineStr">
+        <is>
+          <t>★ 持 MTCSWE（交换）+ MTCINE（ISP 互联）；自述含 switching、高可用、网络监控与安全、远程运维</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" s="3" t="inlineStr">
+        <is>
+          <t>Martin Poisel / MapNet</t>
+        </is>
+      </c>
+      <c r="B531" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C531" s="3" t="inlineStr">
+        <is>
+          <t>Brno</t>
+        </is>
+      </c>
+      <c r="D531" s="3" t="inlineStr">
+        <is>
+          <t>mapnet.cz</t>
+        </is>
+      </c>
+      <c r="E531" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F531" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCTCE+MTCUME+MTCIPv6E+MTCSE</t>
+        </is>
+      </c>
+      <c r="G531" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H531" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I531" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J531" s="3" t="inlineStr">
+        <is>
+          <t>+420 737 429 784 / mpoisel@mapnet.cz</t>
+        </is>
+      </c>
+      <c r="K531" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L531" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M531" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N531" s="3" t="inlineStr"/>
+      <c r="O531" s="3" t="inlineStr"/>
+      <c r="P531" s="3" t="inlineStr"/>
+      <c r="Q531" s="3" t="inlineStr">
+        <is>
+          <t>7 证；布尔诺</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" s="3" t="inlineStr">
+        <is>
+          <t>Martin Klablena</t>
+        </is>
+      </c>
+      <c r="B532" s="3" t="inlineStr">
+        <is>
+          <t>捷克</t>
+        </is>
+      </c>
+      <c r="C532" s="3" t="inlineStr">
+        <is>
+          <t>Prague</t>
+        </is>
+      </c>
+      <c r="D532" s="3" t="inlineStr">
+        <is>
+          <t>fubar.cz</t>
+        </is>
+      </c>
+      <c r="E532" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F532" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCINE</t>
+        </is>
+      </c>
+      <c r="G532" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H532" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I532" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J532" s="3" t="inlineStr">
+        <is>
+          <t>+420 602 242 774 / klablena@fubar.cz</t>
+        </is>
+      </c>
+      <c r="K532" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L532" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M532" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N532" s="3" t="inlineStr"/>
+      <c r="O532" s="3" t="inlineStr"/>
+      <c r="P532" s="3" t="inlineStr"/>
+      <c r="Q532" s="3" t="inlineStr">
+        <is>
+          <t>动态路由 OSPF/RIP/BGP、企业站点互联与集中式 IPSec/SSTP/OpenVPN、CAPsMAN、**高级 LAN 拓扑与双 WAN 备份设计**</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ukrainian consultants: 9 including two strong PoE and switching fits
Andrew Drozd designs and installs CCTV, alarm and access control
systems, so PoE switches are a standing requirement rather than an
upsell. Vitalii Potravka and Vadym Klymenko cover switching and
monitoring respectively. Ukraine produced 18 distributors earlier and
now 9 consultants, the most of any country so far.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q532"/>
+  <dimension ref="A1:Q541"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -27514,7 +27514,7 @@
       </c>
       <c r="K234" s="3" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="L234" s="3" t="inlineStr">
@@ -27532,7 +27532,7 @@
       <c r="P234" s="3" t="inlineStr"/>
       <c r="Q234" s="3" t="inlineStr">
         <is>
-          <t>Lety</t>
+          <t>Lety；店主 Krystof Klima 本人是 MikroTik 认证顾问（7 证：MTCNA+MTCRE+MTCWE+MTCTCE+MTCUME+MTCIPv6E+MTCSE），专长带宽管理与队列、RADIUS、高级防火墙、VPN/隧道、无线、动态路由 → 既是分销又是集成商，技术型老板，可直接聊规格</t>
         </is>
       </c>
     </row>
@@ -49267,6 +49267,661 @@
       <c r="Q532" s="3" t="inlineStr">
         <is>
           <t>动态路由 OSPF/RIP/BGP、企业站点互联与集中式 IPSec/SSTP/OpenVPN、CAPsMAN、**高级 LAN 拓扑与双 WAN 备份设计**</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" s="3" t="inlineStr">
+        <is>
+          <t>Andrew Drozd / Iron Sentinel</t>
+        </is>
+      </c>
+      <c r="B533" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C533" s="3" t="inlineStr">
+        <is>
+          <t>Zhytomyr</t>
+        </is>
+      </c>
+      <c r="D533" s="3" t="inlineStr">
+        <is>
+          <t>ironsentinel.net</t>
+        </is>
+      </c>
+      <c r="E533" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F533" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCTCE+MTCINE+MTCSE</t>
+        </is>
+      </c>
+      <c r="G533" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H533" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I533" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J533" s="3" t="inlineStr">
+        <is>
+          <t>+380 63 418 8971 / support@ironsentinel.net</t>
+        </is>
+      </c>
+      <c r="K533" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L533" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M533" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N533" s="3" t="inlineStr"/>
+      <c r="O533" s="3" t="inlineStr"/>
+      <c r="P533" s="3" t="inlineStr"/>
+      <c r="Q533" s="3" t="inlineStr">
+        <is>
+          <t>★ 做局域网、**视频监控、报警系统、门禁**的设计/安装/维护 → PoE 交换机是刚需，首推 24 口 PoE</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" s="3" t="inlineStr">
+        <is>
+          <t>Vitalii Potravka</t>
+        </is>
+      </c>
+      <c r="B534" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C534" s="3" t="inlineStr">
+        <is>
+          <t>Kyiv</t>
+        </is>
+      </c>
+      <c r="D534" s="3" t="inlineStr"/>
+      <c r="E534" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F534" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSWE</t>
+        </is>
+      </c>
+      <c r="G534" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H534" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I534" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J534" s="3" t="inlineStr">
+        <is>
+          <t>+380 97 931 2131 / webvetal.mob@gmail.com</t>
+        </is>
+      </c>
+      <c r="K534" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L534" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M534" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N534" s="3" t="inlineStr"/>
+      <c r="O534" s="3" t="inlineStr"/>
+      <c r="P534" s="3" t="inlineStr"/>
+      <c r="Q534" s="3" t="inlineStr">
+        <is>
+          <t>★ 持 MTCSWE（交换认证）→ 交换机是正式专长</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" s="3" t="inlineStr">
+        <is>
+          <t>Vadym Klymenko / Explorer</t>
+        </is>
+      </c>
+      <c r="B535" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C535" s="3" t="inlineStr">
+        <is>
+          <t>Odesa</t>
+        </is>
+      </c>
+      <c r="D535" s="3" t="inlineStr">
+        <is>
+          <t>explorer.od.ua</t>
+        </is>
+      </c>
+      <c r="E535" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F535" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCWE+MTCSE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G535" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H535" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I535" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J535" s="3" t="inlineStr">
+        <is>
+          <t>+380 94 946 7003 / vadim@explorer.od.ua</t>
+        </is>
+      </c>
+      <c r="K535" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L535" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M535" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N535" s="3" t="inlineStr"/>
+      <c r="O535" s="3" t="inlineStr"/>
+      <c r="P535" s="3" t="inlineStr"/>
+      <c r="Q535" s="3" t="inlineStr">
+        <is>
+          <t>系统集成公司：网络设计/审计/优化；OSPF、多厂商 VPN、高级防火墙与队列、**The Dude 与 RoMON 监控**、无线 CAPsMAN/PtP/PtMP、CHR 云；英俄德乌四语</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" s="3" t="inlineStr">
+        <is>
+          <t>Oleksandr Kovinia / K2O Services</t>
+        </is>
+      </c>
+      <c r="B536" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C536" s="3" t="inlineStr">
+        <is>
+          <t>Kyiv</t>
+        </is>
+      </c>
+      <c r="D536" s="3" t="inlineStr">
+        <is>
+          <t>k2o.cc</t>
+        </is>
+      </c>
+      <c r="E536" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F536" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCIPv6E+MTCSE</t>
+        </is>
+      </c>
+      <c r="G536" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H536" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I536" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J536" s="3" t="inlineStr">
+        <is>
+          <t>olekovin+mikrotik-consult@gmail.com</t>
+        </is>
+      </c>
+      <c r="K536" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L536" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M536" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N536" s="3" t="inlineStr"/>
+      <c r="O536" s="3" t="inlineStr"/>
+      <c r="P536" s="3" t="inlineStr"/>
+      <c r="Q536" s="3" t="inlineStr">
+        <is>
+          <t>★ 专做 MikroTik 方案的公司：RouterOS 配置、**监控方案、自动化**、企业网络；设计/排障/性能优化/安全加固/长期运维</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" s="3" t="inlineStr">
+        <is>
+          <t>Serhii Antropov</t>
+        </is>
+      </c>
+      <c r="B537" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C537" s="3" t="inlineStr">
+        <is>
+          <t>Chernivtsi</t>
+        </is>
+      </c>
+      <c r="D537" s="3" t="inlineStr"/>
+      <c r="E537" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F537" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCTCE+MTCINE+MTCIPv6E</t>
+        </is>
+      </c>
+      <c r="G537" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H537" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I537" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J537" s="3" t="inlineStr">
+        <is>
+          <t>+380 66 171 2971 / serega12034@gmail.com</t>
+        </is>
+      </c>
+      <c r="K537" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L537" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M537" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N537" s="3" t="inlineStr"/>
+      <c r="O537" s="3" t="inlineStr"/>
+      <c r="P537" s="3" t="inlineStr"/>
+      <c r="Q537" s="3" t="inlineStr">
+        <is>
+          <t>含 MTCINE（ISP 互联）+ MTCTCE（流量控制）</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" s="3" t="inlineStr">
+        <is>
+          <t>Volodymyr Sydorenko / Coders</t>
+        </is>
+      </c>
+      <c r="B538" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C538" s="3" t="inlineStr">
+        <is>
+          <t>Zhytomyr</t>
+        </is>
+      </c>
+      <c r="D538" s="3" t="inlineStr">
+        <is>
+          <t>coders.in.ua</t>
+        </is>
+      </c>
+      <c r="E538" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F538" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCIPv6E</t>
+        </is>
+      </c>
+      <c r="G538" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H538" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I538" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J538" s="3" t="inlineStr">
+        <is>
+          <t>+380 67 760 0368 / vvs@coders.in.ua</t>
+        </is>
+      </c>
+      <c r="K538" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L538" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M538" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N538" s="3" t="inlineStr"/>
+      <c r="O538" s="3" t="inlineStr"/>
+      <c r="P538" s="3" t="inlineStr"/>
+      <c r="Q538" s="3" t="inlineStr">
+        <is>
+          <t>中小企业网络：VLAN、QoS/流量整形、MultiWAN 负载均衡与故障切换、OSPF、脚本、CAPsMAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" s="3" t="inlineStr">
+        <is>
+          <t>Andrii Nagornyi</t>
+        </is>
+      </c>
+      <c r="B539" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C539" s="3" t="inlineStr">
+        <is>
+          <t>Kryvyi Rih</t>
+        </is>
+      </c>
+      <c r="D539" s="3" t="inlineStr"/>
+      <c r="E539" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F539" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCTCE+MTCSE</t>
+        </is>
+      </c>
+      <c r="G539" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H539" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I539" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J539" s="3" t="inlineStr">
+        <is>
+          <t>+380 67 539 2648 / orglink@hotmail.com</t>
+        </is>
+      </c>
+      <c r="K539" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L539" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M539" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N539" s="3" t="inlineStr"/>
+      <c r="O539" s="3" t="inlineStr"/>
+      <c r="P539" s="3" t="inlineStr"/>
+      <c r="Q539" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik IT 外包与网络工程：基础设施设计、RouterOS 部署、VPN、无线、安全、脚本</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" s="3" t="inlineStr">
+        <is>
+          <t>Andrii Chernov / VIP</t>
+        </is>
+      </c>
+      <c r="B540" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C540" s="3" t="inlineStr">
+        <is>
+          <t>Ternopil</t>
+        </is>
+      </c>
+      <c r="D540" s="3" t="inlineStr">
+        <is>
+          <t>vip.te.ua</t>
+        </is>
+      </c>
+      <c r="E540" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F540" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCIPv6E</t>
+        </is>
+      </c>
+      <c r="G540" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H540" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I540" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J540" s="3" t="inlineStr">
+        <is>
+          <t>+380 67 678 0959 / service@vip.te.ua</t>
+        </is>
+      </c>
+      <c r="K540" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L540" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M540" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N540" s="3" t="inlineStr"/>
+      <c r="O540" s="3" t="inlineStr"/>
+      <c r="P540" s="3" t="inlineStr"/>
+      <c r="Q540" s="3" t="inlineStr"/>
+    </row>
+    <row r="541">
+      <c r="A541" s="3" t="inlineStr">
+        <is>
+          <t>Serhii Maksymenko</t>
+        </is>
+      </c>
+      <c r="B541" s="3" t="inlineStr">
+        <is>
+          <t>乌克兰</t>
+        </is>
+      </c>
+      <c r="C541" s="3" t="inlineStr">
+        <is>
+          <t>Dnipro</t>
+        </is>
+      </c>
+      <c r="D541" s="3" t="inlineStr"/>
+      <c r="E541" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F541" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G541" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H541" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I541" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J541" s="3" t="inlineStr">
+        <is>
+          <t>+380 67 551 7229 / studio4face@gmail.com</t>
+        </is>
+      </c>
+      <c r="K541" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L541" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M541" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N541" s="3" t="inlineStr"/>
+      <c r="O541" s="3" t="inlineStr"/>
+      <c r="P541" s="3" t="inlineStr"/>
+      <c r="Q541" s="3" t="inlineStr">
+        <is>
+          <t>含 MTCEWE（企业无线）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
UK consultants: 13, with LinITX holding three of them
LinITX is a UK master distributor, value-added distributor and training
centre with three certified consultants on staff, so its existing
distributor row is enriched with all three names rather than adding
duplicate rows. Ron Touw and Barry Higgins both hold all ten
certifications and are trainers, which makes them reach multipliers.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q541"/>
+  <dimension ref="A1:Q551"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -49922,6 +49922,752 @@
       <c r="Q541" s="3" t="inlineStr">
         <is>
           <t>含 MTCEWE（企业无线）</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" s="3" t="inlineStr">
+        <is>
+          <t>Ron Touw / MikroTik Training UK</t>
+        </is>
+      </c>
+      <c r="B542" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C542" s="3" t="inlineStr">
+        <is>
+          <t>Whitstable</t>
+        </is>
+      </c>
+      <c r="D542" s="3" t="inlineStr">
+        <is>
+          <t>mikrotiktraining.co.uk</t>
+        </is>
+      </c>
+      <c r="E542" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F542" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 10 证全拿</t>
+        </is>
+      </c>
+      <c r="G542" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H542" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I542" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J542" s="3" t="inlineStr">
+        <is>
+          <t>+44 1227 314316 / training@hoka.co.uk</t>
+        </is>
+      </c>
+      <c r="K542" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L542" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M542" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N542" s="3" t="inlineStr"/>
+      <c r="O542" s="3" t="inlineStr"/>
+      <c r="P542" s="3" t="inlineStr"/>
+      <c r="Q542" s="3" t="inlineStr">
+        <is>
+          <t>★ 10 证全拿 + 英国培训讲师；无线勘测与设计、固定网络基础设施设计、BGP/MPLS/VPLS/OSPF、流量管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" s="3" t="inlineStr">
+        <is>
+          <t>Barry Higgins / Allness</t>
+        </is>
+      </c>
+      <c r="B543" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C543" s="3" t="inlineStr">
+        <is>
+          <t>Kidderminster</t>
+        </is>
+      </c>
+      <c r="D543" s="3" t="inlineStr">
+        <is>
+          <t>allness.net</t>
+        </is>
+      </c>
+      <c r="E543" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F543" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 10 证全拿</t>
+        </is>
+      </c>
+      <c r="G543" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H543" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I543" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J543" s="3" t="inlineStr">
+        <is>
+          <t>+44 3333 403 303 / barry@allness.it</t>
+        </is>
+      </c>
+      <c r="K543" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L543" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M543" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N543" s="3" t="inlineStr"/>
+      <c r="O543" s="3" t="inlineStr"/>
+      <c r="P543" s="3" t="inlineStr"/>
+      <c r="Q543" s="3" t="inlineStr">
+        <is>
+          <t>★ 10 证全拿 + 英国 MikroTik 官方讲师；有线+无线设计、OSPF/IS-IS/iBGP/eBGP、RouterOS 脚本</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="3" t="inlineStr">
+        <is>
+          <t>Jono Thompson / LinITX</t>
+        </is>
+      </c>
+      <c r="B544" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C544" s="3" t="inlineStr">
+        <is>
+          <t>Needham Market</t>
+        </is>
+      </c>
+      <c r="D544" s="3" t="inlineStr">
+        <is>
+          <t>linitx.com</t>
+        </is>
+      </c>
+      <c r="E544" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F544" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCTCE+MTCUME+MTCINE+MTCSWE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G544" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H544" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I544" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J544" s="3" t="inlineStr">
+        <is>
+          <t>+44 1449 888000 / training@linitx.com</t>
+        </is>
+      </c>
+      <c r="K544" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L544" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M544" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N544" s="3" t="inlineStr"/>
+      <c r="O544" s="3" t="inlineStr"/>
+      <c r="P544" s="3" t="inlineStr"/>
+      <c r="Q544" s="3" t="inlineStr">
+        <is>
+          <t>LinITX 是英国 MikroTik Master Distributor + VAD + 认证培训中心，公司内有 3 位认证顾问：Jono Thompson（training@linitx.com，7 证含 MTCSWE，交换/VLAN/CAPsMAN/流量管理）；Joel Blakey（MikroTik@LinITX.com，技术销售工程师，有线无线设计与无线勘测）；Luke Cuddehay（shop@linitx.com，技术销售工程师）。同一电话 +44 1449 888000</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" s="3" t="inlineStr">
+        <is>
+          <t>Jason Ede / ASK4</t>
+        </is>
+      </c>
+      <c r="B545" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C545" s="3" t="inlineStr">
+        <is>
+          <t>Sheffield</t>
+        </is>
+      </c>
+      <c r="D545" s="3" t="inlineStr">
+        <is>
+          <t>ask4.com</t>
+        </is>
+      </c>
+      <c r="E545" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F545" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCTCE+MTCINE+MTCSE+MTCSWE</t>
+        </is>
+      </c>
+      <c r="G545" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H545" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I545" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J545" s="3" t="inlineStr">
+        <is>
+          <t>+44 114 321 0555 / jason.ede@ask4.com</t>
+        </is>
+      </c>
+      <c r="K545" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L545" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M545" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N545" s="3" t="inlineStr"/>
+      <c r="O545" s="3" t="inlineStr"/>
+      <c r="P545" s="3" t="inlineStr"/>
+      <c r="Q545" s="3" t="inlineStr">
+        <is>
+          <t>★ 持 MTCSWE；ASK4 是英国大型 ISP（学生公寓/MDU 宽带）；技能含交换、VLAN、防火墙、路由、专线</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" s="3" t="inlineStr">
+        <is>
+          <t>Peter Freeman / Freeclix</t>
+        </is>
+      </c>
+      <c r="B546" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C546" s="3" t="inlineStr">
+        <is>
+          <t>Rackheath (Norwich)</t>
+        </is>
+      </c>
+      <c r="D546" s="3" t="inlineStr">
+        <is>
+          <t>freeclix.com</t>
+        </is>
+      </c>
+      <c r="E546" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F546" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSWE</t>
+        </is>
+      </c>
+      <c r="G546" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H546" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I546" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J546" s="3" t="inlineStr">
+        <is>
+          <t>+44 1603 703340 / sales@freeclix.com</t>
+        </is>
+      </c>
+      <c r="K546" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L546" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M546" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N546" s="3" t="inlineStr"/>
+      <c r="O546" s="3" t="inlineStr"/>
+      <c r="P546" s="3" t="inlineStr"/>
+      <c r="Q546" s="3" t="inlineStr">
+        <is>
+          <t>★ 持 MTCSWE；4G/5G 方案、ISP 服务、光纤专线/xDSL/FTTC、机柜托管、语音；**SimRush Master Distributor**</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" s="3" t="inlineStr">
+        <is>
+          <t>Nick Shore</t>
+        </is>
+      </c>
+      <c r="B547" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C547" s="3" t="inlineStr">
+        <is>
+          <t>Debenham</t>
+        </is>
+      </c>
+      <c r="D547" s="3" t="inlineStr">
+        <is>
+          <t>shore.me.uk</t>
+        </is>
+      </c>
+      <c r="E547" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F547" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G547" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H547" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I547" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J547" s="3" t="inlineStr">
+        <is>
+          <t>+44 7588 286095 / nick@shore.me.uk</t>
+        </is>
+      </c>
+      <c r="K547" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L547" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M547" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N547" s="3" t="inlineStr"/>
+      <c r="O547" s="3" t="inlineStr"/>
+      <c r="P547" s="3" t="inlineStr"/>
+      <c r="Q547" s="3" t="inlineStr">
+        <is>
+          <t>WISP/ISP 方向；BGP、OSPF、防火墙、动态路由、流量管理、**switching**、VPN、CAPsMAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="3" t="inlineStr">
+        <is>
+          <t>Bamidele Richard Amire / Nistech</t>
+        </is>
+      </c>
+      <c r="B548" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C548" s="3" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D548" s="3" t="inlineStr">
+        <is>
+          <t>nistechltd.net</t>
+        </is>
+      </c>
+      <c r="E548" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F548" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCTCE+MTCUME+MTCINE+MTCIPv6E</t>
+        </is>
+      </c>
+      <c r="G548" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H548" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I548" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J548" s="3" t="inlineStr">
+        <is>
+          <t>+44 7498 168213 / richard@nistechltd.net</t>
+        </is>
+      </c>
+      <c r="K548" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L548" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M548" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N548" s="3" t="inlineStr"/>
+      <c r="O548" s="3" t="inlineStr"/>
+      <c r="P548" s="3" t="inlineStr"/>
+      <c r="Q548" s="3" t="inlineStr">
+        <is>
+          <t>多厂商集成、MPLS/VRF、QoS、策略路由、大型无线与**光纤网络**、Hotspot/User-Manager、IPv6 部署</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" s="3" t="inlineStr">
+        <is>
+          <t>Iyiola Folayan / Millie Evolution</t>
+        </is>
+      </c>
+      <c r="B549" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C549" s="3" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D549" s="3" t="inlineStr">
+        <is>
+          <t>millievolution.com</t>
+        </is>
+      </c>
+      <c r="E549" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F549" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCUME+MTCINE</t>
+        </is>
+      </c>
+      <c r="G549" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H549" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I549" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J549" s="3" t="inlineStr">
+        <is>
+          <t>+44 7783 315527 / ifolayan@millievolution.com</t>
+        </is>
+      </c>
+      <c r="K549" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L549" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M549" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N549" s="3" t="inlineStr"/>
+      <c r="O549" s="3" t="inlineStr"/>
+      <c r="P549" s="3" t="inlineStr"/>
+      <c r="Q549" s="3" t="inlineStr">
+        <is>
+          <t>18 年 IP 工程：宽带基础设施设计、IP 网络部署运维、4G/LTE、园区**光纤**网、Hotspot/User-Manager</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="3" t="inlineStr">
+        <is>
+          <t>Adam Reid / HP Networks</t>
+        </is>
+      </c>
+      <c r="B550" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C550" s="3" t="inlineStr">
+        <is>
+          <t>Belfast（北爱）</t>
+        </is>
+      </c>
+      <c r="D550" s="3" t="inlineStr">
+        <is>
+          <t>hpnetworks.net</t>
+        </is>
+      </c>
+      <c r="E550" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F550" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G550" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H550" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I550" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J550" s="3" t="inlineStr">
+        <is>
+          <t>+44 28 9008 0030 / Adam@hpnetworks.net</t>
+        </is>
+      </c>
+      <c r="K550" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L550" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M550" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N550" s="3" t="inlineStr"/>
+      <c r="O550" s="3" t="inlineStr"/>
+      <c r="P550" s="3" t="inlineStr"/>
+      <c r="Q550" s="3" t="inlineStr"/>
+    </row>
+    <row r="551">
+      <c r="A551" s="3" t="inlineStr">
+        <is>
+          <t>Samson Kamwendo / IP Architechs</t>
+        </is>
+      </c>
+      <c r="B551" s="3" t="inlineStr">
+        <is>
+          <t>英国</t>
+        </is>
+      </c>
+      <c r="C551" s="3" t="inlineStr">
+        <is>
+          <t>Peterborough</t>
+        </is>
+      </c>
+      <c r="D551" s="3" t="inlineStr">
+        <is>
+          <t>iparchitechs.com</t>
+        </is>
+      </c>
+      <c r="E551" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F551" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCUME</t>
+        </is>
+      </c>
+      <c r="G551" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H551" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I551" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J551" s="3" t="inlineStr">
+        <is>
+          <t>+44 7778 431460 / samson.kamwendo@iparchitechs.com</t>
+        </is>
+      </c>
+      <c r="K551" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L551" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M551" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N551" s="3" t="inlineStr"/>
+      <c r="O551" s="3" t="inlineStr"/>
+      <c r="P551" s="3" t="inlineStr"/>
+      <c r="Q551" s="3" t="inlineStr">
+        <is>
+          <t>含 MTCUME（用户管理）→ Hotspot 方向</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Dutch consultants: 14, including a presales consultant at a VAD
Aris Vink works as a presales consultant and trainer at a MikroTik
value-added master distributor, which is the same category-manager
entry route found at 100MEGA in Czechia. Three Dutch consultants hold
all ten certifications, and Maher Haddad lists switching explicitly.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q551"/>
+  <dimension ref="A1:Q564"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -50670,6 +50670,961 @@
           <t>含 MTCUME（用户管理）→ Hotspot 方向</t>
         </is>
       </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="3" t="inlineStr">
+        <is>
+          <t>Aris Vink / SDC</t>
+        </is>
+      </c>
+      <c r="B552" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C552" s="3" t="inlineStr">
+        <is>
+          <t>Zoetermeer</t>
+        </is>
+      </c>
+      <c r="D552" s="3" t="inlineStr">
+        <is>
+          <t>sdc.nl</t>
+        </is>
+      </c>
+      <c r="E552" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F552" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G552" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H552" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I552" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J552" s="3" t="inlineStr">
+        <is>
+          <t>+31 6 17552148 / aris@sdc.nl</t>
+        </is>
+      </c>
+      <c r="K552" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L552" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M552" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N552" s="3" t="inlineStr"/>
+      <c r="O552" s="3" t="inlineStr"/>
+      <c r="P552" s="3" t="inlineStr"/>
+      <c r="Q552" s="3" t="inlineStr">
+        <is>
+          <t>★ 自述在某 MikroTik **Value Added Master Distributor 做售前顾问 + 认证讲师**，帮代理商设计/实施/运维 MikroTik 网络 →  distributor 内部的人，最接近「品类经理」入口</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" s="3" t="inlineStr">
+        <is>
+          <t>Maher Haddad / MyNetworkTraining</t>
+        </is>
+      </c>
+      <c r="B553" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C553" s="3" t="inlineStr">
+        <is>
+          <t>Hilversum</t>
+        </is>
+      </c>
+      <c r="D553" s="3" t="inlineStr">
+        <is>
+          <t>mynetworktraining.com</t>
+        </is>
+      </c>
+      <c r="E553" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F553" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 10 证全拿</t>
+        </is>
+      </c>
+      <c r="G553" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H553" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I553" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J553" s="3" t="inlineStr">
+        <is>
+          <t>+31 6 22488675 / info@mynetworktraining.com</t>
+        </is>
+      </c>
+      <c r="K553" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L553" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M553" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N553" s="3" t="inlineStr"/>
+      <c r="O553" s="3" t="inlineStr"/>
+      <c r="P553" s="3" t="inlineStr"/>
+      <c r="Q553" s="3" t="inlineStr">
+        <is>
+          <t>★ 10 证全拿 + 认证讲师，20+ 年 IT；技能清单明确含 **Switching**、MPLS/VPLS、The Dude、CAPsMAN、流量控制</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="3" t="inlineStr">
+        <is>
+          <t>Maurice van der Grijspaarde / GPE Networks</t>
+        </is>
+      </c>
+      <c r="B554" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C554" s="3" t="inlineStr">
+        <is>
+          <t>Haarlem</t>
+        </is>
+      </c>
+      <c r="D554" s="3" t="inlineStr">
+        <is>
+          <t>gpe-networks.com</t>
+        </is>
+      </c>
+      <c r="E554" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F554" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 10 证全拿</t>
+        </is>
+      </c>
+      <c r="G554" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H554" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I554" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J554" s="3" t="inlineStr">
+        <is>
+          <t>+31 23 7640540 / info@gpe-networks.com</t>
+        </is>
+      </c>
+      <c r="K554" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L554" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M554" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N554" s="3" t="inlineStr"/>
+      <c r="O554" s="3" t="inlineStr"/>
+      <c r="P554" s="3" t="inlineStr"/>
+      <c r="Q554" s="3" t="inlineStr">
+        <is>
+          <t>★ 10 证全拿；2015 年起专职 MikroTik，专做复杂场景方案</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" s="3" t="inlineStr">
+        <is>
+          <t>MikroTrain（荷兰 MikroTik 培训）</t>
+        </is>
+      </c>
+      <c r="B555" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C555" s="3" t="inlineStr"/>
+      <c r="D555" s="3" t="inlineStr">
+        <is>
+          <t>mikrotrain.nl</t>
+        </is>
+      </c>
+      <c r="E555" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F555" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 认证讲师（教 MTCNA→MTCINE 全部课程）</t>
+        </is>
+      </c>
+      <c r="G555" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H555" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I555" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J555" s="3" t="inlineStr">
+        <is>
+          <t>+31 6 12224005 / info@mikrotrain.nl</t>
+        </is>
+      </c>
+      <c r="K555" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L555" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M555" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N555" s="3" t="inlineStr"/>
+      <c r="O555" s="3" t="inlineStr"/>
+      <c r="P555" s="3" t="inlineStr"/>
+      <c r="Q555" s="3" t="inlineStr">
+        <is>
+          <t>★ 荷兰 MikroTik 培训机构，教全部等级课程；也接项目支持、WiFi 测试、站点勘测、安全评估</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" s="3" t="inlineStr">
+        <is>
+          <t>Menno van Krimpen / Libernet</t>
+        </is>
+      </c>
+      <c r="B556" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C556" s="3" t="inlineStr">
+        <is>
+          <t>Werkendam</t>
+        </is>
+      </c>
+      <c r="D556" s="3" t="inlineStr">
+        <is>
+          <t>libernet.nl</t>
+        </is>
+      </c>
+      <c r="E556" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F556" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE</t>
+        </is>
+      </c>
+      <c r="G556" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H556" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I556" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J556" s="3" t="inlineStr">
+        <is>
+          <t>+31 85 902 1012 / info@libernet.nl</t>
+        </is>
+      </c>
+      <c r="K556" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L556" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M556" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N556" s="3" t="inlineStr"/>
+      <c r="O556" s="3" t="inlineStr"/>
+      <c r="P556" s="3" t="inlineStr"/>
+      <c r="Q556" s="3" t="inlineStr">
+        <is>
+          <t>★ 荷兰第一位 MikroTik 认证讲师；资深 WISP 运营商，PtP/PtMP、VoIP、Hotspot、流量整形、负载均衡；可上门培训</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" s="3" t="inlineStr">
+        <is>
+          <t>Michiel Visser / Connection Services</t>
+        </is>
+      </c>
+      <c r="B557" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C557" s="3" t="inlineStr">
+        <is>
+          <t>Deventer</t>
+        </is>
+      </c>
+      <c r="D557" s="3" t="inlineStr">
+        <is>
+          <t>connectionservices.nl</t>
+        </is>
+      </c>
+      <c r="E557" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F557" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCINE+MTCIPv6E+MTCSE</t>
+        </is>
+      </c>
+      <c r="G557" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H557" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I557" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J557" s="3" t="inlineStr">
+        <is>
+          <t>+31 6 29047127 / michiel@connectionservices.nl</t>
+        </is>
+      </c>
+      <c r="K557" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L557" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M557" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N557" s="3" t="inlineStr"/>
+      <c r="O557" s="3" t="inlineStr"/>
+      <c r="P557" s="3" t="inlineStr"/>
+      <c r="Q557" s="3" t="inlineStr">
+        <is>
+          <t>含 MTCINE（ISP 互联）+ MTCWE（无线）</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="3" t="inlineStr">
+        <is>
+          <t>Stephan Szarafinski / MNW</t>
+        </is>
+      </c>
+      <c r="B558" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C558" s="3" t="inlineStr">
+        <is>
+          <t>Bussum</t>
+        </is>
+      </c>
+      <c r="D558" s="3" t="inlineStr">
+        <is>
+          <t>mnw.nl</t>
+        </is>
+      </c>
+      <c r="E558" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F558" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE</t>
+        </is>
+      </c>
+      <c r="G558" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H558" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I558" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J558" s="3" t="inlineStr">
+        <is>
+          <t>+31 35 6426800 / stephan@mnw.nl</t>
+        </is>
+      </c>
+      <c r="K558" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L558" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M558" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N558" s="3" t="inlineStr"/>
+      <c r="O558" s="3" t="inlineStr"/>
+      <c r="P558" s="3" t="inlineStr"/>
+      <c r="Q558" s="3" t="inlineStr">
+        <is>
+          <t>自述 2003 年起做 MikroTik 专家 → 荷兰最早一批用户，影响力型</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" s="3" t="inlineStr">
+        <is>
+          <t>Jasper Hagoort / Dside</t>
+        </is>
+      </c>
+      <c r="B559" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C559" s="3" t="inlineStr">
+        <is>
+          <t>Geertruidenberg</t>
+        </is>
+      </c>
+      <c r="D559" s="3" t="inlineStr">
+        <is>
+          <t>dside.nl</t>
+        </is>
+      </c>
+      <c r="E559" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F559" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCWE+MTCTCE+MTCIPv6E+MTCSE</t>
+        </is>
+      </c>
+      <c r="G559" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H559" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I559" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J559" s="3" t="inlineStr">
+        <is>
+          <t>+31 6 50462617 / jasper@dside.nl</t>
+        </is>
+      </c>
+      <c r="K559" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L559" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M559" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N559" s="3" t="inlineStr"/>
+      <c r="O559" s="3" t="inlineStr"/>
+      <c r="P559" s="3" t="inlineStr"/>
+      <c r="Q559" s="3" t="inlineStr">
+        <is>
+          <t>含 MTCTCE（流量控制）+ MTCSE（安全）</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" s="3" t="inlineStr">
+        <is>
+          <t>Corné van Halteren / DAEL</t>
+        </is>
+      </c>
+      <c r="B560" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C560" s="3" t="inlineStr">
+        <is>
+          <t>'s-Hertogenbosch</t>
+        </is>
+      </c>
+      <c r="D560" s="3" t="inlineStr">
+        <is>
+          <t>dael.com</t>
+        </is>
+      </c>
+      <c r="E560" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F560" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G560" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H560" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I560" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J560" s="3" t="inlineStr">
+        <is>
+          <t>+31 6 28026574 / corne.vanhalteren@dael.com</t>
+        </is>
+      </c>
+      <c r="K560" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L560" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M560" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N560" s="3" t="inlineStr"/>
+      <c r="O560" s="3" t="inlineStr"/>
+      <c r="P560" s="3" t="inlineStr"/>
+      <c r="Q560" s="3" t="inlineStr">
+        <is>
+          <t>DAEL 公司有 2 位 MikroTik 顾问；网络规划、实施与 MikroTik 硬件管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" s="3" t="inlineStr">
+        <is>
+          <t>Jeroen Bleuel</t>
+        </is>
+      </c>
+      <c r="B561" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C561" s="3" t="inlineStr">
+        <is>
+          <t>Reduzum</t>
+        </is>
+      </c>
+      <c r="D561" s="3" t="inlineStr"/>
+      <c r="E561" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F561" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCSE</t>
+        </is>
+      </c>
+      <c r="G561" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H561" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I561" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J561" s="3" t="inlineStr">
+        <is>
+          <t>+31 6 38920124 / jeroen.bleuel@gmail.com</t>
+        </is>
+      </c>
+      <c r="K561" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L561" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M561" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N561" s="3" t="inlineStr"/>
+      <c r="O561" s="3" t="inlineStr"/>
+      <c r="P561" s="3" t="inlineStr"/>
+      <c r="Q561" s="3" t="inlineStr">
+        <is>
+          <t>英德荷三语</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" s="3" t="inlineStr">
+        <is>
+          <t>Jan Geert Hek / Qtopia</t>
+        </is>
+      </c>
+      <c r="B562" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C562" s="3" t="inlineStr">
+        <is>
+          <t>Heelweg</t>
+        </is>
+      </c>
+      <c r="D562" s="3" t="inlineStr">
+        <is>
+          <t>qtopia.nl</t>
+        </is>
+      </c>
+      <c r="E562" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F562" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G562" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H562" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I562" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J562" s="3" t="inlineStr">
+        <is>
+          <t>+31 6 47764254 / j.g.hek@qtopia.nl</t>
+        </is>
+      </c>
+      <c r="K562" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L562" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M562" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N562" s="3" t="inlineStr"/>
+      <c r="O562" s="3" t="inlineStr"/>
+      <c r="P562" s="3" t="inlineStr"/>
+      <c r="Q562" s="3" t="inlineStr"/>
+    </row>
+    <row r="563">
+      <c r="A563" s="3" t="inlineStr">
+        <is>
+          <t>Robbin van den Berg / RvdB ICT</t>
+        </is>
+      </c>
+      <c r="B563" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C563" s="3" t="inlineStr">
+        <is>
+          <t>IJsselstein</t>
+        </is>
+      </c>
+      <c r="D563" s="3" t="inlineStr">
+        <is>
+          <t>rvdbict.nl</t>
+        </is>
+      </c>
+      <c r="E563" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F563" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSE</t>
+        </is>
+      </c>
+      <c r="G563" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H563" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I563" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J563" s="3" t="inlineStr">
+        <is>
+          <t>+31 6 19600106 / Info@rvdbict.nl</t>
+        </is>
+      </c>
+      <c r="K563" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L563" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M563" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N563" s="3" t="inlineStr"/>
+      <c r="O563" s="3" t="inlineStr"/>
+      <c r="P563" s="3" t="inlineStr"/>
+      <c r="Q563" s="3" t="inlineStr"/>
+    </row>
+    <row r="564">
+      <c r="A564" s="3" t="inlineStr">
+        <is>
+          <t>Fokko van den Bosch</t>
+        </is>
+      </c>
+      <c r="B564" s="3" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C564" s="3" t="inlineStr">
+        <is>
+          <t>Den Haag</t>
+        </is>
+      </c>
+      <c r="D564" s="3" t="inlineStr">
+        <is>
+          <t>it-support.nl</t>
+        </is>
+      </c>
+      <c r="E564" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F564" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G564" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H564" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I564" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J564" s="3" t="inlineStr">
+        <is>
+          <t>+31 6 24259171 / fokko@it-support.nl</t>
+        </is>
+      </c>
+      <c r="K564" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L564" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M564" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N564" s="3" t="inlineStr"/>
+      <c r="O564" s="3" t="inlineStr"/>
+      <c r="P564" s="3" t="inlineStr"/>
+      <c r="Q564" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
France and Spain consultants, plus a reusable batch import script
France yields two consultants. Spain yields 23 people across 20
companies, led by Fibercli, which runs its own MikroTik certified
training centre and serves IBEX35 customers across hospitality,
telco and oil and gas. Carlos Otin works on hotel and multi-site
networks with switching and GPON, and Carlos Villalobos is an
industrial engineer on IT/OT convergence.

The new script takes a JSON batch so remaining countries can be
imported without repeating the CSV and workbook boilerplate.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q564"/>
+  <dimension ref="A1:Q586"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -51338,7 +51338,7 @@
       <c r="P560" s="3" t="inlineStr"/>
       <c r="Q560" s="3" t="inlineStr">
         <is>
-          <t>DAEL 公司有 2 位 MikroTik 顾问；网络规划、实施与 MikroTik 硬件管理</t>
+          <t>DAEL 公司有 2 位 MikroTik 顾问：Corné van Halteren（网络规划/实施/MikroTik 硬件管理）；Benito Stijger（benito.stijger@dael.com，+31 6 14333514，MTCSE 安全方向：防火墙、VPN、攻击防护）</t>
         </is>
       </c>
     </row>
@@ -51625,6 +51625,1608 @@
       <c r="O564" s="3" t="inlineStr"/>
       <c r="P564" s="3" t="inlineStr"/>
       <c r="Q564" s="3" t="inlineStr"/>
+    </row>
+    <row r="565">
+      <c r="A565" s="3" t="inlineStr">
+        <is>
+          <t>Habib Kanso</t>
+        </is>
+      </c>
+      <c r="B565" s="3" t="inlineStr">
+        <is>
+          <t>法国</t>
+        </is>
+      </c>
+      <c r="C565" s="3" t="inlineStr">
+        <is>
+          <t>Toulouse</t>
+        </is>
+      </c>
+      <c r="D565" s="3" t="inlineStr"/>
+      <c r="E565" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F565" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCTCE+MTCINE+MTCSE</t>
+        </is>
+      </c>
+      <c r="G565" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H565" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I565" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J565" s="3" t="inlineStr">
+        <is>
+          <t>+33 7 55 26 73 43 / habibkanso@gmail.com</t>
+        </is>
+      </c>
+      <c r="K565" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L565" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M565" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N565" s="3" t="inlineStr"/>
+      <c r="O565" s="3" t="inlineStr"/>
+      <c r="P565" s="3" t="inlineStr"/>
+      <c r="Q565" s="3" t="inlineStr">
+        <is>
+          <t>自述专长为「企业核心网络架构与技术」，含 MTCINE（ISP 互联）+ MTCTCE（流量控制）+ MTCSE（安全）</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" s="3" t="inlineStr">
+        <is>
+          <t>Adnan Rihan</t>
+        </is>
+      </c>
+      <c r="B566" s="3" t="inlineStr">
+        <is>
+          <t>法国</t>
+        </is>
+      </c>
+      <c r="C566" s="3" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D566" s="3" t="inlineStr">
+        <is>
+          <t>rihan.fr</t>
+        </is>
+      </c>
+      <c r="E566" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F566" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCIPv6E</t>
+        </is>
+      </c>
+      <c r="G566" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H566" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I566" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J566" s="3" t="inlineStr">
+        <is>
+          <t>+33 6 78 62 26 20 / adnan+mikrotik@rihan.fr</t>
+        </is>
+      </c>
+      <c r="K566" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L566" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M566" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N566" s="3" t="inlineStr"/>
+      <c r="O566" s="3" t="inlineStr"/>
+      <c r="P566" s="3" t="inlineStr"/>
+      <c r="Q566" s="3" t="inlineStr"/>
+    </row>
+    <row r="567">
+      <c r="A567" s="3" t="inlineStr">
+        <is>
+          <t>Fibercli</t>
+        </is>
+      </c>
+      <c r="B567" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C567" s="3" t="inlineStr"/>
+      <c r="D567" s="3" t="inlineStr">
+        <is>
+          <t>fibercli.com</t>
+        </is>
+      </c>
+      <c r="E567" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F567" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 10 证全拿</t>
+        </is>
+      </c>
+      <c r="G567" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H567" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I567" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J567" s="3" t="inlineStr">
+        <is>
+          <t>Víctor Bolaños +34 605 75 90 75 / victor.bolanos@fibercli.com；José Manuel Román Fernández-Checa +34 652 241 431 / facturacion@fibercli.com</t>
+        </is>
+      </c>
+      <c r="K567" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L567" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M567" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N567" s="3" t="inlineStr"/>
+      <c r="O567" s="3" t="inlineStr"/>
+      <c r="P567" s="3" t="inlineStr"/>
+      <c r="Q567" s="3" t="inlineStr">
+        <is>
+          <t>★★ 西班牙最大的 MikroTik 工程团队之一（自述「全球最大之一」），自带 MikroTik 认证培训中心 lo0.es（已在 10+ 时区开课）；客户覆盖 ISP/Telco、数据中心、**酒店 Hospitality**、零售、银行保险、油气，含 IBEX35 上市企业与公共部门；做 RouterOS + 多厂商集成的设计/部署/支持。公司内 2 位 10 证顾问</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" s="3" t="inlineStr">
+        <is>
+          <t>Celenet</t>
+        </is>
+      </c>
+      <c r="B568" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C568" s="3" t="inlineStr">
+        <is>
+          <t>Beniel (Murcia)</t>
+        </is>
+      </c>
+      <c r="D568" s="3" t="inlineStr">
+        <is>
+          <t>celenet.es</t>
+        </is>
+      </c>
+      <c r="E568" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F568" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 10 证全拿 / 9 证（含 MTCSWE）</t>
+        </is>
+      </c>
+      <c r="G568" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H568" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I568" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J568" s="3" t="inlineStr">
+        <is>
+          <t>Carlos Cardenas Cebrian +34 622 330 440 / ccardenas@celenet.es；Javier Prieto Vera +34 649 395 961 / jprietove@celenet.es</t>
+        </is>
+      </c>
+      <c r="K568" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L568" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M568" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N568" s="3" t="inlineStr"/>
+      <c r="O568" s="3" t="inlineStr"/>
+      <c r="P568" s="3" t="inlineStr"/>
+      <c r="Q568" s="3" t="inlineStr">
+        <is>
+          <t>公司内 2 位顾问，均 9–10 证。Carlos：WISP、OSPF/BGP/MPLS、IPv6 规划、**组播 Multicast**、高可用、负载均衡、流量工程、QoS、CAPsMAN、Hotspot、RouterOS v7。Javier：OSPF/BGP/VLAN/EoIP/MPLS/VPLS、WiFi 部署、带宽管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" s="3" t="inlineStr">
+        <is>
+          <t>Carlos Otin / Hotelinking</t>
+        </is>
+      </c>
+      <c r="B569" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C569" s="3" t="inlineStr">
+        <is>
+          <t>Palma（马略卡）</t>
+        </is>
+      </c>
+      <c r="D569" s="3" t="inlineStr">
+        <is>
+          <t>hotelinking.com</t>
+        </is>
+      </c>
+      <c r="E569" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F569" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSE</t>
+        </is>
+      </c>
+      <c r="G569" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H569" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I569" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J569" s="3" t="inlineStr">
+        <is>
+          <t>+34 691 837 651 / c.otin@hotelinking.com</t>
+        </is>
+      </c>
+      <c r="K569" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L569" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M569" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N569" s="3" t="inlineStr"/>
+      <c r="O569" s="3" t="inlineStr"/>
+      <c r="P569" s="3" t="inlineStr"/>
+      <c r="Q569" s="3" t="inlineStr">
+        <is>
+          <t>★★ 高级网络工程师，专注**酒店 hospitality 与多站点 multi-site** 可扩展网络；专长 MikroTik 路由 + **交换 switching** + 无线 + **GPON 集成**；做网络审计、复杂故障排查、配置标准化、对接监控与自动化平台 → 酒店多站点 = PoE 接入交换机批量需求</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" s="3" t="inlineStr">
+        <is>
+          <t>Carlos Villalobos / Hecnys</t>
+        </is>
+      </c>
+      <c r="B570" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C570" s="3" t="inlineStr">
+        <is>
+          <t>Bormujos (Sevilla)</t>
+        </is>
+      </c>
+      <c r="D570" s="3" t="inlineStr">
+        <is>
+          <t>hecnys.com</t>
+        </is>
+      </c>
+      <c r="E570" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F570" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCTCE</t>
+        </is>
+      </c>
+      <c r="G570" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H570" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I570" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J570" s="3" t="inlineStr">
+        <is>
+          <t>+34 645 396 100 / carlosvillalobos@hecnys.com</t>
+        </is>
+      </c>
+      <c r="K570" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L570" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M570" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N570" s="3" t="inlineStr"/>
+      <c r="O570" s="3" t="inlineStr"/>
+      <c r="P570" s="3" t="inlineStr"/>
+      <c r="Q570" s="3" t="inlineStr">
+        <is>
+          <t>★★ 工业工程师出身，专长 **IT/OT 网络融合（工业场景）**；基于 MikroTik 的架构设计、配置与优化 → 推工业导轨交换机</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" s="3" t="inlineStr">
+        <is>
+          <t>Juan Miguel Gallardo Pérez / Codisa Telco Solutions</t>
+        </is>
+      </c>
+      <c r="B571" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C571" s="3" t="inlineStr">
+        <is>
+          <t>Badajoz</t>
+        </is>
+      </c>
+      <c r="D571" s="3" t="inlineStr">
+        <is>
+          <t>codisats.es</t>
+        </is>
+      </c>
+      <c r="E571" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F571" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCTCE+MTCINE</t>
+        </is>
+      </c>
+      <c r="G571" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H571" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I571" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J571" s="3" t="inlineStr">
+        <is>
+          <t>+34 924 11 11 28 / jmgallardo@codisats.es</t>
+        </is>
+      </c>
+      <c r="K571" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L571" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M571" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N571" s="3" t="inlineStr"/>
+      <c r="O571" s="3" t="inlineStr"/>
+      <c r="P571" s="3" t="inlineStr"/>
+      <c r="Q571" s="3" t="inlineStr">
+        <is>
+          <t>ISP/WISP/**FTTx** 工程师；高可用、安全、访问控制、MPLS、动态路由、流量控制、脚本、VPN；可远程支持</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" s="3" t="inlineStr">
+        <is>
+          <t>Jaime Fuentes</t>
+        </is>
+      </c>
+      <c r="B572" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C572" s="3" t="inlineStr">
+        <is>
+          <t>Alcalá la Real</t>
+        </is>
+      </c>
+      <c r="D572" s="3" t="inlineStr"/>
+      <c r="E572" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F572" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCTCE</t>
+        </is>
+      </c>
+      <c r="G572" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H572" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I572" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J572" s="3" t="inlineStr">
+        <is>
+          <t>+34 615 800 589 / jaimefuentesit@gmail.com</t>
+        </is>
+      </c>
+      <c r="K572" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L572" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M572" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N572" s="3" t="inlineStr"/>
+      <c r="O572" s="3" t="inlineStr"/>
+      <c r="P572" s="3" t="inlineStr"/>
+      <c r="Q572" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 讲师，专做 ISP/WISP 网络设计与技术支持；技能含 **FTTH**、OSPF/BGP/MPLS/VPLS、CAPsMAN、Hotspot、The Dude、RADIUS、LibreNMS、Python</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" s="3" t="inlineStr">
+        <is>
+          <t>Darío Noguera / Lanpixel</t>
+        </is>
+      </c>
+      <c r="B573" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C573" s="3" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="D573" s="3" t="inlineStr">
+        <is>
+          <t>lanpixel.com</t>
+        </is>
+      </c>
+      <c r="E573" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F573" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCSE</t>
+        </is>
+      </c>
+      <c r="G573" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H573" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I573" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J573" s="3" t="inlineStr">
+        <is>
+          <t>+34 660 306 934 / dario@lanpixel.com</t>
+        </is>
+      </c>
+      <c r="K573" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L573" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M573" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N573" s="3" t="inlineStr"/>
+      <c r="O573" s="3" t="inlineStr"/>
+      <c r="P573" s="3" t="inlineStr"/>
+      <c r="Q573" s="3" t="inlineStr">
+        <is>
+          <t>15+ 年，既做培训也做生产网络设计；防火墙加固、VPN/IPSec、流量管理、QoS、高可用；兼 Linux/自动化/RADIUS/监控</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" s="3" t="inlineStr">
+        <is>
+          <t>Jorge Castellet Marques</t>
+        </is>
+      </c>
+      <c r="B574" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C574" s="3" t="inlineStr">
+        <is>
+          <t>Castellón de la Plana</t>
+        </is>
+      </c>
+      <c r="D574" s="3" t="inlineStr">
+        <is>
+          <t>yatuaprendes.com</t>
+        </is>
+      </c>
+      <c r="E574" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F574" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCTCE+MTCINE+MTCIPv6E+MTCSE</t>
+        </is>
+      </c>
+      <c r="G574" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H574" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I574" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J574" s="3" t="inlineStr">
+        <is>
+          <t>+34 717 705 653 / j.castellet@yatuaprendes.com</t>
+        </is>
+      </c>
+      <c r="K574" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L574" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M574" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N574" s="3" t="inlineStr"/>
+      <c r="O574" s="3" t="inlineStr"/>
+      <c r="P574" s="3" t="inlineStr"/>
+      <c r="Q574" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 全科目认证讲师；从小型网到企业网与 ISP；还做 MikroTik 与 ACS 系统的集成</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" s="3" t="inlineStr">
+        <is>
+          <t>Giancarlos Bejarano Bordones</t>
+        </is>
+      </c>
+      <c r="B575" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C575" s="3" t="inlineStr">
+        <is>
+          <t>Zaragoza</t>
+        </is>
+      </c>
+      <c r="D575" s="3" t="inlineStr"/>
+      <c r="E575" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F575" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCINE+MTCSE</t>
+        </is>
+      </c>
+      <c r="G575" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H575" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I575" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J575" s="3" t="inlineStr">
+        <is>
+          <t>+34 604 819 851 / giancbeja@gmail.com</t>
+        </is>
+      </c>
+      <c r="K575" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L575" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M575" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N575" s="3" t="inlineStr"/>
+      <c r="O575" s="3" t="inlineStr"/>
+      <c r="P575" s="3" t="inlineStr"/>
+      <c r="Q575" s="3" t="inlineStr">
+        <is>
+          <t>系统与网络安全工程师；**IGMP**、VLAN、OSPF/MPLS、QoS/CoS/DSCP、IPSec、多 WAN 负载均衡、DoS 防护、Hotspot 与强制门户</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" s="3" t="inlineStr">
+        <is>
+          <t>Martin Ruiz / Ibersystems</t>
+        </is>
+      </c>
+      <c r="B576" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C576" s="3" t="inlineStr">
+        <is>
+          <t>Mataró</t>
+        </is>
+      </c>
+      <c r="D576" s="3" t="inlineStr">
+        <is>
+          <t>ibersystems.es</t>
+        </is>
+      </c>
+      <c r="E576" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F576" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCSE</t>
+        </is>
+      </c>
+      <c r="G576" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H576" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I576" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J576" s="3" t="inlineStr">
+        <is>
+          <t>+34 669 379 521 / Martinruiz@ibersystems.es</t>
+        </is>
+      </c>
+      <c r="K576" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L576" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M576" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N576" s="3" t="inlineStr"/>
+      <c r="O576" s="3" t="inlineStr"/>
+      <c r="P576" s="3" t="inlineStr"/>
+      <c r="Q576" s="3" t="inlineStr">
+        <is>
+          <t>高可用、无线 PtP/PtMP/Mesh、HotSpot、QoS、代理/防火墙、VPN；远程与现场支持</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" s="3" t="inlineStr">
+        <is>
+          <t>Santiago Balaguer Garcia</t>
+        </is>
+      </c>
+      <c r="B577" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C577" s="3" t="inlineStr">
+        <is>
+          <t>Castellón de la Plana</t>
+        </is>
+      </c>
+      <c r="D577" s="3" t="inlineStr">
+        <is>
+          <t>cursos-mikrotik.com</t>
+        </is>
+      </c>
+      <c r="E577" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F577" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCTCE+MTCINE</t>
+        </is>
+      </c>
+      <c r="G577" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H577" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I577" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J577" s="3" t="inlineStr">
+        <is>
+          <t>+34 960 802 505 / santiagoayodar@hotmail.com</t>
+        </is>
+      </c>
+      <c r="K577" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L577" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M577" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N577" s="3" t="inlineStr"/>
+      <c r="O577" s="3" t="inlineStr"/>
+      <c r="P577" s="3" t="inlineStr"/>
+      <c r="Q577" s="3" t="inlineStr">
+        <is>
+          <t>开 MikroTik 课程（cursos-mikrotik.com）；Diameter 协议、HotSpot、PPPoE/PPtP/L2TP/OVPN、AAA、高可用、**无线骨干网**</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" s="3" t="inlineStr">
+        <is>
+          <t>Ricardo Bernao Gonzalez / Stratonetworks</t>
+        </is>
+      </c>
+      <c r="B578" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C578" s="3" t="inlineStr">
+        <is>
+          <t>Daganzo de Arriba (Madrid)</t>
+        </is>
+      </c>
+      <c r="D578" s="3" t="inlineStr">
+        <is>
+          <t>stratonetworks.com</t>
+        </is>
+      </c>
+      <c r="E578" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F578" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCWE</t>
+        </is>
+      </c>
+      <c r="G578" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H578" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I578" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J578" s="3" t="inlineStr">
+        <is>
+          <t>+34 657 478 596 / ricardo@stratonetworks.com</t>
+        </is>
+      </c>
+      <c r="K578" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L578" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M578" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N578" s="3" t="inlineStr"/>
+      <c r="O578" s="3" t="inlineStr"/>
+      <c r="P578" s="3" t="inlineStr"/>
+      <c r="Q578" s="3" t="inlineStr">
+        <is>
+          <t>15+ 年 MikroTik/RouterOS 实施经验，同时是 MikroTik 讲师</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" s="3" t="inlineStr">
+        <is>
+          <t>Xavier Poza</t>
+        </is>
+      </c>
+      <c r="B579" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C579" s="3" t="inlineStr">
+        <is>
+          <t>Llinars del Vallès</t>
+        </is>
+      </c>
+      <c r="D579" s="3" t="inlineStr"/>
+      <c r="E579" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F579" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCINE+MTCIPv6E</t>
+        </is>
+      </c>
+      <c r="G579" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H579" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I579" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J579" s="3" t="inlineStr">
+        <is>
+          <t>+34 938 481 901 / xavinetworks@gmail.com</t>
+        </is>
+      </c>
+      <c r="K579" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L579" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M579" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N579" s="3" t="inlineStr"/>
+      <c r="O579" s="3" t="inlineStr"/>
+      <c r="P579" s="3" t="inlineStr"/>
+      <c r="Q579" s="3" t="inlineStr">
+        <is>
+          <t>自述方向：开放、自由、中立的公共/社区网络（含 MTCINE 互联）</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" s="3" t="inlineStr">
+        <is>
+          <t>Enric Perpinyà Pitarch / Perpi.tech</t>
+        </is>
+      </c>
+      <c r="B580" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C580" s="3" t="inlineStr">
+        <is>
+          <t>Palma（马略卡）</t>
+        </is>
+      </c>
+      <c r="D580" s="3" t="inlineStr">
+        <is>
+          <t>perpi.tech</t>
+        </is>
+      </c>
+      <c r="E580" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F580" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCSE</t>
+        </is>
+      </c>
+      <c r="G580" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H580" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I580" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J580" s="3" t="inlineStr">
+        <is>
+          <t>+34 657 334 318 / enric@perpi.tech</t>
+        </is>
+      </c>
+      <c r="K580" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L580" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M580" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N580" s="3" t="inlineStr"/>
+      <c r="O580" s="3" t="inlineStr"/>
+      <c r="P580" s="3" t="inlineStr"/>
+      <c r="Q580" s="3" t="inlineStr">
+        <is>
+          <t>Perpi.tech 的 CEO 兼联合创始人 → 决策人本人</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" s="3" t="inlineStr">
+        <is>
+          <t>Jorge Montero</t>
+        </is>
+      </c>
+      <c r="B581" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C581" s="3" t="inlineStr">
+        <is>
+          <t>Leganés (Madrid)</t>
+        </is>
+      </c>
+      <c r="D581" s="3" t="inlineStr"/>
+      <c r="E581" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F581" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCWE+MTCTCE+MTCINE+MTCSE</t>
+        </is>
+      </c>
+      <c r="G581" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H581" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I581" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J581" s="3" t="inlineStr">
+        <is>
+          <t>+34 609 223 659 / cotiti@gmail.com</t>
+        </is>
+      </c>
+      <c r="K581" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L581" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M581" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N581" s="3" t="inlineStr"/>
+      <c r="O581" s="3" t="inlineStr"/>
+      <c r="P581" s="3" t="inlineStr"/>
+      <c r="Q581" s="3" t="inlineStr">
+        <is>
+          <t>含 MTCINE（ISP 互联）+ MTCTCE（流量控制）+ MTCSE（安全）</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" s="3" t="inlineStr">
+        <is>
+          <t>Adrián González Notario</t>
+        </is>
+      </c>
+      <c r="B582" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C582" s="3" t="inlineStr">
+        <is>
+          <t>Madrid</t>
+        </is>
+      </c>
+      <c r="D582" s="3" t="inlineStr">
+        <is>
+          <t>adrnet.site</t>
+        </is>
+      </c>
+      <c r="E582" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F582" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCINE</t>
+        </is>
+      </c>
+      <c r="G582" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H582" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I582" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J582" s="3" t="inlineStr">
+        <is>
+          <t>services@adrnet.site</t>
+        </is>
+      </c>
+      <c r="K582" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L582" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M582" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N582" s="3" t="inlineStr"/>
+      <c r="O582" s="3" t="inlineStr"/>
+      <c r="P582" s="3" t="inlineStr"/>
+      <c r="Q582" s="3" t="inlineStr"/>
+    </row>
+    <row r="583">
+      <c r="A583" s="3" t="inlineStr">
+        <is>
+          <t>David Forteza Rey Casasnovas</t>
+        </is>
+      </c>
+      <c r="B583" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C583" s="3" t="inlineStr">
+        <is>
+          <t>Colonia de Sant Jordi（马略卡）</t>
+        </is>
+      </c>
+      <c r="D583" s="3" t="inlineStr"/>
+      <c r="E583" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F583" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSE</t>
+        </is>
+      </c>
+      <c r="G583" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H583" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I583" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J583" s="3" t="inlineStr">
+        <is>
+          <t>+34 744 408 692 / davidfortezarey@gmail.com</t>
+        </is>
+      </c>
+      <c r="K583" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L583" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M583" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N583" s="3" t="inlineStr"/>
+      <c r="O583" s="3" t="inlineStr"/>
+      <c r="P583" s="3" t="inlineStr"/>
+      <c r="Q583" s="3" t="inlineStr">
+        <is>
+          <t>各类 MikroTik 网络的搭建/配置/排障</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" s="3" t="inlineStr">
+        <is>
+          <t>Jorge Agulló / IT Consultores</t>
+        </is>
+      </c>
+      <c r="B584" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C584" s="3" t="inlineStr">
+        <is>
+          <t>Benidorm</t>
+        </is>
+      </c>
+      <c r="D584" s="3" t="inlineStr">
+        <is>
+          <t>itconsultores.es</t>
+        </is>
+      </c>
+      <c r="E584" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F584" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G584" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H584" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I584" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J584" s="3" t="inlineStr">
+        <is>
+          <t>+34 966 830 220 / jorge.agullo@itconsultores.es</t>
+        </is>
+      </c>
+      <c r="K584" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L584" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M584" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N584" s="3" t="inlineStr"/>
+      <c r="O584" s="3" t="inlineStr"/>
+      <c r="P584" s="3" t="inlineStr"/>
+      <c r="Q584" s="3" t="inlineStr"/>
+    </row>
+    <row r="585">
+      <c r="A585" s="3" t="inlineStr">
+        <is>
+          <t>Arber Reca Sina</t>
+        </is>
+      </c>
+      <c r="B585" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C585" s="3" t="inlineStr">
+        <is>
+          <t>Seville</t>
+        </is>
+      </c>
+      <c r="D585" s="3" t="inlineStr"/>
+      <c r="E585" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F585" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCIPv6E</t>
+        </is>
+      </c>
+      <c r="G585" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H585" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I585" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J585" s="3" t="inlineStr">
+        <is>
+          <t>+34 636 423 442 / arberreca@gmail.com</t>
+        </is>
+      </c>
+      <c r="K585" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L585" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M585" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N585" s="3" t="inlineStr"/>
+      <c r="O585" s="3" t="inlineStr"/>
+      <c r="P585" s="3" t="inlineStr"/>
+      <c r="Q585" s="3" t="inlineStr">
+        <is>
+          <t>路由、防火墙、无线、网络设计、QoS</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" s="3" t="inlineStr">
+        <is>
+          <t>José María Catalá Ortega / Dualcom CB</t>
+        </is>
+      </c>
+      <c r="B586" s="3" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C586" s="3" t="inlineStr">
+        <is>
+          <t>Santa Cruz de La Palma（加那利）</t>
+        </is>
+      </c>
+      <c r="D586" s="3" t="inlineStr">
+        <is>
+          <t>dualcomcb.com</t>
+        </is>
+      </c>
+      <c r="E586" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F586" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G586" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H586" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I586" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J586" s="3" t="inlineStr">
+        <is>
+          <t>+34 620 823 599 / josecat@dualcomcb.com</t>
+        </is>
+      </c>
+      <c r="K586" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L586" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M586" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N586" s="3" t="inlineStr"/>
+      <c r="O586" s="3" t="inlineStr"/>
+      <c r="P586" s="3" t="inlineStr"/>
+      <c r="Q586" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Italian consultants: 21 people across 19 companies
Donato De Meo has run national ISP-scale fabrics with 40 POPs and about
8000 customers at 20 Gbps, which makes him the largest single-consultant
network found so far. Alessandro Campanella holds MTCSWE and serves
system integrators worldwide, and Elia Spadoni owns his own ISP, so he
has somewhere to deploy hardware. PF Tech has three consultants on one
domain and is merged into a single row.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q586"/>
+  <dimension ref="A1:Q605"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -53227,6 +53227,1383 @@
       <c r="O586" s="3" t="inlineStr"/>
       <c r="P586" s="3" t="inlineStr"/>
       <c r="Q586" s="3" t="inlineStr"/>
+    </row>
+    <row r="587">
+      <c r="A587" s="3" t="inlineStr">
+        <is>
+          <t>Donato De Meo</t>
+        </is>
+      </c>
+      <c r="B587" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C587" s="3" t="inlineStr">
+        <is>
+          <t>Ortona</t>
+        </is>
+      </c>
+      <c r="D587" s="3" t="inlineStr"/>
+      <c r="E587" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F587" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCINE+MTCIPv6E</t>
+        </is>
+      </c>
+      <c r="G587" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H587" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I587" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J587" s="3" t="inlineStr">
+        <is>
+          <t>+39 380 432 3838 / demeodonato@gmail.com</t>
+        </is>
+      </c>
+      <c r="K587" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L587" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M587" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N587" s="3" t="inlineStr"/>
+      <c r="O587" s="3" t="inlineStr"/>
+      <c r="P587" s="3" t="inlineStr"/>
+      <c r="Q587" s="3" t="inlineStr">
+        <is>
+          <t>★★ 资深网络工程师：参与多个**国家级 ISP 规模**基础设施设计与 fabric、路由架构、多厂商环境；实管 **40+ POP、约 8000 客户、20 Gbps 流量**；BGP 架构、OSPF/IS-IS/SRv6/IPv6、网络迁移与高可用 → 规模最大的个人顾问之一</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" s="3" t="inlineStr">
+        <is>
+          <t>Alessandro Campanella / 1off</t>
+        </is>
+      </c>
+      <c r="B588" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C588" s="3" t="inlineStr">
+        <is>
+          <t>Mogliano Veneto</t>
+        </is>
+      </c>
+      <c r="D588" s="3" t="inlineStr">
+        <is>
+          <t>1off.it</t>
+        </is>
+      </c>
+      <c r="E588" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F588" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCIPv6E+MTCSE+MTCSWE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G588" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H588" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I588" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J588" s="3" t="inlineStr">
+        <is>
+          <t>+39 320 299 7787 / a.campanella@1off.it</t>
+        </is>
+      </c>
+      <c r="K588" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L588" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M588" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N588" s="3" t="inlineStr"/>
+      <c r="O588" s="3" t="inlineStr"/>
+      <c r="P588" s="3" t="inlineStr"/>
+      <c r="Q588" s="3" t="inlineStr">
+        <is>
+          <t>★★ 持 MTCSWE；2003 年起做 MikroTik、2007 年起当讲师；**Routing + Switching + Wireless + QoS + VPN + 安全**；网络设计/迁移/排障；为全球运营商与系统集成商服务 → 给 SI 供货的机会</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" s="3" t="inlineStr">
+        <is>
+          <t>Alessandro Del Ferro / Bitmagic</t>
+        </is>
+      </c>
+      <c r="B589" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C589" s="3" t="inlineStr">
+        <is>
+          <t>Pesaro</t>
+        </is>
+      </c>
+      <c r="D589" s="3" t="inlineStr">
+        <is>
+          <t>bitmagic.it</t>
+        </is>
+      </c>
+      <c r="E589" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F589" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 8 证（含 MTCSWE+MTCEWE）</t>
+        </is>
+      </c>
+      <c r="G589" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H589" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I589" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J589" s="3" t="inlineStr">
+        <is>
+          <t>+39 339 651 8864 / mikrotik_consultant@bitmagic.it</t>
+        </is>
+      </c>
+      <c r="K589" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L589" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M589" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N589" s="3" t="inlineStr"/>
+      <c r="O589" s="3" t="inlineStr"/>
+      <c r="P589" s="3" t="inlineStr"/>
+      <c r="Q589" s="3" t="inlineStr">
+        <is>
+          <t>持 MTCSWE（交换）+ MTCEWE（企业无线）+ MTCTCE（流量控制）</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" s="3" t="inlineStr">
+        <is>
+          <t>Davide Toffoletto</t>
+        </is>
+      </c>
+      <c r="B590" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C590" s="3" t="inlineStr">
+        <is>
+          <t>Udine</t>
+        </is>
+      </c>
+      <c r="D590" s="3" t="inlineStr"/>
+      <c r="E590" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F590" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCTCE+MTCINE+MTCIPv6E+MTCSE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G590" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H590" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I590" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J590" s="3" t="inlineStr">
+        <is>
+          <t>+39 347 918 8529 / davide.toffoletto@gmail.com</t>
+        </is>
+      </c>
+      <c r="K590" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L590" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M590" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N590" s="3" t="inlineStr"/>
+      <c r="O590" s="3" t="inlineStr"/>
+      <c r="P590" s="3" t="inlineStr"/>
+      <c r="Q590" s="3" t="inlineStr">
+        <is>
+          <t>★★ 全科目 MikroTik 认证讲师；企业级网络 = **交换 switching、路由、防火墙、防火墙集群**；站点间 PtP 无线；**仓库与办公的室内无线覆盖（CAPsMAN）**；QoS</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" s="3" t="inlineStr">
+        <is>
+          <t>Lorenzo Busatti / Grifonline</t>
+        </is>
+      </c>
+      <c r="B591" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C591" s="3" t="inlineStr">
+        <is>
+          <t>Grosseto</t>
+        </is>
+      </c>
+      <c r="D591" s="3" t="inlineStr">
+        <is>
+          <t>routing.wireless.academy</t>
+        </is>
+      </c>
+      <c r="E591" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F591" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCINE+MTCIPv6E+MTCSE+MTCSWE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G591" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H591" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I591" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J591" s="3" t="inlineStr">
+        <is>
+          <t>+39 340 894 8064 / training@grifonline.it</t>
+        </is>
+      </c>
+      <c r="K591" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L591" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M591" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N591" s="3" t="inlineStr"/>
+      <c r="O591" s="3" t="inlineStr"/>
+      <c r="P591" s="3" t="inlineStr"/>
+      <c r="Q591" s="3" t="inlineStr">
+        <is>
+          <t>★★ 1997 年做 ISP、2006 年做 WISP、2010 年起当讲师；持有 MTCSWE；ISP/WISP 有线无线网络与 NOC 规划/设计/迁移，专精 OSPF 与 BGP；**10+ 次 MUM 大会演讲**，可全球出差</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" s="3" t="inlineStr">
+        <is>
+          <t>Elia Fiumalbo Tino Spadoni / Spadhausen</t>
+        </is>
+      </c>
+      <c r="B592" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C592" s="3" t="inlineStr">
+        <is>
+          <t>Ravenna</t>
+        </is>
+      </c>
+      <c r="D592" s="3" t="inlineStr">
+        <is>
+          <t>spadhausen.com</t>
+        </is>
+      </c>
+      <c r="E592" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F592" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G592" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H592" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I592" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J592" s="3" t="inlineStr">
+        <is>
+          <t>+39 0544 233 0899 / admin@spadhausen.com</t>
+        </is>
+      </c>
+      <c r="K592" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L592" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M592" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N592" s="3" t="inlineStr"/>
+      <c r="O592" s="3" t="inlineStr"/>
+      <c r="P592" s="3" t="inlineStr"/>
+      <c r="Q592" s="3" t="inlineStr">
+        <is>
+          <t>★ **自己拥有一家 ISP**（有实操场景可落设备）；自称「优化专家」，2002 年入行，MikroTik 认证讲师；主攻 BGP 与 ISP/企业冗余方案；常驻摩尔多瓦，可全球接单</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" s="3" t="inlineStr">
+        <is>
+          <t>PF Tech</t>
+        </is>
+      </c>
+      <c r="B593" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C593" s="3" t="inlineStr">
+        <is>
+          <t>Favria / Cuorgnè</t>
+        </is>
+      </c>
+      <c r="D593" s="3" t="inlineStr">
+        <is>
+          <t>pftech.it</t>
+        </is>
+      </c>
+      <c r="E593" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F593" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCSE（公司内 3 人）</t>
+        </is>
+      </c>
+      <c r="G593" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H593" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I593" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J593" s="3" t="inlineStr">
+        <is>
+          <t>Paolo Vacca +39 0124 576161 / info@pftech.it；Stefano Callegari stefano.c@pftech.it；Stefano Vallosio stefano@pftech.it</t>
+        </is>
+      </c>
+      <c r="K593" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L593" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M593" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N593" s="3" t="inlineStr"/>
+      <c r="O593" s="3" t="inlineStr"/>
+      <c r="P593" s="3" t="inlineStr"/>
+      <c r="Q593" s="3" t="inlineStr">
+        <is>
+          <t>公司内 3 位 MikroTik 顾问。Paolo：静态路由与 OSPF、防火墙安全、网络设计、全系列 VPN 隧道（IPsec/PPPoE/L2TP/PPTP/SSTP/oVPN/EoIP/IPIP）、CHR over Proxmox/KVM、虚拟化</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" s="3" t="inlineStr">
+        <is>
+          <t>Alejandro Pablo Falà / MikroTik Training Italia</t>
+        </is>
+      </c>
+      <c r="B594" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C594" s="3" t="inlineStr">
+        <is>
+          <t>Ancona</t>
+        </is>
+      </c>
+      <c r="D594" s="3" t="inlineStr">
+        <is>
+          <t>mikrotik-training.it</t>
+        </is>
+      </c>
+      <c r="E594" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F594" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCINE+MTCIPv6E+MTCSE</t>
+        </is>
+      </c>
+      <c r="G594" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H594" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I594" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J594" s="3" t="inlineStr">
+        <is>
+          <t>info@mikrotik-training.it</t>
+        </is>
+      </c>
+      <c r="K594" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L594" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M594" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N594" s="3" t="inlineStr"/>
+      <c r="O594" s="3" t="inlineStr"/>
+      <c r="P594" s="3" t="inlineStr"/>
+      <c r="Q594" s="3" t="inlineStr">
+        <is>
+          <t>运营商网络顾问工程师：BGP/OSPF/MPLS/VPLS、IPv6、安全、高级无线、HotSpot、QoS 流量管理、PPPoE 与 RADIUS 工程；西/意母语，可全球接单</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" s="3" t="inlineStr">
+        <is>
+          <t>Alfredo Giordano / TikTrain</t>
+        </is>
+      </c>
+      <c r="B595" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C595" s="3" t="inlineStr">
+        <is>
+          <t>Montoro</t>
+        </is>
+      </c>
+      <c r="D595" s="3" t="inlineStr">
+        <is>
+          <t>tiktrain.com</t>
+        </is>
+      </c>
+      <c r="E595" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F595" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCTCE</t>
+        </is>
+      </c>
+      <c r="G595" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H595" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I595" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J595" s="3" t="inlineStr">
+        <is>
+          <t>+39 347 312 5813 / alfredo@tiktrain.com</t>
+        </is>
+      </c>
+      <c r="K595" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L595" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M595" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N595" s="3" t="inlineStr"/>
+      <c r="O595" s="3" t="inlineStr"/>
+      <c r="P595" s="3" t="inlineStr"/>
+      <c r="Q595" s="3" t="inlineStr">
+        <is>
+          <t>ISP/**运营商网络**设计实施与排障；动态路由、隧道、QoS、PPPoE、RouterOS 与现有网集成、PtP/PtMP、负载均衡与故障切换、带宽管理；可服务欧洲与墨西哥</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" s="3" t="inlineStr">
+        <is>
+          <t>CorsiMikrotik（意大利 MikroTik 培训）</t>
+        </is>
+      </c>
+      <c r="B596" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C596" s="3" t="inlineStr">
+        <is>
+          <t>Verona 区号 045</t>
+        </is>
+      </c>
+      <c r="D596" s="3" t="inlineStr">
+        <is>
+          <t>corsimikrotik.it</t>
+        </is>
+      </c>
+      <c r="E596" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F596" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 含 CAPsMAN 与网络自动化</t>
+        </is>
+      </c>
+      <c r="G596" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H596" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I596" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J596" s="3" t="inlineStr">
+        <is>
+          <t>+39 045 485 4174 / marco@corsimikrotik.it</t>
+        </is>
+      </c>
+      <c r="K596" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L596" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M596" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N596" s="3" t="inlineStr"/>
+      <c r="O596" s="3" t="inlineStr"/>
+      <c r="P596" s="3" t="inlineStr"/>
+      <c r="Q596" s="3" t="inlineStr">
+        <is>
+          <t>意大利 MikroTik 培训机构；CAPsMAN 管理 + 脚本化网络自动化</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" s="3" t="inlineStr">
+        <is>
+          <t>Cristian Delogu / Netify</t>
+        </is>
+      </c>
+      <c r="B597" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C597" s="3" t="inlineStr">
+        <is>
+          <t>Lodi</t>
+        </is>
+      </c>
+      <c r="D597" s="3" t="inlineStr">
+        <is>
+          <t>netify.it</t>
+        </is>
+      </c>
+      <c r="E597" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F597" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCSE</t>
+        </is>
+      </c>
+      <c r="G597" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H597" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I597" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J597" s="3" t="inlineStr">
+        <is>
+          <t>+39 335 127 4723 / cristian.delogu@netify.it</t>
+        </is>
+      </c>
+      <c r="K597" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L597" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M597" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N597" s="3" t="inlineStr"/>
+      <c r="O597" s="3" t="inlineStr"/>
+      <c r="P597" s="3" t="inlineStr"/>
+      <c r="Q597" s="3" t="inlineStr">
+        <is>
+          <t>WISP/ISP 咨询：有线无线规划设计与迁移；VLAN、PPPoE、防火墙、OSPF、BGP、MPLS、无线、队列与流量整形、脚本、安全</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" s="3" t="inlineStr">
+        <is>
+          <t>Simone Filippi / Byte Solutions</t>
+        </is>
+      </c>
+      <c r="B598" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C598" s="3" t="inlineStr">
+        <is>
+          <t>Berbenno（Bergamo/Lecco/Milano 一带）</t>
+        </is>
+      </c>
+      <c r="D598" s="3" t="inlineStr">
+        <is>
+          <t>bytesolutions.it</t>
+        </is>
+      </c>
+      <c r="E598" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F598" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCSE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G598" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H598" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I598" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J598" s="3" t="inlineStr">
+        <is>
+          <t>+39 035 199 6065 / info@bytesolutions.it</t>
+        </is>
+      </c>
+      <c r="K598" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L598" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M598" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N598" s="3" t="inlineStr"/>
+      <c r="O598" s="3" t="inlineStr"/>
+      <c r="P598" s="3" t="inlineStr"/>
+      <c r="Q598" s="3" t="inlineStr">
+        <is>
+          <t>企业网络与系统集成（贝加莫/莱科/米兰）；2017 年起用 MikroTik；**VoIP 语音路由与语音流量优先**、多 WAN、带宽管理 QoS → 语音场景 = PoE 话机供电需求</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" s="3" t="inlineStr">
+        <is>
+          <t>Gianpiero Ciacci</t>
+        </is>
+      </c>
+      <c r="B599" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C599" s="3" t="inlineStr">
+        <is>
+          <t>Siena</t>
+        </is>
+      </c>
+      <c r="D599" s="3" t="inlineStr"/>
+      <c r="E599" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F599" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSE</t>
+        </is>
+      </c>
+      <c r="G599" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H599" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I599" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J599" s="3" t="inlineStr">
+        <is>
+          <t>+39 338 248 7996 / gciacci@gmail.com</t>
+        </is>
+      </c>
+      <c r="K599" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L599" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M599" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N599" s="3" t="inlineStr"/>
+      <c r="O599" s="3" t="inlineStr"/>
+      <c r="P599" s="3" t="inlineStr"/>
+      <c r="Q599" s="3" t="inlineStr">
+        <is>
+          <t>WISP、OSPF、防火墙、动态路由、流量管理、带宽整形、**switching**、VPN</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" s="3" t="inlineStr">
+        <is>
+          <t>Valerio Simeraro</t>
+        </is>
+      </c>
+      <c r="B600" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C600" s="3" t="inlineStr">
+        <is>
+          <t>Mazzarrà Sant'Andrea（西西里）</t>
+        </is>
+      </c>
+      <c r="D600" s="3" t="inlineStr"/>
+      <c r="E600" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F600" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCINE+MTCIPv6E</t>
+        </is>
+      </c>
+      <c r="G600" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H600" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I600" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J600" s="3" t="inlineStr">
+        <is>
+          <t>+39 392 000 5977 / valerio.simeraro@gmail.com</t>
+        </is>
+      </c>
+      <c r="K600" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L600" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M600" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N600" s="3" t="inlineStr"/>
+      <c r="O600" s="3" t="inlineStr"/>
+      <c r="P600" s="3" t="inlineStr"/>
+      <c r="Q600" s="3" t="inlineStr">
+        <is>
+          <t>含 MTCINE（ISP 互联）</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" s="3" t="inlineStr">
+        <is>
+          <t>Giorgio Marchetti / Fastnet</t>
+        </is>
+      </c>
+      <c r="B601" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C601" s="3" t="inlineStr">
+        <is>
+          <t>Monsano</t>
+        </is>
+      </c>
+      <c r="D601" s="3" t="inlineStr">
+        <is>
+          <t>fastnet.it</t>
+        </is>
+      </c>
+      <c r="E601" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F601" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCSE</t>
+        </is>
+      </c>
+      <c r="G601" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H601" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I601" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J601" s="3" t="inlineStr">
+        <is>
+          <t>g.marchetti@fastnet.it</t>
+        </is>
+      </c>
+      <c r="K601" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L601" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M601" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N601" s="3" t="inlineStr"/>
+      <c r="O601" s="3" t="inlineStr"/>
+      <c r="P601" s="3" t="inlineStr"/>
+      <c r="Q601" s="3" t="inlineStr"/>
+    </row>
+    <row r="602">
+      <c r="A602" s="3" t="inlineStr">
+        <is>
+          <t>Andrea Somma / Matrix Computers</t>
+        </is>
+      </c>
+      <c r="B602" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C602" s="3" t="inlineStr">
+        <is>
+          <t>Varedo</t>
+        </is>
+      </c>
+      <c r="D602" s="3" t="inlineStr">
+        <is>
+          <t>matrixcomputers.it</t>
+        </is>
+      </c>
+      <c r="E602" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F602" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G602" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H602" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I602" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J602" s="3" t="inlineStr">
+        <is>
+          <t>+39 339 447 6819 / a.somma@matrixcomputers.it</t>
+        </is>
+      </c>
+      <c r="K602" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L602" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M602" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N602" s="3" t="inlineStr"/>
+      <c r="O602" s="3" t="inlineStr"/>
+      <c r="P602" s="3" t="inlineStr"/>
+      <c r="Q602" s="3" t="inlineStr"/>
+    </row>
+    <row r="603">
+      <c r="A603" s="3" t="inlineStr">
+        <is>
+          <t>Zen Vittore</t>
+        </is>
+      </c>
+      <c r="B603" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C603" s="3" t="inlineStr">
+        <is>
+          <t>Pordenone</t>
+        </is>
+      </c>
+      <c r="D603" s="3" t="inlineStr"/>
+      <c r="E603" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F603" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSE</t>
+        </is>
+      </c>
+      <c r="G603" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H603" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I603" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J603" s="3" t="inlineStr">
+        <is>
+          <t>+39 320 057 9027 / vittore@zenfamily.it</t>
+        </is>
+      </c>
+      <c r="K603" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L603" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M603" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N603" s="3" t="inlineStr"/>
+      <c r="O603" s="3" t="inlineStr"/>
+      <c r="P603" s="3" t="inlineStr"/>
+      <c r="Q603" s="3" t="inlineStr"/>
+    </row>
+    <row r="604">
+      <c r="A604" s="3" t="inlineStr">
+        <is>
+          <t>Lorenzo Webber</t>
+        </is>
+      </c>
+      <c r="B604" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C604" s="3" t="inlineStr">
+        <is>
+          <t>Mezzolombardo</t>
+        </is>
+      </c>
+      <c r="D604" s="3" t="inlineStr"/>
+      <c r="E604" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F604" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSE</t>
+        </is>
+      </c>
+      <c r="G604" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H604" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I604" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J604" s="3" t="inlineStr">
+        <is>
+          <t>+39 347 091 9297 / lory76@gmail.com</t>
+        </is>
+      </c>
+      <c r="K604" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L604" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M604" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N604" s="3" t="inlineStr"/>
+      <c r="O604" s="3" t="inlineStr"/>
+      <c r="P604" s="3" t="inlineStr"/>
+      <c r="Q604" s="3" t="inlineStr"/>
+    </row>
+    <row r="605">
+      <c r="A605" s="3" t="inlineStr">
+        <is>
+          <t>Jacopo Cipriani</t>
+        </is>
+      </c>
+      <c r="B605" s="3" t="inlineStr">
+        <is>
+          <t>意大利</t>
+        </is>
+      </c>
+      <c r="C605" s="3" t="inlineStr">
+        <is>
+          <t>Grosseto</t>
+        </is>
+      </c>
+      <c r="D605" s="3" t="inlineStr"/>
+      <c r="E605" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F605" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G605" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H605" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I605" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J605" s="3" t="inlineStr">
+        <is>
+          <t>jacopocipriani@me.com</t>
+        </is>
+      </c>
+      <c r="K605" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L605" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M605" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N605" s="3" t="inlineStr"/>
+      <c r="O605" s="3" t="inlineStr"/>
+      <c r="P605" s="3" t="inlineStr"/>
+      <c r="Q605" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Hungarian and Romanian consultants, including two strong switching fits
Balazs Meretei builds large multicast networks for IPTV and
surveillance, which is where IGMP snooping and multicast VLANs stop
being marketing copy. Veaceslav Samburschii runs the Romanian MikroTik
academy, so what he teaches becomes what his students deploy. Romania's
first page only held two cards, so chunk 0 was checked as well.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q605"/>
+  <dimension ref="A1:Q616"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -54604,6 +54604,811 @@
       <c r="O605" s="3" t="inlineStr"/>
       <c r="P605" s="3" t="inlineStr"/>
       <c r="Q605" s="3" t="inlineStr"/>
+    </row>
+    <row r="606">
+      <c r="A606" s="3" t="inlineStr">
+        <is>
+          <t>Balazs Meretei</t>
+        </is>
+      </c>
+      <c r="B606" s="3" t="inlineStr">
+        <is>
+          <t>匈牙利</t>
+        </is>
+      </c>
+      <c r="C606" s="3" t="inlineStr">
+        <is>
+          <t>Kecskemét</t>
+        </is>
+      </c>
+      <c r="D606" s="3" t="inlineStr">
+        <is>
+          <t>meretei.hu</t>
+        </is>
+      </c>
+      <c r="E606" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F606" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCSE+MTCSWE</t>
+        </is>
+      </c>
+      <c r="G606" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H606" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I606" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J606" s="3" t="inlineStr">
+        <is>
+          <t>+36 30 999 9900 / balazs@meretei.hu</t>
+        </is>
+      </c>
+      <c r="K606" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L606" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M606" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N606" s="3" t="inlineStr"/>
+      <c r="O606" s="3" t="inlineStr"/>
+      <c r="P606" s="3" t="inlineStr"/>
+      <c r="Q606" s="3" t="inlineStr">
+        <is>
+          <t>★★ 持 MTCSWE；专长 **ISP 网络（ADSL/DOCSIS/ETTH/FTTH/WISP）+ 大规模组播网络（IPTV、视频监控系统）+ RADIUS 认证计费系统**的设计实施 → 监控与 IPTV 是最吃交换机的场景，IGMP Snooping/组播 VLAN 是硬需求</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" s="3" t="inlineStr">
+        <is>
+          <t>Laszlo Kalapos / MindenamiMikrotik</t>
+        </is>
+      </c>
+      <c r="B607" s="3" t="inlineStr">
+        <is>
+          <t>匈牙利</t>
+        </is>
+      </c>
+      <c r="C607" s="3" t="inlineStr">
+        <is>
+          <t>Miskolc</t>
+        </is>
+      </c>
+      <c r="D607" s="3" t="inlineStr">
+        <is>
+          <t>mindenamimikrotik.hu</t>
+        </is>
+      </c>
+      <c r="E607" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F607" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCTCE+MTCUME+MTCINE+MTCSE+MTCSWE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G607" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H607" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I607" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J607" s="3" t="inlineStr">
+        <is>
+          <t>+36 20 295 6414 / info@mindenamimikrotik.hu</t>
+        </is>
+      </c>
+      <c r="K607" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L607" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M607" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N607" s="3" t="inlineStr"/>
+      <c r="O607" s="3" t="inlineStr"/>
+      <c r="P607" s="3" t="inlineStr"/>
+      <c r="Q607" s="3" t="inlineStr">
+        <is>
+          <t>★ 持 MTCSWE + MTCEWE；站点名直译「所有关于 MikroTik 的事」→ 纯 MikroTik 专营；有线无线网络设计安装、VPN、PPPoE（含 RADIUS）、防火墙、带宽管理与队列、Hotspot、User Manager、The Dude；现场+远程</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" s="3" t="inlineStr">
+        <is>
+          <t>Tamás Gajdos</t>
+        </is>
+      </c>
+      <c r="B608" s="3" t="inlineStr">
+        <is>
+          <t>匈牙利</t>
+        </is>
+      </c>
+      <c r="C608" s="3" t="inlineStr">
+        <is>
+          <t>Szeged</t>
+        </is>
+      </c>
+      <c r="D608" s="3" t="inlineStr"/>
+      <c r="E608" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F608" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCINE+MTCIPv6E+MTCSE+MTCSWE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G608" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H608" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I608" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J608" s="3" t="inlineStr">
+        <is>
+          <t>+36 30 243 2729 / crowbarlabs@outlook.com</t>
+        </is>
+      </c>
+      <c r="K608" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L608" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M608" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N608" s="3" t="inlineStr"/>
+      <c r="O608" s="3" t="inlineStr"/>
+      <c r="P608" s="3" t="inlineStr"/>
+      <c r="Q608" s="3" t="inlineStr">
+        <is>
+          <t>8 证含 MTCSWE（交换）+ MTCEWE（企业无线）；中小企业 IT、WireGuard VPN；英匈塞三语</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" s="3" t="inlineStr">
+        <is>
+          <t>David Csongradi</t>
+        </is>
+      </c>
+      <c r="B609" s="3" t="inlineStr">
+        <is>
+          <t>匈牙利</t>
+        </is>
+      </c>
+      <c r="C609" s="3" t="inlineStr">
+        <is>
+          <t>Budapest</t>
+        </is>
+      </c>
+      <c r="D609" s="3" t="inlineStr">
+        <is>
+          <t>csongradidavid.hu</t>
+        </is>
+      </c>
+      <c r="E609" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F609" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCTCE+MTCUME+MTCINE+MTCIPv6E+MTCSE</t>
+        </is>
+      </c>
+      <c r="G609" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H609" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I609" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J609" s="3" t="inlineStr">
+        <is>
+          <t>+36 30 616 9819 / mikrotik@csongradidavid.hu</t>
+        </is>
+      </c>
+      <c r="K609" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L609" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M609" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N609" s="3" t="inlineStr"/>
+      <c r="O609" s="3" t="inlineStr"/>
+      <c r="P609" s="3" t="inlineStr"/>
+      <c r="Q609" s="3" t="inlineStr">
+        <is>
+          <t>8 证，含 MTCINE（ISP 互联）+ MTCTCE（流量控制）+ MTCUME（用户管理）</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" s="3" t="inlineStr">
+        <is>
+          <t>András István Németh / LazyBear</t>
+        </is>
+      </c>
+      <c r="B610" s="3" t="inlineStr">
+        <is>
+          <t>匈牙利</t>
+        </is>
+      </c>
+      <c r="C610" s="3" t="inlineStr">
+        <is>
+          <t>Pécs</t>
+        </is>
+      </c>
+      <c r="D610" s="3" t="inlineStr">
+        <is>
+          <t>lazybear.hu</t>
+        </is>
+      </c>
+      <c r="E610" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F610" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCIPv6E</t>
+        </is>
+      </c>
+      <c r="G610" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H610" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I610" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J610" s="3" t="inlineStr">
+        <is>
+          <t>+36 70 226 6213 / andras.nemeth@lazybear.hu</t>
+        </is>
+      </c>
+      <c r="K610" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L610" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M610" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N610" s="3" t="inlineStr"/>
+      <c r="O610" s="3" t="inlineStr"/>
+      <c r="P610" s="3" t="inlineStr"/>
+      <c r="Q610" s="3" t="inlineStr"/>
+    </row>
+    <row r="611">
+      <c r="A611" s="3" t="inlineStr">
+        <is>
+          <t>Richárd Szabolcs Tóth</t>
+        </is>
+      </c>
+      <c r="B611" s="3" t="inlineStr">
+        <is>
+          <t>匈牙利</t>
+        </is>
+      </c>
+      <c r="C611" s="3" t="inlineStr">
+        <is>
+          <t>Pécs</t>
+        </is>
+      </c>
+      <c r="D611" s="3" t="inlineStr"/>
+      <c r="E611" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F611" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCIPv6E</t>
+        </is>
+      </c>
+      <c r="G611" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H611" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I611" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J611" s="3" t="inlineStr">
+        <is>
+          <t>+36 30 930 4158 / toth.richardszabolcs@gmail.com</t>
+        </is>
+      </c>
+      <c r="K611" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L611" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M611" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N611" s="3" t="inlineStr"/>
+      <c r="O611" s="3" t="inlineStr"/>
+      <c r="P611" s="3" t="inlineStr"/>
+      <c r="Q611" s="3" t="inlineStr">
+        <is>
+          <t>有线与无线网络，家庭与中小企业</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" s="3" t="inlineStr">
+        <is>
+          <t>Veaceslav Samburschii / Academia MikroTik</t>
+        </is>
+      </c>
+      <c r="B612" s="3" t="inlineStr">
+        <is>
+          <t>罗马尼亚</t>
+        </is>
+      </c>
+      <c r="C612" s="3" t="inlineStr">
+        <is>
+          <t>Brașov</t>
+        </is>
+      </c>
+      <c r="D612" s="3" t="inlineStr">
+        <is>
+          <t>academia-mikrotik.ro</t>
+        </is>
+      </c>
+      <c r="E612" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F612" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCUME+MTCINE+MTCSE+MTCSWE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G612" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H612" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I612" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J612" s="3" t="inlineStr">
+        <is>
+          <t>+40 748 511 932 / vsamburski@gmail.com</t>
+        </is>
+      </c>
+      <c r="K612" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L612" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M612" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N612" s="3" t="inlineStr"/>
+      <c r="O612" s="3" t="inlineStr"/>
+      <c r="P612" s="3" t="inlineStr"/>
+      <c r="Q612" s="3" t="inlineStr">
+        <is>
+          <t>★★ 8 证含 MTCSWE（交换）+ MTCEWE（企业无线）；**经营罗马尼亚 MikroTik 学院 academia-mikrotik.ro（培训机构）** → 影响力型渠道：他讲什么设备，学员就用什么设备</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" s="3" t="inlineStr">
+        <is>
+          <t>Mircea Enache</t>
+        </is>
+      </c>
+      <c r="B613" s="3" t="inlineStr">
+        <is>
+          <t>罗马尼亚</t>
+        </is>
+      </c>
+      <c r="C613" s="3" t="inlineStr">
+        <is>
+          <t>Chiajna, Ilfov</t>
+        </is>
+      </c>
+      <c r="D613" s="3" t="inlineStr"/>
+      <c r="E613" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F613" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCINE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G613" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H613" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I613" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J613" s="3" t="inlineStr">
+        <is>
+          <t>+40 763 698 949 / mircea.enache@outlook.com</t>
+        </is>
+      </c>
+      <c r="K613" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L613" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M613" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N613" s="3" t="inlineStr"/>
+      <c r="O613" s="3" t="inlineStr"/>
+      <c r="P613" s="3" t="inlineStr"/>
+      <c r="Q613" s="3" t="inlineStr">
+        <is>
+          <t>网络架构师，10+ 年经验；含 MTCINE（ISP 互联）+ MTCEWE（企业无线）；英德罗三语</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="3" t="inlineStr">
+        <is>
+          <t>Holt Andrei Tiberiu / GHT-NET</t>
+        </is>
+      </c>
+      <c r="B614" s="3" t="inlineStr">
+        <is>
+          <t>罗马尼亚</t>
+        </is>
+      </c>
+      <c r="C614" s="3" t="inlineStr">
+        <is>
+          <t>Oradea</t>
+        </is>
+      </c>
+      <c r="D614" s="3" t="inlineStr">
+        <is>
+          <t>ght-net.ro</t>
+        </is>
+      </c>
+      <c r="E614" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F614" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSE</t>
+        </is>
+      </c>
+      <c r="G614" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H614" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I614" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J614" s="3" t="inlineStr">
+        <is>
+          <t>+40 771 125 954 / andrei.holt@ght-net.ro</t>
+        </is>
+      </c>
+      <c r="K614" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L614" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M614" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N614" s="3" t="inlineStr"/>
+      <c r="O614" s="3" t="inlineStr"/>
+      <c r="P614" s="3" t="inlineStr"/>
+      <c r="Q614" s="3" t="inlineStr">
+        <is>
+          <t>★ 10+ 年网络经验，自述专长明确为 **Switching、Routing、Virtualization and Storage**；为小/中/大型企业做设计实施与支持 → 交换是他第一专长</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" s="3" t="inlineStr">
+        <is>
+          <t>George Lupulescu</t>
+        </is>
+      </c>
+      <c r="B615" s="3" t="inlineStr">
+        <is>
+          <t>罗马尼亚</t>
+        </is>
+      </c>
+      <c r="C615" s="3" t="inlineStr">
+        <is>
+          <t>Constanța</t>
+        </is>
+      </c>
+      <c r="D615" s="3" t="inlineStr"/>
+      <c r="E615" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F615" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G615" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H615" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I615" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J615" s="3" t="inlineStr">
+        <is>
+          <t>+40 771 607 498 / georgelupulescu@gmail.com</t>
+        </is>
+      </c>
+      <c r="K615" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L615" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M615" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N615" s="3" t="inlineStr"/>
+      <c r="O615" s="3" t="inlineStr"/>
+      <c r="P615" s="3" t="inlineStr"/>
+      <c r="Q615" s="3" t="inlineStr">
+        <is>
+          <t>全栈网络工程师，15+ 年经验</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" s="3" t="inlineStr">
+        <is>
+          <t>Octavian Nicolae Tolea / Newvision</t>
+        </is>
+      </c>
+      <c r="B616" s="3" t="inlineStr">
+        <is>
+          <t>罗马尼亚</t>
+        </is>
+      </c>
+      <c r="C616" s="3" t="inlineStr">
+        <is>
+          <t>București</t>
+        </is>
+      </c>
+      <c r="D616" s="3" t="inlineStr">
+        <is>
+          <t>newvision.ro</t>
+        </is>
+      </c>
+      <c r="E616" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F616" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSE</t>
+        </is>
+      </c>
+      <c r="G616" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H616" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I616" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J616" s="3" t="inlineStr">
+        <is>
+          <t>+40 724 039 489 / octavian.tolea@newvision.ro</t>
+        </is>
+      </c>
+      <c r="K616" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L616" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M616" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N616" s="3" t="inlineStr"/>
+      <c r="O616" s="3" t="inlineStr"/>
+      <c r="P616" s="3" t="inlineStr"/>
+      <c r="Q616" s="3" t="inlineStr">
+        <is>
+          <t>中小企业/家庭办公网络设计实施与支持；无线设计与部署、PtP 链路、Hotspot 管理、站点间隧道与远程办公、网络安全</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Denmark consultants, and fold Pumait's consultant profile into its row
Pumait was already listed as a distributor, so Stefan Andersen's
profile is merged in rather than duplicated. He designs warehouse
automation, access control and CCTV stacks, all of which need PoE, and
UNIFOSS covers agriculture and grid control.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q616"/>
+  <dimension ref="A1:Q618"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -55407,6 +55407,156 @@
       <c r="Q616" s="3" t="inlineStr">
         <is>
           <t>中小企业/家庭办公网络设计实施与支持；无线设计与部署、PtP 链路、Hotspot 管理、站点间隧道与远程办公、网络安全</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" s="3" t="inlineStr">
+        <is>
+          <t>Troels E. Normolle / UNIFOSS</t>
+        </is>
+      </c>
+      <c r="B617" s="3" t="inlineStr">
+        <is>
+          <t>丹麦</t>
+        </is>
+      </c>
+      <c r="C617" s="3" t="inlineStr">
+        <is>
+          <t>Lemming</t>
+        </is>
+      </c>
+      <c r="D617" s="3" t="inlineStr">
+        <is>
+          <t>unifoss.com</t>
+        </is>
+      </c>
+      <c r="E617" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F617" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G617" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H617" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I617" s="3" t="inlineStr">
+        <is>
+          <t>LT-IS6312XGP-4XS8GT</t>
+        </is>
+      </c>
+      <c r="J617" s="3" t="inlineStr">
+        <is>
+          <t>+45 2279 1234 / troels@unifoss.com</t>
+        </is>
+      </c>
+      <c r="K617" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L617" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M617" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N617" s="3" t="inlineStr"/>
+      <c r="O617" s="3" t="inlineStr"/>
+      <c r="P617" s="3" t="inlineStr"/>
+      <c r="Q617" s="3" t="inlineStr">
+        <is>
+          <t>★★ 网络公司创始人，服务行业列举：**农业、能源与电网控制 Energy and grid control、音乐节 Festivals、医疗、酒店 Hospitality、ISP、办公、零售** → 电网控制与农业是工业级场景，音乐节是临时大容量组网，酒店是 PoE 接入，一家公司覆盖三种需求</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="3" t="inlineStr">
+        <is>
+          <t>Thomas Fossing / CloudPilot</t>
+        </is>
+      </c>
+      <c r="B618" s="3" t="inlineStr">
+        <is>
+          <t>丹麦</t>
+        </is>
+      </c>
+      <c r="C618" s="3" t="inlineStr">
+        <is>
+          <t>Copenhagen</t>
+        </is>
+      </c>
+      <c r="D618" s="3" t="inlineStr">
+        <is>
+          <t>cloudpilot.dk</t>
+        </is>
+      </c>
+      <c r="E618" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F618" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCINE</t>
+        </is>
+      </c>
+      <c r="G618" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H618" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I618" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J618" s="3" t="inlineStr">
+        <is>
+          <t>+45 23 708 070 / tcf@cloudpilot.dk</t>
+        </is>
+      </c>
+      <c r="K618" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L618" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M618" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N618" s="3" t="inlineStr"/>
+      <c r="O618" s="3" t="inlineStr"/>
+      <c r="P618" s="3" t="inlineStr"/>
+      <c r="Q618" s="3" t="inlineStr">
+        <is>
+          <t>面向没有专职 IT 经理的中小企业做 IT 平台规划与选型（预算内最优结构）；含 MTCWE（无线）+ MTCINE（ISP 互联）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Swedish and Finnish consultants; Norway has none
Axbyte's Leo has 21 years of MikroTik experience and is the Swedish
trainer, making it the strongest single influence node in the Nordics.
Fernando Trigueiro focuses on advanced routing and switching. Norway's
list is empty and Finland has exactly one consultant, who holds MTCSWE.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q618"/>
+  <dimension ref="A1:Q622"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -29147,7 +29147,7 @@
       </c>
       <c r="K257" s="3" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="L257" s="3" t="inlineStr">
@@ -29165,7 +29165,7 @@
       <c r="P257" s="3" t="inlineStr"/>
       <c r="Q257" s="3" t="inlineStr">
         <is>
-          <t>Valby</t>
+          <t>同时是 MikroTik 认证顾问（MTCNA+MTCRE，Stefan Andersen，stefan@pumait.dk / +45 60 709 009）：1998 年起做 ISP 网络，实战派；还设计更大的运营技术栈——**仓库自动化 warehouse automation、门禁 access control、CCTV 视频监控** → 这三项全是 PoE 供电场景，交换机需求最硬。分销商身份 + 集成项目能力 + 工业/PoE 场景，三线合一</t>
         </is>
       </c>
     </row>
@@ -55557,6 +55557,306 @@
       <c r="Q618" s="3" t="inlineStr">
         <is>
           <t>面向没有专职 IT 经理的中小企业做 IT 平台规划与选型（预算内最优结构）；含 MTCWE（无线）+ MTCINE（ISP 互联）</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" s="3" t="inlineStr">
+        <is>
+          <t>Axbyte</t>
+        </is>
+      </c>
+      <c r="B619" s="3" t="inlineStr">
+        <is>
+          <t>瑞典</t>
+        </is>
+      </c>
+      <c r="C619" s="3" t="inlineStr">
+        <is>
+          <t>Järfälla / Älvsjö</t>
+        </is>
+      </c>
+      <c r="D619" s="3" t="inlineStr">
+        <is>
+          <t>axbyte.se</t>
+        </is>
+      </c>
+      <c r="E619" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F619" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 公司内 2 人：Leo（瑞典 MikroTik 讲师）+ Fredrik Hellgren（MTCSWE）</t>
+        </is>
+      </c>
+      <c r="G619" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H619" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I619" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J619" s="3" t="inlineStr">
+        <is>
+          <t>Leo +46 70 591 5987 / leo@axbyte.se；Fredrik Hellgren +46 8 586 195 00 / support@axbyte.se</t>
+        </is>
+      </c>
+      <c r="K619" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L619" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M619" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N619" s="3" t="inlineStr"/>
+      <c r="O619" s="3" t="inlineStr"/>
+      <c r="P619" s="3" t="inlineStr"/>
+      <c r="Q619" s="3" t="inlineStr">
+        <is>
+          <t>★★ Leo 自述 **做了 21 年 MikroTik，是瑞典（SE）MikroTik RouterOS 官方讲师**，全领域覆盖：防火墙、流量管理、**switching、VLAN**、CAPsMAN、IPv6、OSPF/OSPFv3/iBGP/eBGP、脚本、有线无线设计、认证培训 → 瑞典最强的个人影响力节点</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="3" t="inlineStr">
+        <is>
+          <t>Fernando Trigueiro / Straznet</t>
+        </is>
+      </c>
+      <c r="B620" s="3" t="inlineStr">
+        <is>
+          <t>瑞典</t>
+        </is>
+      </c>
+      <c r="C620" s="3" t="inlineStr">
+        <is>
+          <t>Kungsbacka</t>
+        </is>
+      </c>
+      <c r="D620" s="3" t="inlineStr">
+        <is>
+          <t>straznet.se</t>
+        </is>
+      </c>
+      <c r="E620" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F620" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSE</t>
+        </is>
+      </c>
+      <c r="G620" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H620" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I620" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J620" s="3" t="inlineStr">
+        <is>
+          <t>+46 300 307 80 / info@straznet.se</t>
+        </is>
+      </c>
+      <c r="K620" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L620" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M620" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N620" s="3" t="inlineStr"/>
+      <c r="O620" s="3" t="inlineStr"/>
+      <c r="P620" s="3" t="inlineStr"/>
+      <c r="Q620" s="3" t="inlineStr">
+        <is>
+          <t>★ 20+ 年 IT，近十年专做 MikroTik，自述聚焦 **advanced routing、switching、network design**；为各种规模企业做规划/实施/监控，强调可靠性、可扩展性与安全；巴西+瑞典两国背景，英葡波瑞四语</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="3" t="inlineStr">
+        <is>
+          <t>Fredrik Soderblom / XPD</t>
+        </is>
+      </c>
+      <c r="B621" s="3" t="inlineStr">
+        <is>
+          <t>瑞典</t>
+        </is>
+      </c>
+      <c r="C621" s="3" t="inlineStr">
+        <is>
+          <t>Järfälla</t>
+        </is>
+      </c>
+      <c r="D621" s="3" t="inlineStr">
+        <is>
+          <t>xpd.se</t>
+        </is>
+      </c>
+      <c r="E621" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F621" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCTCE+MTCINE+MTCIPv6E</t>
+        </is>
+      </c>
+      <c r="G621" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H621" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I621" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J621" s="3" t="inlineStr">
+        <is>
+          <t>+46 70 829 2140 / fredrik@xpd.se</t>
+        </is>
+      </c>
+      <c r="K621" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L621" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M621" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N621" s="3" t="inlineStr"/>
+      <c r="O621" s="3" t="inlineStr"/>
+      <c r="P621" s="3" t="inlineStr"/>
+      <c r="Q621" s="3" t="inlineStr">
+        <is>
+          <t>30+ 年 IT；1992 年就为惠普北欧设计实施第一套防火墙，后组建 HP 欧洲网络安全顾问组；在欧洲与美国做过大量边界安全方案与安全审计 → 资深安全专家，能听懂交换机安全特性</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="3" t="inlineStr">
+        <is>
+          <t>Amin Hamidi Younessi / Netrotik</t>
+        </is>
+      </c>
+      <c r="B622" s="3" t="inlineStr">
+        <is>
+          <t>芬兰</t>
+        </is>
+      </c>
+      <c r="C622" s="3" t="inlineStr">
+        <is>
+          <t>Hämeenlinna</t>
+        </is>
+      </c>
+      <c r="D622" s="3" t="inlineStr">
+        <is>
+          <t>netrotik.com</t>
+        </is>
+      </c>
+      <c r="E622" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F622" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCTCE+MTCUME+MTCSWE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G622" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H622" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I622" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J622" s="3" t="inlineStr">
+        <is>
+          <t>+358 41 723 1250 / info@netrotik.com</t>
+        </is>
+      </c>
+      <c r="K622" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L622" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M622" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N622" s="3" t="inlineStr"/>
+      <c r="O622" s="3" t="inlineStr"/>
+      <c r="P622" s="3" t="inlineStr"/>
+      <c r="Q622" s="3" t="inlineStr">
+        <is>
+          <t>★ 芬兰**唯一**一位 MikroTik 认证顾问（稀缺）；7 证含 **MTCSWE（交换）**+ MTCEWE（企业无线）+ MTCTCE（流量控制）+ MTCUME（用户管理）；域名 netrotik.com → 纯 MikroTik 专营</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Estonian consultants: two, one focused on switching
Martin Soovares lists switching alongside routing and VPN work. Rein
Podra covers the full wired and wireless range and also delivers
MikroTik certification training.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q622"/>
+  <dimension ref="A1:Q624"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -55857,6 +55857,152 @@
       <c r="Q622" s="3" t="inlineStr">
         <is>
           <t>★ 芬兰**唯一**一位 MikroTik 认证顾问（稀缺）；7 证含 **MTCSWE（交换）**+ MTCEWE（企业无线）+ MTCTCE（流量控制）+ MTCUME（用户管理）；域名 netrotik.com → 纯 MikroTik 专营</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="3" t="inlineStr">
+        <is>
+          <t>Martin Soovares</t>
+        </is>
+      </c>
+      <c r="B623" s="3" t="inlineStr">
+        <is>
+          <t>爱沙尼亚</t>
+        </is>
+      </c>
+      <c r="C623" s="3" t="inlineStr">
+        <is>
+          <t>Tartu</t>
+        </is>
+      </c>
+      <c r="D623" s="3" t="inlineStr"/>
+      <c r="E623" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F623" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSE</t>
+        </is>
+      </c>
+      <c r="G623" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H623" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I623" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J623" s="3" t="inlineStr">
+        <is>
+          <t>+372 554 9859 / martin.soovares@gmail.com</t>
+        </is>
+      </c>
+      <c r="K623" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L623" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M623" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N623" s="3" t="inlineStr"/>
+      <c r="O623" s="3" t="inlineStr"/>
+      <c r="P623" s="3" t="inlineStr"/>
+      <c r="Q623" s="3" t="inlineStr">
+        <is>
+          <t>★ 专做网络安全分析与运维；技能明确含 **Switching** + Routing + VPN（OpenVPN/WireGuard/IPSec）+ 防火墙（NAT/Layer-7/Mangle）+ User Manager + Hotspot</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="3" t="inlineStr">
+        <is>
+          <t>Rein Podra</t>
+        </is>
+      </c>
+      <c r="B624" s="3" t="inlineStr">
+        <is>
+          <t>爱沙尼亚</t>
+        </is>
+      </c>
+      <c r="C624" s="3" t="inlineStr">
+        <is>
+          <t>Põltsamaa</t>
+        </is>
+      </c>
+      <c r="D624" s="3" t="inlineStr">
+        <is>
+          <t>ccisrd.eu</t>
+        </is>
+      </c>
+      <c r="E624" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F624" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCUME+MTCIPv6E+MTCSE</t>
+        </is>
+      </c>
+      <c r="G624" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H624" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I624" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J624" s="3" t="inlineStr">
+        <is>
+          <t>+372 505 1372 / rein.podra@ccisrd.eu</t>
+        </is>
+      </c>
+      <c r="K624" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L624" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M624" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N624" s="3" t="inlineStr"/>
+      <c r="O624" s="3" t="inlineStr"/>
+      <c r="P624" s="3" t="inlineStr"/>
+      <c r="Q624" s="3" t="inlineStr">
+        <is>
+          <t>有线无线全领域：路由、隧道、防火墙、无线、CAPsMAN、The Dude；网络设计与 MikroTik 认证培训</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Latvian and Lithuanian consultants, completing the Baltics
Latvia has one consultant, NetPro, who does 802.1x and RADIUS for access
layer security. Lithuania has three: Kestutis Viselga runs the national
MikroTik training site and holds MTCSWE, and Robertas Stauskas sells
MikroTik router and switch configuration as his first listed service.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q624"/>
+  <dimension ref="A1:Q628"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -56003,6 +56003,306 @@
       <c r="Q624" s="3" t="inlineStr">
         <is>
           <t>有线无线全领域：路由、隧道、防火墙、无线、CAPsMAN、The Dude；网络设计与 MikroTik 认证培训</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="3" t="inlineStr">
+        <is>
+          <t>Oļegs Žakovs / NetPro</t>
+        </is>
+      </c>
+      <c r="B625" s="3" t="inlineStr">
+        <is>
+          <t>拉脱维亚</t>
+        </is>
+      </c>
+      <c r="C625" s="3" t="inlineStr">
+        <is>
+          <t>Rīga</t>
+        </is>
+      </c>
+      <c r="D625" s="3" t="inlineStr">
+        <is>
+          <t>netpro.lv</t>
+        </is>
+      </c>
+      <c r="E625" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F625" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCWE</t>
+        </is>
+      </c>
+      <c r="G625" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H625" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I625" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J625" s="3" t="inlineStr">
+        <is>
+          <t>+371 27 866 444 / oleg@netpro.lv</t>
+        </is>
+      </c>
+      <c r="K625" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L625" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M625" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N625" s="3" t="inlineStr"/>
+      <c r="O625" s="3" t="inlineStr"/>
+      <c r="P625" s="3" t="inlineStr"/>
+      <c r="Q625" s="3" t="inlineStr">
+        <is>
+          <t>★ 拉脱维亚**唯一**认证顾问（稀缺）；15+ 年 MikroTik 经验；专长含 **802.1x 端口认证 + RADIUS**（→ 交换机接入层安全是他的活）、CAPsMAN、RoMON、The Dude 监控、PtP/PtMP 远距离无线、各类 VPN 隧道、流量管理、安全策略设计</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="3" t="inlineStr">
+        <is>
+          <t>Kęstutis Viselga / MikroTik Training Lietuva</t>
+        </is>
+      </c>
+      <c r="B626" s="3" t="inlineStr">
+        <is>
+          <t>立陶宛</t>
+        </is>
+      </c>
+      <c r="C626" s="3" t="inlineStr">
+        <is>
+          <t>Alytus</t>
+        </is>
+      </c>
+      <c r="D626" s="3" t="inlineStr">
+        <is>
+          <t>mikrotik-training.lt</t>
+        </is>
+      </c>
+      <c r="E626" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F626" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCTCE+MTCSE+MTCSWE</t>
+        </is>
+      </c>
+      <c r="G626" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H626" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I626" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J626" s="3" t="inlineStr">
+        <is>
+          <t>+370 684 43770 / trainer@mikrotik-training.lt</t>
+        </is>
+      </c>
+      <c r="K626" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L626" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M626" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N626" s="3" t="inlineStr"/>
+      <c r="O626" s="3" t="inlineStr"/>
+      <c r="P626" s="3" t="inlineStr"/>
+      <c r="Q626" s="3" t="inlineStr">
+        <is>
+          <t>★★ 立陶宛 MikroTik 培训机构（mikrotik-training.lt）；6 证含 **MTCSWE（交换）**+ MTCTCE（流量控制）+ MTCSE（安全）+ MTCWE（无线）→ 他教什么，立陶宛的工程师就用什么</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="3" t="inlineStr">
+        <is>
+          <t>Robertas Stauskas / Magit</t>
+        </is>
+      </c>
+      <c r="B627" s="3" t="inlineStr">
+        <is>
+          <t>立陶宛</t>
+        </is>
+      </c>
+      <c r="C627" s="3" t="inlineStr">
+        <is>
+          <t>Vilnius</t>
+        </is>
+      </c>
+      <c r="D627" s="3" t="inlineStr">
+        <is>
+          <t>magit.lt</t>
+        </is>
+      </c>
+      <c r="E627" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F627" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G627" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H627" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I627" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J627" s="3" t="inlineStr">
+        <is>
+          <t>+370 674 47188 / robertas@magit.lt</t>
+        </is>
+      </c>
+      <c r="K627" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L627" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M627" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N627" s="3" t="inlineStr"/>
+      <c r="O627" s="3" t="inlineStr"/>
+      <c r="P627" s="3" t="inlineStr"/>
+      <c r="Q627" s="3" t="inlineStr">
+        <is>
+          <t>★ 服务项目第一条就是「**MikroTik router and switch configuration from scratch（从零配置路由器与交换机）**」；技能含 **VLANs、Bridges、Link Bonding（链路聚合）**、QoS/流量整形、防火墙加固、DDoS 防护、无线规划、网络审计与优化 → 接入层交换是他日常生意</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="3" t="inlineStr">
+        <is>
+          <t>Dovydas Rimeisis</t>
+        </is>
+      </c>
+      <c r="B628" s="3" t="inlineStr">
+        <is>
+          <t>立陶宛</t>
+        </is>
+      </c>
+      <c r="C628" s="3" t="inlineStr">
+        <is>
+          <t>Vilnius</t>
+        </is>
+      </c>
+      <c r="D628" s="3" t="inlineStr">
+        <is>
+          <t>atitic.eu</t>
+        </is>
+      </c>
+      <c r="E628" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F628" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G628" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H628" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I628" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J628" s="3" t="inlineStr">
+        <is>
+          <t>+370 623 74543 / dovydas.rimeisis@atitic.eu</t>
+        </is>
+      </c>
+      <c r="K628" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L628" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M628" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N628" s="3" t="inlineStr"/>
+      <c r="O628" s="3" t="inlineStr"/>
+      <c r="P628" s="3" t="inlineStr"/>
+      <c r="Q628" s="3" t="inlineStr">
+        <is>
+          <t>10+ 年 MikroTik 实操、15+ 年 IT 基础设施；做本地/混合/公有云融合的完整方案（网络+计算+云+安全协同），擅长 MikroTik 作为大架构一环的复杂环境</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
US consultants: 19 people across 15 companies
Link Technologies and IP ArchiTechs are the two finds of the sweep.
Both describe themselves as among the largest MikroTik consultancies,
both spell out switching expertise down to QinQ, spanning tree and LACP,
and LinkTechs also runs its own hardware shop, so it consults,
integrates and resells. Michael Jezierski works at IndyCar on IP video
multicast and Dante audio for motorsports.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q628"/>
+  <dimension ref="A1:Q641"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -56305,6 +56305,953 @@
           <t>10+ 年 MikroTik 实操、15+ 年 IT 基础设施；做本地/混合/公有云融合的完整方案（网络+计算+云+安全协同），擅长 MikroTik 作为大架构一环的复杂环境</t>
         </is>
       </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="3" t="inlineStr">
+        <is>
+          <t>Michael Jezierski / IndyCar</t>
+        </is>
+      </c>
+      <c r="B629" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C629" s="3" t="inlineStr">
+        <is>
+          <t>Indianapolis</t>
+        </is>
+      </c>
+      <c r="D629" s="3" t="inlineStr">
+        <is>
+          <t>indycar.com</t>
+        </is>
+      </c>
+      <c r="E629" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F629" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCIPv6E+MTCSWE</t>
+        </is>
+      </c>
+      <c r="G629" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H629" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I629" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J629" s="3" t="inlineStr">
+        <is>
+          <t>+1 317 492 5005 / mjezierski@indycar.com</t>
+        </is>
+      </c>
+      <c r="K629" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L629" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M629" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N629" s="3" t="inlineStr"/>
+      <c r="O629" s="3" t="inlineStr"/>
+      <c r="P629" s="3" t="inlineStr"/>
+      <c r="Q629" s="3" t="inlineStr">
+        <is>
+          <t>★★ 持 MTCSWE；**专做美国赛车运动产业与车队（邮箱是 @indycar.com，人在 IndyCar 赛事方）**；业务：Layer 2/3、无线 LAN、PtP、**IP 视频与组播 IP Video &amp; Multicast**、IP 对讲、**Audinate Dante 认证 1/2/3 级（专业音频 over IP）** → 赛事转播+ Dante 音频对交换机的 IGMP Snooping/组播/低时延要求极高，是极高门槛高单价的细分市场</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="3" t="inlineStr">
+        <is>
+          <t>Michael Omondi / McCharles Tech</t>
+        </is>
+      </c>
+      <c r="B630" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C630" s="3" t="inlineStr">
+        <is>
+          <t>Pelham</t>
+        </is>
+      </c>
+      <c r="D630" s="3" t="inlineStr">
+        <is>
+          <t>mccharlestech.net</t>
+        </is>
+      </c>
+      <c r="E630" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F630" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 10 证全拿</t>
+        </is>
+      </c>
+      <c r="G630" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H630" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I630" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J630" s="3" t="inlineStr">
+        <is>
+          <t>+1 833 622 4275 / support@mccharlestech.com</t>
+        </is>
+      </c>
+      <c r="K630" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L630" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M630" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N630" s="3" t="inlineStr"/>
+      <c r="O630" s="3" t="inlineStr"/>
+      <c r="P630" s="3" t="inlineStr"/>
+      <c r="Q630" s="3" t="inlineStr">
+        <is>
+          <t>★★ 10 证全拿；服务清单含 **L2 的 VLAN 与 L3 的 VRF、从二层扁平桥接网迁移到三层分段网、网络准入控制与设备加固、.1X 与 RADIUS 用户认证、高可用（负载均衡/首跳冗余/绑定）**、QoS、室内外无线规划 → 接入层交换与准入控制是主业</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="3" t="inlineStr">
+        <is>
+          <t>Juan Manuel Díaz Gómez</t>
+        </is>
+      </c>
+      <c r="B631" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C631" s="3" t="inlineStr">
+        <is>
+          <t>Tampa, FL</t>
+        </is>
+      </c>
+      <c r="D631" s="3" t="inlineStr"/>
+      <c r="E631" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F631" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 10 证全拿</t>
+        </is>
+      </c>
+      <c r="G631" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H631" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I631" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J631" s="3" t="inlineStr">
+        <is>
+          <t>+57 315 649 0735 / sutik.oficial@gmail.com</t>
+        </is>
+      </c>
+      <c r="K631" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L631" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M631" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N631" s="3" t="inlineStr"/>
+      <c r="O631" s="3" t="inlineStr"/>
+      <c r="P631" s="3" t="inlineStr"/>
+      <c r="Q631" s="3" t="inlineStr">
+        <is>
+          <t>★★ 10 证全拿 + 认证讲师，18+ 年 MikroTik；VPN 隧道、负载均衡与故障切换、BGP/OSPF、VLAN、PPPoE、防火墙、PtP/PtMP、CAPsMAN、QoS、The Dude；提供 24/7 支持；英西双语（拉美市场）</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" s="3" t="inlineStr">
+        <is>
+          <t>Mohammad Tayyebi / Tayyebi.net</t>
+        </is>
+      </c>
+      <c r="B632" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C632" s="3" t="inlineStr">
+        <is>
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="D632" s="3" t="inlineStr">
+        <is>
+          <t>tayyebi.net</t>
+        </is>
+      </c>
+      <c r="E632" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F632" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCTCE+MTCUME+MTCINE+MTCIPv6E+MTCSWE</t>
+        </is>
+      </c>
+      <c r="G632" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H632" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I632" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J632" s="3" t="inlineStr">
+        <is>
+          <t>1-512-713-6825 / MohammadTayyebi@Gmail.Com</t>
+        </is>
+      </c>
+      <c r="K632" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L632" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M632" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N632" s="3" t="inlineStr"/>
+      <c r="O632" s="3" t="inlineStr"/>
+      <c r="P632" s="3" t="inlineStr"/>
+      <c r="Q632" s="3" t="inlineStr">
+        <is>
+          <t>★★ 8 证含 **MTCSWE**；20+ 年 ISP/WISP 与数据中心；**MikroTik 认证讲师 + 学术讲师（Academy Trainer）**；做托管网络服务（设计/实施/迁移/监控/加固/安全，24/7）；专长含 **交换（MAC-based VLAN、QinQ）**、高可用 VRRP/LACP/绑定、DDoS 防护、组播、MPLS/VPLS/VRF；**还能把 MikroTik 与别的品牌集成并做双向迁移** → 最懂多厂商替代的人</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="3" t="inlineStr">
+        <is>
+          <t>Kyle Heppler / The ISP Academy</t>
+        </is>
+      </c>
+      <c r="B633" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C633" s="3" t="inlineStr">
+        <is>
+          <t>Tucson, AZ</t>
+        </is>
+      </c>
+      <c r="D633" s="3" t="inlineStr">
+        <is>
+          <t>theispacademy.com</t>
+        </is>
+      </c>
+      <c r="E633" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F633" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCINE+MTCSE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G633" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H633" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I633" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J633" s="3" t="inlineStr">
+        <is>
+          <t>+1 805 394 5953 / hello@theispacademy.com</t>
+        </is>
+      </c>
+      <c r="K633" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L633" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M633" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N633" s="3" t="inlineStr"/>
+      <c r="O633" s="3" t="inlineStr"/>
+      <c r="P633" s="3" t="inlineStr"/>
+      <c r="Q633" s="3" t="inlineStr">
+        <is>
+          <t>★ 经营 **The ISP Academy（ISP 学院，培训机构）**；专攻各规模 ISP，尤其 WISP；兼做网络监控、数据库、**网络自动化与编程**、无线工程、团队培训 → 他教出来的 WISP 就是他的渠道</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="3" t="inlineStr">
+        <is>
+          <t>Rick Frey / Rick Frey Consulting</t>
+        </is>
+      </c>
+      <c r="B634" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C634" s="3" t="inlineStr">
+        <is>
+          <t>Rexburg, ID</t>
+        </is>
+      </c>
+      <c r="D634" s="3" t="inlineStr">
+        <is>
+          <t>rickfreyconsulting.com</t>
+        </is>
+      </c>
+      <c r="E634" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F634" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCTCE+MTCINE+MTCSE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G634" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H634" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I634" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J634" s="3" t="inlineStr">
+        <is>
+          <t>+1 430 236 5829 / rickfrey1000@gmail.com</t>
+        </is>
+      </c>
+      <c r="K634" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L634" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M634" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N634" s="3" t="inlineStr"/>
+      <c r="O634" s="3" t="inlineStr"/>
+      <c r="P634" s="3" t="inlineStr"/>
+      <c r="Q634" s="3" t="inlineStr">
+        <is>
+          <t>**30+ 年网络、19 年 MikroTik**，提供 MikroTik 全科目咨询与培训（含 ROS7 迁移）；路由/无线/QoS/VPN/防火墙/监控/OSPF/BGP/MPLS/VPLS/TE/负载均衡/VLAN/安全/CAPsMAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="3" t="inlineStr">
+        <is>
+          <t>Joshua Moore / Archous Networks</t>
+        </is>
+      </c>
+      <c r="B635" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C635" s="3" t="inlineStr">
+        <is>
+          <t>Lake Stevens, WA</t>
+        </is>
+      </c>
+      <c r="D635" s="3" t="inlineStr">
+        <is>
+          <t>archous.tech</t>
+        </is>
+      </c>
+      <c r="E635" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F635" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCTCE+MTCUME+MTCINE+MTCIPv6E+MTCSE</t>
+        </is>
+      </c>
+      <c r="G635" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H635" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I635" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J635" s="3" t="inlineStr">
+        <is>
+          <t>+1 912 218 3720 / mikrotik@archous.tech</t>
+        </is>
+      </c>
+      <c r="K635" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L635" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M635" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N635" s="3" t="inlineStr"/>
+      <c r="O635" s="3" t="inlineStr"/>
+      <c r="P635" s="3" t="inlineStr"/>
+      <c r="Q635" s="3" t="inlineStr">
+        <is>
+          <t>多厂商网络与系统集成商，专做 **MikroTik 及他牌的自动化网络方案**（端到端开通自动化：用户开通/停用/限速）；OSPF/BGP/MPLS 规模部署、WireGuard/IPIP/GRE/L2TP/PPP 隧道；为企业与 ISP 定制监控与报表</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="3" t="inlineStr">
+        <is>
+          <t>Andres Ocampo</t>
+        </is>
+      </c>
+      <c r="B636" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C636" s="3" t="inlineStr">
+        <is>
+          <t>Lake Grove, NY</t>
+        </is>
+      </c>
+      <c r="D636" s="3" t="inlineStr"/>
+      <c r="E636" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F636" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCTCE+MTCINE+MTCIPv6E+MTCSE</t>
+        </is>
+      </c>
+      <c r="G636" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H636" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I636" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J636" s="3" t="inlineStr">
+        <is>
+          <t>+1 551 219 8239 / sriandres@hotmail.com</t>
+        </is>
+      </c>
+      <c r="K636" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L636" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M636" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N636" s="3" t="inlineStr"/>
+      <c r="O636" s="3" t="inlineStr"/>
+      <c r="P636" s="3" t="inlineStr"/>
+      <c r="Q636" s="3" t="inlineStr">
+        <is>
+          <t>★ 技能清单明确含 **Switching（VRRP、SPT 生成树、L2 过滤器）**、Routing &amp; Switching；高级防火墙与 Mangle、OSPF/BGP/路由过滤、带宽管理与队列树、PtP/PtMP、MPLS 与 VPLS、VRF、HotSpot、运营商支持</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="3" t="inlineStr">
+        <is>
+          <t>John Ellis</t>
+        </is>
+      </c>
+      <c r="B637" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C637" s="3" t="inlineStr">
+        <is>
+          <t>Woodland, WA</t>
+        </is>
+      </c>
+      <c r="D637" s="3" t="inlineStr">
+        <is>
+          <t>ellis.me</t>
+        </is>
+      </c>
+      <c r="E637" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F637" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCINE</t>
+        </is>
+      </c>
+      <c r="G637" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H637" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I637" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J637" s="3" t="inlineStr">
+        <is>
+          <t>john@ellis.me</t>
+        </is>
+      </c>
+      <c r="K637" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L637" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M637" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N637" s="3" t="inlineStr"/>
+      <c r="O637" s="3" t="inlineStr"/>
+      <c r="P637" s="3" t="inlineStr"/>
+      <c r="Q637" s="3" t="inlineStr">
+        <is>
+          <t>★ 2007 年起持 MikroTik 认证；近 30 年任首席工程师/系统架构师；专长明确含 **routing、switching、bridging**、防火墙、园区与固定无线、VPN、脚本；运营本地 WISP、全国性企业网络、**区域学区的安全防火墙** → 学区是 PoE 交换机的大宗场景</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="3" t="inlineStr">
+        <is>
+          <t>Jun Baay</t>
+        </is>
+      </c>
+      <c r="B638" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C638" s="3" t="inlineStr">
+        <is>
+          <t>Green Valley, AZ</t>
+        </is>
+      </c>
+      <c r="D638" s="3" t="inlineStr"/>
+      <c r="E638" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F638" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G638" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H638" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I638" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J638" s="3" t="inlineStr">
+        <is>
+          <t>+1 951 433 0197 / junbaay2011@gmail.com</t>
+        </is>
+      </c>
+      <c r="K638" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L638" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M638" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N638" s="3" t="inlineStr"/>
+      <c r="O638" s="3" t="inlineStr"/>
+      <c r="P638" s="3" t="inlineStr"/>
+      <c r="Q638" s="3" t="inlineStr">
+        <is>
+          <t>资深网络工程师 10+ 年：企业路由、大规模网络架构、专家级排障；**多厂商高性能环境**，擅长用 MikroTik RouterOS/CCR 搭配传统企业设备以最大化基础设施价值；**擅长定位 Layer 2 到 Layer 7 异常**、数据中心迁移</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="3" t="inlineStr">
+        <is>
+          <t>Andrei Zhernosek</t>
+        </is>
+      </c>
+      <c r="B639" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C639" s="3" t="inlineStr">
+        <is>
+          <t>Newcastle, WA</t>
+        </is>
+      </c>
+      <c r="D639" s="3" t="inlineStr"/>
+      <c r="E639" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F639" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCTCE+MTCSE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G639" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H639" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I639" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J639" s="3" t="inlineStr">
+        <is>
+          <t>+1 206 412 4111 / master226@gmail.com</t>
+        </is>
+      </c>
+      <c r="K639" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L639" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M639" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N639" s="3" t="inlineStr"/>
+      <c r="O639" s="3" t="inlineStr"/>
+      <c r="P639" s="3" t="inlineStr"/>
+      <c r="Q639" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证讲师（TR0232），10+ 年 ISP 与企业网络设计实施排障；英俄双语</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="3" t="inlineStr">
+        <is>
+          <t>Ray Evelyn</t>
+        </is>
+      </c>
+      <c r="B640" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C640" s="3" t="inlineStr">
+        <is>
+          <t>Melbourne, FL</t>
+        </is>
+      </c>
+      <c r="D640" s="3" t="inlineStr"/>
+      <c r="E640" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F640" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCTCE+MTCUME+MTCIPv6E+MTCSE</t>
+        </is>
+      </c>
+      <c r="G640" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H640" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I640" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J640" s="3" t="inlineStr">
+        <is>
+          <t>+1 754 317 8108 / rayfevelyn@gmail.com</t>
+        </is>
+      </c>
+      <c r="K640" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L640" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M640" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N640" s="3" t="inlineStr"/>
+      <c r="O640" s="3" t="inlineStr"/>
+      <c r="P640" s="3" t="inlineStr"/>
+      <c r="Q640" s="3" t="inlineStr">
+        <is>
+          <t>2008 年起用 MikroTik，熟悉运营商与企业级软件栈；架构到工程实施与特定场景支持；路由与云</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="3" t="inlineStr">
+        <is>
+          <t>Christopher Schiessl</t>
+        </is>
+      </c>
+      <c r="B641" s="3" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C641" s="3" t="inlineStr">
+        <is>
+          <t>Minot, ND</t>
+        </is>
+      </c>
+      <c r="D641" s="3" t="inlineStr"/>
+      <c r="E641" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F641" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCTCE</t>
+        </is>
+      </c>
+      <c r="G641" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H641" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I641" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J641" s="3" t="inlineStr">
+        <is>
+          <t>+1 701 858 5464 / cschiessl@gmail.com</t>
+        </is>
+      </c>
+      <c r="K641" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L641" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M641" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N641" s="3" t="inlineStr"/>
+      <c r="O641" s="3" t="inlineStr"/>
+      <c r="P641" s="3" t="inlineStr"/>
+      <c r="Q641" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Canadian consultants: 15, including a CCIE and a national ISP veteran
Jody Lemoine holds both a current Cisco CCIE and MikroTik trainer
status, so he can read switching silicon specs without any education.
Payam Poursaied spent 16 years at a national ISP with over a million
subscribers. Two consultants work inside education and healthcare
networks, and Hani Rahrouh calls out L3 hardware offloading by name.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q641"/>
+  <dimension ref="A1:Q655"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -37362,7 +37362,7 @@
       <c r="P372" s="3" t="inlineStr"/>
       <c r="Q372" s="3" t="inlineStr">
         <is>
-          <t>USDittmer</t>
+          <t>★★★ 【升级：这不只是总代，还是北美最大的 MikroTik 工程公司之一】自述「北美领先的 MikroTik 工程与咨询公司之一」，客户从单人创业到全国性 ISP、**市政公用事业 utilities、园区/工业/多站点企业**，项目跨多洲。公司内 2 位认证顾问：Dennis Burgess（314-735-0270 / dmburgess@linktechs.net，6 证）、Dan Parrish（support@linktechs.net，5 证）。★**交换专长（逐条列出）：VLAN/Q-in-Q、VLAN 翻译与重写、LACP/绑定、生成树 RSTP/MSTP、二层传输与冗余、GPON 集成、EVPN/VXLAN、10G/25G/40G/100G/200G/400G 交换矩阵**。路由：BGP/OSPF/MPLS-TE/策略路由/路由反射器/CGNAT。★**另开网店 shop.linktechs.net 卖设备 → 总代 + 咨询集成 + 零售，三线合一，北美第一优先账号**</t>
         </is>
       </c>
     </row>
@@ -50649,7 +50649,7 @@
       </c>
       <c r="K551" s="3" t="inlineStr">
         <is>
-          <t>★★</t>
+          <t>★★★</t>
         </is>
       </c>
       <c r="L551" s="3" t="inlineStr">
@@ -50667,7 +50667,7 @@
       <c r="P551" s="3" t="inlineStr"/>
       <c r="Q551" s="3" t="inlineStr">
         <is>
-          <t>含 MTCUME（用户管理）→ Hotspot 方向</t>
+          <t>★★★ 【升级：这家是跨国大所，不是普通顾问】自述「全球最大的 MikroTik 咨询公司之一，3 国设办公室、6 大洲有在建项目，客户含财富 500 强与上市公司，提供全球 24/7 支持」。公司内已知 3 位认证顾问：英国 Samson Kamwendo（MTCNA+MTCUME）、美国 Thomas Murdock（+1-855-645-7684 / thomas.murdock@iparchitechs.com，9 证）、Abraham Rios Velez（+1 303 590 9940 / abraham.rios@gmail.com，6 证，波多黎各出身，服务西语市场；西语站 es.iparchitechs.com）。★**交换专长（逐条列出）：VLAN（Q-in-Q、s/c tag、重写/翻译）、生成树、LACP 与绑定、GPON、二层传输设计、二层冗余**。无线含体育场/大型场馆；服务含 IPTV 与实时视频、SIP/H.323。→ 一家公司同时覆盖欧美与拉美</t>
         </is>
       </c>
     </row>
@@ -57252,6 +57252,1020 @@
       <c r="O641" s="3" t="inlineStr"/>
       <c r="P641" s="3" t="inlineStr"/>
       <c r="Q641" s="3" t="inlineStr"/>
+    </row>
+    <row r="642">
+      <c r="A642" s="3" t="inlineStr">
+        <is>
+          <t>Payam Poursaied / MoLuke</t>
+        </is>
+      </c>
+      <c r="B642" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C642" s="3" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="D642" s="3" t="inlineStr">
+        <is>
+          <t>moluke.net</t>
+        </is>
+      </c>
+      <c r="E642" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F642" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCIPv6E（自述可教全部证书）</t>
+        </is>
+      </c>
+      <c r="G642" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H642" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I642" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J642" s="3" t="inlineStr">
+        <is>
+          <t>+1 778-300-2288 / payam@moluke.net</t>
+        </is>
+      </c>
+      <c r="K642" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L642" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M642" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N642" s="3" t="inlineStr"/>
+      <c r="O642" s="3" t="inlineStr"/>
+      <c r="P642" s="3" t="inlineStr"/>
+      <c r="Q642" s="3" t="inlineStr">
+        <is>
+          <t>★★ 19 年 IT，**其中 16 年在一家全国性 ISP（用户 100 万+）**；MikroTik 认证讲师（自称可教所有证书）；带团队；场景：DDoS 防护、VPN 与站点互联、互联网冗余、VoIP、QoS</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="3" t="inlineStr">
+        <is>
+          <t>Jody Lemoine / Tishco Networks</t>
+        </is>
+      </c>
+      <c r="B643" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C643" s="3" t="inlineStr">
+        <is>
+          <t>Ontario</t>
+        </is>
+      </c>
+      <c r="D643" s="3" t="inlineStr">
+        <is>
+          <t>tishco.ca</t>
+        </is>
+      </c>
+      <c r="E643" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F643" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 多证 + MikroTik 认证讲师 + **Cisco CCIE（41436）**</t>
+        </is>
+      </c>
+      <c r="G643" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H643" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I643" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J643" s="3" t="inlineStr">
+        <is>
+          <t>+1 905 378 1134 / jody.lemoine@tishco.ca</t>
+        </is>
+      </c>
+      <c r="K643" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L643" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M643" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N643" s="3" t="inlineStr"/>
+      <c r="O643" s="3" t="inlineStr"/>
+      <c r="P643" s="3" t="inlineStr"/>
+      <c r="Q643" s="3" t="inlineStr">
+        <is>
+          <t>★★★ **同时持有 Cisco CCIE（证书号 41436，仍在有效期内）和 MikroTik 认证讲师资格** —— 极少见的双料，说明他真看得懂交换芯片/转发架构这类硬指标，不用给他做科普；1980 年代末入行，2007 年起独立经营 tishco networks；专做**多厂商**企业网络设计与实施 + 配套培训</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="3" t="inlineStr">
+        <is>
+          <t>Amir Seifi / Magenta Networks</t>
+        </is>
+      </c>
+      <c r="B644" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C644" s="3" t="inlineStr">
+        <is>
+          <t>Scarborough, ON</t>
+        </is>
+      </c>
+      <c r="D644" s="3" t="inlineStr">
+        <is>
+          <t>magentanetworks.net</t>
+        </is>
+      </c>
+      <c r="E644" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F644" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCTCE+MTCUME+MTCINE</t>
+        </is>
+      </c>
+      <c r="G644" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H644" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I644" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J644" s="3" t="inlineStr">
+        <is>
+          <t>+1-647-812-5170 / support@magentanetworks.net</t>
+        </is>
+      </c>
+      <c r="K644" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L644" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M644" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N644" s="3" t="inlineStr"/>
+      <c r="O644" s="3" t="inlineStr"/>
+      <c r="P644" s="3" t="inlineStr"/>
+      <c r="Q644" s="3" t="inlineStr">
+        <is>
+          <t>★★ 精通 RouterOS 与 **SwitchOS**；核心能力明确包含「**二层交换、VLAN 配置、链路聚合、端口优化管理**」；另有高级路由 OSPF/BGP、防火墙加固、DDoS 缓解、定制脚本与自动化</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="3" t="inlineStr">
+        <is>
+          <t>Wilmer Almazan / Arawi</t>
+        </is>
+      </c>
+      <c r="B645" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C645" s="3" t="inlineStr">
+        <is>
+          <t>Winnipeg</t>
+        </is>
+      </c>
+      <c r="D645" s="3" t="inlineStr">
+        <is>
+          <t>arawi.ca</t>
+        </is>
+      </c>
+      <c r="E645" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F645" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 10 证全拿</t>
+        </is>
+      </c>
+      <c r="G645" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H645" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I645" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J645" s="3" t="inlineStr">
+        <is>
+          <t>1-431-990-6625 / info@arawi.ca</t>
+        </is>
+      </c>
+      <c r="K645" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L645" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M645" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N645" s="3" t="inlineStr"/>
+      <c r="O645" s="3" t="inlineStr"/>
+      <c r="P645" s="3" t="inlineStr"/>
+      <c r="Q645" s="3" t="inlineStr">
+        <is>
+          <t>★★ 10 证全拿 + 全资格 MikroTik 讲师；2008 年起在**加拿大与拉丁美洲**设计/优化/防护 MikroTik 网络；路由 OSPF/BGP/MPLS、无线 CAPsMAN/Mesh、企业安全；英西双语，可线上或现场</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="3" t="inlineStr">
+        <is>
+          <t>Yvan Laverdiere</t>
+        </is>
+      </c>
+      <c r="B646" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C646" s="3" t="inlineStr">
+        <is>
+          <t>Rouyn-Noranda, QC</t>
+        </is>
+      </c>
+      <c r="D646" s="3" t="inlineStr">
+        <is>
+          <t>cegepat.qc.ca</t>
+        </is>
+      </c>
+      <c r="E646" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F646" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCINE+MTCSWE</t>
+        </is>
+      </c>
+      <c r="G646" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H646" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I646" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J646" s="3" t="inlineStr">
+        <is>
+          <t>819-763-1411 / yvan.laverdiere@cegepat.qc.ca</t>
+        </is>
+      </c>
+      <c r="K646" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L646" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M646" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N646" s="3" t="inlineStr"/>
+      <c r="O646" s="3" t="inlineStr"/>
+      <c r="P646" s="3" t="inlineStr"/>
+      <c r="Q646" s="3" t="inlineStr">
+        <is>
+          <t>★ 持 **MTCSWE**；技能含 **VXLAN、VLAN**、RADIUS、MPLS/VPLS/VRF、IPSec/GRE/EoIP/IPIP、PPPoE、Hotspot、网络监控、Proxmox 集成；**任职于教育系统（cegepat.qc.ca 魁北克 CEGEP 学院）→ 校园网场景**；英法双语</t>
+        </is>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="3" t="inlineStr">
+        <is>
+          <t>Alain Casault, B.Ing.</t>
+        </is>
+      </c>
+      <c r="B647" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C647" s="3" t="inlineStr">
+        <is>
+          <t>Prévost, QC</t>
+        </is>
+      </c>
+      <c r="D647" s="3" t="inlineStr">
+        <is>
+          <t>educationhmo.com</t>
+        </is>
+      </c>
+      <c r="E647" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F647" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE</t>
+        </is>
+      </c>
+      <c r="G647" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H647" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I647" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J647" s="3" t="inlineStr">
+        <is>
+          <t>1-514-394-0419 / casault.alain@educationhmo.com</t>
+        </is>
+      </c>
+      <c r="K647" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L647" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M647" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N647" s="3" t="inlineStr"/>
+      <c r="O647" s="3" t="inlineStr"/>
+      <c r="P647" s="3" t="inlineStr"/>
+      <c r="Q647" s="3" t="inlineStr">
+        <is>
+          <t>★ 工程师（B.Ing.）；专长明确为「**培训、企业网络设计与架构、Routing、Switching、VLANs、无线、高可用与冗余**」；**任职于教育/卫生系统（educationhmo.com）→ 校园与医疗机构网络**；英法双语</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" s="3" t="inlineStr">
+        <is>
+          <t>MohammadMahdi Raeesi / Commander IT</t>
+        </is>
+      </c>
+      <c r="B648" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C648" s="3" t="inlineStr">
+        <is>
+          <t>Markham, ON</t>
+        </is>
+      </c>
+      <c r="D648" s="3" t="inlineStr">
+        <is>
+          <t>commanderit.ca</t>
+        </is>
+      </c>
+      <c r="E648" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F648" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCTCE</t>
+        </is>
+      </c>
+      <c r="G648" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H648" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I648" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J648" s="3" t="inlineStr">
+        <is>
+          <t>647 562 2246 / admin@commanderit.ca</t>
+        </is>
+      </c>
+      <c r="K648" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L648" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M648" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N648" s="3" t="inlineStr"/>
+      <c r="O648" s="3" t="inlineStr"/>
+      <c r="P648" s="3" t="inlineStr"/>
+      <c r="Q648" s="3" t="inlineStr">
+        <is>
+          <t>★ 自述专长含 **switching**；RouterOS 7.xx、动态路由 BGP/OSPF、高性能无线与 CAPsMAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="3" t="inlineStr">
+        <is>
+          <t>Sylvain Caron</t>
+        </is>
+      </c>
+      <c r="B649" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C649" s="3" t="inlineStr">
+        <is>
+          <t>Lévis, QC</t>
+        </is>
+      </c>
+      <c r="D649" s="3" t="inlineStr"/>
+      <c r="E649" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F649" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCWE+MTCRE+MTCTCE+MTCINE+MTCSE</t>
+        </is>
+      </c>
+      <c r="G649" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H649" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I649" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J649" s="3" t="inlineStr">
+        <is>
+          <t>581-681-5641 / scaron999@hotmail.com</t>
+        </is>
+      </c>
+      <c r="K649" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L649" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M649" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N649" s="3" t="inlineStr"/>
+      <c r="O649" s="3" t="inlineStr"/>
+      <c r="P649" s="3" t="inlineStr"/>
+      <c r="Q649" s="3" t="inlineStr">
+        <is>
+          <t>6 证含 MTCINE（ISP 互联）</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" s="3" t="inlineStr">
+        <is>
+          <t>Hussein Khalil</t>
+        </is>
+      </c>
+      <c r="B650" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C650" s="3" t="inlineStr">
+        <is>
+          <t>Calgary</t>
+        </is>
+      </c>
+      <c r="D650" s="3" t="inlineStr"/>
+      <c r="E650" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F650" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCTCE</t>
+        </is>
+      </c>
+      <c r="G650" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H650" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I650" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J650" s="3" t="inlineStr">
+        <is>
+          <t>+1 403 973 6789 / hkhalil_7@hotmail.com</t>
+        </is>
+      </c>
+      <c r="K650" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L650" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M650" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N650" s="3" t="inlineStr"/>
+      <c r="O650" s="3" t="inlineStr"/>
+      <c r="P650" s="3" t="inlineStr"/>
+      <c r="Q650" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 顾问兼讲师，覆盖防火墙、QoS、桥接、高级路由协议、无线等全部特性</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" s="3" t="inlineStr">
+        <is>
+          <t>Frédéric Gauthier / ProRéseau</t>
+        </is>
+      </c>
+      <c r="B651" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C651" s="3" t="inlineStr">
+        <is>
+          <t>Québec</t>
+        </is>
+      </c>
+      <c r="D651" s="3" t="inlineStr">
+        <is>
+          <t>proreseau.net</t>
+        </is>
+      </c>
+      <c r="E651" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F651" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G651" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H651" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I651" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J651" s="3" t="inlineStr">
+        <is>
+          <t>+1 418 933 1285 / fgauthier@proreseau.net</t>
+        </is>
+      </c>
+      <c r="K651" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L651" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M651" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N651" s="3" t="inlineStr"/>
+      <c r="O651" s="3" t="inlineStr"/>
+      <c r="P651" s="3" t="inlineStr"/>
+      <c r="Q651" s="3" t="inlineStr"/>
+    </row>
+    <row r="652">
+      <c r="A652" s="3" t="inlineStr">
+        <is>
+          <t>Simon Miners / JMR</t>
+        </is>
+      </c>
+      <c r="B652" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C652" s="3" t="inlineStr">
+        <is>
+          <t>Niagara Falls, ON</t>
+        </is>
+      </c>
+      <c r="D652" s="3" t="inlineStr">
+        <is>
+          <t>jmr.ca</t>
+        </is>
+      </c>
+      <c r="E652" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F652" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G652" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H652" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I652" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J652" s="3" t="inlineStr">
+        <is>
+          <t>+1 905 374 2878 / simon@jmr.ca</t>
+        </is>
+      </c>
+      <c r="K652" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L652" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M652" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N652" s="3" t="inlineStr"/>
+      <c r="O652" s="3" t="inlineStr"/>
+      <c r="P652" s="3" t="inlineStr"/>
+      <c r="Q652" s="3" t="inlineStr"/>
+    </row>
+    <row r="653">
+      <c r="A653" s="3" t="inlineStr">
+        <is>
+          <t>Gerald Paul Mamaril</t>
+        </is>
+      </c>
+      <c r="B653" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C653" s="3" t="inlineStr">
+        <is>
+          <t>Hamilton, ON</t>
+        </is>
+      </c>
+      <c r="D653" s="3" t="inlineStr"/>
+      <c r="E653" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F653" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCUME</t>
+        </is>
+      </c>
+      <c r="G653" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H653" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I653" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J653" s="3" t="inlineStr">
+        <is>
+          <t>+1 289 921 6314 / mamarilgeraldpaul22@gmail.com</t>
+        </is>
+      </c>
+      <c r="K653" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L653" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M653" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N653" s="3" t="inlineStr"/>
+      <c r="O653" s="3" t="inlineStr"/>
+      <c r="P653" s="3" t="inlineStr"/>
+      <c r="Q653" s="3" t="inlineStr"/>
+    </row>
+    <row r="654">
+      <c r="A654" s="3" t="inlineStr">
+        <is>
+          <t>Afshin Yadollahi</t>
+        </is>
+      </c>
+      <c r="B654" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C654" s="3" t="inlineStr">
+        <is>
+          <t>Toronto</t>
+        </is>
+      </c>
+      <c r="D654" s="3" t="inlineStr"/>
+      <c r="E654" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F654" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G654" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H654" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I654" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J654" s="3" t="inlineStr">
+        <is>
+          <t>+1 647 463 9762 / yadollahi.afshin@gmail.com</t>
+        </is>
+      </c>
+      <c r="K654" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L654" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M654" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N654" s="3" t="inlineStr"/>
+      <c r="O654" s="3" t="inlineStr"/>
+      <c r="P654" s="3" t="inlineStr"/>
+      <c r="Q654" s="3" t="inlineStr">
+        <is>
+          <t>英西波斯法四语</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="3" t="inlineStr">
+        <is>
+          <t>Falak Sheth</t>
+        </is>
+      </c>
+      <c r="B655" s="3" t="inlineStr">
+        <is>
+          <t>加拿大</t>
+        </is>
+      </c>
+      <c r="C655" s="3" t="inlineStr">
+        <is>
+          <t>Brampton, ON</t>
+        </is>
+      </c>
+      <c r="D655" s="3" t="inlineStr"/>
+      <c r="E655" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F655" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G655" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H655" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I655" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J655" s="3" t="inlineStr">
+        <is>
+          <t>+1 647 615 2151 / sheth2151@gmail.com</t>
+        </is>
+      </c>
+      <c r="K655" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L655" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M655" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N655" s="3" t="inlineStr"/>
+      <c r="O655" s="3" t="inlineStr"/>
+      <c r="P655" s="3" t="inlineStr"/>
+      <c r="Q655" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Austrian, Swiss, Belgian, Portuguese and Irish consultants
Bernhard Kroll has 23 years of MikroTik experience and holds MTCSWE.
Narrowin builds its own open source automation platform for MikroTik,
so it cares about manageability. Urbino Lobo specialises in hospitality
and multi-dwelling captive portal networks with a field engineer
database behind him. Belgium and Ireland each turned up very few
consultants.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q655"/>
+  <dimension ref="A1:Q668"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -58266,6 +58266,949 @@
       <c r="O655" s="3" t="inlineStr"/>
       <c r="P655" s="3" t="inlineStr"/>
       <c r="Q655" s="3" t="inlineStr"/>
+    </row>
+    <row r="656">
+      <c r="A656" s="3" t="inlineStr">
+        <is>
+          <t>Bernhard Kröll / Giganet</t>
+        </is>
+      </c>
+      <c r="B656" s="3" t="inlineStr">
+        <is>
+          <t>奥地利</t>
+        </is>
+      </c>
+      <c r="C656" s="3" t="inlineStr">
+        <is>
+          <t>Mayrhofen</t>
+        </is>
+      </c>
+      <c r="D656" s="3" t="inlineStr">
+        <is>
+          <t>giganet.at</t>
+        </is>
+      </c>
+      <c r="E656" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F656" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCTCE+MTCIPv6E+MTCSWE</t>
+        </is>
+      </c>
+      <c r="G656" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H656" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I656" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J656" s="3" t="inlineStr">
+        <is>
+          <t>+43 5285 2022 / bk@giganet.at</t>
+        </is>
+      </c>
+      <c r="K656" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L656" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M656" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N656" s="3" t="inlineStr"/>
+      <c r="O656" s="3" t="inlineStr"/>
+      <c r="P656" s="3" t="inlineStr"/>
+      <c r="Q656" s="3" t="inlineStr">
+        <is>
+          <t>★★ 持 MTCSWE；**23 年 MikroTik/RouterOS 经验**；从 SOHO 到企业网与数据中心（HC3 Scale Computing）；专长含 **switching、VLANs**、BGP、防火墙、隧道 VPN/IPsec/WireGuard、PPPoE、CAPsMAN、QoS 与队列、高可用与负载均衡、数据中心托管、监控、备份、自动化、网络审计</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" s="3" t="inlineStr">
+        <is>
+          <t>Khalil / Aulaf</t>
+        </is>
+      </c>
+      <c r="B657" s="3" t="inlineStr">
+        <is>
+          <t>奥地利</t>
+        </is>
+      </c>
+      <c r="C657" s="3" t="inlineStr"/>
+      <c r="D657" s="3" t="inlineStr">
+        <is>
+          <t>aulaf.com</t>
+        </is>
+      </c>
+      <c r="E657" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F657" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 含 Routing/Switching 多方向</t>
+        </is>
+      </c>
+      <c r="G657" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H657" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I657" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J657" s="3" t="inlineStr">
+        <is>
+          <t>+43 688 9131190 / khalil@aulaf.com</t>
+        </is>
+      </c>
+      <c r="K657" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L657" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M657" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N657" s="3" t="inlineStr"/>
+      <c r="O657" s="3" t="inlineStr"/>
+      <c r="P657" s="3" t="inlineStr"/>
+      <c r="Q657" s="3" t="inlineStr">
+        <is>
+          <t>★ 服务行业明确含 **政府、教育、医疗 Government; Education, Health**；多厂商环境；技能含 **Routing/Switching**、BGP/OSPF/MPLS/VPLS、流量工程、无线、防火墙、HotSpot、隧道与 VPN、负载均衡、带宽管理、队列 QoS、RADIUS、培训</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="3" t="inlineStr">
+        <is>
+          <t>Florian Valentin / Formatik</t>
+        </is>
+      </c>
+      <c r="B658" s="3" t="inlineStr">
+        <is>
+          <t>奥地利</t>
+        </is>
+      </c>
+      <c r="C658" s="3" t="inlineStr">
+        <is>
+          <t>Ehrwald</t>
+        </is>
+      </c>
+      <c r="D658" s="3" t="inlineStr">
+        <is>
+          <t>formatik.at</t>
+        </is>
+      </c>
+      <c r="E658" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F658" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCTCE</t>
+        </is>
+      </c>
+      <c r="G658" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H658" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I658" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J658" s="3" t="inlineStr">
+        <is>
+          <t>+43 5673 21939 / florian@formatik.at</t>
+        </is>
+      </c>
+      <c r="K658" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L658" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M658" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N658" s="3" t="inlineStr"/>
+      <c r="O658" s="3" t="inlineStr"/>
+      <c r="P658" s="3" t="inlineStr"/>
+      <c r="Q658" s="3" t="inlineStr">
+        <is>
+          <t>小型系统集成商（system house），**主要就用 MikroTik 设备** → 品牌忠诚度高的小 ISV，替换决策链短</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="3" t="inlineStr">
+        <is>
+          <t>Gunther Engetsberger</t>
+        </is>
+      </c>
+      <c r="B659" s="3" t="inlineStr">
+        <is>
+          <t>奥地利</t>
+        </is>
+      </c>
+      <c r="C659" s="3" t="inlineStr">
+        <is>
+          <t>Oberndorf</t>
+        </is>
+      </c>
+      <c r="D659" s="3" t="inlineStr">
+        <is>
+          <t>sei-ned.org</t>
+        </is>
+      </c>
+      <c r="E659" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F659" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCWE+MTCTCE</t>
+        </is>
+      </c>
+      <c r="G659" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H659" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I659" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J659" s="3" t="inlineStr">
+        <is>
+          <t>+43 664 2772011 / office@sei-ned.org</t>
+        </is>
+      </c>
+      <c r="K659" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L659" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M659" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N659" s="3" t="inlineStr"/>
+      <c r="O659" s="3" t="inlineStr"/>
+      <c r="P659" s="3" t="inlineStr"/>
+      <c r="Q659" s="3" t="inlineStr"/>
+    </row>
+    <row r="660">
+      <c r="A660" s="3" t="inlineStr">
+        <is>
+          <t>Tomas Horyl / Narrowin</t>
+        </is>
+      </c>
+      <c r="B660" s="3" t="inlineStr">
+        <is>
+          <t>瑞士</t>
+        </is>
+      </c>
+      <c r="C660" s="3" t="inlineStr">
+        <is>
+          <t>Lugano</t>
+        </is>
+      </c>
+      <c r="D660" s="3" t="inlineStr">
+        <is>
+          <t>narrowin.ch</t>
+        </is>
+      </c>
+      <c r="E660" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F660" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSWE</t>
+        </is>
+      </c>
+      <c r="G660" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H660" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I660" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J660" s="3" t="inlineStr">
+        <is>
+          <t>info@narrowin.ch（另 +41 61 511 23 30）</t>
+        </is>
+      </c>
+      <c r="K660" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L660" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M660" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N660" s="3" t="inlineStr"/>
+      <c r="O660" s="3" t="inlineStr"/>
+      <c r="P660" s="3" t="inlineStr"/>
+      <c r="Q660" s="3" t="inlineStr">
+        <is>
+          <t>★★ 持 MTCSWE；公司为 MikroTik 提供**网络设计、可视化 visibility 与自动化**，并自研 **network explorer 工具 + MikroTik 开源自动化平台**（narrowin.ch/en/mikrotik_lightweight_sdn.html）→ 做工具的，会看重设备的 API/可管理性；英捷意德四语</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" s="3" t="inlineStr">
+        <is>
+          <t>Philipp Marcel Albrecht / Portup</t>
+        </is>
+      </c>
+      <c r="B661" s="3" t="inlineStr">
+        <is>
+          <t>瑞士</t>
+        </is>
+      </c>
+      <c r="C661" s="3" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+      <c r="D661" s="3" t="inlineStr">
+        <is>
+          <t>portup.ch</t>
+        </is>
+      </c>
+      <c r="E661" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F661" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCIPv6E+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G661" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H661" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I661" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J661" s="3" t="inlineStr">
+        <is>
+          <t>+41 44 500 4699 / info@portup.ch</t>
+        </is>
+      </c>
+      <c r="K661" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L661" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M661" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N661" s="3" t="inlineStr"/>
+      <c r="O661" s="3" t="inlineStr"/>
+      <c r="P661" s="3" t="inlineStr"/>
+      <c r="Q661" s="3" t="inlineStr">
+        <is>
+          <t>含 MTCINE 方向外的路由与 IPv6、企业无线；英葡德三语</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="3" t="inlineStr">
+        <is>
+          <t>Jonathan De Graeve / Smarteye</t>
+        </is>
+      </c>
+      <c r="B662" s="3" t="inlineStr">
+        <is>
+          <t>比利时</t>
+        </is>
+      </c>
+      <c r="C662" s="3" t="inlineStr">
+        <is>
+          <t>Wilrijk (Antwerpen)</t>
+        </is>
+      </c>
+      <c r="D662" s="3" t="inlineStr">
+        <is>
+          <t>smarteye.eu</t>
+        </is>
+      </c>
+      <c r="E662" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F662" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCINE+MTCSE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G662" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H662" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I662" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J662" s="3" t="inlineStr">
+        <is>
+          <t>+32 9 395 6202 / jonathan@smarteye.eu</t>
+        </is>
+      </c>
+      <c r="K662" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L662" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M662" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N662" s="3" t="inlineStr"/>
+      <c r="O662" s="3" t="inlineStr"/>
+      <c r="P662" s="3" t="inlineStr"/>
+      <c r="Q662" s="3" t="inlineStr">
+        <is>
+          <t>★ 比利时**唯一**认证顾问（稀缺）；专做**骨干网设计**与 RouterOS 全栈运维诊断：BGP、MPLS、VPLS、OSPF、流量管理、带宽整形、防火墙、Hotspots、VPN、无线</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="3" t="inlineStr">
+        <is>
+          <t>Urbino Lobo / MiniMeLabs</t>
+        </is>
+      </c>
+      <c r="B663" s="3" t="inlineStr">
+        <is>
+          <t>葡萄牙</t>
+        </is>
+      </c>
+      <c r="C663" s="3" t="inlineStr">
+        <is>
+          <t>Funchal（马德拉）</t>
+        </is>
+      </c>
+      <c r="D663" s="3" t="inlineStr">
+        <is>
+          <t>minimelabs.com</t>
+        </is>
+      </c>
+      <c r="E663" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F663" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCUME</t>
+        </is>
+      </c>
+      <c r="G663" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H663" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I663" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J663" s="3" t="inlineStr">
+        <is>
+          <t>+351 919 379 550 / urbino@minimelabs.com</t>
+        </is>
+      </c>
+      <c r="K663" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L663" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M663" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N663" s="3" t="inlineStr"/>
+      <c r="O663" s="3" t="inlineStr"/>
+      <c r="P663" s="3" t="inlineStr"/>
+      <c r="Q663" s="3" t="inlineStr">
+        <is>
+          <t>★★ 自述「**酒店 Hospitality、多住户公寓 Multi-Dwelling Properties、公共接入 Public Access 的网络与强制门户 Captive Portal 环境专家**」，且「**手上有大量现场工程师与生态方案的数据库**」→ 酒店+MDU 是 PoE 接入交换机批量出货场景；他还有外场工程师网络，能铺量。同事 João Martins（+351 968 850 581 / joao@minimelabs.com，MTCNA+MTCUME）</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" s="3" t="inlineStr">
+        <is>
+          <t>Rogério Costa</t>
+        </is>
+      </c>
+      <c r="B664" s="3" t="inlineStr">
+        <is>
+          <t>葡萄牙</t>
+        </is>
+      </c>
+      <c r="C664" s="3" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="D664" s="3" t="inlineStr"/>
+      <c r="E664" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F664" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCIPv6E</t>
+        </is>
+      </c>
+      <c r="G664" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H664" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I664" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J664" s="3" t="inlineStr">
+        <is>
+          <t>+351 914 846 382 / costa_rogerio@yahoo.com</t>
+        </is>
+      </c>
+      <c r="K664" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L664" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M664" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N664" s="3" t="inlineStr"/>
+      <c r="O664" s="3" t="inlineStr"/>
+      <c r="P664" s="3" t="inlineStr"/>
+      <c r="Q664" s="3" t="inlineStr">
+        <is>
+          <t>认证网络顾问，做 MikroTik RouterOS 基础设施的运维/设计/实施/排障/优化；有 LinkedIn 主页；英西葡三语</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="3" t="inlineStr">
+        <is>
+          <t>Bruno Caiola Ricardo / Sinaltech</t>
+        </is>
+      </c>
+      <c r="B665" s="3" t="inlineStr">
+        <is>
+          <t>葡萄牙</t>
+        </is>
+      </c>
+      <c r="C665" s="3" t="inlineStr">
+        <is>
+          <t>Sintra</t>
+        </is>
+      </c>
+      <c r="D665" s="3" t="inlineStr">
+        <is>
+          <t>sinaltech.pt</t>
+        </is>
+      </c>
+      <c r="E665" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F665" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G665" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H665" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I665" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J665" s="3" t="inlineStr">
+        <is>
+          <t>+351 931 048 461 / bruno.ricardo@sinaltech.pt</t>
+        </is>
+      </c>
+      <c r="K665" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L665" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M665" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N665" s="3" t="inlineStr"/>
+      <c r="O665" s="3" t="inlineStr"/>
+      <c r="P665" s="3" t="inlineStr"/>
+      <c r="Q665" s="3" t="inlineStr"/>
+    </row>
+    <row r="666">
+      <c r="A666" s="3" t="inlineStr">
+        <is>
+          <t>Camacho / Engenheiros</t>
+        </is>
+      </c>
+      <c r="B666" s="3" t="inlineStr">
+        <is>
+          <t>葡萄牙</t>
+        </is>
+      </c>
+      <c r="C666" s="3" t="inlineStr"/>
+      <c r="D666" s="3" t="inlineStr">
+        <is>
+          <t>engenheiros.pt</t>
+        </is>
+      </c>
+      <c r="E666" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F666" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MikroTik 认证顾问 </t>
+        </is>
+      </c>
+      <c r="G666" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H666" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I666" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J666" s="3" t="inlineStr">
+        <is>
+          <t>+351 965 869 277 / camacho@engenheiros.pt</t>
+        </is>
+      </c>
+      <c r="K666" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L666" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M666" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N666" s="3" t="inlineStr"/>
+      <c r="O666" s="3" t="inlineStr"/>
+      <c r="P666" s="3" t="inlineStr"/>
+      <c r="Q666" s="3" t="inlineStr"/>
+    </row>
+    <row r="667">
+      <c r="A667" s="3" t="inlineStr">
+        <is>
+          <t>M Ciantar</t>
+        </is>
+      </c>
+      <c r="B667" s="3" t="inlineStr">
+        <is>
+          <t>爱尔兰</t>
+        </is>
+      </c>
+      <c r="C667" s="3" t="inlineStr"/>
+      <c r="D667" s="3" t="inlineStr"/>
+      <c r="E667" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F667" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 含认证讲师（Certified Trainer）</t>
+        </is>
+      </c>
+      <c r="G667" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H667" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I667" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J667" s="3" t="inlineStr">
+        <is>
+          <t>+353 86 040 6099 / mciantar@gmail.com</t>
+        </is>
+      </c>
+      <c r="K667" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L667" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M667" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N667" s="3" t="inlineStr"/>
+      <c r="O667" s="3" t="inlineStr"/>
+      <c r="P667" s="3" t="inlineStr"/>
+      <c r="Q667" s="3" t="inlineStr">
+        <is>
+          <t>★ **MikroTik 认证讲师**；中大型企业网络排障与支持；**ISP 与 WISP 核心网设计与实施**（BGP/OSPF/MPLS/VPLS/VRF）、流量工程与 QoS、IPv6 实施</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" s="3" t="inlineStr">
+        <is>
+          <t>Oskar Siejk</t>
+        </is>
+      </c>
+      <c r="B668" s="3" t="inlineStr">
+        <is>
+          <t>爱尔兰</t>
+        </is>
+      </c>
+      <c r="C668" s="3" t="inlineStr">
+        <is>
+          <t>Saggart (Dublin)</t>
+        </is>
+      </c>
+      <c r="D668" s="3" t="inlineStr">
+        <is>
+          <t>vit.ie</t>
+        </is>
+      </c>
+      <c r="E668" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F668" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G668" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H668" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I668" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J668" s="3" t="inlineStr">
+        <is>
+          <t>+353 85 157 7369 / oskar@vit.ie</t>
+        </is>
+      </c>
+      <c r="K668" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L668" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M668" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N668" s="3" t="inlineStr"/>
+      <c r="O668" s="3" t="inlineStr"/>
+      <c r="P668" s="3" t="inlineStr"/>
+      <c r="Q668" s="3" t="inlineStr">
+        <is>
+          <t>英波双语</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Croatian, Serbian and Bulgarian consultants; Slovenia has none
Sasa Blagojevic's switching paragraph is word for word the one used by
IP ArchiTechs and Link Technologies, which places him in the same
technical circle. Nenad Marinkovic runs routerboard.rs, a business named
after the hardware, and Goran Stojkovic repairs RouterBOARDs at board
level.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q668"/>
+  <dimension ref="A1:Q677"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -59207,6 +59207,665 @@
       <c r="Q668" s="3" t="inlineStr">
         <is>
           <t>英波双语</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" s="3" t="inlineStr">
+        <is>
+          <t>Sasa Blagojevic</t>
+        </is>
+      </c>
+      <c r="B669" s="3" t="inlineStr">
+        <is>
+          <t>塞尔维亚</t>
+        </is>
+      </c>
+      <c r="C669" s="3" t="inlineStr">
+        <is>
+          <t>Niš</t>
+        </is>
+      </c>
+      <c r="D669" s="3" t="inlineStr"/>
+      <c r="E669" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F669" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCTCE+MTCSWE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G669" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H669" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I669" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J669" s="3" t="inlineStr">
+        <is>
+          <t>+381 64 910 8717 / sajberista@gmail.com</t>
+        </is>
+      </c>
+      <c r="K669" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L669" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M669" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N669" s="3" t="inlineStr"/>
+      <c r="O669" s="3" t="inlineStr"/>
+      <c r="P669" s="3" t="inlineStr"/>
+      <c r="Q669" s="3" t="inlineStr">
+        <is>
+          <t>★★ 持 MTCSWE；**简历的交换专长段落与 IP ArchiTechs / LinkTechs 完全一致**（VLAN q-in-q、s/c tag、重写翻译、生成树、LACP 绑定、GPON、二层传输与冗余），说明他属于同一技术体系/合作网络；设计方向：运营商 WISP/Wireline、企业园区分支、数据中心；服务含 IPTV 与实时视频</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" s="3" t="inlineStr">
+        <is>
+          <t>Igor Stojković / Netis</t>
+        </is>
+      </c>
+      <c r="B670" s="3" t="inlineStr">
+        <is>
+          <t>塞尔维亚</t>
+        </is>
+      </c>
+      <c r="C670" s="3" t="inlineStr">
+        <is>
+          <t>Beograd</t>
+        </is>
+      </c>
+      <c r="D670" s="3" t="inlineStr">
+        <is>
+          <t>netis.rs</t>
+        </is>
+      </c>
+      <c r="E670" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F670" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE（自述可教 MTCNA/MTCRE/MTCTE/MTCWE/MTCINE）</t>
+        </is>
+      </c>
+      <c r="G670" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H670" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I670" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J670" s="3" t="inlineStr">
+        <is>
+          <t>+381 63 546 126 / igor.stojkovic@netis.rs</t>
+        </is>
+      </c>
+      <c r="K670" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L670" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M670" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N670" s="3" t="inlineStr"/>
+      <c r="O670" s="3" t="inlineStr"/>
+      <c r="P670" s="3" t="inlineStr"/>
+      <c r="Q670" s="3" t="inlineStr">
+        <is>
+          <t>★ **塞尔维亚 MikroTik 讲师**（可教 5 门课）；网络架构师，电信背景；网络设计、OSPF/BGP、带宽管理、Hotspot、PPPoE、PtP、防火墙、VLAN、DNS、代理缓存；**企业级与大规模 WISP 工程支持**</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="3" t="inlineStr">
+        <is>
+          <t>Nenad Marinkovic / Routerboard.rs</t>
+        </is>
+      </c>
+      <c r="B671" s="3" t="inlineStr">
+        <is>
+          <t>塞尔维亚</t>
+        </is>
+      </c>
+      <c r="C671" s="3" t="inlineStr">
+        <is>
+          <t>Kragujevac</t>
+        </is>
+      </c>
+      <c r="D671" s="3" t="inlineStr">
+        <is>
+          <t>routerboard.rs</t>
+        </is>
+      </c>
+      <c r="E671" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F671" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSE</t>
+        </is>
+      </c>
+      <c r="G671" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H671" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I671" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J671" s="3" t="inlineStr">
+        <is>
+          <t>+381 66 341 442 / tech@routerboard.rs</t>
+        </is>
+      </c>
+      <c r="K671" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L671" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M671" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N671" s="3" t="inlineStr"/>
+      <c r="O671" s="3" t="inlineStr"/>
+      <c r="P671" s="3" t="inlineStr"/>
+      <c r="Q671" s="3" t="inlineStr">
+        <is>
+          <t>★ 域名直接叫 **routerboard.rs** → 塞尔维亚本地以 MikroTik 为主业的专营店/服务商，品牌绑定极深</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="3" t="inlineStr">
+        <is>
+          <t>Goran Stojkovic</t>
+        </is>
+      </c>
+      <c r="B672" s="3" t="inlineStr">
+        <is>
+          <t>塞尔维亚</t>
+        </is>
+      </c>
+      <c r="C672" s="3" t="inlineStr">
+        <is>
+          <t>Ćuprija</t>
+        </is>
+      </c>
+      <c r="D672" s="3" t="inlineStr"/>
+      <c r="E672" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F672" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCTCE</t>
+        </is>
+      </c>
+      <c r="G672" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H672" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I672" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J672" s="3" t="inlineStr">
+        <is>
+          <t>+381 35 847 7077 / intercom@beotel.net</t>
+        </is>
+      </c>
+      <c r="K672" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L672" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M672" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N672" s="3" t="inlineStr"/>
+      <c r="O672" s="3" t="inlineStr"/>
+      <c r="P672" s="3" t="inlineStr"/>
+      <c r="Q672" s="3" t="inlineStr">
+        <is>
+          <t>★ 专长含 **RouterBOARD 硬件维修** → 懂板级硬件，能评估做工与方案；另有有线无线网络设计（PtP/PtMP/Mesh）、PPPoE、队列与流量整形、QoS、负载均衡与多路径故障切换、高可用、静态/RIP/OSPF/BGP、WISP 运维</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" s="3" t="inlineStr">
+        <is>
+          <t>Tomislav Vrebac / Kerberos</t>
+        </is>
+      </c>
+      <c r="B673" s="3" t="inlineStr">
+        <is>
+          <t>克罗地亚</t>
+        </is>
+      </c>
+      <c r="C673" s="3" t="inlineStr">
+        <is>
+          <t>Kraljevica</t>
+        </is>
+      </c>
+      <c r="D673" s="3" t="inlineStr">
+        <is>
+          <t>kerberos.hr</t>
+        </is>
+      </c>
+      <c r="E673" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F673" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G673" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H673" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I673" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J673" s="3" t="inlineStr">
+        <is>
+          <t>+385 98 983 8091 / mikrotik@kerberos.hr</t>
+        </is>
+      </c>
+      <c r="K673" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L673" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M673" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N673" s="3" t="inlineStr"/>
+      <c r="O673" s="3" t="inlineStr"/>
+      <c r="P673" s="3" t="inlineStr"/>
+      <c r="Q673" s="3" t="inlineStr">
+        <is>
+          <t>为**小型到大型、多站点**系统做 IT 基础设施设计与实施 → 多站点 = 每台点都要接入交换机</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" s="3" t="inlineStr">
+        <is>
+          <t>Dejan Liovic</t>
+        </is>
+      </c>
+      <c r="B674" s="3" t="inlineStr">
+        <is>
+          <t>克罗地亚</t>
+        </is>
+      </c>
+      <c r="C674" s="3" t="inlineStr">
+        <is>
+          <t>Osijek</t>
+        </is>
+      </c>
+      <c r="D674" s="3" t="inlineStr"/>
+      <c r="E674" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F674" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE</t>
+        </is>
+      </c>
+      <c r="G674" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H674" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I674" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J674" s="3" t="inlineStr">
+        <is>
+          <t>+385 95 287 2886 / liovicd@outlook.com</t>
+        </is>
+      </c>
+      <c r="K674" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L674" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M674" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N674" s="3" t="inlineStr"/>
+      <c r="O674" s="3" t="inlineStr"/>
+      <c r="P674" s="3" t="inlineStr"/>
+      <c r="Q674" s="3" t="inlineStr">
+        <is>
+          <t>项目规划与实施、基础与高级配置、现场与远程支持</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="3" t="inlineStr">
+        <is>
+          <t>Stanimir Konakchiev / Nebo Systems</t>
+        </is>
+      </c>
+      <c r="B675" s="3" t="inlineStr">
+        <is>
+          <t>保加利亚</t>
+        </is>
+      </c>
+      <c r="C675" s="3" t="inlineStr">
+        <is>
+          <t>Sofia</t>
+        </is>
+      </c>
+      <c r="D675" s="3" t="inlineStr">
+        <is>
+          <t>nebosystems.eu</t>
+        </is>
+      </c>
+      <c r="E675" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F675" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCUME+MTCIPv6E+MTCSE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G675" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H675" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I675" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J675" s="3" t="inlineStr">
+        <is>
+          <t>+359 898 428 927 / s.konakchiev@nebosystems.eu</t>
+        </is>
+      </c>
+      <c r="K675" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L675" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M675" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N675" s="3" t="inlineStr"/>
+      <c r="O675" s="3" t="inlineStr"/>
+      <c r="P675" s="3" t="inlineStr"/>
+      <c r="Q675" s="3" t="inlineStr">
+        <is>
+          <t>6 证含 MTCEWE（企业无线）+ MTCSE（安全）+ MTCUME（用户管理）</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="3" t="inlineStr">
+        <is>
+          <t>Mihail Gyoshev / Digit Consult</t>
+        </is>
+      </c>
+      <c r="B676" s="3" t="inlineStr">
+        <is>
+          <t>保加利亚</t>
+        </is>
+      </c>
+      <c r="C676" s="3" t="inlineStr">
+        <is>
+          <t>Plovdiv</t>
+        </is>
+      </c>
+      <c r="D676" s="3" t="inlineStr">
+        <is>
+          <t>digitconsult.eu</t>
+        </is>
+      </c>
+      <c r="E676" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F676" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCUME+MTCINE+MTCIPv6E+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G676" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H676" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I676" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J676" s="3" t="inlineStr">
+        <is>
+          <t>+359 898 737 844 / mihail.gyoshev@digitconsult.eu</t>
+        </is>
+      </c>
+      <c r="K676" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L676" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M676" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N676" s="3" t="inlineStr"/>
+      <c r="O676" s="3" t="inlineStr"/>
+      <c r="P676" s="3" t="inlineStr"/>
+      <c r="Q676" s="3" t="inlineStr">
+        <is>
+          <t>含 MTCINE（ISP 互联）+ MTCEWE（企业无线）</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" s="3" t="inlineStr">
+        <is>
+          <t>Georgi Vasilev</t>
+        </is>
+      </c>
+      <c r="B677" s="3" t="inlineStr">
+        <is>
+          <t>保加利亚</t>
+        </is>
+      </c>
+      <c r="C677" s="3" t="inlineStr">
+        <is>
+          <t>Sofia</t>
+        </is>
+      </c>
+      <c r="D677" s="3" t="inlineStr"/>
+      <c r="E677" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F677" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G677" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H677" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I677" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J677" s="3" t="inlineStr">
+        <is>
+          <t>+359 889 895 830 / georgi.petkov.vasilev@gmail.com</t>
+        </is>
+      </c>
+      <c r="K677" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L677" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M677" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N677" s="3" t="inlineStr"/>
+      <c r="O677" s="3" t="inlineStr"/>
+      <c r="P677" s="3" t="inlineStr"/>
+      <c r="Q677" s="3" t="inlineStr">
+        <is>
+          <t>电信硕士，10+ 年 IT，电子爱好者</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Greek consultants: 20, plus Slovak, Bosnian and Albanian
Hellascom has been the first Greek MikroTik distributor since 2001 and
runs the national training centre, making it the origin point of the
Greek ecosystem. Apostolas Georgios does hotel WiFi end to end on
Rhodes, Christos Kargiotis lists PIM-SM multicast routing, and Rom
Digital has specialised in MikroTik since 1983.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q677"/>
+  <dimension ref="A1:Q702"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -59868,6 +59868,1813 @@
           <t>电信硕士，10+ 年 IT，电子爱好者</t>
         </is>
       </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="3" t="inlineStr">
+        <is>
+          <t>Matej Sojka / 365IT</t>
+        </is>
+      </c>
+      <c r="B678" s="3" t="inlineStr">
+        <is>
+          <t>斯洛伐克</t>
+        </is>
+      </c>
+      <c r="C678" s="3" t="inlineStr">
+        <is>
+          <t>Bratislava</t>
+        </is>
+      </c>
+      <c r="D678" s="3" t="inlineStr">
+        <is>
+          <t>365it.sk</t>
+        </is>
+      </c>
+      <c r="E678" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F678" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSWE</t>
+        </is>
+      </c>
+      <c r="G678" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H678" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I678" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J678" s="3" t="inlineStr">
+        <is>
+          <t>+421 905 303 903 / ms@365it.sk（另 sojka.matej@gmail.com）</t>
+        </is>
+      </c>
+      <c r="K678" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L678" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M678" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N678" s="3" t="inlineStr"/>
+      <c r="O678" s="3" t="inlineStr"/>
+      <c r="P678" s="3" t="inlineStr"/>
+      <c r="Q678" s="3" t="inlineStr">
+        <is>
+          <t>★ 持 MTCSWE（交换认证）；**有自己的团队**，客户从小型企业到大型企业基础设施；提供 MikroTik 咨询、实施与支持；英捷匈斯四语</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="3" t="inlineStr">
+        <is>
+          <t>Michal Petkáč / Alfac</t>
+        </is>
+      </c>
+      <c r="B679" s="3" t="inlineStr">
+        <is>
+          <t>斯洛伐克</t>
+        </is>
+      </c>
+      <c r="C679" s="3" t="inlineStr">
+        <is>
+          <t>Bratislava</t>
+        </is>
+      </c>
+      <c r="D679" s="3" t="inlineStr">
+        <is>
+          <t>alfac.sk</t>
+        </is>
+      </c>
+      <c r="E679" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F679" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G679" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H679" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I679" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J679" s="3" t="inlineStr">
+        <is>
+          <t>+421 948 768 927 / petkac@alfac.sk</t>
+        </is>
+      </c>
+      <c r="K679" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L679" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M679" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N679" s="3" t="inlineStr"/>
+      <c r="O679" s="3" t="inlineStr"/>
+      <c r="P679" s="3" t="inlineStr"/>
+      <c r="Q679" s="3" t="inlineStr"/>
+    </row>
+    <row r="680">
+      <c r="A680" s="3" t="inlineStr">
+        <is>
+          <t>Oltion Nikolla / Router.al</t>
+        </is>
+      </c>
+      <c r="B680" s="3" t="inlineStr">
+        <is>
+          <t>阿尔巴尼亚</t>
+        </is>
+      </c>
+      <c r="C680" s="3" t="inlineStr">
+        <is>
+          <t>Tirana</t>
+        </is>
+      </c>
+      <c r="D680" s="3" t="inlineStr">
+        <is>
+          <t>router.al</t>
+        </is>
+      </c>
+      <c r="E680" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F680" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G680" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H680" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I680" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J680" s="3" t="inlineStr">
+        <is>
+          <t>+355 695 250 949 / oltionnikolla@gmail.com</t>
+        </is>
+      </c>
+      <c r="K680" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L680" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M680" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N680" s="3" t="inlineStr"/>
+      <c r="O680" s="3" t="inlineStr"/>
+      <c r="P680" s="3" t="inlineStr"/>
+      <c r="Q680" s="3" t="inlineStr">
+        <is>
+          <t>★★ 域名 **router.al**（阿尔巴尼亚国别域名做 MikroTik 生意）；资深网络工程师与 IT 顾问，**业务覆盖整个巴尔干地区与国际**；核心专长明确含「**复杂路由与交换：BGP、OSPF、MPLS/VPLS、VLAN Filtering、RSTP/MSTP、多 WAN 负载均衡**」；高密度 Wi-Fi、CAPsMAN、Asterisk/VoIP 集成；服务含 ISP/WISP 建网与企业 IT 外包</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="3" t="inlineStr">
+        <is>
+          <t>Olisian Sulaj</t>
+        </is>
+      </c>
+      <c r="B681" s="3" t="inlineStr">
+        <is>
+          <t>阿尔巴尼亚</t>
+        </is>
+      </c>
+      <c r="C681" s="3" t="inlineStr">
+        <is>
+          <t>Tirana</t>
+        </is>
+      </c>
+      <c r="D681" s="3" t="inlineStr"/>
+      <c r="E681" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F681" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G681" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H681" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I681" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J681" s="3" t="inlineStr">
+        <is>
+          <t>+355 69 299 6257 / olisian.sulaj@gmail.com</t>
+        </is>
+      </c>
+      <c r="K681" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L681" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M681" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N681" s="3" t="inlineStr"/>
+      <c r="O681" s="3" t="inlineStr"/>
+      <c r="P681" s="3" t="inlineStr"/>
+      <c r="Q681" s="3" t="inlineStr">
+        <is>
+          <t>★ 专长含 **Switching（MAC-based VLAN）**、PPPoE 与 RADIUS 认证计费、HotSpot、WISP 有线无线 NOC 规划设计迁移、PtP/Mesh、队列与流量整形；英西双语</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" s="3" t="inlineStr">
+        <is>
+          <t>Dritan / Vreshta</t>
+        </is>
+      </c>
+      <c r="B682" s="3" t="inlineStr">
+        <is>
+          <t>阿尔巴尼亚</t>
+        </is>
+      </c>
+      <c r="C682" s="3" t="inlineStr"/>
+      <c r="D682" s="3" t="inlineStr">
+        <is>
+          <t>vreshta.com</t>
+        </is>
+      </c>
+      <c r="E682" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F682" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 含 Switching</t>
+        </is>
+      </c>
+      <c r="G682" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H682" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I682" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J682" s="3" t="inlineStr">
+        <is>
+          <t>+355 682 059 505 / dritan@vreshta.com</t>
+        </is>
+      </c>
+      <c r="K682" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L682" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M682" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N682" s="3" t="inlineStr"/>
+      <c r="O682" s="3" t="inlineStr"/>
+      <c r="P682" s="3" t="inlineStr"/>
+      <c r="Q682" s="3" t="inlineStr">
+        <is>
+          <t>★ 专长 BGP/OSPF/MPLS/**Switching**；Hotspot（公共场所大型部署、企业项目）；**熟悉「Made for MikroTik」生态软件、扇区天线、链路、机柜外壳与配件 → 卖配件的人，进货渠道意识强**；WISP 规划与硬件选型</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" s="3" t="inlineStr">
+        <is>
+          <t>Samir Zildzic / Wirac</t>
+        </is>
+      </c>
+      <c r="B683" s="3" t="inlineStr">
+        <is>
+          <t>波黑</t>
+        </is>
+      </c>
+      <c r="C683" s="3" t="inlineStr">
+        <is>
+          <t>Gracanica</t>
+        </is>
+      </c>
+      <c r="D683" s="3" t="inlineStr">
+        <is>
+          <t>wirac.ba</t>
+        </is>
+      </c>
+      <c r="E683" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F683" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCTCE</t>
+        </is>
+      </c>
+      <c r="G683" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H683" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I683" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J683" s="3" t="inlineStr">
+        <is>
+          <t>+387 35 708 296 / samir@wirac.ba</t>
+        </is>
+      </c>
+      <c r="K683" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L683" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M683" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N683" s="3" t="inlineStr"/>
+      <c r="O683" s="3" t="inlineStr"/>
+      <c r="P683" s="3" t="inlineStr"/>
+      <c r="Q683" s="3" t="inlineStr">
+        <is>
+          <t>波黑**唯一**认证顾问（稀缺）；MikroTik 路由器搭建配置、远程排障、无线、路由、VPN、OSPF；英德塞克波五语</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="3" t="inlineStr">
+        <is>
+          <t>Eleftherios Liodakis / MikroTik Training Greece</t>
+        </is>
+      </c>
+      <c r="B684" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C684" s="3" t="inlineStr">
+        <is>
+          <t>Chania</t>
+        </is>
+      </c>
+      <c r="D684" s="3" t="inlineStr">
+        <is>
+          <t>mikrotiktraining.gr</t>
+        </is>
+      </c>
+      <c r="E684" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F684" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCTCE+MTCUME+MTCINE+MTCIPv6E+MTCSE+MTCSWE</t>
+        </is>
+      </c>
+      <c r="G684" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H684" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I684" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J684" s="3" t="inlineStr">
+        <is>
+          <t>+30 28210 98579 / el@dce.gr</t>
+        </is>
+      </c>
+      <c r="K684" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L684" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M684" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N684" s="3" t="inlineStr"/>
+      <c r="O684" s="3" t="inlineStr"/>
+      <c r="P684" s="3" t="inlineStr"/>
+      <c r="Q684" s="3" t="inlineStr">
+        <is>
+          <t>★ 9 证含 **MTCSWE**；经营 **mikrotiktraining.gr（希腊 MikroTik 培训机构）**；防火墙安全、PPPoE、各类隧道 VPN、负载均衡与多路径故障切换、队列与 QoS、User Manager + RADIUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="3" t="inlineStr">
+        <is>
+          <t>Christos Kargiotis / Novelcomm</t>
+        </is>
+      </c>
+      <c r="B685" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C685" s="3" t="inlineStr">
+        <is>
+          <t>Athens</t>
+        </is>
+      </c>
+      <c r="D685" s="3" t="inlineStr">
+        <is>
+          <t>novelcomm.gr</t>
+        </is>
+      </c>
+      <c r="E685" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F685" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCTCE</t>
+        </is>
+      </c>
+      <c r="G685" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H685" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I685" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J685" s="3" t="inlineStr">
+        <is>
+          <t>+30 698 352 4337 / ckariotis@novelcomm.gr</t>
+        </is>
+      </c>
+      <c r="K685" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L685" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M685" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N685" s="3" t="inlineStr"/>
+      <c r="O685" s="3" t="inlineStr"/>
+      <c r="P685" s="3" t="inlineStr"/>
+      <c r="Q685" s="3" t="inlineStr">
+        <is>
+          <t>★★ 大型网络工程师；技能清单含 **PIM-SM（组播路由协议）→ IPTV/监控组播的核心**、OSPF、MPLS、MP-BGP、IPSec（PSK 与数字证书）、负载均衡、流量整形与 QoS、PtP/PtMP、**Switching**</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" s="3" t="inlineStr">
+        <is>
+          <t>Apostolas Georgios</t>
+        </is>
+      </c>
+      <c r="B686" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C686" s="3" t="inlineStr">
+        <is>
+          <t>Rodos（罗德岛）</t>
+        </is>
+      </c>
+      <c r="D686" s="3" t="inlineStr">
+        <is>
+          <t>apostolas.gr</t>
+        </is>
+      </c>
+      <c r="E686" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F686" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G686" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H686" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I686" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J686" s="3" t="inlineStr">
+        <is>
+          <t>+30 22410 38089 / george@apostolas.gr</t>
+        </is>
+      </c>
+      <c r="K686" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L686" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M686" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N686" s="3" t="inlineStr"/>
+      <c r="O686" s="3" t="inlineStr"/>
+      <c r="P686" s="3" t="inlineStr"/>
+      <c r="Q686" s="3" t="inlineStr">
+        <is>
+          <t>★★ 信息与通信系统工程师；自述「**酒店 WiFi 网络专家，从结构化布线规划到 RouterOS 编程全包**」；技能含 Routing、**Switching**、HotSpot、CAPsMAN 集中管理、无线、VLAN、脚本、防火墙 → 罗德岛是旅游岛，酒店密度极高，PoE 接入交换机是刚需</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" s="3" t="inlineStr">
+        <is>
+          <t>Charalampos Marinakis / SystemCon</t>
+        </is>
+      </c>
+      <c r="B687" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C687" s="3" t="inlineStr">
+        <is>
+          <t>Heraklion（克里特）</t>
+        </is>
+      </c>
+      <c r="D687" s="3" t="inlineStr">
+        <is>
+          <t>systemcon.gr</t>
+        </is>
+      </c>
+      <c r="E687" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F687" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCINE</t>
+        </is>
+      </c>
+      <c r="G687" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H687" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I687" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J687" s="3" t="inlineStr">
+        <is>
+          <t>+30 281 121 7219 / info@systemcon.gr</t>
+        </is>
+      </c>
+      <c r="K687" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L687" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M687" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N687" s="3" t="inlineStr"/>
+      <c r="O687" s="3" t="inlineStr"/>
+      <c r="P687" s="3" t="inlineStr"/>
+      <c r="Q687" s="3" t="inlineStr">
+        <is>
+          <t>★ 公司**同时交付硬件与软件网络系统**（从小型企业到企业级），并提供安装/配置/支持/管理的认证专业服务；核心服务：网络设计、**Routing、Switching**、防火墙安全、HotSpot 与用户管理、VPN、负载均衡与故障切换、高可用、流量整形与 QoS、无线、**SLA 支持服务**</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="3" t="inlineStr">
+        <is>
+          <t>Vasileios Tzamichas / Rom Digital</t>
+        </is>
+      </c>
+      <c r="B688" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C688" s="3" t="inlineStr">
+        <is>
+          <t>Athens</t>
+        </is>
+      </c>
+      <c r="D688" s="3" t="inlineStr">
+        <is>
+          <t>rom-psifiaki.gr</t>
+        </is>
+      </c>
+      <c r="E688" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F688" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G688" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H688" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I688" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J688" s="3" t="inlineStr">
+        <is>
+          <t>+30 693 220 1024 / technical@rom-psifiaki.gr</t>
+        </is>
+      </c>
+      <c r="K688" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L688" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M688" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N688" s="3" t="inlineStr"/>
+      <c r="O688" s="3" t="inlineStr"/>
+      <c r="P688" s="3" t="inlineStr"/>
+      <c r="Q688" s="3" t="inlineStr">
+        <is>
+          <t>★ **公司成立于 1983 年（40+ 年）**，自述「**专营 MikroTik 产品**」，为中型与大型组织提供技术服务 → 老牌公司、品牌专营、客户偏大中型</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="3" t="inlineStr">
+        <is>
+          <t>Georgios Argyrides</t>
+        </is>
+      </c>
+      <c r="B689" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C689" s="3" t="inlineStr">
+        <is>
+          <t>Thessaloniki</t>
+        </is>
+      </c>
+      <c r="D689" s="3" t="inlineStr"/>
+      <c r="E689" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F689" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G689" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H689" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I689" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328XG-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J689" s="3" t="inlineStr">
+        <is>
+          <t>+30 697 962 3656 / argeorge86@gmail.com</t>
+        </is>
+      </c>
+      <c r="K689" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L689" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M689" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N689" s="3" t="inlineStr"/>
+      <c r="O689" s="3" t="inlineStr"/>
+      <c r="P689" s="3" t="inlineStr"/>
+      <c r="Q689" s="3" t="inlineStr">
+        <is>
+          <t>2011 年起认证顾问、**2012 年起认证讲师**；WISP 室外无线 PtP/PtMP/Mesh，覆盖 2.4/5/24/**60GHz** 频段；专长 VLAN、高级带宽管理与 QoS、虚拟化、VoIP、RADIUS Hotspot、The Dude；**10+ 年国际出差做培训与现场勘测**</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="3" t="inlineStr">
+        <is>
+          <t>Katsariotis Dimitrios / IME</t>
+        </is>
+      </c>
+      <c r="B690" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C690" s="3" t="inlineStr">
+        <is>
+          <t>Patra</t>
+        </is>
+      </c>
+      <c r="D690" s="3" t="inlineStr">
+        <is>
+          <t>ime.com.gr</t>
+        </is>
+      </c>
+      <c r="E690" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F690" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCTCE+MTCSE</t>
+        </is>
+      </c>
+      <c r="G690" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H690" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I690" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J690" s="3" t="inlineStr">
+        <is>
+          <t>+30 697 762 8291 / dkats@ime.com.gr</t>
+        </is>
+      </c>
+      <c r="K690" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L690" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M690" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N690" s="3" t="inlineStr"/>
+      <c r="O690" s="3" t="inlineStr"/>
+      <c r="P690" s="3" t="inlineStr"/>
+      <c r="Q690" s="3" t="inlineStr">
+        <is>
+          <t>20+ 年网络基础设施设计实施管理支持；专长明确含 **switching**；路由、防火墙、无线、流量与带宽管理、IPSec/L2TP/SSTP/PPP/EoIP；云架构与 IT 管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="3" t="inlineStr">
+        <is>
+          <t>George Tatsis / GTA</t>
+        </is>
+      </c>
+      <c r="B691" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C691" s="3" t="inlineStr">
+        <is>
+          <t>Galatsi (Athens)</t>
+        </is>
+      </c>
+      <c r="D691" s="3" t="inlineStr">
+        <is>
+          <t>gta.gr</t>
+        </is>
+      </c>
+      <c r="E691" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F691" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCSE</t>
+        </is>
+      </c>
+      <c r="G691" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H691" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I691" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J691" s="3" t="inlineStr">
+        <is>
+          <t>+30 210 291 1011 / george@gta.gr</t>
+        </is>
+      </c>
+      <c r="K691" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L691" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M691" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N691" s="3" t="inlineStr"/>
+      <c r="O691" s="3" t="inlineStr"/>
+      <c r="P691" s="3" t="inlineStr"/>
+      <c r="Q691" s="3" t="inlineStr">
+        <is>
+          <t>★ 自述场景「**楼宇自控跑在网络上（controls running on the network），你需要为你的建筑提供稳定的承载网**」→ 楼宇自动化/弱电集成方向，帮客户设计、维护甚至翻新网络基础设施</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="3" t="inlineStr">
+        <is>
+          <t>George Karoubalis</t>
+        </is>
+      </c>
+      <c r="B692" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C692" s="3" t="inlineStr">
+        <is>
+          <t>Athens</t>
+        </is>
+      </c>
+      <c r="D692" s="3" t="inlineStr"/>
+      <c r="E692" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F692" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCWE+MTCTCE+MTCUME+MTCIPv6E+MTCSE</t>
+        </is>
+      </c>
+      <c r="G692" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H692" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I692" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J692" s="3" t="inlineStr">
+        <is>
+          <t>+30 210 440 0091 / g.karoub@gmail.com</t>
+        </is>
+      </c>
+      <c r="K692" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L692" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M692" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N692" s="3" t="inlineStr"/>
+      <c r="O692" s="3" t="inlineStr"/>
+      <c r="P692" s="3" t="inlineStr"/>
+      <c r="Q692" s="3" t="inlineStr">
+        <is>
+          <t>7 证含 MTCUME（用户管理）+ MTCTCE（流量控制）</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="3" t="inlineStr">
+        <is>
+          <t>Georgios Papageorgiou / DSlab</t>
+        </is>
+      </c>
+      <c r="B693" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C693" s="3" t="inlineStr">
+        <is>
+          <t>Chania</t>
+        </is>
+      </c>
+      <c r="D693" s="3" t="inlineStr">
+        <is>
+          <t>dslab.gr</t>
+        </is>
+      </c>
+      <c r="E693" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F693" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCWE+MTCIPv6E+MTCSE+MTCEWE</t>
+        </is>
+      </c>
+      <c r="G693" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H693" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I693" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J693" s="3" t="inlineStr">
+        <is>
+          <t>+30 694 240 0212 / info@dslab.gr</t>
+        </is>
+      </c>
+      <c r="K693" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L693" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M693" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N693" s="3" t="inlineStr"/>
+      <c r="O693" s="3" t="inlineStr"/>
+      <c r="P693" s="3" t="inlineStr"/>
+      <c r="Q693" s="3" t="inlineStr">
+        <is>
+          <t>负载均衡与故障切换、队列树 QoS、Hotspot、无线、隧道 VPN、CAPsMAN、防火墙、The Dude 监控</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" s="3" t="inlineStr">
+        <is>
+          <t>George Alexander Kontaxakis / EXA Solutions</t>
+        </is>
+      </c>
+      <c r="B694" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C694" s="3" t="inlineStr">
+        <is>
+          <t>Heraklion（克里特）</t>
+        </is>
+      </c>
+      <c r="D694" s="3" t="inlineStr">
+        <is>
+          <t>exasolutions.gr</t>
+        </is>
+      </c>
+      <c r="E694" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F694" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G694" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H694" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I694" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J694" s="3" t="inlineStr">
+        <is>
+          <t>+30 694 610 4339 / geokodax@exasolutions.gr</t>
+        </is>
+      </c>
+      <c r="K694" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L694" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M694" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N694" s="3" t="inlineStr"/>
+      <c r="O694" s="3" t="inlineStr"/>
+      <c r="P694" s="3" t="inlineStr"/>
+      <c r="Q694" s="3" t="inlineStr">
+        <is>
+          <t>IT 服务与**企业级规模网络**</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" s="3" t="inlineStr">
+        <is>
+          <t>Spiros Potsikas / Tele-Net</t>
+        </is>
+      </c>
+      <c r="B695" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C695" s="3" t="inlineStr">
+        <is>
+          <t>Rethimno（克里特）</t>
+        </is>
+      </c>
+      <c r="D695" s="3" t="inlineStr">
+        <is>
+          <t>tele-net.gr</t>
+        </is>
+      </c>
+      <c r="E695" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F695" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G695" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H695" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I695" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J695" s="3" t="inlineStr">
+        <is>
+          <t>+30 690 766 9554 / spyros.potsikas@gmail.com</t>
+        </is>
+      </c>
+      <c r="K695" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L695" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M695" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N695" s="3" t="inlineStr"/>
+      <c r="O695" s="3" t="inlineStr"/>
+      <c r="P695" s="3" t="inlineStr"/>
+      <c r="Q695" s="3" t="inlineStr"/>
+    </row>
+    <row r="696">
+      <c r="A696" s="3" t="inlineStr">
+        <is>
+          <t>Ioannis Orfanos</t>
+        </is>
+      </c>
+      <c r="B696" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C696" s="3" t="inlineStr">
+        <is>
+          <t>Asini Nafpliou</t>
+        </is>
+      </c>
+      <c r="D696" s="3" t="inlineStr"/>
+      <c r="E696" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F696" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCINE</t>
+        </is>
+      </c>
+      <c r="G696" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H696" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I696" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J696" s="3" t="inlineStr">
+        <is>
+          <t>+30 694 747 4659 / fearasini@gmail.com</t>
+        </is>
+      </c>
+      <c r="K696" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L696" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M696" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N696" s="3" t="inlineStr"/>
+      <c r="O696" s="3" t="inlineStr"/>
+      <c r="P696" s="3" t="inlineStr"/>
+      <c r="Q696" s="3" t="inlineStr">
+        <is>
+          <t>含 MTCINE（ISP 互联）</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="3" t="inlineStr">
+        <is>
+          <t>Konstantinos Analytis / Alfa-Tech</t>
+        </is>
+      </c>
+      <c r="B697" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C697" s="3" t="inlineStr">
+        <is>
+          <t>Argostoli</t>
+        </is>
+      </c>
+      <c r="D697" s="3" t="inlineStr">
+        <is>
+          <t>alfa-tech.gr</t>
+        </is>
+      </c>
+      <c r="E697" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F697" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSE</t>
+        </is>
+      </c>
+      <c r="G697" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H697" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I697" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J697" s="3" t="inlineStr">
+        <is>
+          <t>+30 26710 23655 / ka@alfa-tech.gr</t>
+        </is>
+      </c>
+      <c r="K697" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L697" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M697" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N697" s="3" t="inlineStr"/>
+      <c r="O697" s="3" t="inlineStr"/>
+      <c r="P697" s="3" t="inlineStr"/>
+      <c r="Q697" s="3" t="inlineStr"/>
+    </row>
+    <row r="698">
+      <c r="A698" s="3" t="inlineStr">
+        <is>
+          <t>Christos Kotoufos</t>
+        </is>
+      </c>
+      <c r="B698" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C698" s="3" t="inlineStr">
+        <is>
+          <t>Nea Makri</t>
+        </is>
+      </c>
+      <c r="D698" s="3" t="inlineStr"/>
+      <c r="E698" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F698" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSE</t>
+        </is>
+      </c>
+      <c r="G698" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H698" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I698" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J698" s="3" t="inlineStr">
+        <is>
+          <t>+30 211 800 0313 / chriskotoufos@gmail.com</t>
+        </is>
+      </c>
+      <c r="K698" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L698" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M698" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N698" s="3" t="inlineStr"/>
+      <c r="O698" s="3" t="inlineStr"/>
+      <c r="P698" s="3" t="inlineStr"/>
+      <c r="Q698" s="3" t="inlineStr"/>
+    </row>
+    <row r="699">
+      <c r="A699" s="3" t="inlineStr">
+        <is>
+          <t>Nikolaos Giovanopoulos</t>
+        </is>
+      </c>
+      <c r="B699" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C699" s="3" t="inlineStr">
+        <is>
+          <t>Athens</t>
+        </is>
+      </c>
+      <c r="D699" s="3" t="inlineStr">
+        <is>
+          <t>ien.gr</t>
+        </is>
+      </c>
+      <c r="E699" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F699" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSE</t>
+        </is>
+      </c>
+      <c r="G699" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H699" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I699" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J699" s="3" t="inlineStr">
+        <is>
+          <t>+30 694 347 5654 / ngiovanopoulos@ien.gr</t>
+        </is>
+      </c>
+      <c r="K699" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L699" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M699" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N699" s="3" t="inlineStr"/>
+      <c r="O699" s="3" t="inlineStr"/>
+      <c r="P699" s="3" t="inlineStr"/>
+      <c r="Q699" s="3" t="inlineStr"/>
+    </row>
+    <row r="700">
+      <c r="A700" s="3" t="inlineStr">
+        <is>
+          <t>Georgios Floros</t>
+        </is>
+      </c>
+      <c r="B700" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C700" s="3" t="inlineStr">
+        <is>
+          <t>Pallini</t>
+        </is>
+      </c>
+      <c r="D700" s="3" t="inlineStr"/>
+      <c r="E700" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F700" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSE</t>
+        </is>
+      </c>
+      <c r="G700" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H700" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I700" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J700" s="3" t="inlineStr">
+        <is>
+          <t>+30 215 555 2222 / giorgosfloros@yahoo.co.uk</t>
+        </is>
+      </c>
+      <c r="K700" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L700" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M700" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N700" s="3" t="inlineStr"/>
+      <c r="O700" s="3" t="inlineStr"/>
+      <c r="P700" s="3" t="inlineStr"/>
+      <c r="Q700" s="3" t="inlineStr"/>
+    </row>
+    <row r="701">
+      <c r="A701" s="3" t="inlineStr">
+        <is>
+          <t>Panagiotis Taxiarchis Chatzinikolaou</t>
+        </is>
+      </c>
+      <c r="B701" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C701" s="3" t="inlineStr">
+        <is>
+          <t>Mytilene</t>
+        </is>
+      </c>
+      <c r="D701" s="3" t="inlineStr"/>
+      <c r="E701" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F701" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCSE</t>
+        </is>
+      </c>
+      <c r="G701" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H701" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I701" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J701" s="3" t="inlineStr">
+        <is>
+          <t>+30 698 290 3349 / controlfieldgr@gmail.com</t>
+        </is>
+      </c>
+      <c r="K701" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L701" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M701" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N701" s="3" t="inlineStr"/>
+      <c r="O701" s="3" t="inlineStr"/>
+      <c r="P701" s="3" t="inlineStr"/>
+      <c r="Q701" s="3" t="inlineStr"/>
+    </row>
+    <row r="702">
+      <c r="A702" s="3" t="inlineStr">
+        <is>
+          <t>Lechouritis Ioannis</t>
+        </is>
+      </c>
+      <c r="B702" s="3" t="inlineStr">
+        <is>
+          <t>希腊</t>
+        </is>
+      </c>
+      <c r="C702" s="3" t="inlineStr">
+        <is>
+          <t>Neo Herakleio</t>
+        </is>
+      </c>
+      <c r="D702" s="3" t="inlineStr"/>
+      <c r="E702" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F702" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE+MTCSE</t>
+        </is>
+      </c>
+      <c r="G702" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H702" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I702" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J702" s="3" t="inlineStr">
+        <is>
+          <t>+30 697 734 2230 / lechjohnny@gmail.com</t>
+        </is>
+      </c>
+      <c r="K702" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L702" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M702" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N702" s="3" t="inlineStr"/>
+      <c r="O702" s="3" t="inlineStr"/>
+      <c r="P702" s="3" t="inlineStr"/>
+      <c r="Q702" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Final countries: North Macedonia, Kosovo, Montenegro, Malta, Moldova
Malta's only consultant holds MTCSWE and names hospitality, online
gaming, retail and manufacturing as his verticals, which matters
because Malta is an iGaming hub. A Moldovan consultant ships his own
centralised backup and traffic control software for MikroTik, making
him a tooling vendor as well as an integrator. Iceland has none.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -11188,7 +11188,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q702"/>
+  <dimension ref="A1:Q708"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -61675,6 +61675,432 @@
       <c r="O702" s="3" t="inlineStr"/>
       <c r="P702" s="3" t="inlineStr"/>
       <c r="Q702" s="3" t="inlineStr"/>
+    </row>
+    <row r="703">
+      <c r="A703" s="3" t="inlineStr">
+        <is>
+          <t>Aleksandar Cvetanoski</t>
+        </is>
+      </c>
+      <c r="B703" s="3" t="inlineStr">
+        <is>
+          <t>北马其顿</t>
+        </is>
+      </c>
+      <c r="C703" s="3" t="inlineStr">
+        <is>
+          <t>Skopje</t>
+        </is>
+      </c>
+      <c r="D703" s="3" t="inlineStr"/>
+      <c r="E703" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F703" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCRE</t>
+        </is>
+      </c>
+      <c r="G703" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H703" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I703" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J703" s="3" t="inlineStr">
+        <is>
+          <t>+389 78 299 716 / acvetanoskiii@gmail.com</t>
+        </is>
+      </c>
+      <c r="K703" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L703" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M703" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N703" s="3" t="inlineStr"/>
+      <c r="O703" s="3" t="inlineStr"/>
+      <c r="P703" s="3" t="inlineStr"/>
+      <c r="Q703" s="3" t="inlineStr">
+        <is>
+          <t>★ 北马其顿**唯一**认证顾问（稀缺）；10+ 年 RouterOS 经验；为**中小企业与大型企业**做设计/实施/**迁移**/排障；专长含 **Routing、Switching**、VPN 隧道、防火墙、NAT、Mangle、QoS → 做迁移的人会评估替代方案</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="3" t="inlineStr">
+        <is>
+          <t>Dan Erhan</t>
+        </is>
+      </c>
+      <c r="B704" s="3" t="inlineStr">
+        <is>
+          <t>摩尔多瓦</t>
+        </is>
+      </c>
+      <c r="C704" s="3" t="inlineStr">
+        <is>
+          <t>Hancesti</t>
+        </is>
+      </c>
+      <c r="D704" s="3" t="inlineStr"/>
+      <c r="E704" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F704" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSWE</t>
+        </is>
+      </c>
+      <c r="G704" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H704" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I704" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J704" s="3" t="inlineStr">
+        <is>
+          <t>+373 798 117 28 / dan.erhan.off@gmail.com</t>
+        </is>
+      </c>
+      <c r="K704" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L704" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M704" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N704" s="3" t="inlineStr"/>
+      <c r="O704" s="3" t="inlineStr"/>
+      <c r="P704" s="3" t="inlineStr"/>
+      <c r="Q704" s="3" t="inlineStr">
+        <is>
+          <t>持 MTCSWE（交换认证）；英俄罗三语</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="3" t="inlineStr">
+        <is>
+          <t>Radion Gareev / Meganet</t>
+        </is>
+      </c>
+      <c r="B705" s="3" t="inlineStr">
+        <is>
+          <t>摩尔多瓦</t>
+        </is>
+      </c>
+      <c r="C705" s="3" t="inlineStr">
+        <is>
+          <t>Chisinau</t>
+        </is>
+      </c>
+      <c r="D705" s="3" t="inlineStr">
+        <is>
+          <t>meganet.md</t>
+        </is>
+      </c>
+      <c r="E705" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F705" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCINE</t>
+        </is>
+      </c>
+      <c r="G705" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H705" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I705" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J705" s="3" t="inlineStr">
+        <is>
+          <t>+373 685 666 11 / radeon_service@mail.ru</t>
+        </is>
+      </c>
+      <c r="K705" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L705" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M705" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N705" s="3" t="inlineStr"/>
+      <c r="O705" s="3" t="inlineStr"/>
+      <c r="P705" s="3" t="inlineStr"/>
+      <c r="Q705" s="3" t="inlineStr">
+        <is>
+          <t>承接任何 MikroTik 配置或咨询任务；含 MTCINE（ISP 互联）；英俄罗三语</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="3" t="inlineStr">
+        <is>
+          <t>（摩尔多瓦）MikroTik 集中管理软件开发者</t>
+        </is>
+      </c>
+      <c r="B706" s="3" t="inlineStr">
+        <is>
+          <t>摩尔多瓦</t>
+        </is>
+      </c>
+      <c r="C706" s="3" t="inlineStr"/>
+      <c r="D706" s="3" t="inlineStr"/>
+      <c r="E706" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F706" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 含 Security Engineer 方向</t>
+        </is>
+      </c>
+      <c r="G706" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H706" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I706" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328GP-4GX24GT-S</t>
+        </is>
+      </c>
+      <c r="J706" s="3" t="inlineStr">
+        <is>
+          <t>+373 795 065 44 / Vovcik81@mail.ru</t>
+        </is>
+      </c>
+      <c r="K706" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L706" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M706" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N706" s="3" t="inlineStr"/>
+      <c r="O706" s="3" t="inlineStr"/>
+      <c r="P706" s="3" t="inlineStr"/>
+      <c r="Q706" s="3" t="inlineStr">
+        <is>
+          <t>★★ **自研软件产品**：集中化设备备份、集中软件升级、流量控制、版本变更比对等，一套软件搞定 → 做 MikroTik 生态工具的，会非常看重设备的 API/SNMP/可管理性，且他自己就是渠道；同时承接有线无线网络、控制器与流量优先级、防火墙、CAPsMAN、OSPF 项目，并有 MikroTik 安全工程师资质（安全审计）</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="3" t="inlineStr">
+        <is>
+          <t>Jeton Syla</t>
+        </is>
+      </c>
+      <c r="B707" s="3" t="inlineStr">
+        <is>
+          <t>科索沃</t>
+        </is>
+      </c>
+      <c r="C707" s="3" t="inlineStr"/>
+      <c r="D707" s="3" t="inlineStr"/>
+      <c r="E707" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F707" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MikroTik 认证顾问 </t>
+        </is>
+      </c>
+      <c r="G707" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H707" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I707" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J707" s="3" t="inlineStr">
+        <is>
+          <t>+383 45 512 344 / jetoonsyla@gmail.com</t>
+        </is>
+      </c>
+      <c r="K707" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L707" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M707" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N707" s="3" t="inlineStr"/>
+      <c r="O707" s="3" t="inlineStr"/>
+      <c r="P707" s="3" t="inlineStr"/>
+      <c r="Q707" s="3" t="inlineStr">
+        <is>
+          <t>科索沃**唯一**认证顾问（稀缺）</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="3" t="inlineStr">
+        <is>
+          <t>Andrey Glushchenko / Core-Bridge</t>
+        </is>
+      </c>
+      <c r="B708" s="3" t="inlineStr">
+        <is>
+          <t>黑山</t>
+        </is>
+      </c>
+      <c r="C708" s="3" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
+      <c r="D708" s="3" t="inlineStr">
+        <is>
+          <t>core-bridge.me</t>
+        </is>
+      </c>
+      <c r="E708" s="3" t="inlineStr">
+        <is>
+          <t>集成商/顾问（MikroTik 认证）</t>
+        </is>
+      </c>
+      <c r="F708" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问 MTCNA+MTCSE</t>
+        </is>
+      </c>
+      <c r="G708" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H708" s="3" t="inlineStr">
+        <is>
+          <t>MikroTik 认证顾问：自己做方案/集成/运维并自行采购设备 → 用 ERPS/IGMP/VLAN/CLI/MIB 这类技术语言切入，不打价格战</t>
+        </is>
+      </c>
+      <c r="I708" s="3" t="inlineStr">
+        <is>
+          <t>LT-S8328G-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J708" s="3" t="inlineStr">
+        <is>
+          <t>+382 068 176 243 / AndreiGL@core-bridge.me</t>
+        </is>
+      </c>
+      <c r="K708" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="L708" s="3" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M708" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="N708" s="3" t="inlineStr"/>
+      <c r="O708" s="3" t="inlineStr"/>
+      <c r="P708" s="3" t="inlineStr"/>
+      <c r="Q708" s="3" t="inlineStr">
+        <is>
+          <t>黑山**唯一**认证顾问（稀缺）；英俄塞三语</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add a per-customer dossier under profile/, one file each
705 dossiers plus an index. Each carries the grade and why, company
overview, the named people with their direct lines, certifications and
brands, the follow-up play, the cautions, and an empty log to fill in
after contact.

A Chinese ambiguity is fixed along the way: the word 监控 covers both
video surveillance and network monitoring, so matching it bare was
crediting NMS integrators with a CCTV requirement. Requiring 视频监控
or 摄像头 moves eight such accounts out of A, including Hotelinking,
which is really a hotel and multi-site networking shop, and K2O, whose
monitoring practice is RouterOS monitoring rather than cameras.

This drops A from 96 to 88.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -12657,12 +12657,12 @@
       </c>
       <c r="R18" s="3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="S18" s="3" t="inlineStr">
         <is>
-          <t>有明确交换/供电需求（PoE/监控/门禁），三星重点</t>
+          <t>通用分销商信号，无差异化切入点，慢慢跟</t>
         </is>
       </c>
     </row>
@@ -33334,7 +33334,7 @@
       </c>
       <c r="S274" s="3" t="inlineStr">
         <is>
-          <t>有明确交换/供电需求（PoE/监控/门禁、工业/楼宇、组播/IPTV），且有具体人直联</t>
+          <t>有明确交换/供电需求（工业/楼宇、组播/IPTV），且有具体人直联</t>
         </is>
       </c>
     </row>
@@ -34468,7 +34468,7 @@
       </c>
       <c r="S288" s="3" t="inlineStr">
         <is>
-          <t>有信号（PoE/监控/门禁）但需先验证需求或联系人不具体</t>
+          <t>通用分销商信号，无差异化切入点，慢慢跟</t>
         </is>
       </c>
     </row>
@@ -52989,12 +52989,12 @@
       </c>
       <c r="R510" s="3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="S510" s="3" t="inlineStr">
         <is>
-          <t>有明确交换/供电需求（PoE/监控/门禁），且有具体人直联</t>
+          <t>有信号（ISP/骨干）但需先验证需求或联系人不具体</t>
         </is>
       </c>
     </row>
@@ -54516,7 +54516,7 @@
       </c>
       <c r="S528" s="3" t="inlineStr">
         <is>
-          <t>有明确交换/供电需求（交换认证 MTCSWE、交换专长、PoE/监控/门禁），且有具体人直联</t>
+          <t>有明确交换/供电需求（交换认证 MTCSWE、交换专长），且有具体人直联</t>
         </is>
       </c>
     </row>
@@ -54932,12 +54932,12 @@
       </c>
       <c r="R533" s="3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="S533" s="3" t="inlineStr">
         <is>
-          <t>有明确交换/供电需求（PoE/监控/门禁），且有具体人直联</t>
+          <t>通用分销商信号，无差异化切入点，慢慢跟</t>
         </is>
       </c>
     </row>
@@ -55017,12 +55017,12 @@
       </c>
       <c r="R534" s="3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="S534" s="3" t="inlineStr">
         <is>
-          <t>有明确交换/供电需求（PoE/监控/门禁），且有具体人直联</t>
+          <t>通用分销商信号，无差异化切入点，慢慢跟</t>
         </is>
       </c>
     </row>
@@ -58106,12 +58106,12 @@
       </c>
       <c r="R571" s="3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="S571" s="3" t="inlineStr">
         <is>
-          <t>有明确交换/供电需求（PoE/监控/门禁），且有具体人直联</t>
+          <t>有信号（影响力/渠道）但需先验证需求或联系人不具体</t>
         </is>
       </c>
     </row>
@@ -62006,7 +62006,7 @@
       </c>
       <c r="S618" s="3" t="inlineStr">
         <is>
-          <t>有明确交换/供电需求（交换专长、PoE/监控/门禁），且有具体人直联</t>
+          <t>有明确交换/供电需求（交换专长），且有具体人直联</t>
         </is>
       </c>
     </row>
@@ -62427,7 +62427,7 @@
       </c>
       <c r="S623" s="3" t="inlineStr">
         <is>
-          <t>有明确交换/供电需求（交换专长、PoE/监控/门禁），且有具体人直联</t>
+          <t>有明确交换/供电需求（交换专长），且有具体人直联</t>
         </is>
       </c>
     </row>
@@ -63018,7 +63018,7 @@
       </c>
       <c r="S630" s="3" t="inlineStr">
         <is>
-          <t>有明确交换/供电需求（交换认证 MTCSWE、交换专长、PoE/监控/门禁），且有具体人直联</t>
+          <t>有明确交换/供电需求（交换认证 MTCSWE、交换专长、组播/IPTV），且有具体人直联</t>
         </is>
       </c>
     </row>
@@ -63098,12 +63098,12 @@
       </c>
       <c r="R631" s="3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="S631" s="3" t="inlineStr">
         <is>
-          <t>有明确交换/供电需求（PoE/监控/门禁），且有具体人直联</t>
+          <t>有信号（ISP/骨干、校园/教育、影响力/渠道）但需先验证需求或联系人不具体</t>
         </is>
       </c>
     </row>
@@ -63183,12 +63183,12 @@
       </c>
       <c r="R632" s="3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="S632" s="3" t="inlineStr">
         <is>
-          <t>有明确交换/供电需求（PoE/监控/门禁），且有具体人直联</t>
+          <t>有信号（ISP/骨干、影响力/渠道）但需先验证需求或联系人不具体</t>
         </is>
       </c>
     </row>
@@ -63268,12 +63268,12 @@
       </c>
       <c r="R633" s="3" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="S633" s="3" t="inlineStr">
         <is>
-          <t>有明确交换/供电需求（PoE/监控/门禁），且有具体人直联</t>
+          <t>有信号（ISP/骨干）但需先验证需求或联系人不具体</t>
         </is>
       </c>
     </row>
@@ -68075,7 +68075,7 @@
       </c>
       <c r="S691" s="3" t="inlineStr">
         <is>
-          <t>有信号（PoE/监控/门禁）但需先验证需求或联系人不具体</t>
+          <t>通用分销商信号，无差异化切入点，慢慢跟</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mine Teltonika and Allied Telesis channels; A 118 -> 122
Following the scope correction, this round targets vendors that are
genuinely inside the Marvell access-layer ecosystem rather than the
broader WISP space.

Allied Telesis builds on Marvell Prestera, which makes its reseller list
a clean fit for the rule. Teltonika is a European vendor with its own
TSW access switch line and an established channel on both continents.

27 new accounts: 4 Teltonika distributors including Capestone, the
Diamond partner and largest European value-added distributor, and 23
Allied Telesis partners across the US, Sweden and Spain. A goes 118 to
122.

Deliberately excluded Graybar and Ingram Micro from the Allied Telesis
list as too large to be worth the effort, and flagged the two Security
101 entities as separate operations so outreach does not double up.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/MikroTik_vs_SmartByte_替代对照表.xlsx
+++ b/MikroTik_vs_SmartByte_替代对照表.xlsx
@@ -5212,7 +5212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U780"/>
+  <dimension ref="A1:U807"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -75266,6 +75266,2355 @@
         </is>
       </c>
       <c r="U780" t="inlineStr"/>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>Capestone</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>荷兰</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr"/>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>capestone.com</t>
+        </is>
+      </c>
+      <c r="E781" t="inlineStr">
+        <is>
+          <t>分销（Teltonika 授权）</t>
+        </is>
+      </c>
+      <c r="F781" t="inlineStr">
+        <is>
+          <t>Teltonika Networks（含 TSW 系列交换机）</t>
+        </is>
+      </c>
+      <c r="G781" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H781" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I781" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J781" t="inlineStr">
+        <is>
+          <t>见 capestone.com</t>
+        </is>
+      </c>
+      <c r="K781" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L781" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M781" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N781" t="inlineStr"/>
+      <c r="O781" t="inlineStr"/>
+      <c r="P781" t="inlineStr"/>
+      <c r="Q781" t="inlineStr">
+        <is>
+          <t>Teltonika **Diamond 级伙伴，连续 7 年**、**欧洲最大增值分销**。备货型分销，提供售前咨询/项目支持/配置/培训/云管平台全托管。</t>
+        </is>
+      </c>
+      <c r="R781" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S781" t="inlineStr">
+        <is>
+          <t>备注含「最大」，决策链长或存在品牌冲突</t>
+        </is>
+      </c>
+      <c r="T781" t="inlineStr">
+        <is>
+          <t>C-320</t>
+        </is>
+      </c>
+      <c r="U781" t="inlineStr">
+        <is>
+          <t>太难·规模过大/决策链长</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>NTS Direct</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>Bolton, MA</t>
+        </is>
+      </c>
+      <c r="D782" t="inlineStr">
+        <is>
+          <t>shop.ntsdirect.com</t>
+        </is>
+      </c>
+      <c r="E782" t="inlineStr">
+        <is>
+          <t>分销（Teltonika 授权）</t>
+        </is>
+      </c>
+      <c r="F782" t="inlineStr">
+        <is>
+          <t>Teltonika Networks（含 TSW 系列交换机）</t>
+        </is>
+      </c>
+      <c r="G782" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H782" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I782" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J782" t="inlineStr">
+        <is>
+          <t>见 shop.ntsdirect.com</t>
+        </is>
+      </c>
+      <c r="K782" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L782" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M782" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N782" t="inlineStr"/>
+      <c r="O782" t="inlineStr"/>
+      <c r="P782" t="inlineStr"/>
+      <c r="Q782" t="inlineStr">
+        <is>
+          <t>2025 年与 Teltonika 达成**北美战略分销合作**，备货并提供预配置、技术培训、集成支持。</t>
+        </is>
+      </c>
+      <c r="R782" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="S782" t="inlineStr">
+        <is>
+          <t>有明确交换/供电需求（交换专长），三星重点</t>
+        </is>
+      </c>
+      <c r="T782" t="inlineStr">
+        <is>
+          <t>A-119</t>
+        </is>
+      </c>
+      <c r="U782" t="inlineStr"/>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>5Gstore</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr"/>
+      <c r="D783" t="inlineStr">
+        <is>
+          <t>5gstore.com</t>
+        </is>
+      </c>
+      <c r="E783" t="inlineStr">
+        <is>
+          <t>分销（Teltonika 授权）</t>
+        </is>
+      </c>
+      <c r="F783" t="inlineStr">
+        <is>
+          <t>Teltonika Networks（含 TSW212 工业 PoE+ 交换机）</t>
+        </is>
+      </c>
+      <c r="G783" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H783" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I783" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J783" t="inlineStr">
+        <is>
+          <t>见 5gstore.com</t>
+        </is>
+      </c>
+      <c r="K783" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L783" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M783" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N783" t="inlineStr"/>
+      <c r="O783" t="inlineStr"/>
+      <c r="P783" t="inlineStr"/>
+      <c r="Q783" t="inlineStr">
+        <is>
+          <t>Teltonika 授权分销，主营工业蜂窝路由与 IoT 网关，**亦供 TSW212 等工业 PoE+ 交换机**。</t>
+        </is>
+      </c>
+      <c r="R783" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="S783" t="inlineStr">
+        <is>
+          <t>有明确交换/供电需求（交换专长、PoE/监控/门禁、工业/楼宇），三星重点</t>
+        </is>
+      </c>
+      <c r="T783" t="inlineStr">
+        <is>
+          <t>A-120</t>
+        </is>
+      </c>
+      <c r="U783" t="inlineStr"/>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>A3 Communications</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>Cumberland Foreside, ME</t>
+        </is>
+      </c>
+      <c r="D784" t="inlineStr"/>
+      <c r="E784" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F784" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G784" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H784" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I784" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J784" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com/us/en/resellers</t>
+        </is>
+      </c>
+      <c r="K784" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L784" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M784" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N784" t="inlineStr"/>
+      <c r="O784" t="inlineStr"/>
+      <c r="P784" t="inlineStr"/>
+      <c r="Q784" t="inlineStr"/>
+      <c r="R784" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S784" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T784" t="inlineStr">
+        <is>
+          <t>C-321</t>
+        </is>
+      </c>
+      <c r="U784" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>Amplitel Technologies</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>Kaukauna, WI</t>
+        </is>
+      </c>
+      <c r="D785" t="inlineStr"/>
+      <c r="E785" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F785" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G785" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H785" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I785" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J785" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com 代理商名录</t>
+        </is>
+      </c>
+      <c r="K785" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L785" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M785" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N785" t="inlineStr"/>
+      <c r="O785" t="inlineStr"/>
+      <c r="P785" t="inlineStr"/>
+      <c r="Q785" t="inlineStr"/>
+      <c r="R785" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S785" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T785" t="inlineStr">
+        <is>
+          <t>C-322</t>
+        </is>
+      </c>
+      <c r="U785" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>BCL Enterprises, Inc.</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>Middletown</t>
+        </is>
+      </c>
+      <c r="D786" t="inlineStr"/>
+      <c r="E786" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F786" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G786" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H786" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I786" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J786" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com 代理商名录</t>
+        </is>
+      </c>
+      <c r="K786" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L786" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M786" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N786" t="inlineStr"/>
+      <c r="O786" t="inlineStr"/>
+      <c r="P786" t="inlineStr"/>
+      <c r="Q786" t="inlineStr"/>
+      <c r="R786" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S786" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T786" t="inlineStr">
+        <is>
+          <t>C-323</t>
+        </is>
+      </c>
+      <c r="U786" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>Davis Ulmer Family of Companies</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>East Syracuse, NY / Fargo, ND</t>
+        </is>
+      </c>
+      <c r="D787" t="inlineStr"/>
+      <c r="E787" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F787" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G787" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H787" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I787" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J787" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com 代理商名录</t>
+        </is>
+      </c>
+      <c r="K787" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L787" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M787" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N787" t="inlineStr"/>
+      <c r="O787" t="inlineStr"/>
+      <c r="P787" t="inlineStr"/>
+      <c r="Q787" t="inlineStr">
+        <is>
+          <t>多地经营。</t>
+        </is>
+      </c>
+      <c r="R787" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S787" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T787" t="inlineStr">
+        <is>
+          <t>C-324</t>
+        </is>
+      </c>
+      <c r="U787" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>Gemellaro Systems Integration (GSI)</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>Troy, MI</t>
+        </is>
+      </c>
+      <c r="D788" t="inlineStr"/>
+      <c r="E788" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F788" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G788" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H788" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I788" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J788" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com 代理商名录</t>
+        </is>
+      </c>
+      <c r="K788" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L788" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M788" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N788" t="inlineStr"/>
+      <c r="O788" t="inlineStr"/>
+      <c r="P788" t="inlineStr"/>
+      <c r="Q788" t="inlineStr">
+        <is>
+          <t>系统集成商。</t>
+        </is>
+      </c>
+      <c r="R788" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S788" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T788" t="inlineStr">
+        <is>
+          <t>C-325</t>
+        </is>
+      </c>
+      <c r="U788" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>Griffon Security Technologies, LLC</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>Kennebunk, ME</t>
+        </is>
+      </c>
+      <c r="D789" t="inlineStr"/>
+      <c r="E789" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F789" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G789" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H789" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I789" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J789" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com 代理商名录</t>
+        </is>
+      </c>
+      <c r="K789" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L789" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M789" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N789" t="inlineStr"/>
+      <c r="O789" t="inlineStr"/>
+      <c r="P789" t="inlineStr"/>
+      <c r="Q789" t="inlineStr"/>
+      <c r="R789" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S789" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T789" t="inlineStr">
+        <is>
+          <t>C-326</t>
+        </is>
+      </c>
+      <c r="U789" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>Heartland Business Systems</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>Little Chute, WI</t>
+        </is>
+      </c>
+      <c r="D790" t="inlineStr"/>
+      <c r="E790" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F790" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G790" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H790" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I790" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J790" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com 代理商名录</t>
+        </is>
+      </c>
+      <c r="K790" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L790" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M790" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N790" t="inlineStr"/>
+      <c r="O790" t="inlineStr"/>
+      <c r="P790" t="inlineStr"/>
+      <c r="Q790" t="inlineStr"/>
+      <c r="R790" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S790" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T790" t="inlineStr">
+        <is>
+          <t>C-327</t>
+        </is>
+      </c>
+      <c r="U790" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>ITC Technologies</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>Maybrook, NY</t>
+        </is>
+      </c>
+      <c r="D791" t="inlineStr"/>
+      <c r="E791" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F791" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G791" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H791" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I791" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J791" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com 代理商名录</t>
+        </is>
+      </c>
+      <c r="K791" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L791" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M791" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N791" t="inlineStr"/>
+      <c r="O791" t="inlineStr"/>
+      <c r="P791" t="inlineStr"/>
+      <c r="Q791" t="inlineStr"/>
+      <c r="R791" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S791" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T791" t="inlineStr">
+        <is>
+          <t>C-328</t>
+        </is>
+      </c>
+      <c r="U791" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>Kidwell Inc.</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>Lincoln, NE</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr"/>
+      <c r="E792" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F792" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G792" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H792" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I792" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J792" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com 代理商名录</t>
+        </is>
+      </c>
+      <c r="K792" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L792" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M792" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N792" t="inlineStr"/>
+      <c r="O792" t="inlineStr"/>
+      <c r="P792" t="inlineStr"/>
+      <c r="Q792" t="inlineStr"/>
+      <c r="R792" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S792" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T792" t="inlineStr">
+        <is>
+          <t>C-329</t>
+        </is>
+      </c>
+      <c r="U792" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>Nexware Technologies</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>Chandler, AZ</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr"/>
+      <c r="E793" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F793" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G793" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H793" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I793" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J793" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com 代理商名录</t>
+        </is>
+      </c>
+      <c r="K793" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L793" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M793" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N793" t="inlineStr"/>
+      <c r="O793" t="inlineStr"/>
+      <c r="P793" t="inlineStr"/>
+      <c r="Q793" t="inlineStr"/>
+      <c r="R793" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S793" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T793" t="inlineStr">
+        <is>
+          <t>C-330</t>
+        </is>
+      </c>
+      <c r="U793" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>Paramount Security Partners</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr"/>
+      <c r="D794" t="inlineStr"/>
+      <c r="E794" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F794" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G794" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H794" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I794" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J794" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com 代理商名录</t>
+        </is>
+      </c>
+      <c r="K794" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L794" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M794" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N794" t="inlineStr"/>
+      <c r="O794" t="inlineStr"/>
+      <c r="P794" t="inlineStr"/>
+      <c r="Q794" t="inlineStr"/>
+      <c r="R794" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S794" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T794" t="inlineStr">
+        <is>
+          <t>C-331</t>
+        </is>
+      </c>
+      <c r="U794" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>Professional Cabling Solutions (PCS), LLC</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>Cincinnati, OH</t>
+        </is>
+      </c>
+      <c r="D795" t="inlineStr"/>
+      <c r="E795" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F795" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G795" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H795" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I795" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J795" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com 代理商名录</t>
+        </is>
+      </c>
+      <c r="K795" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L795" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M795" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N795" t="inlineStr"/>
+      <c r="O795" t="inlineStr"/>
+      <c r="P795" t="inlineStr"/>
+      <c r="Q795" t="inlineStr">
+        <is>
+          <t>综合布线+网络，接入层落地能力强。</t>
+        </is>
+      </c>
+      <c r="R795" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S795" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T795" t="inlineStr">
+        <is>
+          <t>C-332</t>
+        </is>
+      </c>
+      <c r="U795" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>Riverside Technologies Inc</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>North Sioux City, SD</t>
+        </is>
+      </c>
+      <c r="D796" t="inlineStr"/>
+      <c r="E796" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F796" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G796" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H796" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I796" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J796" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com 代理商名录</t>
+        </is>
+      </c>
+      <c r="K796" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L796" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M796" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N796" t="inlineStr"/>
+      <c r="O796" t="inlineStr"/>
+      <c r="P796" t="inlineStr"/>
+      <c r="Q796" t="inlineStr"/>
+      <c r="R796" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S796" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T796" t="inlineStr">
+        <is>
+          <t>C-333</t>
+        </is>
+      </c>
+      <c r="U796" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>Security 101 - CT</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>Southington, CT</t>
+        </is>
+      </c>
+      <c r="D797" t="inlineStr"/>
+      <c r="E797" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F797" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G797" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H797" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I797" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J797" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com 代理商名录</t>
+        </is>
+      </c>
+      <c r="K797" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L797" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M797" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N797" t="inlineStr"/>
+      <c r="O797" t="inlineStr"/>
+      <c r="P797" t="inlineStr"/>
+      <c r="Q797" t="inlineStr"/>
+      <c r="R797" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S797" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T797" t="inlineStr">
+        <is>
+          <t>C-334</t>
+        </is>
+      </c>
+      <c r="U797" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>Security 101 - Rochester NY</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>Rochester, NY</t>
+        </is>
+      </c>
+      <c r="D798" t="inlineStr"/>
+      <c r="E798" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F798" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G798" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H798" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I798" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J798" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com 代理商名录</t>
+        </is>
+      </c>
+      <c r="K798" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L798" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M798" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N798" t="inlineStr"/>
+      <c r="O798" t="inlineStr"/>
+      <c r="P798" t="inlineStr"/>
+      <c r="Q798" t="inlineStr">
+        <is>
+          <t>与 Security 101 - CT 同品牌不同实体，**注意别重复触达**。</t>
+        </is>
+      </c>
+      <c r="R798" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S798" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T798" t="inlineStr">
+        <is>
+          <t>C-335</t>
+        </is>
+      </c>
+      <c r="U798" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>Shea Electric</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>Oshkosh, WI</t>
+        </is>
+      </c>
+      <c r="D799" t="inlineStr"/>
+      <c r="E799" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F799" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G799" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H799" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I799" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J799" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com 代理商名录</t>
+        </is>
+      </c>
+      <c r="K799" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L799" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M799" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N799" t="inlineStr"/>
+      <c r="O799" t="inlineStr"/>
+      <c r="P799" t="inlineStr"/>
+      <c r="Q799" t="inlineStr"/>
+      <c r="R799" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S799" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T799" t="inlineStr">
+        <is>
+          <t>C-336</t>
+        </is>
+      </c>
+      <c r="U799" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>Silco Fire Protection &amp; Security</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr"/>
+      <c r="D800" t="inlineStr"/>
+      <c r="E800" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F800" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G800" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H800" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I800" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J800" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com 代理商名录</t>
+        </is>
+      </c>
+      <c r="K800" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L800" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M800" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N800" t="inlineStr"/>
+      <c r="O800" t="inlineStr"/>
+      <c r="P800" t="inlineStr"/>
+      <c r="Q800" t="inlineStr"/>
+      <c r="R800" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S800" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T800" t="inlineStr">
+        <is>
+          <t>C-337</t>
+        </is>
+      </c>
+      <c r="U800" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>UberData Networks</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr"/>
+      <c r="D801" t="inlineStr"/>
+      <c r="E801" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F801" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G801" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H801" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I801" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J801" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com 代理商名录</t>
+        </is>
+      </c>
+      <c r="K801" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L801" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M801" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N801" t="inlineStr"/>
+      <c r="O801" t="inlineStr"/>
+      <c r="P801" t="inlineStr"/>
+      <c r="Q801" t="inlineStr"/>
+      <c r="R801" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S801" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T801" t="inlineStr">
+        <is>
+          <t>C-338</t>
+        </is>
+      </c>
+      <c r="U801" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>VARtek Services Inc</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr"/>
+      <c r="D802" t="inlineStr"/>
+      <c r="E802" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F802" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G802" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H802" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I802" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J802" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com 代理商名录</t>
+        </is>
+      </c>
+      <c r="K802" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L802" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M802" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N802" t="inlineStr"/>
+      <c r="O802" t="inlineStr"/>
+      <c r="P802" t="inlineStr"/>
+      <c r="Q802" t="inlineStr"/>
+      <c r="R802" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S802" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T802" t="inlineStr">
+        <is>
+          <t>C-339</t>
+        </is>
+      </c>
+      <c r="U802" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>Wire Technologies, Inc.</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>美国</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr"/>
+      <c r="D803" t="inlineStr"/>
+      <c r="E803" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F803" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）</t>
+        </is>
+      </c>
+      <c r="G803" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H803" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I803" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J803" t="inlineStr">
+        <is>
+          <t>见 alliedtelesis.com 代理商名录</t>
+        </is>
+      </c>
+      <c r="K803" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L803" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M803" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N803" t="inlineStr"/>
+      <c r="O803" t="inlineStr"/>
+      <c r="P803" t="inlineStr"/>
+      <c r="Q803" t="inlineStr"/>
+      <c r="R803" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S803" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T803" t="inlineStr">
+        <is>
+          <t>C-340</t>
+        </is>
+      </c>
+      <c r="U803" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>BRS Networks AB</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>瑞典</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr"/>
+      <c r="D804" t="inlineStr"/>
+      <c r="E804" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F804" t="inlineStr">
+        <is>
+          <t>Allied Telesis（Marvell Prestera 接入层）+ Fortinet</t>
+        </is>
+      </c>
+      <c r="G804" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H804" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I804" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J804" t="inlineStr">
+        <is>
+          <t>见 elioplus 渠道库</t>
+        </is>
+      </c>
+      <c r="K804" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L804" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M804" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N804" t="inlineStr"/>
+      <c r="O804" t="inlineStr"/>
+      <c r="P804" t="inlineStr"/>
+      <c r="Q804" t="inlineStr">
+        <is>
+          <t>**光纤网络方案商，业务覆盖瑞典、丹麦、德国** —— 北欧+德语区三地经营。</t>
+        </is>
+      </c>
+      <c r="R804" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="S804" t="inlineStr">
+        <is>
+          <t>有明确交换/供电需求（光纤接入），三星重点</t>
+        </is>
+      </c>
+      <c r="T804" t="inlineStr">
+        <is>
+          <t>A-121</t>
+        </is>
+      </c>
+      <c r="U804" t="inlineStr"/>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>Berdin Grupo</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr"/>
+      <c r="D805" t="inlineStr"/>
+      <c r="E805" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F805" t="inlineStr">
+        <is>
+          <t>Allied Telesis + Bosch + Comnet + Genetec + Hanwha + Commscope + Fortinet</t>
+        </is>
+      </c>
+      <c r="G805" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H805" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I805" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J805" t="inlineStr">
+        <is>
+          <t>见 elioplus 渠道库</t>
+        </is>
+      </c>
+      <c r="K805" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L805" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M805" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N805" t="inlineStr"/>
+      <c r="O805" t="inlineStr"/>
+      <c r="P805" t="inlineStr"/>
+      <c r="Q805" t="inlineStr">
+        <is>
+          <t>西班牙，覆盖照明/楼控、电气、安防、工业自动化、通信与能源。</t>
+        </is>
+      </c>
+      <c r="R805" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="S805" t="inlineStr">
+        <is>
+          <t>有明确交换/供电需求（工业/楼宇），三星重点</t>
+        </is>
+      </c>
+      <c r="T805" t="inlineStr">
+        <is>
+          <t>A-122</t>
+        </is>
+      </c>
+      <c r="U805" t="inlineStr"/>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>DeInta</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>Zaragoza</t>
+        </is>
+      </c>
+      <c r="D806" t="inlineStr"/>
+      <c r="E806" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F806" t="inlineStr">
+        <is>
+          <t>Allied Telesis + Axis + 3CX + HP</t>
+        </is>
+      </c>
+      <c r="G806" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H806" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I806" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J806" t="inlineStr">
+        <is>
+          <t>见 elioplus 渠道库</t>
+        </is>
+      </c>
+      <c r="K806" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L806" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M806" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N806" t="inlineStr"/>
+      <c r="O806" t="inlineStr"/>
+      <c r="P806" t="inlineStr"/>
+      <c r="Q806" t="inlineStr">
+        <is>
+          <t>西班牙 Zaragoza，VOIP 与网络。</t>
+        </is>
+      </c>
+      <c r="R806" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S806" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T806" t="inlineStr">
+        <is>
+          <t>C-341</t>
+        </is>
+      </c>
+      <c r="U806" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>Nexus Technology</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>西班牙</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr"/>
+      <c r="D807" t="inlineStr"/>
+      <c r="E807" t="inlineStr">
+        <is>
+          <t>集成商/代理（Allied Telesis）</t>
+        </is>
+      </c>
+      <c r="F807" t="inlineStr">
+        <is>
+          <t>Allied Telesis 等</t>
+        </is>
+      </c>
+      <c r="G807" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="H807" t="inlineStr">
+        <is>
+          <t>Marvell 接入层生态切入</t>
+        </is>
+      </c>
+      <c r="I807" t="inlineStr">
+        <is>
+          <t>LT-S8328XGP-4XS24GT-S</t>
+        </is>
+      </c>
+      <c r="J807" t="inlineStr">
+        <is>
+          <t>见 elioplus 渠道库</t>
+        </is>
+      </c>
+      <c r="K807" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="L807" t="inlineStr">
+        <is>
+          <t>未触达</t>
+        </is>
+      </c>
+      <c r="M807" t="inlineStr">
+        <is>
+          <t>厂商官方渠道名录</t>
+        </is>
+      </c>
+      <c r="N807" t="inlineStr"/>
+      <c r="O807" t="inlineStr"/>
+      <c r="P807" t="inlineStr"/>
+      <c r="Q807" t="inlineStr">
+        <is>
+          <t>西语区批发分销，覆盖综合布线、网络、安全、数据中心。</t>
+        </is>
+      </c>
+      <c r="R807" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="S807" t="inlineStr">
+        <is>
+          <t>【2026-09-23 复核下放】无邮箱（群发触达不到），按「B 只做群发」原则沉 C 待命；全量信息保留，出现以下任一情形可重评：①补到邮箱 ②对方主动询价 ③出现 EOL 替换需求 ④冒出内部联系人。原判：通用分销商信号，无差异化切入点，慢慢跟</t>
+        </is>
+      </c>
+      <c r="T807" t="inlineStr">
+        <is>
+          <t>C-342</t>
+        </is>
+      </c>
+      <c r="U807" t="inlineStr">
+        <is>
+          <t>B下放·无邮箱（群发触达不到）</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>